<commit_message>
radial distances plots added
</commit_message>
<xml_diff>
--- a/results/forces/force_results.xlsx
+++ b/results/forces/force_results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,65 +452,385 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>6500</v>
+        <v>3000</v>
       </c>
       <c r="B2" t="n">
-        <v>6727</v>
+        <v>5552</v>
       </c>
       <c r="C2" t="n">
-        <v>1341</v>
+        <v>1306</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>{6500: {'frame': 6500, 'ionic_force': [10.081943392753601, 8.897971272468567, -2.1222930885851383], 'ionic_force_magnitude': 13.613361204868552, 'motion_vector': [0.8403472900390625, -0.8082695007324219, 0.09564208984375], 'cosine_ionic_motion': 0.06764976203132832, 'ionic_motion_component': 0.9209406459558744, 'ionic_force_x': 10.081943392753601, 'ionic_force_y': 8.897971272468567, 'ionic_force_z': -2.1222930885851383, 'radial_force': 13.446913227219245, 'axial_force': -2.1222930885851383, 'before_closest_residue': None, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1327, 'force': [0.9640901684761047, 1.2501052618026733, -0.017418090254068375], 'magnitude': 1.5787769556045532, 'distance': 14.501358032226562, 'before_closest_residue': None, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.10932251628727493, 'motion_component': np.float64(-0.1725958601939592)}, {'ion': 1330, 'force': [1.6772516965866089, 2.190032482147217, -0.4691789448261261], 'magnitude': 2.7981324195861816, 'distance': 10.892683982849121, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.12388473780067283, 'motion_component': np.float64(-0.3466458872142508)}, {'ion': 1355, 'force': [6.430893898010254, 2.644869804382324, 1.5276371240615845], 'magnitude': 7.119368553161621, 'distance': 6.828861236572266, 'before_closest_residue': None, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.40972363875095874, 'motion_component': np.float64(2.9169735660942946)}, {'ion': 1359, 'force': [0.31147414445877075, 0.8422232866287231, -1.251532793045044], 'magnitude': 1.5403540134429932, 'distance': 14.681105613708496, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.29893736937806575, 'motion_component': np.float64(-0.4604693817881386)}, {'ion': 1465, 'force': [0.6982334852218628, 1.9707404375076294, -1.9118003845214844], 'magnitude': 2.8330776691436768, 'distance': 10.825296401977539, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.3587341555448995, 'motion_component': np.float64(-1.0163216937527935)}]}, 6501: {'frame': 6501, 'ionic_force': [10.483401834964752, 8.962290287017822, -2.592883415520191], 'ionic_force_magnitude': 14.033795125645664, 'motion_vector': [-0.46063232421875, -0.98577880859375, -0.43386077880859375], 'cosine_ionic_motion': -0.7627435020819218, 'ionic_motion_component': -10.704186041635177, 'ionic_force_x': 10.483401834964752, 'ionic_force_y': 8.962290287017822, 'ionic_force_z': -2.592883415520191, 'radial_force': 13.792184787846931, 'axial_force': -2.592883415520191, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1327, 'force': [1.1554293632507324, 1.1262601613998413, -0.06863195449113846], 'magnitude': 1.614988923072815, 'distance': 14.337858200073242, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.8524669734757304, 'motion_component': np.float64(-1.3767247427129778)}, {'ion': 1330, 'force': [2.076904535293579, 4.1037421226501465, -0.780176043510437], 'magnitude': 4.665072917938232, 'distance': 8.436062812805176, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8534071025520663, 'motion_component': np.float64(-3.9812064706752075)}, {'ion': 1355, 'force': [5.77974796295166, 0.7983136177062988, 1.5908108949661255], 'magnitude': 6.047600269317627, 'distance': 7.409305572509766, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.5843306382230081, 'motion_component': np.float64(-3.533798194344239)}, {'ion': 1359, 'force': [0.37562042474746704, 0.8487633466720581, -1.3221392631530762], 'magnitude': 1.6154077053070068, 'distance': 14.33599853515625, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.2304572530784242, 'motion_component': np.float64(-0.37228242942476975)}, {'ion': 1465, 'force': [1.0956995487213135, 2.0852110385894775, -2.012747049331665], 'magnitude': 3.0983564853668213, 'distance': 10.35150146484375, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.46481876014102497, 'motion_component': np.float64(-1.4401742463094678)}]}, 6502: {'frame': 6502, 'ionic_force': [11.625001072883606, 8.640661895275116, -4.613270215690136], 'ionic_force_magnitude': 15.201445655462445, 'motion_vector': [-0.4776763916015625, 0.31816864013671875, -0.33734130859375], 'cosine_ionic_motion': -0.12327419183801153, 'ionic_motion_component': -1.8739459279465842, 'ionic_force_x': 11.625001072883606, 'ionic_force_y': 8.640661895275116, 'ionic_force_z': -4.613270215690136, 'radial_force': 14.484532713657156, 'axial_force': -4.613270215690136, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 455, 'contributions': [{'ion': 1327, 'force': [1.3942028284072876, 1.1995381116867065, -0.08850883692502975], 'magnitude': 1.8413383960723877, 'distance': 13.427719116210938, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.20758287483310087, 'motion_component': np.float64(-0.3822303140483485)}, {'ion': 1330, 'force': [2.795842409133911, 4.828749656677246, -1.6259845495224], 'magnitude': 5.811831474304199, 'distance': 7.558098316192627, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.19367581937819087, 'motion_component': np.float64(1.1256112010987422)}, {'ion': 1355, 'force': [5.975592613220215, 0.20818573236465454, 0.7748331427574158], 'magnitude': 6.0292134284973145, 'distance': 7.420594215393066, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.7597521300040813, 'motion_component': np.float64(-4.580707757849028)}, {'ion': 1359, 'force': [0.39647555351257324, 0.6920130252838135, -1.412355661392212], 'magnitude': 1.6219812631607056, 'distance': 14.30691909790039, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.46974438467694246, 'motion_component': np.float64(0.7619166176325294)}, {'ion': 1465, 'force': [1.0628876686096191, 1.7121753692626953, -2.26125431060791], 'magnitude': 3.028951406478882, 'distance': 10.469426155090332, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.39666013784961557, 'motion_component': np.float64(1.2014642251812404)}]}, 6503: {'frame': 6503, 'ionic_force': [11.245525926351547, 9.056975424289703, -5.633130252361298], 'ionic_force_magnitude': 15.499122995721422, 'motion_vector': [0.24894332885742188, 0.13856887817382812, -0.48906707763671875], 'cosine_ionic_motion': 0.7762256271430822, 'ionic_motion_component': 12.030816467521626, 'ionic_force_x': 11.245525926351547, 'ionic_force_y': 9.056975424289703, 'ionic_force_z': -5.633130252361298, 'radial_force': 14.439205559740207, 'axial_force': -5.633130252361298, 'before_closest_residue': 423, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1327, 'force': [1.3975937366485596, 1.4927356243133545, -0.144304096698761], 'magnitude': 2.0499637126922607, 'distance': 12.726118087768555, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1105, 'cosine_with_motion': 0.538954731470277, 'motion_component': np.float64(1.1048376877525996)}, {'ion': 1330, 'force': [2.3191373348236084, 4.516908645629883, -2.2384073734283447], 'magnitude': 5.5489935874938965, 'distance': 7.7350287437438965, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.7316614144844448, 'motion_component': np.float64(4.059984459355739)}, {'ion': 1355, 'force': [6.450555324554443, 0.437552273273468, 0.7234834432601929], 'magnitude': 6.50573205947876, 'distance': 7.14366340637207, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 130, 'cosine_with_motion': 0.3564707452300667, 'motion_component': np.float64(2.3191030089353406)}, {'ion': 1359, 'force': [0.3285345733165741, 0.7057961225509644, -1.4670779705047607], 'magnitude': 1.6608434915542603, 'distance': 14.138544082641602, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.9543033380850897, 'motion_component': np.float64(1.5849484307332196)}, {'ion': 1465, 'force': [0.7497049570083618, 1.9039827585220337, -2.506824254989624], 'magnitude': 3.235950469970703, 'distance': 10.129035949707031, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.9153239264090328, 'motion_component': np.float64(2.9619429278287637)}]}, 6504: {'frame': 6504, 'ionic_force': [9.827082395553589, 8.0006403028965, -3.616157114505768], 'ionic_force_magnitude': 13.177950748964033, 'motion_vector': [-1.3946723937988281, 1.9302940368652344, 2.1039581298828125], 'cosine_ionic_motion': -0.14018226200391393, 'ionic_motion_component': -1.8473149445659498, 'ionic_force_x': 9.827082395553589, 'ionic_force_y': 8.0006403028965, 'ionic_force_z': -3.616157114505768, 'radial_force': 12.672087186621274, 'axial_force': -3.616157114505768, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 423, 'contributions': [{'ion': 1327, 'force': [1.2314133644104004, 1.187270998954773, -0.10812932252883911], 'magnitude': 1.7139670848846436, 'distance': 13.917710304260254, 'before_closest_residue': 1073, 'closest_residue': 1105, 'next_closest_residue': 1073, 'cosine_with_motion': 0.0636860082514764, 'motion_component': np.float64(0.10915572342171842)}, {'ion': 1330, 'force': [2.0249695777893066, 4.583828449249268, -1.6436532735824585], 'magnitude': 5.273858547210693, 'distance': 7.934230327606201, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.15310153127654202, 'motion_component': np.float64(0.8074357779586236)}, {'ion': 1355, 'force': [5.697000026702881, 0.46980372071266174, 0.2337888479232788], 'magnitude': 5.72111701965332, 'distance': 7.617783069610596, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 98, 'cosine_with_motion': -0.36010487446415945, 'motion_component': np.float64(-2.060202192659389)}, {'ion': 1465, 'force': [0.873699426651001, 1.7597371339797974, -2.098163366317749], 'magnitude': 2.8744242191314697, 'distance': 10.747157096862793, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.24481573853975963, 'motion_component': np.float64(-0.7037043046516871)}]}, 6505: {'frame': 6505, 'ionic_force': [8.95492085814476, 11.337874174118042, 0.06668233871459961], 'ionic_force_magnitude': 14.447921819350539, 'motion_vector': [1.2258834838867188, -0.9209442138671875, -0.31507110595703125], 'cosine_ionic_motion': 0.02277776321583095, 'ionic_motion_component': 0.3290913421620041, 'ionic_force_x': 8.95492085814476, 'ionic_force_y': 11.337874174118042, 'ionic_force_z': 0.06668233871459961, 'radial_force': 14.447767937081801, 'axial_force': 0.06668233871459961, 'before_closest_residue': 455, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1327, 'force': [0.9046583771705627, 1.2874258756637573, 0.10324346274137497], 'magnitude': 1.5768738985061646, 'distance': 14.51010513305664, 'before_closest_residue': 1105, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.04422916059227101, 'motion_component': np.float64(-0.06974381009018105)}, {'ion': 1330, 'force': [0.6813580989837646, 3.155944347381592, 0.12422109395265579], 'magnitude': 3.2310469150543213, 'distance': 10.13671875, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': 455, 'cosine_with_motion': -0.41725808914305246, 'motion_component': np.float64(-1.348180480801879)}, {'ion': 1355, 'force': [6.1667399406433105, 2.169691562652588, 2.961028575897217], 'magnitude': 7.176624298095703, 'distance': 6.801566123962402, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.41203043851929855, 'motion_component': np.float64(2.956987567178629)}, {'ion': 1359, 'force': [0.27677449584007263, 1.2362631559371948, -1.4230068922042847], 'magnitude': 1.9052294492721558, 'distance': 13.200652122497559, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.11765770814868194, 'motion_component': np.float64(-0.22416493275781235)}, {'ion': 1465, 'force': [0.9253899455070496, 3.48854923248291, -1.6988039016723633], 'magnitude': 3.9890170097351074, 'distance': 9.122966766357422, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.24713040678039583, 'motion_component': np.float64(-0.9858074052864723)}]}, 6506: {'frame': 6506, 'ionic_force': [8.623957008123398, 13.234449625015259, -0.39382988307625055], 'ionic_force_magnitude': 15.80121493214465, 'motion_vector': [0.202423095703125, -0.7250022888183594, -0.397186279296875], 'cosine_ionic_motion': -0.5720341661698859, 'ionic_motion_component': -9.038834808180514, 'ionic_force_x': 8.623957008123398, 'ionic_force_y': 13.234449625015259, 'ionic_force_z': -0.39382988307625055, 'radial_force': 15.796306256686314, 'axial_force': -0.39382988307625055, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1327, 'force': [1.1759207248687744, 1.295444130897522, 0.006512581370770931], 'magnitude': 1.7495734691619873, 'distance': 13.775360107421875, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.4726186239400156, 'motion_component': np.float64(-0.8268810240048633)}, {'ion': 1330, 'force': [0.41796424984931946, 5.998465061187744, 1.121175765991211], 'magnitude': 6.116641998291016, 'distance': 7.36737060546875, 'before_closest_residue': None, 'closest_residue': 455, 'next_closest_residue': 780, 'cosine_with_motion': -0.9046792344213612, 'motion_component': np.float64(-5.533599219691718)}, {'ion': 1355, 'force': [5.303382396697998, 1.6648468971252441, 1.7273120880126953], 'magnitude': 5.8207550048828125, 'distance': 7.552302837371826, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 130, 'cosine_with_motion': -0.16543281645221253, 'motion_component': np.float64(-0.9629438695954278)}, {'ion': 1359, 'force': [0.40036541223526, 1.0453904867172241, -1.4302330017089844], 'magnitude': 1.816232442855835, 'distance': 13.520206451416016, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.07038395043073115, 'motion_component': np.float64(-0.12783361201448695)}, {'ion': 1465, 'force': [1.326324224472046, 3.2303030490875244, -1.8185973167419434], 'magnitude': 3.9371676445007324, 'distance': 9.182841300964355, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.403228158784902, 'motion_component': np.float64(-1.587576905024907)}]}, 6507: {'frame': 6507, 'ionic_force': [7.709233671426773, 10.224741399288177, -1.3882663254626095], 'ionic_force_magnitude': 12.880407752605946, 'motion_vector': [-0.5508842468261719, 0.7071418762207031, 0.5803451538085938], 'cosine_ionic_motion': 0.15833213834327778, 'ionic_motion_component': 2.039382502203432, 'ionic_force_x': 7.709233671426773, 'ionic_force_y': 10.224741399288177, 'ionic_force_z': -1.3882663254626095, 'radial_force': 12.805374671714134, 'axial_force': -1.3882663254626095, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1327, 'force': [1.2036428451538086, 1.2521858215332031, 0.005354940425604582], 'magnitude': 1.7368805408477783, 'distance': 13.825602531433105, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.12158704527623818, 'motion_component': np.float64(0.21118217619887092)}, {'ion': 1330, 'force': [-0.9935824275016785, 3.679025411605835, 0.9656086564064026], 'magnitude': 3.9312636852264404, 'distance': 9.18973445892334, 'before_closest_residue': 455, 'closest_residue': 780, 'next_closest_residue': 748, 'cosine_with_motion': 0.8835863573943219, 'motion_component': np.float64(3.47361095217196)}, {'ion': 1355, 'force': [5.284008026123047, 0.8967590928077698, 1.443036437034607], 'magnitude': 5.550429821014404, 'distance': 7.734027862548828, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 98, 'cosine_with_motion': -0.24283154513861926, 'motion_component': np.float64(-1.3478194638669372)}, {'ion': 1359, 'force': [0.4560973346233368, 1.0773588418960571, -1.6211364269256592], 'magnitude': 1.9992023706436157, 'distance': 12.886669158935547, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.20152537909680956, 'motion_component': np.float64(-0.402890018093796)}, {'ion': 1465, 'force': [1.7590678930282593, 3.3194122314453125, -2.1811299324035645], 'magnitude': 4.343977928161621, 'distance': 8.742290496826172, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.024240219321329245, 'motion_component': np.float64(0.10529898037360397)}]}, 6508: {'frame': 6508, 'ionic_force': [8.196879386901855, 9.545158863067627, -0.8453916572034359], 'ionic_force_magnitude': 12.610058543031597, 'motion_vector': [0.4479179382324219, -0.00655364990234375, -0.4083099365234375], 'cosine_ionic_motion': 0.5173359934108689, 'ionic_motion_component': 6.523637163328465, 'ionic_force_x': 8.196879386901855, 'ionic_force_y': 9.545158863067627, 'ionic_force_z': -0.8453916572034359, 'radial_force': 12.581688654732123, 'axial_force': -0.8453916572034359, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1327, 'force': [1.1328179836273193, 1.335171103477478, 0.0463273860514164], 'magnitude': 1.7516005039215088, 'distance': 13.767386436462402, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.4518662415614668, 'motion_component': np.float64(0.7914891829820513)}, {'ion': 1330, 'force': [-0.5327326059341431, 1.9765138626098633, 0.0836285948753357], 'magnitude': 2.0487568378448486, 'distance': 12.729866027832031, 'before_closest_residue': 780, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.2300841228810292, 'motion_component': np.float64(-0.4713864334961526)}, {'ion': 1355, 'force': [6.056460857391357, 1.6252504587173462, 2.4695639610290527], 'magnitude': 6.739502906799316, 'distance': 7.018674850463867, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.41463880587954705, 'motion_component': np.float64(2.7944595573921855)}, {'ion': 1359, 'force': [0.32606077194213867, 1.136378526687622, -1.499696135520935], 'magnitude': 1.9096492528915405, 'distance': 13.185367584228516, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.6487670122404887, 'motion_component': np.float64(1.2389174423903972)}, {'ion': 1465, 'force': [1.214272379875183, 3.4718449115753174, -1.9452154636383057], 'magnitude': 4.160772323608398, 'distance': 8.932685852050781, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5215755781755362, 'motion_component': np.float64(2.1701573164389067)}]}, 6509: {'frame': 6509, 'ionic_force': [8.639954075217247, 9.225626826286316, -1.5821315594948828], 'ionic_force_magnitude': 12.738294117789343, 'motion_vector': [0.6326484680175781, 0.24243927001953125, -0.14005279541015625], 'cosine_ionic_motion': 0.8991798414206716, 'ionic_motion_component': 11.454017284803696, 'ionic_force_x': 8.639954075217247, 'ionic_force_y': 9.225626826286316, 'ionic_force_z': -1.5821315594948828, 'radial_force': 12.63965967737094, 'axial_force': -1.5821315594948828, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1327, 'force': [1.1541346311569214, 1.2506356239318848, -0.005397135857492685], 'magnitude': 1.7018065452575684, 'distance': 13.967348098754883, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.8783315356447652, 'motion_component': np.float64(1.4947503104034952)}, {'ion': 1330, 'force': [-0.1657009869813919, 2.027735710144043, 0.1610119342803955], 'magnitude': 2.040856122970581, 'distance': 12.75448226928711, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 455, 'cosine_with_motion': 0.2579594262839983, 'motion_component': np.float64(0.5264580781231629)}, {'ion': 1355, 'force': [5.690523624420166, 1.5907838344573975, 1.5250321626663208], 'magnitude': 6.102325439453125, 'distance': 7.376007556915283, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.8935009839525232, 'motion_component': np.float64(5.452433759382151)}, {'ion': 1359, 'force': [0.4454243779182434, 1.0431405305862427, -1.415763020515442], 'magnitude': 1.8140920400619507, 'distance': 13.528180122375488, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5840209254987284, 'motion_component': np.float64(1.0594677191690547)}, {'ion': 1465, 'force': [1.515572428703308, 3.313331127166748, -1.8470155000686646], 'magnitude': 4.084921836853027, 'distance': 9.015236854553223, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.7150459892242651, 'motion_component': np.float64(2.92090721985379)}]}, 6510: {'frame': 6510, 'ionic_force': [8.169408738613129, 10.510639429092407, -0.9569092690944672], 'ionic_force_magnitude': 13.34647727665242, 'motion_vector': [-0.5427474975585938, -0.5374031066894531, -0.217681884765625], 'cosine_ionic_motion': -0.9315300525098844, 'ionic_motion_component': -12.432644678342008, 'ionic_force_x': 8.169408738613129, 'ionic_force_y': 10.510639429092407, 'ionic_force_z': -0.9569092690944672, 'radial_force': 13.312129068895047, 'axial_force': -0.9569092690944672, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1327, 'force': [1.0011017322540283, 1.0972646474838257, 0.06368693709373474], 'magnitude': 1.4866911172866821, 'distance': 14.943717956542969, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.9713265624370541, 'motion_component': np.float64(-1.4440625503671303)}, {'ion': 1330, 'force': [-0.3688025176525116, 4.693726539611816, 0.4749440550804138], 'magnitude': 4.732088088989258, 'distance': 8.376114845275879, 'before_closest_residue': 748, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': -0.6454182627521611, 'motion_component': np.float64(-3.0541759575970087)}, {'ion': 1355, 'force': [5.465493679046631, 0.39318275451660156, 1.7694438695907593], 'magnitude': 5.758224010467529, 'distance': 7.593198776245117, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.7790707398781728, 'motion_component': np.float64(-4.486063954346015)}, {'ion': 1359, 'force': [0.4867585003376007, 1.0545459985733032, -1.4388798475265503], 'magnitude': 1.8491555452346802, 'distance': 13.399306297302246, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.35250023319791834, 'motion_component': np.float64(-0.6518277691022636)}, {'ion': 1465, 'force': [1.5848573446273804, 3.2719194889068604, -1.8261042833328247], 'magnitude': 4.068401336669922, 'distance': 9.033523559570312, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6873743841577581, 'motion_component': np.float64(-2.7965146404573744)}]}, 6511: {'frame': 6511, 'ionic_force': [9.239876329898834, 10.888403117656708, -0.996029619127512], 'ionic_force_magnitude': 14.3151916524579, 'motion_vector': [-0.13922500610351562, -0.4607810974121094, -0.42333984375], 'cosine_ionic_motion': -0.6409801106238094, 'ionic_motion_component': -9.175753128993499, 'ionic_force_x': 9.239876329898834, 'ionic_force_y': 10.888403117656708, 'ionic_force_z': -0.996029619127512, 'radial_force': 14.280498487252505, 'axial_force': -0.996029619127512, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1327, 'force': [0.9707937836647034, 1.2145224809646606, -0.004816416651010513], 'magnitude': 1.5548404455184937, 'distance': 14.612554550170898, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.6950428688930558, 'motion_component': np.float64(-1.0806807223558081)}, {'ion': 1330, 'force': [0.5534781217575073, 3.8982489109039307, 0.9348843097686768], 'magnitude': 4.046812534332275, 'distance': 9.057586669921875, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 780, 'cosine_with_motion': -0.874695048431411, 'motion_component': np.float64(-3.5397268411039313)}, {'ion': 1355, 'force': [5.989511966705322, 1.8379708528518677, 1.4910531044006348], 'magnitude': 6.440157413482666, 'distance': 7.1799397468566895, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.5600356041623372, 'motion_component': np.float64(-3.6067175481792972)}, {'ion': 1359, 'force': [0.3790135383605957, 0.935649573802948, -1.3818391561508179], 'magnitude': 1.7113068103790283, 'distance': 13.928524017333984, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.09215119369332977, 'motion_component': np.float64(0.15769896108285408)}, {'ion': 1465, 'force': [1.3470789194107056, 3.002011299133301, -2.035311460494995], 'magnitude': 3.8690032958984375, 'distance': 9.26338005065918, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.2859462078220281, 'motion_component': np.float64(-1.106326809160759)}]}, 6512: {'frame': 6512, 'ionic_force': [9.70670634508133, 9.800261974334717, -2.381965771317482], 'ionic_force_magnitude': 13.997822822530697, 'motion_vector': [0.5918121337890625, 0.91455078125, 0.193389892578125], 'cosine_ionic_motion': 0.9199332606195443, 'ionic_motion_component': 12.877062790705336, 'ionic_force_x': 9.70670634508133, 'ionic_force_y': 9.800261974334717, 'ionic_force_z': -2.381965771317482, 'radial_force': 13.793668215352765, 'axial_force': -2.381965771317482, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1327, 'force': [1.3225460052490234, 1.2799756526947021, -0.04935155808925629], 'magnitude': 1.8411684036254883, 'distance': 13.428338050842285, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.9542232735745532, 'motion_component': np.float64(1.7568857654786743)}, {'ion': 1330, 'force': [0.5024370551109314, 3.6082277297973633, 0.4674486815929413], 'magnitude': 3.6729087829589844, 'distance': 9.507448196411133, 'before_closest_residue': 455, 'closest_residue': 780, 'next_closest_residue': 'SF', 'cosine_with_motion': 0.9074896578601978, 'motion_component': np.float64(3.3331266960591543)}, {'ion': 1355, 'force': [6.186309337615967, 0.9965171813964844, 1.0365417003631592], 'magnitude': 6.3512115478515625, 'distance': 7.230040550231934, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.679254058319942, 'motion_component': np.float64(4.314086234341268)}, {'ion': 1359, 'force': [0.3710061311721802, 0.939140796661377, -1.5384976863861084], 'magnitude': 1.840273380279541, 'distance': 13.431604385375977, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.38355716263184525, 'motion_component': np.float64(0.7058500364331834)}, {'ion': 1465, 'force': [1.3244078159332275, 2.97640061378479, -2.2981069087982178], 'magnitude': 3.986767053604126, 'distance': 9.125540733337402, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.6940747888775192, 'motion_component': np.float64(2.767114544662796)}]}, 6513: {'frame': 6513, 'ionic_force': [8.1560879945755, 11.545685350894928, -1.4180030822753906], 'ionic_force_magnitude': 14.206877008634617, 'motion_vector': [0.8010101318359375, -0.8122329711914062, -0.20128631591796875], 'cosine_ionic_motion': -0.15551117028458428, 'ionic_motion_component': -2.209328069701923, 'ionic_force_x': 8.1560879945755, 'ionic_force_y': 11.545685350894928, 'ionic_force_z': -1.4180030822753906, 'radial_force': 14.135933700931409, 'axial_force': -1.4180030822753906, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1330, 'force': [1.3748646974563599, 6.309800148010254, 0.5138952732086182], 'magnitude': 6.478265285491943, 'distance': 7.1587910652160645, 'before_closest_residue': 780, 'closest_residue': 'SF', 'next_closest_residue': 780, 'cosine_with_motion': -0.5499744294061559, 'motion_component': np.float64(-3.562880172717495)}, {'ion': 1355, 'force': [4.779118061065674, 1.3160141706466675, 1.0592595338821411], 'magnitude': 5.068914413452148, 'distance': 8.093037605285645, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 130, 'cosine_with_motion': 0.43360080452607963, 'motion_component': np.float64(2.1978853749391742)}, {'ion': 1359, 'force': [0.449627161026001, 0.992048442363739, -1.3071831464767456], 'magnitude': 1.7014853954315186, 'distance': 13.968666076660156, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.09259397836105233, 'motion_component': np.float64(-0.15754729980454307)}, {'ion': 1465, 'force': [1.5524780750274658, 2.9278225898742676, -1.6839747428894043], 'magnitude': 3.717271089553833, 'distance': 9.450546264648438, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.184755329899073, 'motion_component': np.float64(-0.686785643310678)}]}, 6514: {'frame': 6514, 'ionic_force': [7.400987505912781, 7.646649926900864, -1.3441858291625977], 'ionic_force_magnitude': 10.726262476304205, 'motion_vector': [-0.7476043701171875, -0.9638442993164062, 0.5952987670898438], 'cosine_ionic_motion': -0.9412403328787488, 'ionic_motion_component': -10.095990863741402, 'ionic_force_x': 7.400987505912781, 'ionic_force_y': 7.646649926900864, 'ionic_force_z': -1.3441858291625977, 'radial_force': 10.64170433564333, 'axial_force': -1.3441858291625977, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1330, 'force': [0.8154507875442505, 3.8844902515411377, 1.2020996809005737], 'magnitude': 4.147200107574463, 'distance': 8.947290420532227, 'before_closest_residue': 'SF', 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.6463045514988436, 'motion_component': np.float64(-2.6803542596674426)}, {'ion': 1355, 'force': [4.358066082000732, 0.3850259482860565, 0.6954754590988159], 'magnitude': 4.42997407913208, 'distance': 8.657020568847656, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 130, 'cosine_with_motion': -0.534721682356506, 'motion_component': np.float64(-2.368803236348027)}, {'ion': 1359, 'force': [0.5083365440368652, 0.913629412651062, -1.3647812604904175], 'magnitude': 1.7192302942276, 'distance': 13.896390914916992, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8883906186024271, 'motion_component': np.float64(-1.5273480207018046)}, {'ion': 1465, 'force': [1.7191340923309326, 2.4635043144226074, -1.8769797086715698], 'magnitude': 3.5422208309173584, 'distance': 9.681245803833008, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.9935816073151836, 'motion_component': np.float64(-3.51</t>
+          <t>{3000: {'frame': 3000, 'ionic_force': [-2.0055387914180756, -9.355347752571106, -5.252918437123299], 'ionic_force_magnitude': 10.915029524581682, 'motion_vector': [0.024631500244140625, 0.30776214599609375, -0.1444854736328125], 'cosine_ionic_motion': -0.5831245588979053, 'ionic_motion_component': -6.364821776879306, 'ionic_force_x': -2.0055387914180756, 'ionic_force_y': -9.355347752571106, 'ionic_force_z': -5.252918437123299, 'radial_force': 9.567900366089727, 'axial_force': -5.252918437123299, 'before_closest_residue': None, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1305, 'force': [-1.338510513305664, -4.348547458648682, -1.8191893100738525], 'magnitude': 4.900094509124756, 'distance': 8.231269836425781, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6635973801547728, 'motion_component': -3.251689807117941}, {'ion': 1307, 'force': [0.29505655169487, -1.8750426769256592, 0.13831393420696259], 'magnitude': 1.9031484127044678, 'distance': 13.207867622375488, 'before_closest_residue': None, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.9091102591232869, 'motion_component': -1.7301718117342832}, {'ion': 1313, 'force': [-0.332777202129364, -1.0366517305374146, -1.5025314092636108], 'magnitude': 1.8555290699005127, 'distance': 13.376274108886719, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.17413794403402547, 'motion_component': -0.32311801654238526}, {'ion': 2433, 'force': [-0.6293076276779175, -2.0951058864593506, -2.069511651992798], 'magnitude': 3.0113744735717773, 'distance': 10.499937057495117, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.3519462991251713, 'motion_component': -1.0598420441839398}]}, 3001: {'frame': 3001, 'ionic_force': [-1.7987768054008484, -9.250487446784973, -5.685618311166763], 'ionic_force_magnitude': 11.006060674875878, 'motion_vector': [0.4005584716796875, 0.21022796630859375, 0.6815719604492188], 'cosine_ionic_motion': -0.7264385017949461, 'ionic_motion_component': -7.995226227321106, 'ionic_force_x': -1.7987768054008484, 'ionic_force_y': -9.250487446784973, 'ionic_force_z': -5.685618311166763, 'radial_force': 9.423752755605086, 'axial_force': -5.685618311166763, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1305, 'force': [-1.2598000764846802, -4.045856952667236, -1.9470460414886475], 'magnitude': 4.66337251663208, 'distance': 8.437601089477539, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7031096133565167, 'motion_component': -3.278862029990396}, {'ion': 1307, 'force': [0.42661887407302856, -1.954982876777649, 0.08282431960105896], 'magnitude': 2.0027036666870117, 'distance': 12.875399589538574, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.11210237590554617, 'motion_component': -0.22450782817503345}, {'ion': 1313, 'force': [-0.310261070728302, -1.0852751731872559, -1.5717225074768066], 'magnitude': 1.9350441694259644, 'distance': 13.09856128692627, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8993886874713677, 'motion_component': -1.7403567977253491}, {'ion': 2433, 'force': [-0.6553345322608948, -2.164372444152832, -2.249674081802368], 'magnitude': 3.1898281574249268, 'distance': 10.202001571655273, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.862585429192802, 'motion_component': -2.7514994560726382}]}, 3002: {'frame': 3002, 'ionic_force': [-2.6747649759054184, -12.456079721450806, -6.5811577886343], 'ionic_force_magnitude': 14.339453530116488, 'motion_vector': [0.13358688354492188, -0.9328022003173828, -0.378326416015625], 'cosine_ionic_motion': 0.9444306854503265, 'ionic_motion_component': 13.54261992643102, 'ionic_force_x': -2.6747649759054184, 'ionic_force_y': -12.456079721450806, 'ionic_force_z': -6.5811577886343, 'radial_force': 12.740027068396216, 'axial_force': -6.5811577886343, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1305, 'force': [-1.6123325824737549, -5.863553047180176, -0.9820989370346069], 'magnitude': 6.159982681274414, 'distance': 7.34140682220459, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.8993891749766614, 'motion_component': 5.540221915483258}, {'ion': 1307, 'force': [0.4164557456970215, -1.7535215616226196, 0.1588585525751114], 'magnitude': 1.8092842102050781, 'distance': 13.546142578125, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.8878845784434418, 'motion_component': 1.606435533939714}, {'ion': 1313, 'force': [-0.403207391500473, -1.379842758178711, -1.9157507419586182], 'magnitude': 2.3951289653778076, 'distance': 11.773472785949707, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.8050858417995584, 'motion_component': 1.9282844835756299}, {'ion': 1460, 'force': [-0.19490917026996613, -0.6853560209274292, -1.3463873863220215], 'magnitude': 1.523306131362915, 'distance': 14.763028144836426, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.7257766907021649, 'motion_component': 1.1055800553786388}, {'ion': 2433, 'force': [-0.8807715773582458, -2.77380633354187, -2.495779275894165], 'magnitude': 3.8338849544525146, 'distance': 9.305709838867188, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.8769428583860391, 'motion_component': 3.3620980875768307}]}, 3003: {'frame': 3003, 'ionic_force': [-1.1474620401859283, -9.749491453170776, -5.080912113189697], 'ionic_force_magnitude': 11.0537288111784, 'motion_vector': [-0.7327499389648438, 0.2111797332763672, -0.0490264892578125], 'cosine_ionic_motion': -0.11471866276502497, 'ionic_motion_component': -1.2680689877856153, 'ionic_force_x': -1.1474620401859283, 'ionic_force_y': -9.749491453170776, 'ionic_force_z': -5.080912113189697, 'radial_force': 9.81678423564039, 'axial_force': -5.080912113189697, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1305, 'force': [-0.8707835078239441, -4.788753032684326, -1.3522531986236572], 'magnitude': 5.051634311676025, 'distance': 8.106867790222168, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.07951011180184486, 'motion_component': -0.4016560011896875}, {'ion': 1307, 'force': [0.4663363993167877, -1.546359658241272, 0.07744836807250977], 'magnitude': 1.6170021295547485, 'distance': 14.32892894744873, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.5439046782712613, 'motion_component': -0.8794950554476717}, {'ion': 1313, 'force': [-0.258034348487854, -1.1367427110671997, -1.6128792762756348], 'magnitude': 1.99001145362854, 'distance': 12.916393280029297, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.018473133544180807, 'motion_component': 0.036761745900474097}, {'ion': 2433, 'force': [-0.48498058319091797, -2.2776360511779785, -2.193228006362915], 'magnitude': 3.1989188194274902, 'distance': 10.187495231628418, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.0074024147240997155, 'motion_component': -0.023679723333129843}]}, 3004: {'frame': 3004, 'ionic_force': [-2.022185653448105, -9.561164498329163, -4.9194693602621555], 'ionic_force_magnitude': 10.941036521631734, 'motion_vector': [-0.24576187133789062, 0.10697555541992188, -0.01856231689453125], 'cosine_ionic_motion': -0.14781520566090017, 'ionic_motion_component': -1.6172515635884146, 'ionic_force_x': -2.022185653448105, 'ionic_force_y': -9.561164498329163, 'ionic_force_z': -4.9194693602621555, 'radial_force': 9.772671148724964, 'axial_force': -4.9194693602621555, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 1105, 'contributions': [{'ion': 1305, 'force': [-1.385051965713501, -4.45631217956543, -1.491028904914856], 'magnitude': 4.89900541305542, 'distance': 8.232184410095215, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.08254255206962378, 'motion_component': -0.4043764123249529}, {'ion': 1307, 'force': [0.3731239438056946, -1.9103577136993408, 0.05936693772673607], 'magnitude': 1.9473603963851929, 'distance': 13.057074546813965, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.5679609815258614, 'motion_component': -1.1060247208930802}, {'ion': 1313, 'force': [-0.36821165680885315, -1.061498761177063, -1.5287107229232788], 'magnitude': 1.8971863985061646, 'distance': 13.228605270385742, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.010425866150245287, 'motion_component': 0.01977981059531242}, {'ion': 2433, 'force': [-0.6420459747314453, -2.132995843887329, -1.9590966701507568], 'magnitude': 2.9664714336395264, 'distance': 10.579105377197266, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.04268717739586549, 'motion_component': -0.12663030168172362}]}, 3005: {'frame': 3005, 'ionic_force': [-2.272895395755768, -9.669207692146301, -4.632208496332169], 'ionic_force_magnitude': 10.95978952477651, 'motion_vector': [0.5893363952636719, 0.39318084716796875, 0.4419708251953125], 'cosine_ionic_motion': -0.7854991608957079, 'ionic_motion_component': -8.608905475305518, 'ionic_force_x': -2.272895395755768, 'ionic_force_y': -9.669207692146301, 'ionic_force_z': -4.632208496332169, 'radial_force': 9.932755452235243, 'axial_force': -4.632208496332169, 'before_closest_residue': 780, 'closest_residue': 1105, 'next_closest_residue': 780, 'contributions': [{'ion': 1305, 'force': [-1.5205748081207275, -4.809185981750488, -1.187056064605713], 'magnitude': 5.181652069091797, 'distance': 8.004512786865234, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7653911936741354, 'motion_component': -3.9659909723783358}, {'ion': 1307, 'force': [0.34922900795936584, -1.6264971494674683, 0.19030365347862244], 'magnitude': 1.674416184425354, 'distance': 14.081124305725098, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 130, 'cosine_with_motion': -0.25003267788013345, 'motion_component': -0.4186587474770729}, {'ion': 1313, 'force': [-0.39352306723594666, -1.1050562858581543, -1.597266674041748], 'magnitude': 1.981734275817871, 'distance': 12.943339347839355, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.829327631882084, 'motion_component': -1.6435069704258574}, {'ion': 2433, 'force': [-0.7080265283584595, -2.1284682750701904, -2.03818941116333], 'magnitude': 3.0308241844177246, 'distance': 10.466191291809082, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8515007583172389, 'motion_component': -2.5807490354166873}]}, 3006: {'frame': 3006, 'ionic_force': [-2.148721843957901, -10.554901480674744, -6.08821539580822], 'ionic_force_magnitude': 12.37292679745613, 'motion_vector': [0.427276611328125, 1.7292823791503906, -1.6639404296875], 'cosine_ionic_motion': -0.2997401968827221, 'ionic_motion_component': -3.708663514285008, 'ionic_force_x': -2.148721843957901, 'ionic_force_y': -10.554901480674744, 'ionic_force_z': -6.08821539580822, 'radial_force': 10.771395027082228, 'axial_force': -6.08821539580822, 'before_closest_residue': 1105, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1305, 'force': [-1.4315390586853027, -5.059445858001709, -2.0888192653656006], 'magnitude': 5.657778739929199, 'distance': 7.660305023193359, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.42673747944869317, 'motion_component': -2.414386318704686}, {'ion': 1307, 'force': [0.4035383462905884, -1.9195414781570435, 0.24027784168720245], 'magnitude': 1.9761619567871094, 'distance': 12.96157455444336, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 98, 'cosine_with_motion': -0.736311037040692, 'motion_component': -1.4550698681541725}, {'ion': 1313, 'force': [-0.3729988634586334, -1.161724328994751, -1.7436925172805786], 'magnitude': 2.128190517425537, 'distance': 12.49003791809082, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.14131385137704483, 'motion_component': 0.3007428079462997}, {'ion': 2433, 'force': [-0.7477222681045532, -2.4141898155212402, -2.495981454849243], 'magnitude': 3.5520873069763184, 'distance': 9.667790412902832, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.039399304406863365, 'motion_component': -0.13994977043029166}]}, 3007: {'frame': 3007, 'ionic_force': [-1.2613288164138794, -9.13017863035202, -8.179755677469075], 'ionic_force_magnitude': 12.323129275810599, 'motion_vector': [0.9349288940429688, -0.6350440979003906, 0.477752685546875], 'cosine_ionic_motion': 0.047015133551017024, 'ionic_motion_component': 0.5793735686686831, 'ionic_force_x': -1.2613288164138794, 'ionic_force_y': -9.13017863035202, 'ionic_force_z': -8.179755677469075, 'radial_force': 9.216892763033144, 'axial_force': -8.179755677469075, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1305, 'force': [-0.9955459237098694, -4.762621879577637, -3.790351390838623], 'magnitude': 6.167693614959717, 'distance': 7.336816310882568, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.03737578009319252, 'motion_component': 0.23052235415094915}, {'ion': 1307, 'force': [0.4332018792629242, -1.9774179458618164, -0.002815951593220234], 'magnitude': 2.024315595626831, 'distance': 12.806485176086426, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 130, 'cosine_with_motion': 0.6680654760734864, 'motion_component': 1.3523753455646768}, {'ion': 1313, 'force': [-0.21243613958358765, -0.746026337146759, -1.7458677291870117], 'magnitude': 1.9104288816452026, 'distance': 13.182676315307617, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.23844116329659729, 'motion_component': -0.4555248865019088}, {'ion': 2433, 'force': [-0.48654863238334656, -1.644112467765808, -2.6407206058502197], 'magnitude': 3.1485297679901123, 'distance': 10.268692016601562, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.1740493160935444, 'motion_component': -0.5479994803640693}]}, 3008: {'frame': 3008, 'ionic_force': [0.005047585815191269, -11.746112525463104, -6.980247122235596], 'ionic_force_magnitude': 13.663639150184043, 'motion_vector': [-0.9179306030273438, 0.7456550598144531, -0.105194091796875], 'cosine_ionic_motion': -0.4949164773646154, 'ionic_motion_component': -6.762360156190334, 'ionic_force_x': 0.005047585815191269, 'ionic_force_y': -11.746112525463104, 'ionic_force_z': -6.980247122235596, 'radial_force': 11.746113609997298, 'axial_force': -6.980247122235596, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1305, 'force': [-0.47162288427352905, -6.657526016235352, -2.6302850246429443], 'magnitude': 7.173804759979248, 'distance': 6.802902698516846, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.49951949610591684, 'motion_component': -3.5834555261181933}, {'ion': 1307, 'force': [0.693957507610321, -2.034898281097412, 0.0119145093485713], 'magnitude': 2.1500070095062256, 'distance': 12.426507949829102, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 130, 'cosine_with_motion': -0.844439576304053, 'motion_component': -1.815550978973864}, {'ion': 1313, 'force': [-0.06039971485733986, -0.998511016368866, -1.829248070716858], 'magnitude': 2.0849030017852783, 'distance': 12.619033813476562, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.20064552868436059, 'motion_component': -0.41832648202185685}, {'ion': 2433, 'force': [-0.15688732266426086, -2.0551772117614746, -2.5326285362243652], 'magnitude': 3.265359878540039, 'distance': 10.083319664001465, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.2894098793691679, 'motion_component': -0.9450273717580888}]}, 3009: {'frame': 3009, 'ionic_force': [-2.8977731317281723, -12.583130359649658, -9.118463832885027], 'ionic_force_magnitude': 15.807550140440325, 'motion_vector': [0.6446266174316406, -0.28569793701171875, -0.4042816162109375], 'cosine_ionic_motion': 0.4213417086883455, 'ionic_motion_component': 6.660380186349822, 'ionic_force_x': -2.8977731317281723, 'ionic_force_y': -12.583130359649658, 'ionic_force_z': -9.118463832885027, 'radial_force': 12.912484608738266, 'axial_force': -9.118463832885027, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1305, 'force': [-2.659644603729248, -7.628777503967285, -4.108871936798096], 'magnitude': 9.06392765045166, 'distance': 6.052165985107422, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.28861099210636953, 'motion_component': 2.615949147813012}, {'ion': 1307, 'force': [0.5262024998664856, -2.080961227416992, 0.009617727249860764], 'magnitude': 2.1464810371398926, 'distance': 12.4367094039917, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 98, 'cosine_with_motion': 0.5329782250495367, 'motion_component': 1.1440276978173094}, {'ion': 1313, 'force': [-0.22009967267513275, -0.8663344383239746, -1.9290385246276855], 'magnitude': 2.1260688304901123, 'distance': 12.496269226074219, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.51243623983977, 'motion_component': 1.0894747391248973}, {'ion': 2433, 'force': [-0.5442313551902771, -2.0070571899414062, -3.0901710987091064], 'magnitude': 3.724731206893921, 'distance': 9.44107723236084, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.48619036356088124, 'motion_component': 1.8109284971392512}]}, 3010: {'frame': 3010, 'ionic_force': [-1.4288375824689865, -11.894582986831665, -8.427950035780668], 'ionic_force_magnitude': 14.647628581900774, 'motion_vector': [-0.03083038330078125, 0.14577102661132812, -0.056365966796875], 'cosine_ionic_motion': -0.5206108707521561, 'ionic_motion_component': -7.625714670477531, 'ionic_force_x': -1.4288375824689865, 'ionic_force_y': -11.894582986831665, 'ionic_force_z': -8.427950035780668, 'radial_force': 11.98009521112838, 'axial_force': -8.427950035780668, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1305, 'force': [-1.6354900598526, -7.113887786865234, -3.7080366611480713], 'magnitude': 8.18729305267334, 'distance': 6.36793851852417, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5961834304625964, 'motion_component': -4.881128295598728}, {'ion': 1307, 'force': [0.6026757955551147, -1.9631599187850952, 0.01580892875790596], 'magnitude': 2.0536468029022217, 'distance': 12.714701652526855, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.9342669475811238, 'motion_component': -1.9186542645450393}, {'ion': 1313, 'force': [-0.1381060630083084, -0.8840373754501343, -1.8939621448516846], 'magnitude': 2.0946810245513916, 'distance': 12.589547157287598, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.05350608717478665, 'motion_component': -0.11207817755057192}, {'ion': 2433, 'force': [-0.25791725516319275, -1.9334979057312012, -2.8417601585388184], 'magnitude': 3.446815252304077, 'distance': 9.814315795898438, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.2071054553698344, 'motion_component': -0.713854268755469}]}, 3011: {'frame': 3011, 'ionic_force': [-0.9096110463142395, -11.761033356189728, -8.9583909958601], 'ionic_force_magnitude': 14.812226945861031, 'motion_vector': [0.000152587890625, -0.8182907104492188, 0.11767578125], 'cosine_ionic_motion': 0.6998237472618103, 'ionic_motion_component': 10.365948166544827, 'ionic_force_x': -0.9096110463142395, 'ionic_force_y': -11.761033356189728, 'ionic_force_z': -8.9583909958601, 'radial_force': 11.796156062929326, 'axial_force': -8.9583909958601, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1305, 'force': [-1.3281829357147217, -7.1350812911987305, -4.085694789886475], 'magnitude': 8.328646659851074, 'distance': 6.313669204711914, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.7781113738897705, 'motion_component': 6.480614773345758}, {'ion': 1307, 'force': [0.8396745920181274, -2.035407304763794, -0.0728185623884201], 'magnitude': 2.2030067443847656, 'distance': 12.27612018585205, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.9098798401350634, 'motion_component': 2.0044714541324913}, {'ion': 1313, 'force': [-0.13250839710235596, -0.7889592051506042, -1.8526458740234375], 'magnitude': 2.0179970264434814, 'distance': 12.826518058776855, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.25628922882923555, 'motion_component': 0.5171908914312319}, {'ion': 2433, 'force': [-0.2885943055152893, -1.8015855550765991, -2.9472317695617676], 'magnitude': 3.4662909507751465, 'distance': 9.78670597076416, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.3934093462392622, 'motion_component': 1.363671218998477}]}, 3012: {'frame': 3012, 'ionic_force': [-0.3800518661737442, -10.41212683916092, -7.1678599789738655], 'ionic_force_magnitude': 12.646542666433879, 'motion_vector': [-0.6113166809082031, 0.6762008666992188, 0.26922607421875], 'cosine_ionic_motion': -0.7269382448602062, 'ionic_motion_component': -9.193255529487155, 'ionic_force_x': -0.3800518661737442, 'ionic_force_y': -10.41212683916092, 'ionic_force_z': -7.1678599789738655, 'radial_force': 10.419060645555208, 'axial_force': -7.1678599789738655, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1305, 'force': [-0.663364052772522, -5.617071151733398, -2.9004411697387695], 'magnitude': 6.356421947479248, 'distance': 7.227077007293701, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6907973392269726, 'motion_component': -4.390999324572796}, {'ion': 1307, 'force': [0.7231239676475525, -1.9537044763565063, -0.054674215614795685], 'magnitude': 2.0839526653289795, 'distance': 12.62191104888916, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 130, 'cosine_with_motion': -0.8975608458534442, 'motion_component': -1.8704743196047122}, {'ion': 1313, 'force': [-0.15532906353473663, -0.9136618971824646, -1.7275465726852417], 'magnitude': 1.9604393243789673, 'distance': 13.013446807861328, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5301986263598378, 'motion_component': -1.0394222363832712}, {'ion': 2433, 'force': [-0.2844827175140381, -1.9276893138885498, -2.4851980209350586], 'magnitude': 3.1580255031585693, 'distance': 10.253242492675781, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5992224932426599, 'motion_component': -1.8923599756961522}]}, 3013: {'frame': 3013, 'ionic_force': [-2.4495624005794525, -12.213647663593292, -7.546032872051001], 'ionic_force_magnitude': 14.564208090754702, 'motion_vector': [0.26108551025390625, -0.7062110900878906, -0.43798828125], 'cosine_ionic_motion': 0.8900177668723809, 'ionic_motion_component': 12.962403961198161, 'ionic_force_x': -2.4495624005794525, 'ionic_force_y': -12.213647663593292, 'ionic_force_z': -7.546032872051001, 'radial_force': 12.45686739131193, 'axial_force': -7.546032872051001, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1305, 'force': [-2.3178341388702393, -6.814496040344238, -2.8570826053619385], 'magnitude': 7.744199752807617, 'distance': 6.547579288482666, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.8092209569229076, 'motion_component': 6.266768869452655}, {'ion': 1307, 'force': [0.6791321635246277, -2.255999803543091, -0.028292980045080185], 'magnitude': 2.3561739921569824, 'distance': 11.870400428771973, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 130, 'cosine_with_motion': 0.8687179447280861, 'motion_component': 2.046850668541632}, {'ion': 1313, 'force': [-0.2513520419597626, -0.9746912121772766, -1.8853918313980103], 'magnitude': 2.137265205383301, 'distance': 12.463494300842285, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.7780603653831658, 'motion_component': 1.6629214572641589}, {'ion': 2433, 'force': [-0.5595083832740784, -2.1684606075286865, -2.7752654552459717], 'magnitude': 3.5661420822143555, 'distance': 9.648720741271973, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.8372809684401377, 'motion_component': 2.9858629001710906}]}, 3014: {'frame': 3014, 'ionic_force': [-0.759348452091217, -10.030214369297028, -6.846714980900288], 'ionic_force_magnitude': 12.167962705212007, 'motion_vector': [-0.043239593505859375, 0.11359786987304688, 0.687835693359375], 'cosine_ionic_motion': -0.6842960866567757, 'ionic_motion_component': -8.32648926176217, 'ionic_force_x': -0.759348452091217, 'ionic_force_y': -10.030214369297028, 'ionic_force_z': -6.846714980900288, 'radial_force': 10.058916957890938, 'axial_force': -6.846714980900288, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1305, 'force': [-0.8984873294830322, -5.705676555633545, -2.774850606918335], 'magnitude': 6.407949924468994, 'distance': 7.19796085357666, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5625550746086877, 'motion_component': -3.604824664226517}, {'ion': 1307, 'force': [0.5754648447036743, -1.8000924587249756, -0.07871926575899124], 'magnitude': 1.8914780616760254, 'distance': 13.248551368713379, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 130, 'cosine_with_motion': -0.2145920117416949, 'motion_component': -0.405896088799083}, {'ion': 1313, 'force': [-0.14402753114700317, -0.8609333634376526, -1.6557806730270386], 'magnitude': 1.8717797994613647, 'distance': 13.31808090209961, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.9411460896000108, 'motion_component': -1.761618290520553}, {'ion': 2433, 'force': [-0.29229843616485596, -1.6635119915008545, -2.337364435195923], 'magnitude': 2.883744478225708, 'distance': 10.729775428771973, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8857060610732216, 'motion_component': -2.5541500871685643}]}, 3015: {'frame': 3015, 'ionic_force': [-1.0981189906597137, -12.061806082725525, -7.414692517369986], 'ionic_force_magnitude': 14.201080818799126, 'motion_vector': [-0.32537841796875, -0.43274688720703125, 0.7002716064453125], 'cosine_ionic_motion': 0.030604965603512557, 'ionic_motion_component': 0.4346235899920492, 'ionic_force_x': -1.0981189906597137, 'ionic_force_y': -12.061806082725525, 'ionic_force_z': -7.414692517369986, 'radial_force': 12.111689861242402, 'axial_force': -7.414692517369986, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1305, 'force': [-1.1908631324768066, -6.918148040771484, -2.9930710792541504], 'magnitude': 7.631343364715576, 'distance': 6.595816135406494, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.19027719091390694, 'motion_component': 1.4520705814493056}, {'ion': 1307, 'force': [0.6159889101982117, -2.011329174041748, 0.03404975309967995], 'magnitude': 2.1038172245025635, 'distance': 12.562180519104004, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 98, 'cosine_with_motion': 0.37256992229827496, 'motion_component': 0.7838190070599007}, {'ion': 1313, 'force': [-0.15704071521759033, -1.0099607706069946, -1.7739356756210327], 'magnitude': 2.0473227500915527, 'distance': 12.734323501586914, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.4161086266890991, 'motion_component': -0.8519086459994227}, {'ion': 2433, 'force': [-0.36620405316352844, -2.122368097305298, -2.6817355155944824], 'magnitude': 3.43951416015625, 'distance': 9.824727058410645, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.2760149597521022, 'motion_component': -0.9493573410840455}]}, 3016: {'frame': 3016, 'ionic_force': [-1.516221433877945, -12.025810241699219, -6.379298746585846], 'ionic_force_magnitude': 13.697243952857832, 'motion_vector': [0.7737503051757812, 0.16421127319335938, -1.1707305908203125], 'cosine_ionic_motion': 0.22324959715390397, 'ionic_motion_component': 3.057904194594258, 'ionic_force_x': -1.516221433877945, 'ionic_force_y': -12.025810241699219, 'ionic_force_z': -6.379298746585846, 'radial_force': 12.121016434520197, 'axial_force': -6.379298746585846, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1305, 'force': [-1.2403539419174194, -6.43123722076416, -1.9104478359222412], 'magnitude': 6.822690486907959, 'distance': 6.975754737854004, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.022906645209660924, 'motion_component': 0.15628494287961558}, {'ion': 1307, 'force': [0.4378458559513092, -1.8139464855194092, 0.1359662413597107], 'magnitude': 1.8709884881973267, 'distance': 13.320898056030273, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 130, 'cosine_with_motion': -0.04473867597191927, 'motion_component': -0.08370554463273727}, {'ion': 1313, 'force': [-0.2837839126586914, -1.2178921699523926, -1.8668174743652344], 'magnitude': 2.2469539642333984, 'distance': 12.155475616455078, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5562630835268899, 'motion_component': 1.249897542163712}, {'ion': 2433, 'force': [-0.4299294352531433, -2.562734365463257, -2.737999677658081], 'magnitude': 3.774796485900879, 'distance': 9.378259658813477, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.45974060530945204, 'motion_component': 1.7354272500976844}]}, 3017: {'frame': 3017, 'ionic_force': [-0.832437627017498, -10.54514217376709, -6.56848693266511], 'ionic_force_magnitude': 12.451425478732471, 'motion_vector': [-0.13201904296875, 0.3127250671386719, 0.21350860595703125], 'cosine_ionic_motion': -0.9193040516053272, 'ionic_motion_component': -11.446645890860562, 'ionic_force_x': -0.832437627017498, 'ionic_force_y': -10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>6500</v>
+        <v>3000</v>
       </c>
       <c r="B3" t="n">
-        <v>6562</v>
+        <v>5178</v>
       </c>
       <c r="C3" t="n">
-        <v>1355</v>
+        <v>1307</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">{6500: {'frame': 6500, 'ionic_force': [-6.289812058210373, 8.96427071094513, -9.324965178966522], 'ionic_force_magnitude': 14.383145021018715, 'motion_vector': [-0.07231521606445312, 0.7506103515625, -0.3880615234375], 'cosine_ionic_motion': 0.8855674625804343, 'ionic_motion_component': 12.73724524018995, 'ionic_force_x': -6.289812058210373, 'ionic_force_y': 8.96427071094513, 'ionic_force_z': -9.324965178966522, 'radial_force': 10.950793811715993, 'axial_force': -9.324965178966522, 'before_closest_residue': None, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1327, 'force': [1.0468125343322754, 3.485199213027954, -0.6332185864448547], 'magnitude': 3.6936967372894287, 'distance': 9.480656623840332, 'before_closest_residue': None, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.8893899870605828, 'motion_component': np.float64(3.2851369207949244)}, {'ion': 1330, 'force': [0.373801052570343, 6.2043938636779785, -3.4104108810424805], 'magnitude': 7.0897908210754395, 'distance': 6.843091011047363, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.9901543538498361, 'motion_component': np.float64(7.019987174897452)}, {'ion': 1341, 'force': [-6.430893898010254, -2.644869804382324, -1.5276371240615845], 'magnitude': 7.119368553161621, 'distance': 6.828861236572266, 'before_closest_residue': None, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.15359908600446906, 'motion_component': np.float64(-1.0935284940286643)}, {'ion': 1359, 'force': [-0.32606586813926697, 0.5594664812088013, -1.3648302555084229], 'magnitude': 1.5106565952301025, 'distance': 14.824708938598633, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.7595948298763611, 'motion_component': np.float64(1.1474869323154466)}, {'ion': 1465, 'force': [-0.9534658789634705, 1.3600809574127197, -2.3888683319091797], 'magnitude': 2.909572124481201, 'distance': 10.682046890258789, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.8173583481576957, 'motion_component': np.float64(2.3781629745923936)}]}, 6501: {'frame': 6501, 'ionic_force': [-7.690910220146179, 7.941129207611084, -6.768357813358307], 'ionic_force_magnitude': 12.962341632435525, 'motion_vector': [-0.7340888977050781, -0.2639427185058594, 0.5615005493164062], 'cosine_ionic_motion': -0.020116340046945916, 'ionic_motion_component': -0.26075487208275705, 'ionic_force_x': -7.690910220146179, 'ionic_force_y': 7.941129207611084, 'ionic_force_z': -6.768357813358307, 'radial_force': 11.054937046691979, 'axial_force': -6.768357813358307, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1327, 'force': [1.086919903755188, 3.0864734649658203, -0.8753246665000916], 'magnitude': 3.387315511703491, 'distance': 9.900136947631836, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.6462517880524703, 'motion_component': np.float64(-2.189058727415901)}, {'ion': 1330, 'force': [-2.163508176803589, 4.191789627075195, -2.1859216690063477], 'magnitude': 5.199049949645996, 'distance': 7.9911088943481445, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.14920166887626987, 'motion_component': np.float64(-0.7757069444527929)}, {'ion': 1341, 'force': [-5.77974796295166, -0.7983136177062988, -1.5908108949661255], 'magnitude': 6.047600269317627, 'distance': 7.409305572509766, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.6125030968041318, 'motion_component': np.float64(3.704173965785848)}, {'ion': 1465, 'force': [-0.8345739841461182, 1.4611797332763672, -2.116300582885742], 'magnitude': 2.703754425048828, 'distance': 11.081165313720703, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.3699163734030524, 'motion_component': np.float64(-1.0001630392920333)}]}, 6502: {'frame': 6502, 'ionic_force': [-8.320663332939148, 9.290036618709564, -5.847688913345337], 'ionic_force_magnitude': 13.774385078991534, 'motion_vector': [-0.20615386962890625, 0.09394073486328125, -0.17812347412109375], 'cosine_ionic_motion': 0.9143617562565562, 'ionic_motion_component': 12.594770932180802, 'ionic_force_x': -8.320663332939148, 'ionic_force_y': 9.290036618709564, 'ionic_force_z': -5.847688913345337, 'radial_force': 12.47149624852939, 'axial_force': -5.847688913345337, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1327, 'force': [1.2445228099822998, 3.7574269771575928, -0.7076037526130676], 'magnitude': 4.0209197998046875, 'distance': 9.086702346801758, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.19197172373628854, 'motion_component': np.float64(0.7719029419149344)}, {'ion': 1330, 'force': [-2.6883904933929443, 4.354552745819092, -2.218109607696533], 'magnitude': 5.577596664428711, 'distance': 7.715169906616211, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.8450870621748968, 'motion_component': np.float64(4.713554683820419)}, {'ion': 1341, 'force': [-5.975592613220215, -0.20818573236465454, -0.7748331427574158], 'magnitude': 6.0292134284973145, 'distance': 7.420594215393066, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 455, 'cosine_with_motion': 0.7771593925339317, 'motion_component': np.float64(4.685659859152084)}, {'ion': 1465, 'force': [-0.9012030363082886, 1.3862426280975342, -2.1471424102783203], 'magnitude': 2.709991931915283, 'distance': 11.068405151367188, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.894339778827869, 'motion_component': np.float64(2.4236535512828468)}]}, 6503: {'frame': 6503, 'ionic_force': [-9.341203212738037, 8.49120157957077, -6.012524783611298], 'ionic_force_magnitude': 13.982454577080258, 'motion_vector': [-0.2536506652832031, -0.006526947021484375, -0.0059356689453125], 'cosine_ionic_motion': 0.6621017489640658, 'ionic_motion_component': 9.257807630295446, 'ionic_force_x': -9.341203212738037, 'ionic_force_y': 8.49120157957077, 'ionic_force_z': -6.012524783611298, 'radial_force': 12.623730895681062, 'axial_force': -6.012524783611298, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 130, 'contributions': [{'ion': 1327, 'force': [0.7046209573745728, 3.8860714435577393, -0.7475729584693909], 'magnitude': 4.019565582275391, 'distance': 9.088233947753906, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1105, 'cosine_with_motion': -0.19570468620753045, 'motion_component': np.float64(-0.7866478164911828)}, {'ion': 1330, 'force': [-2.498203992843628, 3.7735369205474854, -2.5399537086486816], 'magnitude': 5.189601898193359, 'distance': 7.998379707336426, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.473842396353421, 'motion_component': np.float64(2.4590534479954007)}, {'ion': 1341, 'force': [-6.450555324554443, -0.437552273273468, -0.7234834432601929], 'magnitude': 6.50573205947876, 'distance': 7.14366340637207, 'before_closest_residue': 423, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': 0.9952499266486445, 'motion_component': np.float64(6.474828945763575)}, {'ion': 1465, 'force': [-1.0970648527145386, 1.2691454887390137, -2.0015146732330322], 'magnitude': 2.6115784645080566, 'distance': 11.2750244140625, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.4252496629338461, 'motion_component': np.float64(1.1105729003106086)}]}, 6504: {'frame': 6504, 'ionic_force': [-8.524013698101044, 8.355697840452194, -4.412104159593582], 'ionic_force_magnitude': 12.725688941721572, 'motion_vector': [0.3465385437011719, 0.4995460510253906, -0.39102935791015625], 'cosine_ionic_motion': 0.32018892773106106, 'ionic_motion_component': 4.0746246968888515, 'ionic_force_x': -8.524013698101044, 'ionic_force_y': 8.355697840452194, 'ionic_force_z': -4.412104159593582, 'radial_force': 11.936351868404001, 'axial_force': -4.412104159593582, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 98, 'contributions': [{'ion': 1327, 'force': [0.9622270464897156, 3.5940864086151123, -0.4741422235965729], 'magnitude': 3.750753164291382, 'distance': 9.408270835876465, 'before_closest_residue': 1073, 'closest_residue': 1105, 'next_closest_residue': 1073, 'cosine_with_motion': 0.8535618129631807, 'motion_component': np.float64(3.201499619725597)}, {'ion': 1330, 'force': [-2.706892728805542, 3.7393574714660645, -1.6602447032928467], 'magnitude': 4.905759334564209, 'distance': 8.226515769958496, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.4453031668656395, 'motion_component': np.float64(2.184550184391945)}, {'ion': 1341, 'force': [-5.697000026702881, -0.46980372071266174, -0.2337888479232788], 'magnitude': 5.72111701965332, 'distance': 7.617783069610596, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 423, 'cosine_with_motion': -0.5120156164827646, 'motion_component': np.float64(-2.9293013523443108)}, {'ion': 1465, 'force': [-1.0823479890823364, 1.4920576810836792, -2.043928384780884], 'magnitude': 2.7523365020751953, 'distance': 10.982931137084961, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5878192153180595, 'motion_component': np.float64(1.617876316536755)}]}, 6505: {'frame': 6505, 'ionic_force': [-8.858785659074783, 7.233338713645935, -8.38033264875412], 'ionic_force_magnitude': 14.17847832468394, 'motion_vector': [0.18931961059570312, -1.0247459411621094, 0.25006103515625], 'cosine_ionic_motion': -0.7361189969277341, 'ionic_motion_component': -10.437047242327962, 'ionic_force_x': -8.858785659074783, 'ionic_force_y': 7.233338713645935, 'ionic_force_z': -8.38033264875412, 'radial_force': 11.436750950324925, 'axial_force': -8.38033264875412, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1327, 'force': [0.760402500629425, 3.0018088817596436, -0.5691439509391785], 'magnitude': 3.1484906673431396, 'distance': 10.268755912780762, 'before_closest_residue': 1105, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.9111803809742021, 'motion_component': np.float64(-2.8688429084164335)}, {'ion': 1330, 'force': [-1.6843782663345337, 3.5646517276763916, -1.0980793237686157], 'magnitude': 4.0926337242126465, 'distance': 9.006739616394043, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': 455, 'cosine_with_motion': -0.9681670240901964, 'motion_component': np.float64(-3.962352952482247)}, {'ion': 1341, 'force': [-6.1667399406433105, -2.169691562652588, -2.961028575897217], 'magnitude': 7.176624298095703, 'distance': 6.801566123962402, 'before_closest_residue': 455, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.04101690603007464, 'motion_component': np.float64(0.29436291554315375)}, {'ion': 1359, 'force': [-0.4044402539730072, 0.6704288721084595, -1.30451500415802], 'magnitude': 1.5214487314224243, 'distance': 14.772037506103516, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6683852195464322, 'motion_component': np.float64(-1.0169138323690374)}, {'ion': 1465, 'force': [-1.363629698753357, 2.1661407947540283, -2.447565793991089], 'magnitude': 3.541501045227051, 'distance': 9.682229042053223, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8141463853674326, 'motion_component': np.float64(-2.883300339182952)}]}, 6506: {'frame': 6506, 'ionic_force': [-9.954873085021973, 8.362967014312744, -7.493973672389984], 'ionic_force_magnitude': 15.006610437532258, 'motion_vector': [-0.2793464660644531, 0.185546875, -0.166778564453125], 'cosine_ionic_motion': 0.9932212824235008, 'ionic_motion_component': 14.904884863595681, 'ionic_force_x': -9.954873085021973, 'ionic_force_y': 8.362967014312744, 'ionic_force_z': -7.493973672389984, 'radial_force': 13.001488969398002, 'axial_force': -7.493973672389984, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 130, 'contributions': [{'ion': 1327, 'force': [1.2132747173309326, 4.102494239807129, -1.1174546480178833], 'magnitude': 4.421673774719238, 'distance': 8.665142059326172, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.36752452508670613, 'motion_component': np.float64(1.6250735727482741)}, {'ion': 1330, 'force': [-3.8504509925842285, 3.057932138442993, -0.5377671122550964], 'magnitude': 4.946323394775391, 'distance': 8.192713737487793, 'before_closest_residue': None, 'closest_residue': 455, 'next_closest_residue': 780, 'cosine_with_motion': 0.935285634250728, 'motion_component': np.float64(4.6262252277617595)}, {'ion': 1341, 'force': [-5.303382396697998, -1.6648468971252441, -1.7273120880126953], 'magnitude': 5.8207550048828125, 'distance': 7.552302837371826, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.6699989475694714, 'motion_component': np.float64(3.8998996271321857)}, {'ion': 1359, 'force': [-0.4168241024017334, 0.6007530689239502, -1.3772019147872925], 'magnitude': 1.5592727661132812, 'distance': 14.59177017211914, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.7835462945155544, 'motion_component': np.float64(1.2217624324779344)}, {'ion': 1465, 'force': [-1.5974903106689453, 2.266634464263916, -2.7342379093170166], 'magnitude': 3.8943119049072266, 'distance': 9.233230590820312, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.9069443256084724, 'motion_component': np.float64(3.531923946820477)}]}, 6507: {'frame': 6507, 'ionic_force': [-8.23822170495987, 7.098378419876099, -6.328981697559357], 'ionic_force_magnitude': 12.582181145567564, 'motion_vector': [0.5045700073242188, 0.26412200927734375, 0.01922607421875], 'cosine_ionic_motion': -0.3352367732455727, 'ionic_motion_component': -4.218009807631353, 'ionic_force_x': -8.23822170495987, 'ionic_force_y': 7.098378419876099, 'ionic_force_z': -6.328981697559357, 'radial_force': 10.874524037944585, 'axial_force': -6.328981697559357, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 98, 'contributions': [{'ion': 1327, 'force': [0.9431630373001099, 3.706730842590332, -0.8368191123008728], 'magnitude': 3.9153130054473877, 'distance': 9.208434104919434, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.6448942427064687, 'motion_component': np.float64(2.5249628444662635)}, {'ion': 1330, 'force': [-1.7877682447433472, 1.3567931652069092, 0.0454939603805542], 'magnitude': 2.2447879314422607, 'distance': 12.161338806152344, 'before_closest_residue': 455, 'closest_residue': 780, 'next_closest_residue': 748, 'cosine_with_motion': -0.42435162498048673, 'motion_component': np.float64(-0.9525793906921981)}, {'ion': 1341, 'force': [-5.284008026123047, -0.8967590928077698, -1.443036437034607], 'magnitude': 5.550429821014404, 'distance': 7.734027862548828, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.926609918586174, 'motion_component': np.float64(-5.143083378931156)}, {'ion': 1359, 'force': [-0.49212461709976196, 0.6336775422096252, -1.3864613771438599], 'magnitude': 1.6018767356872559, 'distance': 14.396419525146484, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.11787599555012783, 'motion_component': np.float64(-0.18882281276867507)}, {'ion': 1465, 'force': [-1.6174838542938232, 2.297935962677002, -2.7081587314605713], 'magnitude': 3.902677059173584, 'distance': 9.223329544067383, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.11748015924481388, 'motion_component': np.float64(-0.4584871102622854)}]}, 6508: {'frame': 6508, 'ionic_force': [-7.880869120359421, 5.787855565547943, -7.391227334737778], 'ionic_force_magnitude': 12.257145330526757, 'motion_vector': [-0.12299728393554688, -0.23679351806640625, 0.32021331787109375], 'cosine_ionic_motion': -0.5417852045691541, 'ionic_motion_component': -6.640739990333292, 'ionic_force_x': -7.880869120359421, 'ionic_force_y': 5.787855565547943, 'ionic_force_z': -7.391227334737778, 'radial_force': 9.777902133887359, 'axial_force': -7.391227334737778, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1327, 'force': [1.0252001285552979, 3.475285530090332, -0.871704638004303], 'magnitude': 3.72672963142395, 'distance': 9.438546180725098, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.7906417068880925, 'motion_component': np.float64(-2.9465078821428534)}, {'ion': 1330, 'force': [-1.0581204891204834, 1.1649466753005981, -0.22578909993171692], 'magnitude': 1.5898743867874146, 'distance': 14.450658798217773, 'before_closest_residue': 780, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.32897413435374084, 'motion_component': np.float64(-0.5230275374690159)}, {'ion': 1341, 'force': [-6.056460857391357, -1.6252504587173462, -2.4695639610290527], 'magnitude': 6.739502906799316, 'distance': 7.018674850463867, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.12067398511185845, 'motion_component': np.float64(0.81328270833)}, {'ion': 1359, 'force': [-0.40871426463127136, 0.6200887560844421, -1.3025858402252197], 'magnitude': 1.4994289875030518, 'distance': 14.880107879638672, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8218854183146611, 'motion_component': np.float64(-1.232358820113542)}, {'ion': 1465, 'force': [-1.3827736377716064, 2.152785062789917, -2.5215837955474854], 'magnitude': 3.592343330383301, 'distance': 9.613468170166016, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7661095677045854, 'motion_component': np.float64(-2.7521286699421736)}]}, 6509: {'frame': 6509, 'ionic_force': [-7.748109370470047, 7.134311139583588, -6.899723134934902], 'ionic_force_magnitude': 12.591178403624822, 'motion_vector': [0.30371856689453125, 1.6467742919921875, -0.6300277709960938], 'cosine_ionic_motion': 0.6100275251247687, 'ionic_motion_component': 7.680965399967685, 'ionic_force_x': -7.748109370470047, 'ionic_force_y': 7.134311139583588, 'ionic_force_z': -6.899723134934902, 'radial_force': 10.532406859457728, 'axial_force': -6.899723134934902, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1327, 'force': [1.206465721130371, 3.8794455528259277, -0.8778850436210632], 'magnitude': 4.156481742858887, 'distance': 8.937294960021973, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.9827251048591827, 'motion_component': np.float64(4.084678838935654)}, {'ion': 1330, 'force': [-1.0981571674346924, 1.4916738271713257, -0.11615731567144394], 'magnitude': 1.855945110321045, 'distance': 13.374774932861328, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 455, 'cosine_with_motion': 0.6613652660136579, 'motion_component': np.float64(1.2274576744480303)}, {'ion': 1341, 'force': [-5.690523624420166, -1.5907838344573975, -1.5250321626663208], 'magnitude': 6.102325439453125, 'distance': 7.376007556915283, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.31023823222513514, 'motion_component': np.float64(-1.8931746480597589)}, {'ion': 1359, 'force': [-0.41519561409950256, 0.6836457848548889, -1.4476933479309082], 'magnitude': 1.653957486152649, 'distance': 14.167945861816406, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.646057281422398, 'motion_component': np.float64(1.0685512030240307)}, {'ion': 1465, 'force': [-1.7506986856460571, 2.6703298091888428, -2.932955265045166], 'magnitude': 4.335647106170654, 'distance': 8.750685691833496, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.7365572665382815, 'motion_component': np.float64(3.1934522058137915)}]}, 6510: {'frame': 6510, 'ionic_force': [-7.857691705226898, 6.3123403787612915, -4.668317198753357], 'ionic_force_magnitude': 11.107751593365249, 'motion_vector': [-0.013092041015625, -2.068023681640625, 0.45330047607421875], 'cosine_ionic_motion': -0.6407026655708375, 'ionic_motion_component': -7.116766054367833, 'ionic_force_x': -7.857691705226898, 'ionic_force_y': 6.3123403787612915, 'ionic_force_z': -4.668317198753357, 'radial_force': 10.079134883100426, 'axial_force': -4.668317198753357, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1327, 'force': [0.7078949809074402, 2.60565447807312, -0.4197348356246948], 'magnitude': 2.7325315475463867, 'distance': 11.022661209106445, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.9659264590732278, 'motion_component': np.float64(-2.6394243871698735)}, {'ion': 1330, 'force': [-1.8742456436157227, 1.8574930429458618, -0.35592353343963623], 'magnitude': 2.6626601219177246, 'distance': 11.166348457336426, 'before_closest_residue': 748, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': -0.7056843576031504, 'motion_component': np.float64(-1.8789975677039947)}, {'ion': 1341, 'force': [-5.465493679046631, -0.39318275451660156, -1.7694438695907593], 'magnitude': 5.758224010467529, 'distance': 7.593198776245117, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.006773466801259861, 'motion_component': np.float64(0.03900314016137085)}, {'ion': 1465, 'force': [-1.2258473634719849, 2.242375612258911, -2.1232149600982666], 'magnitude': 3.322497844696045, 'distance': 9.996240615844727, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7937844963782316, 'motion_component': np.float64(-2.6373472764298405)}]}, 6511: {'frame': 6511, 'ionic_force': [-9.91338911652565, 7.838640451431274, -6.242726296186447], 'ionic_force_magnitude': 14.095786587188444, 'motion_vector': [-0.5040168762207031, 0.45391082763671875, 0.05902099609375], 'cosine_ionic_motion': 0.8529805459805472, 'ionic_motion_component': 12.023431739165273, 'ionic_force_x': -9.91338911652565, 'ionic_force_y': 7.838640451431274, 'ionic_force_z': -6.242726296186447, 'radial_force': 12.638020727252503, 'axial_force': -6.242726296186447, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1327, 'force': [0.8552926182746887, 3.274571418762207, -0.5970718264579773], 'magnitude': 3.436690092086792, 'distance': 9.828763008117676, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.43594189268299505, 'motion_component': np.float64(1.4981971462915187)}, {'ion': 1330, 'force': [-2.817471742630005, 3.458409547805786, 0.222823828458786], 'magnitude': 4.466362476348877, 'distance': 8.621683120727539, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 780, 'cosine_with_motion': 0.9875394002999975, 'motion_component': np.float64(4.4107089556061)}, {'ion': 1341, 'force': [-5.989511966705322, -1.8379708528518677, -1.4910531044006348], 'magnitude': 6.440157413482666, 'distance': 7.1799397468566895, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.47814214261356464, 'motion_component': np.float64(3.0793107500152885)}, {'ion': 1359, 'force': [-0.39044126868247986, 0.6049216985702515, -1.4029350280761719], 'magnitude': 1.576896071434021, 'distance': 14.510003089904785, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.3619209476488102, 'motion_component': np.float64(0.5707117341262276)}, {'ion': 1465, 'force': [-1.5712567567825317, 2.3387086391448975, -2.974490165710449], 'magnitude': 4.097071647644043, 'distance': 9.001859664916992, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.60152803654643, 'motion_component': np.float64(2.4645035779143)}]}, 6512: {'frame': 6512, 'ionic_force': [-8.842867404222488, 8.652108788490295, -5.702980926260352], 'ionic_force_magnitude': 13.62274868966689, 'motion_vector': [0.0037841796875, -0.05219268798828125, -0.3178558349609375], 'cosine_ionic_motion': 0.3025472302265823, 'ionic_motion_component': 4.121524884131521, 'ionic_force_x': -8.842867404222488, 'ionic_force_y': 8.652108788490295, 'ionic_force_z': -5.702980926260352, 'radial_force': 12.371551657594596, 'axial_force': -5.702980926260352, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1327, 'force': [1.2942389249801636, 4.0767974853515625, -0.7655097246170044], 'magnitude': 4.345265865325928, 'distance': 8.740994453430176, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.025318867713297652, 'motion_component': np.float64(0.1100172169536805)}, {'ion': 1330, 'force': [-1.897695779800415, 2.7120249271392822, 0.009927460923790932], 'magnitude': 3.310049295425415, 'distance': 10.015019416809082, 'before_closest_residue': 455, 'closest_residue': 780, 'next_closest_residue': 'SF', 'cosine_with_motion': -0.14244322695982675, 'motion_component': np.float64(-0.47149411797842333)}, {'ion': 1341, 'force': [-6.186309337615967, -0.9965171813964844, -1.0365417003631592], 'magnitude': 6.3512115478515625, 'distance': 7.230040550231934, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.17501525512030888, 'motion_component': np.float64(1.1115589132904602)}, {'ion': 1359, 'force': [-0.4885233938694, 0.6446949243545532, -1.39858078956604], 'magnitude': 1.6156468391418457, 'distance': 14.334938049316406, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.7859457482091414, 'motion_component': np.float64(1.2698108046839687)}, {'ion': 1465, 'force': [-1.5645778179168701, 2.215108633041382, -2.5122761726379395], 'magnitude': 3.696774482727051, 'distance': 9.476709365844727, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5685043020976622, 'motion_component': np.float64(2.1016321970041183)}]}, 6513: {'frame': 6513, 'ionic_force': [-9.518068015575409, 8.962327480316162, -6.766226708889008], 'ionic_force_magnitude': 14.720691440609466, 'motion_vector': [-0.08514022827148438, 0.5365028381347656, 0.13083648681640625], 'cosine_ionic_motion': 0.5754774721577084, 'ionic_motion_component': 8.47142629865555, 'ionic_force_x': -9.518068015575409, 'ionic_force_y': 8.962327480316162, 'ionic_force_z': -6.766226708889008, 'radial_force': 13.073520283900196, 'axial_force': -6.766226708889008, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 130, 'contributions': [{'ion': 1327, 'force': [1.6071330308914185, 3.729818344116211, -0.6672799587249756], 'magnitude': 4.115784645080566, 'distance': 8.981372833251953, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.7726763203040994, 'motion_component': np.float64(3.1801694058504886)}, {'ion': 1330, 'force': [-4.122141361236572, 3.285998582839966, -0.7577335238456726], 'magnitude': 5.325786113739014, 'distance': 7.895455360412598, 'before_closest_residue': 780, 'closest_residue': 'SF', 'next_closest_residue': 780, 'cosine_with_motion': 0.6770540584150978, 'motion_component': np.float64(3.605845004180625)}, {'ion': 1341, 'force': [-4.779118061065674, -1.3160141706466675, -1.0592595338821411], 'magnitude': 5.068914413452148, 'distance': 8.093037605285645, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.15455502589751444, 'motion_component': np.float64(-0.7834262010071082)}, {'ion': 1359, 'force': [-0.4411465525627136, 0.676803708076477, -1.391266942024231], 'magnitude': 1.608818531036377, 'distance': 14.365326881408691, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.24322060934406917, 'motion_component': np.float64(0.3912978369179019)}, {'ion': 1465, 'force': [-1.7827950716018677, 2.585721015930176, -2.8906867504119873], 'magnitude': 4.268533706665039, 'distance': 8.819210052490234, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.4867104389111577, 'motion_component': np.float64(2.0775399893396376)}]}, 6514: {'frame': 6514, 'ionic_force': [-7.190410137176514, 8.119711190462112, -4.648743212223053], 'ionic_force_magnitude': 11.800106830470492, 'motion_vector': [-0.034603118896484375, 0.70941162109375, -0.40940093994140625], 'cosine_ionic_motion': 0.8179093619358464, 'ionic_motion_component': 9.651417848484943, 'ionic_force_x': -7.190410137176514, 'ionic_force_y': 8.119711190462112, 'ionic_force_z': -4.648743212223053, 'radial_force': 10.84581521866044, 'axial_force': -4.648743212223053, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 130, 'contributions': [{'ion': 1327, 'force': [1.1255909204483032, 3.2406394481658936, -0.6212179064750671], 'magnitude': 3.4863462448120117, 'distance': 9.758516311645508, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.8797176687793233, 'motion_component': np.float64(3.067000454355637)}, {'ion': 1330, 'force': [-2.07405948638916, 2.3413660526275635, 0.3788716793060303], 'magnitude': 3.1507556438446045, 'distance': 10.265064239501953, 'before_closest_residue': 'SF', 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.6107851738046798, 'motion_component': np.float64(1.9244348691757835)}, {'ion': 1341, 'force': [-4.358066082000732, -0.3850259482860565, -0.6954754590988159], 'magnitude': 4.42997407913208, 'distance': 8.657020568847656, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.04471446363204596, 'motion_component': np.float64(0.19808391852817842)}, {'ion': 1359, 'force': [-0.4579681158065796, 0.6891224384307861, -1.2874083518981934], 'magnitude': 1.5303740501403809, 'distance': 14.728897094726562, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.8224014246805668, 'motion_component': np.float64(1.2585818156376751)}, {'ion': 1465, 'force': [-1.4259073734283447, 2.233609199523926, -2.423513174057007], 'magnitude': 3.5910496711730957, 'distance': 9.61520004272461, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.8920280207972249, 'motion_component': np.float64(3.2033169627790716)}]}, 6515: {'frame': 6515, 'ionic_force': [-6.946783423423767, 6.875458121299744, -4.343691200017929], 'ionic_force_magnitude': 10.695670972445583, 'motion_vector': [-0.9353866577148438, -0.8836402893066406, 0.4879302978515625], 'cosine_ionic_motion': -0.11528735159234577, 'ionic_motion_component': -1.2330755799163806, 'ionic_force_x': -6.946783423423767, 'ionic_force_y': 6.875458121299744, 'ionic_force_z': -4.343691200017929, 'radial_force': 9.773930852512812, 'axial_force': -4.343691200017929, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 98, 'contributions': [{'ion': 1327, 'force': [0.5734409093856812, 2.937873363494873, </t>
+          <t>{3000: {'frame': 3000, 'ionic_force': [-4.559090405702591, 7.512245416641235, -6.194559022784233], 'ionic_force_magnitude': 10.751357961391399, 'motion_vector': [-0.67041015625, -0.13644790649414062, 0.28293609619140625], 'cosine_ionic_motion': 0.03502179671396994, 'ionic_motion_component': 0.37653187292297186, 'ionic_force_x': -4.559090405702591, 'ionic_force_y': 7.512245416641235, 'ionic_force_z': -6.194559022784233, 'radial_force': 8.78744197859745, 'axial_force': -6.194559022784233, 'before_closest_residue': None, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1305, 'force': [-2.591191053390503, 3.442763328552246, -2.422104835510254], 'magnitude': 4.943023681640625, 'distance': 8.19544792175293, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.15906271144856737, 'motion_component': 0.7862507355347361}, {'ion': 1306, 'force': [-0.29505655169487, 1.8750426769256592, -0.13831393420696259], 'magnitude': 1.9031484127044678, 'distance': 13.207867622375488, 'before_closest_residue': None, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.06896437793450658, 'motion_component': -0.13124945133843413}, {'ion': 1313, 'force': [-0.5659236311912537, 0.7050395011901855, -1.5006968975067139], 'magnitude': 1.7519820928573608, 'distance': 13.765887260437012, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.10901502951116973, 'motion_component': -0.19099238512717776}, {'ion': 2433, 'force': [-1.1069191694259644, 1.4893999099731445, -2.1334433555603027], 'magnitude': 2.8275718688964844, 'distance': 10.835830688476562, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.0309371619834855, 'motion_component': -0.08747704902143738}]}, 3001: {'frame': 3001, 'ionic_force': [-5.316149055957794, 7.246454656124115, -6.096022456884384], 'ionic_force_magnitude': 10.859743812045592, 'motion_vector': [0.0252838134765625, 0.7702713012695312, 0.0246734619140625], 'cosine_ionic_motion': 0.6325622732381134, 'ionic_motion_component': 6.869464232531095, 'ionic_force_x': -5.316149055957794, 'ionic_force_y': 7.246454656124115, 'ionic_force_z': -6.096022456884384, 'radial_force': 8.987354775929557, 'axial_force': -6.096022456884384, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1305, 'force': [-2.895693302154541, 3.026092767715454, -2.338249683380127], 'magnitude': 4.796841621398926, 'distance': 8.319387435913086, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5947964728156222, 'motion_component': 2.8531444262245547}, {'ion': 1306, 'force': [-0.42661887407302856, 1.954982876777649, -0.08282431960105896], 'magnitude': 2.0027036666870117, 'distance': 12.875399589538574, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.9668384403055922, 'motion_component': 1.9362907938011529}, {'ion': 1313, 'force': [-0.6913728713989258, 0.7455218434333801, -1.5948574542999268], 'magnitude': 1.8913935422897339, 'distance': 13.248847007751465, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.35478374279946634, 'motion_component': 0.6710356832350675}, {'ion': 2433, 'force': [-1.3024640083312988, 1.5198571681976318, -2.0800909996032715], 'magnitude': 2.886720657348633, 'distance': 10.7242431640625, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.488094789931222, 'motion_component': 1.4089933735214455}]}, 3002: {'frame': 3002, 'ionic_force': [-5.37500536441803, 7.8116095662117, -4.815210834145546], 'ionic_force_magnitude': 10.634762905665804, 'motion_vector': [-0.8808021545410156, -0.35851287841796875, 0.12474822998046875], 'cosine_ionic_motion': 0.1306927962960198, 'ionic_motion_component': 1.3898869020866484, 'ionic_force_x': -5.37500536441803, 'ionic_force_y': 7.8116095662117, 'ionic_force_z': -4.815210834145546, 'radial_force': 9.482189972915156, 'axial_force': -4.815210834145546, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1305, 'force': [-2.940093755722046, 3.5823886394500732, -1.3767294883728027], 'magnitude': 4.834567546844482, 'distance': 8.286864280700684, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.24446495439083782, 'motion_component': 1.18188234433633}, {'ion': 1306, 'force': [-0.4164557456970215, 1.7535215616226196, -0.1588585525751114], 'magnitude': 1.8092842102050781, 'distance': 13.546142578125, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.16231181261522235, 'motion_component': -0.2936681970762114}, {'ion': 1313, 'force': [-0.708341121673584, 0.8813830018043518, -1.4731264114379883], 'magnitude': 1.8570634126663208, 'distance': 13.370746612548828, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.06970321418611172, 'motion_component': 0.1294432896723503}, {'ion': 2433, 'force': [-1.3101147413253784, 1.5943163633346558, -1.8064963817596436], 'magnitude': 2.7425670623779297, 'distance': 11.00247573852539, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.1357229932285359, 'motion_component': 0.37222942042426865}]}, 3003: {'frame': 3003, 'ionic_force': [-5.220101922750473, 6.779296398162842, -4.533165335655212], 'ionic_force_magnitude': 9.682866915249475, 'motion_vector': [0.8978500366210938, -0.6827850341796875, 0.23921966552734375], 'cosine_ionic_motion': -0.9314937323200955, 'ionic_motion_component': -9.019529842444504, 'ionic_force_x': -5.220101922750473, 'ionic_force_y': 6.779296398162842, 'ionic_force_z': -4.533165335655212, 'radial_force': 8.556186284674197, 'axial_force': -4.533165335655212, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1305, 'force': [-2.8291804790496826, 3.0789058208465576, -1.4613944292068481], 'magnitude': 4.429401397705078, 'distance': 8.657580375671387, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.977409692743869, 'motion_component': -4.329339878191837}, {'ion': 1306, 'force': [-0.4663363993167877, 1.546359658241272, -0.07744836807250977], 'magnitude': 1.6170021295547485, 'distance': 14.32892894744873, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.8007794302619649, 'motion_component': -1.2948620917512237}, {'ion': 1313, 'force': [-0.6911757588386536, 0.752778172492981, -1.3276585340499878], 'magnitude': 1.6754330396652222, 'distance': 14.076849937438965, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7516817720995196, 'motion_component': -1.2593925254665255}, {'ion': 2433, 'force': [-1.2334092855453491, 1.4012527465820312, -1.6666640043258667], 'magnitude': 2.502514123916626, 'distance': 11.518097877502441, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8535158715968457, 'motion_component': -2.1359354705181435}]}, 3004: {'frame': 3004, 'ionic_force': [-6.019017517566681, 8.081940829753876, -5.979864832013845], 'ionic_force_magnitude': 11.717726864096692, 'motion_vector': [-0.6808280944824219, 0.9761505126953125, -1.2208786010742188], 'cosine_ionic_motion': 0.9654306726604445, 'ionic_motion_component': 11.31265292845623, 'ionic_force_x': -6.019017517566681, 'ionic_force_y': 8.081940829753876, 'ionic_force_z': -5.979864832013845, 'radial_force': 10.077020365783595, 'axial_force': -5.979864832013845, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1305, 'force': [-3.444451093673706, 3.7949910163879395, -2.0709657669067383], 'magnitude': 5.5276665687561035, 'distance': 7.749936103820801, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.9101730806416061, 'motion_component': 5.031133446600975}, {'ion': 1306, 'force': [-0.3731239438056946, 1.9103577136993408, -0.05936693772673607], 'magnitude': 1.9473603963851929, 'distance': 13.057074546813965, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 1105, 'cosine_with_motion': 0.659992934280571, 'motion_component': 1.2852441006915112}, {'ion': 1313, 'force': [-0.7134701013565063, 0.7610639929771423, -1.556267261505127], 'magnitude': 1.873559594154358, 'distance': 13.31175422668457, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.979433723811407, 'motion_component': 1.835027508457479}, {'ion': 2433, 'force': [-1.487972378730774, 1.6155281066894531, -2.293264865875244], 'magnitude': 3.1753828525543213, 'distance': 10.225180625915527, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.9955485343981766, 'motion_component': 3.161247799586725}]}, 3005: {'frame': 3005, 'ionic_force': [-4.469300419092178, 6.485483527183533, -4.737789124250412], 'ionic_force_magnitude': 9.191451931187583, 'motion_vector': [0.8794097900390625, -0.69476318359375, 0.46636962890625], 'cosine_ionic_motion': -0.9541350510901858, 'ionic_motion_component': -8.769886457956652, 'ionic_force_x': -4.469300419092178, 'ionic_force_y': 6.485483527183533, 'ionic_force_z': -4.737789124250412, 'radial_force': 7.876302610836285, 'axial_force': -4.737789124250412, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 130, 'contributions': [{'ion': 1305, 'force': [-2.509575128555298, 2.966874599456787, -1.6304306983947754], 'magnitude': 4.214097499847412, 'distance': 8.875988960266113, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.9830128520237679, 'motion_component': -4.142511854934142}, {'ion': 1306, 'force': [-0.34922900795936584, 1.6264971494674683, -0.19030365347862244], 'magnitude': 1.674416184425354, 'distance': 14.081124305725098, 'before_closest_residue': 780, 'closest_residue': 1105, 'next_closest_residue': 780, 'cosine_with_motion': -0.7507206326202612, 'motion_component': -1.2570187322021518}, {'ion': 1313, 'force': [-0.5725502967834473, 0.6716901063919067, -1.2509846687316895], 'magnitude': 1.5309944152832031, 'distance': 14.725913047790527, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8359494889208097, 'motion_component': -1.2798340489967686}, {'ion': 2433, 'force': [-1.0379459857940674, 1.2204216718673706, -1.6660701036453247], 'magnitude': 2.3113956451416016, 'distance': 11.984829902648926, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.9044412036581045, 'motion_component': -2.0905215941200908}]}, 3006: {'frame': 3006, 'ionic_force': [-4.481074392795563, 7.026353359222412, -5.908306911587715], 'ionic_force_magnitude': 10.215564585667273, 'motion_vector': [0.3334922790527344, 1.6488761901855469, -0.07015228271484375], 'cosine_ionic_motion': 0.6107871495547678, 'ionic_motion_component': 6.239535574372346, 'ionic_force_x': -4.481074392795563, 'ionic_force_y': 7.026353359222412, 'ionic_force_z': -5.908306911587715, 'radial_force': 8.333646815315861, 'axial_force': -5.908306911587715, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 98, 'contributions': [{'ion': 1305, 'force': [-2.4223365783691406, 3.0325369834899902, -2.3267641067504883], 'magnitude': 4.525243282318115, 'distance': 8.565408706665039, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5716659414311396, 'motion_component': 2.5869274295736986}, {'ion': 1306, 'force': [-0.4035383462905884, 1.9195414781570435, -0.24027784168720245], 'magnitude': 1.9761619567871094, 'distance': 12.96157455444336, 'before_closest_residue': 1105, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.9158634707675024, 'motion_component': 1.809894558980031}, {'ion': 1313, 'force': [-0.5843501687049866, 0.6974948644638062, -1.4270141124725342], 'magnitude': 1.6924341917037964, 'distance': 14.00596809387207, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.37033857249325824, 'motion_component': 0.626773661452849}, {'ion': 2433, 'force': [-1.0708492994308472, 1.3767800331115723, -1.9142508506774902], 'magnitude': 2.589709997177124, 'distance': 11.322529792785645, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.4695274573912474, 'motion_component': 1.2159399441461698}]}, 3007: {'frame': 3007, 'ionic_force': [-3.4469441771507263, 7.1588616371154785, -4.899470458738506], 'ionic_force_magnitude': 9.334641657600377, 'motion_vector': [-0.33539581298828125, -1.3836326599121094, 0.39107513427734375], 'cosine_ionic_motion': -0.7738491981948528, 'ionic_motion_component': -7.223604962170323, 'ionic_force_x': -3.4469441771507263, 'ionic_force_y': 7.1588616371154785, 'ionic_force_z': -4.899470458738506, 'radial_force': 7.945484510069666, 'axial_force': -4.899470458738506, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 130, 'contributions': [{'ion': 1305, 'force': [-1.741471290588379, 3.0368943214416504, -1.9926906824111938], 'magnitude': 4.028183937072754, 'distance': 9.078506469726562, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.73934532148256, 'motion_component': -2.9782189204535285}, {'ion': 1306, 'force': [-0.4332018792629242, 1.9774179458618164, 0.002815951593220234], 'magnitude': 2.024315595626831, 'distance': 12.806485176086426, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.8664497558775278, 'motion_component': -1.7539677321843956}, {'ion': 1313, 'force': [-0.43810316920280457, 0.76674485206604, -1.2528533935546875], 'magnitude': 1.5327993631362915, 'distance': 14.717240333557129, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.620355029914809, 'motion_component': -0.9508797529127636}, {'ion': 2433, 'force': [-0.8341678380966187, 1.3778045177459717, -1.6567423343658447], 'magnitude': 2.310622453689575, 'distance': 11.986835479736328, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6667201047343652, 'motion_component': -1.5405384890820315}]}, 3008: {'frame': 3008, 'ionic_force': [-6.099629461765289, 8.671195447444916, -5.837015765719116], 'ionic_force_magnitude': 12.102308172736226, 'motion_vector': [0.044155120849609375, 1.041534423828125, -0.0920562744140625], 'cosine_ionic_motion': 0.7342336025818584, 'ionic_motion_component': 8.885921329223988, 'ionic_force_x': -6.099629461765289, 'ionic_force_y': 8.671195447444916, 'ionic_force_z': -5.837015765719116, 'radial_force': 10.601656005484452, 'axial_force': -5.837015765719116, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 130, 'contributions': [{'ion': 1305, 'force': [-3.520183801651001, 4.301698207855225, -2.023888349533081], 'magnitude': 5.915439605712891, 'distance': 7.491616249084473, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.7287172989395309, 'motion_component': 4.310683158667021}, {'ion': 1306, 'force': [-0.693957507610321, 2.034898281097412, -0.0119145093485713], 'magnitude': 2.1500070095062256, 'distance': 12.426507949829102, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.9288156065375995, 'motion_component': 1.996960032494214}, {'ion': 1313, 'force': [-0.6225230693817139, 0.8132948279380798, -1.584661841392517], 'magnitude': 1.8868324756622314, 'distance': 13.264851570129395, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.48893709202128266, 'motion_component': 0.9225423590883679}, {'ion': 2433, 'force': [-1.2629650831222534, 1.5213041305541992, -2.2165510654449463], 'magnitude': 2.9702770709991455, 'distance': 10.57232666015625, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5574348863284022, 'motion_component': 1.6557360432367907}]}, 3009: {'frame': 3009, 'ionic_force': [-4.289487838745117, 7.724954307079315, -4.442825596779585], 'ionic_force_magnitude': 9.89006189306242, 'motion_vector': [-0.037891387939453125, -0.18831253051757812, -0.44643402099609375], 'cosine_ionic_motion': 0.14381369028517, 'ionic_motion_component': 1.4223262979900408, 'ionic_force_x': -4.289487838745117, 'ionic_force_y': 7.724954307079315, 'ionic_force_z': -4.442825596779585, 'radial_force': 8.835984663024576, 'axial_force': -4.442825596779585, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 98, 'contributions': [{'ion': 1305, 'force': [-2.255481004714966, 3.25519061088562, -1.3086310625076294], 'magnitude': 4.170848369598389, 'distance': 8.921889305114746, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.02796551695509831, 'motion_component': 0.11663992949438828}, {'ion': 1306, 'force': [-0.5262024998664856, 2.080961227416992, -0.009617727249860764], 'magnitude': 2.1464810371398926, 'distance': 12.4367094039917, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.35241447004123666, 'motion_component': -0.7564510066078423}, {'ion': 1313, 'force': [-0.5206497311592102, 0.8350910544395447, -1.3660943508148193], 'magnitude': 1.6836469173431396, 'distance': 14.042470932006836, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5772501674325248, 'motion_component': 0.9718854726153299}, {'ion': 2433, 'force': [-0.9871546030044556, 1.5537114143371582, -1.7584824562072754], 'magnitude': 2.5457324981689453, 'distance': 11.419909477233887, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.42826652079334576, 'motion_component': 1.0902519969871483}]}, 3010: {'frame': 3010, 'ionic_force': [-4.548879444599152, 7.443653404712677, -4.621647346764803], 'ionic_force_magnitude': 9.872178301106876, 'motion_vector': [-0.9785308837890625, -0.6665191650390625, 0.44728851318359375], 'cosine_ionic_motion': -0.2062754538621916, 'ionic_motion_component': -2.0363880596693003, 'ionic_force_x': -4.548879444599152, 'ionic_force_y': 7.443653404712677, 'ionic_force_z': -4.621647346764803, 'radial_force': 8.723547455650557, 'axial_force': -4.621647346764803, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1305, 'force': [-2.422109603881836, 3.2053823471069336, -1.4435312747955322], 'magnitude': 4.269060134887695, 'distance': 8.818666458129883, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.07625550117973197, 'motion_component': -0.3255393114924843}, {'ion': 1306, 'force': [-0.6026757955551147, 1.9631599187850952, -0.01580892875790596], 'magnitude': 2.0536468029022217, 'distance': 12.714701652526855, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.27924973124076724, 'motion_component': -0.5734802982223999}, {'ion': 1313, 'force': [-0.5377405881881714, 0.8065060973167419, -1.3534986972808838], 'magnitude': 1.6648050546646118, 'distance': 14.121712684631348, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.2927142623326544, 'motion_component': -0.48731217283988926}, {'ion': 2433, 'force': [-0.9863534569740295, 1.4686050415039062, -1.808808445930481], 'magnitude': 2.5301148891448975, 'distance': 11.455101013183594, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.2569275351755479, 'motion_component': -0.6500562101965954}]}, 3011: {'frame': 3011, 'ionic_force': [-5.611195087432861, 7.195566117763519, -4.379134848713875], 'ionic_force_magnitude': 10.121190843352245, 'motion_vector': [0.29943084716796875, -0.3274383544921875, 0.0430450439453125], 'cosine_ionic_motion': -0.9363588422319269, 'ionic_motion_component': -9.477066540089687, 'ionic_force_x': -5.611195087432861, 'ionic_force_y': 7.195566117763519, 'ionic_force_z': -4.379134848713875, 'radial_force': 9.124783946173029, 'axial_force': -4.379134848713875, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1305, 'force': [-2.919311046600342, 3.046348810195923, -1.3818751573562622], 'magnitude': 4.4398417472839355, 'distance': 8.647395133972168, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.9756848654458751, 'motion_component': -4.331886647199135}, {'ion': 1306, 'force': [-0.8396745920181274, 2.035407304763794, 0.0728185623884201], 'magnitude': 2.2030067443847656, 'distance': 12.27612018585205, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.9314562894247654, 'motion_component': -2.052004518142707}, {'ion': 1313, 'force': [-0.6490916013717651, 0.7438748478889465, -1.336652398109436], 'magnitude': 1.6617188453674316, 'distance': 14.134819984436035, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.668849733604304, 'motion_component': -1.1114401685326927}, {'ion': 2433, 'force': [-1.203117847442627, 1.369935154914856, -1.7334258556365967], 'magnitude': 2.515746593475342, 'distance': 11.48776626586914, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7877326239859699, 'motion_component': -1.9817355335246472}]}, 3012: {'frame': 3012, 'ionic_force': [-6.049041509628296, 7.594256043434143, -5.260452680289745], 'ionic_force_magnitude': 11.042463060386924, 'motion_vector': [0.3469734191894531, 0.20888900756835938, 0.08061981201171875], 'cosine_ionic_motion': -0.20539647540249492, 'ionic_motion_component': -2.2680829923657218, 'ionic_force_x': -6.049041509628296, 'ionic_force_y': 7.594256043434143, 'ionic_force_z': -5.260452680289745, 'radial_force': 9.708945773792445, 'axial_force': -5.260452680289745, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 130, 'contributions': [{'ion': 1305, 'force': [-3.265826940536499, 3.464674711227417, -1.8870964050292969], 'magnitude': 5.121594429016113, 'distance': 8.051308631896973, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.2655200365688773, 'motion_component': -1.3598859350726258}, {'ion': 1306, 'force': [-0.7231239676475525, 1.9537044763565063, 0.054674215614795685], 'magnitude': 2.0839526653289795, 'distance': 12.62191104888916, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.18779666302852827, 'motion_component': 0.39135935700082647}, {'ion': 1313, 'force': [-0.7049381136894226, 0.7514866590499878, -1.450873851776123], 'magnitude': 1.7795237302780151, 'distance': 13.658944129943848, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.2784067888137741, 'motion_component': -0.49543150066343955}, {'ion': 2433, 'force': [-1.3551524877548218, 1.424390196800232, -1.977156639099121], 'magnitude': 2.7882742881774902, 'distance': 10.911922454833984, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.28839512733415656, 'motion_component': -0.8041247477162372}]}, 3013: {'frame': 3013, 'ionic_force': [-6.196957647800446, 8.193085849285126, -5.1182726956903934], 'ionic_force_magnitude': 11.477179758539918, 'motion_vector': [-0.34819793701171875, 0.5365219116210938, -0.02915191650390625], 'cosine_ionic_motion': 0.9121231123486542, 'ionic_motion_component': 10.468600922344406, 'ionic_force_x': -6.196957647800446, 'ionic_force_y': 8.193085849285126, 'ionic_force_z': -5.1182726956903934, 'radial_force': 10.272727964001996, 'axial_force': -5.1182726956903934, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 130, 'contributions': [{'ion': 1305, 'force': [-3.3678054809570312, 3.507394313812256, -1.4226062297821045], 'magnitude': 5.066333770751953, 'distance': 8.095098495483398, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.9544057502036403, 'motion_component': 4.835338011528242}, {'ion': 1306, 'force': [-0.6791321635246277, 2.255999803543091, 0.028292980045080185], 'magnitude': 2.3561739921569824, 'distance': 11.870400428771973, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.9585375764212114, 'motion_component': 2.2584813529253673}, {'ion': 1313, 'force': [-0.7073150873184204, 0.8223105072975159, -1.570601224899292], 'magnitude': 1.9087371826171875, 'distance': 13.188517570495605, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5999946408263227, 'motion_component': 1.1452320455045228}, {'ion': 2433, 'force': [-1.4427049160003662, 1.6073812246322632, -2.153358221054077], 'magnitude': 3.049921751022339, 'distance': 10.433371543884277, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.7310185168992356, 'motion_component': 2.2295493729750344}]}, 3014: {'frame': 3014, 'ionic_force': [-5.128503501415253, 7.459451794624329, -4.494173161685467], 'ionic_force_magnitude': 10.106560327211557, 'motion_vector': [0.309356689453125, -0.4849357604980469, -0.06685638427734375], 'cosine_ionic_motion': -0.837833215388072, 'ionic_motion_component': -8.467611935461184, 'ionic_force_x': -5.128503501415253, 'ionic_force_y': 7.459451794624329, 'ionic_force_z': -4.494173161685467, 'radial_force': 9.052346062781329, 'axial_force': -4.494173161685467, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 130, 'contributions': [{'ion': 1305, 'force': [-2.8318116664886475, 3.483206033706665, -1.4415103197097778], 'magnitude': 4.714852333068848, 'distance': 8.391410827636719, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.9042290210606279, 'motion_component': -4.263306411882647}, {'ion': 1306, 'force': [-0.5754648447036743, 1.8000924587249756, 0.07871926575899124], 'magnitude': 1.8914780616760254, 'distance': 13.248551368713379, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.9643009774094256, 'motion_component': -1.8239541722865034}, {'ion': 1313, 'force': [-0.6226338744163513, 0.7984076738357544, -1.3830528259277344], 'magnitude': 1.7140486240386963, 'distance': 13.917379379272461, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.4909734898007002, 'motion_component': -0.8415524616936167}, {'ion': 2433, 'force': [-1.0985931158065796, 1.3777456283569336, -1.7483292818069458], 'magnitude': 2.482286214828491, 'distance': 11.564932823181152, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6199120152515205, 'motion_component': -1.5387990843100372}]}, 3015: {'frame': 3015, 'ionic_force': [-5.346394121646881, 8.012602269649506, -5.28259539976716], 'ionic_force_magnitude': 10.985970116162427, 'motion_vector': [0.23543930053710938, 0.47210693359375, -0.064453125], 'cosine_ionic_motion': 0.4906013195606233, 'ionic_motion_component': 5.389731435642861, 'ionic_force_x': -5.346394121646881, 'ionic_force_y': 8.012602269649506, 'ionic_force_z': -5.28259539976716, 'radial_force': 9.632534725375908, 'axial_force': -5.28259539976716, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 98, 'contributions': [{'ion': 1305, 'force': [-2.894195556640625, 3.707658052444458, -1.715484857559204], 'magnitude': 5.006593704223633, 'distance': 8.143251419067383, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.4432974937621314, 'motion_component': 2.219410615410636}, {'ion': 1306, 'force': [-0.6159889101982117, 2.011329174041748, -0.03404975309967995], 'magnitude': 2.1038172245025635, 'distance': 12.562180519104004, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.7214942822630875, 'motion_component': 1.5178920736121577}, {'ion': 1313, 'force': [-0.6359555721282959, 0.7825525403022766, -1.5352153778076172], 'magnitude': 1.836767315864563, 'distance': 13.444416999816895, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.32643658538632897, 'motion_component': 0.5995880553327027}, {'ion': 2433, 'force': [-1.2002540826797485, 1.511062502861023, -1.9978454113006592], 'magnitude': 2.777643918991089, 'distance': 10.932783126831055, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.37904081224136815, 'motion_component': 1.0528404274558927}]}, 3016: {'frame': 3016, 'ionic_force': [-4.702168673276901, 8.04951399564743, -5.281480491161346], 'ionic_force_magnitude': 10.714434281686943, 'motion_vector': [-0.16048431396484375, -0.3881187438964844, -0.0879364013671875], 'cosine_ionic_motion': -0.4143764525793021, 'ionic_motion_component': -4.439809269039499, 'ionic_force_x': -4.702168673276901, 'ionic_force_y': 8.04951399564743, 'ionic_force_z': -5.281480491161346, 'radial_force': 9.322288656658863, 'axial_force': -5.281480491161346, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 130, 'contributions': [{'ion': 1305, 'force': [-2.5992252826690674, 3.7571747303009033, -1.7314361333847046], 'magnitude': 4.885714530944824, 'distance': 8.24337387084961, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.42397427634892976, 'motion_component': -2.0714172232695276}, {'ion': 1306, 'force': [-0.4378458559513092, 1.8139464855194092, -0.1359662413597107], 'magnitude': 1.8709884881973267, 'distance': 13.320898056030273, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.7745085217710622, 'motion_component': -1.4490964747869315}, {'ion': 1313, 'force': [-0.6181272864341736, 0.8404967188835144, -1.470349669456482], 'magnitude': 1.80289888381958, 'distance': 13.570110321044922, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.12630974740547024, 'motion_component': -0.2277236970740173}, {'ion': 2433, 'force': [-1.046970248222351, 1.6378960609436035, -1.9437284469604492], 'magnitude': 2.7489871978759766, 'distance': 10.989620208740234, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.251573340095654, 'motion_component': -0.6915718852352448}]}, 3017: {'frame': 3017, 'ionic_force': [-5.671230614185333, 7.587991833686829, -5.028748389333487], 'ionic_force_magnitude': 10.725147416730229, 'motion_vector': [-0.14921188354492188, 0.14101409912109375, 0.17226409912109375], 'cosine_ionic_motion': 0.3652858024533034, 'ionic_motion_component': 3.9177440805502757, 'ionic_force_x': -5.671230614185333, 'ionic_force_y': 7.587991833686829, 'ionic_force_z': -5.028748389333487, 'radial_force': 9.473145029364375, 'axial_force': -5.028748389333487, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 130, 'contributions': [{'ion': 1305, 'force': [-3.1320512294769287, 3.454732894897461, -1.6151375770568848], 'magnitude': 4.934936046600342, 'distance': 8.202160835266113, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosi</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>6569</v>
+        <v>3045</v>
       </c>
       <c r="B4" t="n">
-        <v>6670</v>
+        <v>3171</v>
       </c>
       <c r="C4" t="n">
-        <v>1465</v>
+        <v>1305</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>{6569: {'frame': 6569, 'ionic_force': [8.93659296631813, 4.198592029511929, -11.964962244033813], 'ionic_force_magnitude': 15.51293622681027, 'motion_vector': [0.9375572204589844, 4.542621612548828, 3.9090347290039062], 'cosine_ionic_motion': -0.20531702194883455, 'ionic_motion_component': -3.185069867770875, 'ionic_force_x': 8.93659296631813, 'ionic_force_y': 4.198592029511929, 'ionic_force_z': -11.964962244033813, 'radial_force': 9.87374644579897, 'axial_force': -11.964962244033813, 'before_closest_residue': None, 'closest_residue': 455, 'next_closest_residue': 423, 'contributions': [{'ion': 1327, 'force': [2.5776994228363037, 1.23420250415802, -1.3029985427856445], 'magnitude': 3.1409544944763184, 'distance': 10.281067848205566, 'before_closest_residue': 1105, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.15377313307214993, 'motion_component': np.float64(0.4829944183947106)}, {'ion': 1330, 'force': [3.5478971004486084, -3.1198573112487793, -2.1965181827545166], 'magnitude': 5.210160732269287, 'distance': 7.982583522796631, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.6148617942807654, 'motion_component': np.float64(-3.20352882053065)}, {'ion': 1341, 'force': [1.5748634338378906, 5.740958213806152, -3.378621816635132], 'magnitude': 6.844989776611328, 'distance': 6.964383125305176, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.3455697276985564, 'motion_component': np.float64(2.365421161972364)}, {'ion': 1359, 'force': [1.0105098485946655, 0.24263377487659454, -3.6123909950256348], 'magnitude': 3.7589054107666016, 'distance': 9.398062705993652, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5294201717457786, 'motion_component': np.float64(-1.990040356360307)}, {'ion': 1374, 'force': [0.22562316060066223, 0.10065484791994095, -1.4744327068328857], 'magnitude': 1.494987964630127, 'distance': 14.902193069458008, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5618215292436758, 'motion_component': np.float64(-0.8399164247898128)}]}, 6570: {'frame': 6570, 'ionic_force': [12.36908807605505, 9.55480182170868, -1.3525466732680798], 'ionic_force_magnitude': 15.68814712414131, 'motion_vector': [0.08165740966796875, 0.8572654724121094, 0.46636962890625], 'cosine_ionic_motion': 0.5578220936822563, 'ionic_motion_component': 8.751195074783773, 'ionic_force_x': 12.36908807605505, 'ionic_force_y': 9.55480182170868, 'ionic_force_z': -1.3525466732680798, 'radial_force': 15.629733768856548, 'axial_force': -1.3525466732680798, 'before_closest_residue': 455, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1327, 'force': [1.5750916004180908, 1.4534358978271484, -0.05986563488841057], 'magnitude': 2.1440553665161133, 'distance': 12.443742752075195, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.6413605881302702, 'motion_component': np.float64(1.3751126016324602)}, {'ion': 1330, 'force': [8.851373672485352, -0.5448993444442749, 0.612082302570343], 'magnitude': 8.889227867126465, 'distance': 6.1113481521606445, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.06215821404243742, 'motion_component': np.float64(0.5525385419218214)}, {'ion': 1341, 'force': [-0.1118030920624733, 4.923777103424072, 3.27870774269104], 'magnitude': 5.9165873527526855, 'distance': 7.490889549255371, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.9908006826356204, 'motion_component': np.float64(5.862158742332892)}, {'ion': 1359, 'force': [1.5930393934249878, 2.9040167331695557, -3.243910789489746], 'magnitude': 4.636167049407959, 'distance': 8.462321281433105, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.24375800960093685, 'motion_component': np.float64(1.130102852027684)}, {'ion': 1374, 'force': [0.461386501789093, 0.8184714317321777, -1.9395602941513062], 'magnitude': 2.155148983001709, 'distance': 12.411674499511719, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.07828589813614696, 'motion_component': np.float64(-0.16871777346652062)}]}, 6571: {'frame': 6571, 'ionic_force': [10.874882698059082, 11.021745324134827, -1.573933221399784], 'ionic_force_magnitude': 15.563393250575485, 'motion_vector': [-0.7143974304199219, 2.6378211975097656, 0.46242523193359375], 'cosine_ionic_motion': 0.47700528588108876, 'ionic_motion_component': 7.423820846770567, 'ionic_force_x': 10.874882698059082, 'ionic_force_y': 11.021745324134827, 'ionic_force_z': -1.573933221399784, 'radial_force': 15.483602413089555, 'axial_force': -1.573933221399784, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1327, 'force': [0.9435465931892395, 1.386662483215332, -0.0861724391579628], 'magnitude': 1.6794459819793701, 'distance': 14.060022354125977, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.6324180818544546, 'motion_component': np.float64(1.0621119874398648)}, {'ion': 1330, 'force': [7.051734924316406, 1.6229393482208252, 0.9881018400192261], 'magnitude': 7.3032355308532715, 'distance': 6.742351531982422, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.014810253427721524, 'motion_component': np.float64(-0.10816276256291779)}, {'ion': 1341, 'force': [0.5937607288360596, 3.663236141204834, 2.101393938064575], 'magnitude': 4.264704704284668, 'distance': 8.82316780090332, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.8637998705639303, 'motion_component': np.float64(3.683851482704153)}, {'ion': 1359, 'force': [1.727159023284912, 3.332382917404175, -2.602457284927368], 'magnitude': 4.567344665527344, 'distance': 8.525839805603027, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5018376696551394, 'motion_component': np.float64(2.2920656488424704)}, {'ion': 1374, 'force': [0.5586814284324646, 1.0165244340896606, -1.9747992753982544], 'magnitude': 2.290257453918457, 'distance': 12.040011405944824, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.21567643245512247, 'motion_component': np.float64(0.49395454936455074)}]}, 6572: {'frame': 6572, 'ionic_force': [4.297864869236946, 8.788159370422363, -1.3208140432834625], 'ionic_force_magnitude': 9.871572179298408, 'motion_vector': [0.8923988342285156, -0.882781982421875, -0.6154251098632812], 'cosine_ionic_motion': -0.2253358702880056, 'ionic_motion_component': -2.2244193081330708, 'ionic_force_x': 4.297864869236946, 'ionic_force_y': 8.788159370422363, 'ionic_force_z': -1.3208140432834625, 'radial_force': 9.782810820728544, 'axial_force': -1.3208140432834625, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1330, 'force': [3.4389588832855225, 2.7700512409210205, 0.2946772277355194], 'magnitude': 4.425658702850342, 'distance': 8.661239624023438, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.07147438925554626, 'motion_component': np.float64(0.31632126731567206)}, {'ion': 1341, 'force': [-0.10774736106395721, 2.0299341678619385, 1.3322513103485107], 'magnitude': 2.430459976196289, 'distance': 11.687585830688477, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.7969983098200872, 'motion_component': np.float64(-1.9370725058540001)}, {'ion': 1359, 'force': [0.6919946074485779, 2.870731830596924, -1.4831961393356323], 'magnitude': 3.304516315460205, 'distance': 10.02340030670166, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.21730627483870296, 'motion_component': np.float64(-0.718092146719588)}, {'ion': 1374, 'force': [0.274658739566803, 1.1174421310424805, -1.4645464420318604], 'magnitude': 1.8625279664993286, 'distance': 13.351118087768555, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.06143491221927885, 'motion_component': np.float64(0.11442424533271733)}]}, 6573: {'frame': 6573, 'ionic_force': [6.707516558468342, 9.176944851875305, -0.19504992105066776], 'ionic_force_magnitude': 11.368603241743884, 'motion_vector': [-0.3231239318847656, -0.48430633544921875, 0.06146240234375], 'cosine_ionic_motion': -0.9952177524802688, 'ionic_motion_component': -11.314235767088245, 'ionic_force_x': 6.707516558468342, 'ionic_force_y': 9.176944851875305, 'ionic_force_z': -0.19504992105066776, 'radial_force': 11.366929893180817, 'axial_force': -0.19504992105066776, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1327, 'force': [0.9881269335746765, 1.1771571636199951, 0.006705602630972862], 'magnitude': 1.5369250774383545, 'distance': 14.697473526000977, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.9880008358344904, 'motion_component': np.float64(-1.5184832920336617)}, {'ion': 1330, 'force': [4.258534908294678, 1.36393404006958, 1.1857856512069702], 'magnitude': 4.62617826461792, 'distance': 8.471452713012695, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.7250604061209903, 'motion_component': np.float64(-3.354258527189531)}, {'ion': 1341, 'force': [-0.05445399135351181, 2.8371944427490234, 1.6453436613082886], 'magnitude': 3.28021240234375, 'distance': 10.060464859008789, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 'SF', 'cosine_with_motion': -0.6537031557818106, 'motion_component': np.float64(-2.144285189327313)}, {'ion': 1359, 'force': [1.1280900239944458, 2.8237078189849854, -1.7318087816238403], 'magnitude': 3.499296188354492, 'distance': 9.740442276000977, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8974276319060125, 'motion_component': np.float64(-3.14036519314781)}, {'ion': 1374, 'force': [0.3872186839580536, 0.9749513864517212, -1.301076054573059], 'magnitude': 1.67130708694458, 'distance': 14.094215393066406, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6921791202753821, 'motion_component': np.float64(-1.1568438766190443)}]}, 6574: {'frame': 6574, 'ionic_force': [9.922765731811523, 10.655503392219543, -1.8789063915610313], 'ionic_force_magnitude': 14.680985032969149, 'motion_vector': [0.2715606689453125, -0.07678985595703125, -0.05289459228515625], 'cosine_ionic_motion': 0.46872233966314086, 'ionic_motion_component': 6.881305653212853, 'ionic_force_x': 9.922765731811523, 'ionic_force_y': 10.655503392219543, 'ionic_force_z': -1.8789063915610313, 'radial_force': 14.560255228189348, 'axial_force': -1.8789063915610313, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1327, 'force': [0.8655595779418945, 1.3287379741668701, -0.031944431364536285], 'magnitude': 1.5861142873764038, 'distance': 14.467777252197266, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.29579496872987926, 'motion_component': np.float64(0.4691646168085734)}, {'ion': 1330, 'force': [6.645339488983154, 1.9468575716018677, 1.6377795934677124], 'magnitude': 7.115694999694824, 'distance': 6.830624103546143, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.7677054146793523, 'motion_component': np.float64(5.462757472369846)}, {'ion': 1341, 'force': [0.776921272277832, 3.7414114475250244, 0.194529190659523], 'magnitude': 3.826174020767212, 'distance': 9.315082550048828, 'before_closest_residue': 780, 'closest_residue': 'SF', 'next_closest_residue': 780, 'cosine_with_motion': -0.0788385563843854, 'motion_component': np.float64(-0.3016500388670462)}, {'ion': 1359, 'force': [1.2521162033081055, 2.632829427719116, -2.2195000648498535], 'magnitude': 3.664118766784668, 'distance': 9.518845558166504, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.24262122220108004, 'motion_component': np.float64(0.8889929729182668)}, {'ion': 1374, 'force': [0.3828291893005371, 1.005666971206665, -1.459770679473877], 'magnitude': 1.8135199546813965, 'distance': 13.530313491821289, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.19963431493602773, 'motion_component': np.float64(0.3620408168458269)}]}, 6575: {'frame': 6575, 'ionic_force': [6.102406769990921, 8.403478920459747, -1.6997588761150837], 'ionic_force_magnitude': 10.52364036776126, 'motion_vector': [-0.7413291931152344, 0.8488311767578125, 0.4405517578125], 'cosine_ionic_motion': 0.14609900437198084, 'ionic_motion_component': 1.5374933800987063, 'ionic_force_x': 6.102406769990921, 'ionic_force_y': 8.403478920459747, 'ionic_force_z': -1.6997588761150837, 'radial_force': 10.385462259959464, 'axial_force': -1.6997588761150837, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1330, 'force': [3.698859691619873, 1.877339243888855, -0.03207122161984444], 'magnitude': 4.148131370544434, 'distance': 8.94628620147705, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.2316347697950632, 'motion_component': np.float64(-0.96085146489291)}, {'ion': 1341, 'force': [0.6937668323516846, 2.8005433082580566, 1.644039273262024], 'magnitude': 3.320725917816162, 'distance': 9.998907089233398, 'before_closest_residue': 'SF', 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.6438655630588777, 'motion_component': np.float64(2.1381010385898946)}, {'ion': 1359, 'force': [1.2716120481491089, 2.7411482334136963, -1.8873075246810913], 'magnitude': 3.5626986026763916, 'distance': 9.653382301330566, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.12819220190672265, 'motion_component': np.float64(0.45671016417391286)}, {'ion': 1374, 'force': [0.4381681978702545, 0.9844481348991394, -1.4244194030761719], 'magnitude': 1.7860851287841797, 'distance': 13.633832931518555, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.05400995022278874, 'motion_component': np.float64(-0.09646636963300992)}]}, 6576: {'frame': 6576, 'ionic_force': [5.697530130855739, 9.966541528701782, -1.1423418633639812], 'ionic_force_magnitude': 11.536842920320106, 'motion_vector': [0.1239013671875, -0.14241409301757812, -0.3520050048828125], 'cosine_ionic_motion': -0.06756220567549721, 'ionic_motion_component': -0.7794545542285709, 'ionic_force_x': 5.697530130855739, 'ionic_force_y': 9.966541528701782, 'ionic_force_z': -1.1423418633639812, 'radial_force': 11.480148066786693, 'axial_force': -1.1423418633639812, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1327, 'force': [0.8476411700248718, 1.4078731536865234, 0.05625929310917854], 'magnitude': 1.6443136930465698, 'distance': 14.209431648254395, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.17552367847627473, 'motion_component': np.float64(-0.28861598567276614)}, {'ion': 1330, 'force': [3.670255661010742, 1.709186315536499, 0.31133517622947693], 'magnitude': 4.060667991638184, 'distance': 9.042120933532715, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.06273120196461206, 'motion_component': np.float64(0.25473058028006434)}, {'ion': 1341, 'force': [0.002328316681087017, 2.6095755100250244, 1.5804171562194824], 'magnitude': 3.050837278366089, 'distance': 10.431806564331055, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.7612668469814414, 'motion_component': np.float64(-2.322501282066058)}, {'ion': 1359, 'force': [0.9095866680145264, 3.105701446533203, -1.6332862377166748], 'magnitude': 3.624962568283081, 'distance': 9.570117950439453, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.16943698437349575, 'motion_component': np.float64(0.6142027188966424)}, {'ion': 1374, 'force': [0.2677183151245117, 1.1342051029205322, -1.4570672512054443], 'magnitude': 1.8657810688018799, 'distance': 13.339473724365234, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5159927105714089, 'motion_component': np.float64(0.9627294710664245)}]}, 6577: {'frame': 6577, 'ionic_force': [10.770041853189468, 11.033284544944763, -1.4359604306519032], 'ionic_force_magnitude': 15.48512679081343, 'motion_vector': [2.2769126892089844, -2.477092742919922, -0.91888427734375], 'cosine_ionic_motion': -0.027561089715659084, 'ionic_motion_component': -0.42678696873996497, 'ionic_force_x': 10.770041853189468, 'ionic_force_y': 11.033284544944763, 'ionic_force_z': -1.4359604306519032, 'radial_force': 15.41840359340648, 'axial_force': -1.4359604306519032, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1327, 'force': [1.0223180055618286, 1.2306550741195679, 0.052624136209487915], 'magnitude': 1.6007546186447144, 'distance': 14.401464462280273, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1105, 'cosine_with_motion': -0.13775037653817027, 'motion_component': np.float64(-0.22050455002434874)}, {'ion': 1330, 'force': [7.852027416229248, 3.727412223815918, 1.5429376363754272], 'magnitude': 8.827717781066895, 'distance': 6.132602691650391, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.23473986102912722, 'motion_component': np.float64(2.0722171355634664)}, {'ion': 1341, 'force': [0.4523809254169464, 1.9864200353622437, 0.05863363668322563], 'magnitude': 2.0381243228912354, 'distance': 12.76302719116211, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 'SF', 'cosine_with_motion': -0.5548802485993717, 'motion_component': np.float64(-1.1309149590530434)}, {'ion': 1359, 'force': [1.0853403806686401, 2.987722158432007, -1.669343113899231], 'magnitude': 3.5904252529144287, 'distance': 9.616036415100098, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.27116527483362757, 'motion_component': np.float64(-0.9735986645634576)}, {'ion': 1374, 'force': [0.3579751253128052, 1.1010750532150269, -1.420812726020813], 'magnitude': 1.832817792892456, 'distance': 13.458894729614258, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.09492783318420045, 'motion_component': np.float64(-0.17398542697419472)}]}, 6578: {'frame': 6578, 'ionic_force': [11.297083020210266, 8.097006872296333, -3.7768772915005684], 'ionic_force_magnitude': 14.40313879439443, 'motion_vector': [-1.2792587280273438, 0.96728515625, 1.4186248779296875], 'cosine_ionic_motion': -0.38838770907447234, 'ionic_motion_component': -5.59400207983651, 'ionic_force_x': 11.297083020210266, 'ionic_force_y': 8.097006872296333, 'ionic_force_z': -3.7768772915005684, 'radial_force': 13.899122456311304, 'axial_force': -3.7768772915005684, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1327, 'force': [1.3949049711227417, 1.2103791236877441, -0.1234259158372879], 'magnitude': 1.8509488105773926, 'distance': 13.392813682556152, 'before_closest_residue': 1073, 'closest_residue': 1105, 'next_closest_residue': 1073, 'cosine_with_motion': -0.19901993161504958, 'motion_component': np.float64(-0.3683757034914823)}, {'ion': 1330, 'force': [4.5826263427734375, 0.2037651091814041, 0.11392490565776825], 'magnitude': 4.588568687438965, 'distance': 8.506098747253418, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.5601713361052677, 'motion_component': np.float64(-2.57038469530253)}, {'ion': 1341, 'force': [2.695676326751709, 3.7334976196289062, 0.10549106448888779], 'magnitude': 4.606170177459717, 'distance': 8.48983097076416, 'before_closest_residue': 780, 'closest_residue': 'SF', 'next_closest_residue': 780, 'cosine_with_motion': 0.031689497765525536, 'motion_component': np.float64(0.1459672195302515)}, {'ion': 1359, 'force': [2.0399694442749023, 2.267669677734375, -2.4146974086761475], 'magnitude': 3.8903167247772217, 'distance': 9.237970352172852, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.46119819915256116, 'motion_component': np.float64(-1.7942070947055129)}, {'ion': 1374, 'force': [0.5839059352874756, 0.6816953420639038, -1.458169937133789], 'magnitude': 1.7122833728790283, 'distance': 13.924551963806152, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5881046115313526, 'motion_component': np.float64(-1.0070017301809386)}]}, 6579: {'frame': 6579, 'ionic_force': [9.608516097068787, 8.373697221279144, -1.9300379157066345], 'ionic_force_magnitude': 12.890594753437611, 'motion_vector': [2.924358367919922, -6.608238220214844, -2.4186172485351562], 'cosine_ionic_motion': -0.2297495323581236, 'ionic_motion_component': -2.9616081164203725, 'ionic_force_x': 9.608516097068787, 'ionic_force_y': 8.373697221279144, 'ionic_force_z': -1.9300379157066345, 'radial_force': 12.745288805723, 'axial_force': -1.9300379157066345, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 455, 'contributions': [{'ion': 1327, 'force': [1.3253157138824463, 1.562822699546814, 0.09811156988143921], 'magnitude': 2.0514633655548096, 'distance': 12.721465110778809, 'before_closest_residue': 1105, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.4278845029472088, 'motion_component': np.float64(-0.8777894316682975)}, {'ion': 1330, 'force': [5.451991558074951, 0.6885251402854919, 1.5081236362457275], 'magnitude': 5.698483943939209, 'distance': 7.632896900177002, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.17837929729573904, 'motion_component': np.float64(1.0164915061803086)}, {'ion': 1341, 'force': [0.3505029082298279, 1.43211030960083, 0.5435124635696411], 'magnitude': 1.5713682174682617, 'distance': 14.535503387451172, 'before_closest_residue': 'SF', 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.8145078473890567, 'motion_component': np.float64(-1.2798917314959368)}, {'ion': 1359, 'force': [1.873288631439209, 3.515359878540039, -2.291175127029419], 'magnitude': 4.595263957977295, 'distance': 8.499899864196777, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.3487003992758554, 'motion_component': np.float64(-1.6023703007219012)}, {'ion': 1374, 'force': [0.6074172854423523, 1.1748791933059692, -1.7886104583740234], 'magnitude': 2.2245054244995117, 'distance': 12.216654777526855, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.09802088427497478, 'motion_component': np.float64(-0.21804798582489582)}]}, 6580: {'frame': 6580, 'ionic_force': [9.401102423667908, 2.1901233000680804, -3.3302337273489684], 'ionic_force_magnitude': 10.211161712977045, 'motion_vector': [0.0558624267578125, 1.9655532836914062, -0.0980682373046875], 'cosine_ionic_motion': 0.25649892462915785, 'ionic_motion_component': 2.6191519985930416, 'ionic_force_x': 9.401102423667908, 'ionic_force_y': 2.1901233000680804, 'ionic_force_z': -3.3302337273489684, 'radial_force': 9.652842423338097, 'axial_force': -3.3302337273489684, 'before_closest_residue': 423, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1327, 'force': [1.994491696357727, 0.5432167649269104, -0.318158358335495], 'magnitude': 2.091484308242798, 'distance': 12.599164009094238, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1105, 'cosine_with_motion': 0.2939362459607358, 'motion_component': np.float64(0.6147630256647435)}, {'ion': 1330, 'force': [1.8411482572555542, -1.1111571788787842, 0.0030383423436433077], 'magnitude': 2.1504666805267334, 'distance': 12.425180435180664, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.4916330977797622, 'motion_component': np.float64(-1.0572405351031535)}, {'ion': 1341, 'force': [3.1475207805633545, 2.842928171157837, 0.6421310901641846], 'magnitude': 4.289692401885986, 'distance': 8.797432899475098, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.6750076766192781, 'motion_component': np.float64(2.89557522958656)}, {'ion': 1359, 'force': [1.743165135383606, -0.0841091051697731, -2.3038322925567627], 'magnitude': 2.8902149200439453, 'distance': 10.717759132385254, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.0277650151279751, 'motion_component': np.float64(0.08024686087711674)}, {'ion': 1374, 'force': [0.674776554107666, -0.0007553519681096077, -1.3534125089645386], 'magnitude': 1.5122994184494019, 'distance': 14.816655158996582, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.05673966670334128, 'motion_component': np.float64(0.08580736227417984)}]}, 6581: {'frame': 6581, 'ionic_force': [8.237632155418396, 2.801070511341095, -3.125244453549385], 'ionic_force_magnitude': 9.245092343072026, 'motion_vector': [-1.0904083251953125, 0.6786651611328125, -0.0248260498046875], 'cosine_ionic_motion': -0.589733052245308, 'ionic_motion_component': -5.452136525769592, 'ionic_force_x': 8.237632155418396, 'ionic_force_y': 2.801070511341095, 'ionic_force_z': -3.125244453549385, 'radial_force': 8.700837864107559, 'axial_force': -3.125244453549385, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1327, 'force': [1.5015419721603394, 0.9385555386543274, -0.21082422137260437], 'magnitude': 1.7832446098327637, 'distance': 13.644686698913574, 'before_closest_residue': 1073, 'closest_residue': 1105, 'next_closest_residue': 1105, 'cosine_with_motion': -0.434396371589925, 'motion_component': np.float64(-0.7746350255753975)}, {'ion': 1330, 'force': [2.607945680618286, -0.777786374092102, -0.1844618171453476], 'magnitude': 2.7277021408081055, 'distance': 11.032414436340332, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 780, 'cosine_with_motion': -0.9609020723946794, 'motion_component': np.float64(-2.621054553634242)}, {'ion': 1341, 'force': [1.963555932044983, 2.088361978530884, 0.7296456098556519], 'magnitude': 2.9579031467437744, 'distance': 10.594417572021484, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 'SF', 'cosine_with_motion': -0.1952496148674068, 'motion_component': np.float64(-0.5775294285032408)}, {'ion': 1359, 'force': [1.4981328248977661, 0.38405388593673706, -2.148705005645752], 'magnitude': 2.6474199295043945, 'distance': 11.198442459106445, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.38801482743793303, 'motion_component': np.float64(-1.0272382066311811)}, {'ion': 1374, 'force': [0.6664557456970215, 0.16788548231124878, -1.310899019241333], 'magnitude': 1.480136752128601, 'distance': 14.976768493652344, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.3051604361312931, 'motion_component': np.float64(-0.45167920050142335)}]}, 6582: {'frame': 6582, 'ionic_force': [13.439600765705109, 8.873755604028702, -5.538107115775347], 'ionic_force_magnitude': 17.03047379515243, 'motion_vector': [-3.5965843200683594, -4.00225830078125, 1.7977447509765625], 'cosine_ionic_motion': -0.9709190347276151, 'ionic_motion_component': -16.535211178143342, 'ionic_force_x': 13.439600765705109, 'ionic_force_y': 8.873755604028702, 'ionic_force_z': -5.538107115775347, 'radial_force': 16.104856635859015, 'axial_force': -5.538107115775347, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 'SF', 'contributions': [{'ion': 1327, 'force': [1.7381343841552734, 1.2546632289886475, -0.4241744577884674], 'magnitude': 2.1852266788482666, 'distance': 12.32596206665039, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 1105, 'cosine_with_motion': -0.9708103909504258, 'motion_component': np.float64(-2.1214406083064645)}, {'ion': 1330, 'force': [7.226672649383545, 3.7144134044647217, -0.0353500135242939], 'magnitude': 8.125448226928711, 'distance': 6.392126560211182, 'before_closest_residue': 98, 'closest_residue': 780, 'next_closest_residue': 130, 'cosine_with_motion': -0.8877053409310843, 'motion_component': np.float64(-7.213004075589314)}, {'ion': 1341, 'force': [2.3823862075805664, 2.991396427154541, -1.2005852460861206], 'magnitude': 4.008194446563721, 'distance': 9.101116180419922, 'before_closest_residue': 780, 'closest_residue': 'SF', 'next_closest_residue': 780, 'cosine_with_motion': -0.9982316294542771, 'motion_component': np.float64(-4.0011063288809225)}, {'ion': 1359, 'force': [1.5048085451126099, 0.7228309512138367, -2.4776906967163086], 'magnitude': 2.987621784210205, 'distance': 10.541592597961426, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7527915131617094, 'motion_component': np.float64(-2.249056399859022)}, {'ion': 1374, 'force': [0.587598979473114, 0.19045159220695496, -1.4003067016601562], 'magnitude': 1.5304911136627197, 'distance': 14.728333473205566, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6211101904690303, 'motion_component': np.float64(-0.950603663513693)}]}, 6583: {'frame': 6583, 'ionic_force': [16.05817210674286, 6.1076273918151855, 3.6224589943885803], 'ionic_force_magnitude': 17.558195036308607, 'motion_vector': [-2.217937469482422, 1.4410781860351562, 1.8284072875976562], 'cosine_ionic_motion': -0.35763561505257213, 'ionic_motion_component': -6.279435881023248, 'ionic_force_x': 16.05817210674286, 'ionic_force_y': 6.1076273918151855, 'ionic_force_z': 3.6224589943885803, 'radial_force': 17.180454119930168, 'axial_force': 3.6224589943885803, 'before_closest_residue': 455, 'closest_residue': 'SF', 'next_closest_residue': 'SF', 'contributions': [{'ion': 1327, 'force': [4.602260112762451, 2.496872901916504, -0.22734969854354858], 'magnitude': 5.2408833503723145, 'distance': 7.959151744842529, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 1105, 'cosine_with_motion': -0.41687272413751025, 'motion_component': np.float64(-2.1847813997755807)}, {'ion': 1330, 'force': [9.457734107971191, -11.10282039642334, 7.554731369018555], 'magnitude': 16.425447463989258, 'distance': 4.495835781097412, 'before_closest_residue': 780, 'closest_residue': 130, 'next_closest_residue': 98, 'cosine_with_motion': -0.43857960139192076, 'motion_component': np.float64(-7.203866159760764)}, {'ion': 1341, 'force': [-2.9511709213256836, 18.338525772094727, 8.4227876663208], 'magnitude': 20.394956588745117, 'distance': 4.034666538238525, 'before_closest_residue': 'SF', 'closest_residue': 780, 'next_closest_residue': 748, 'cosine_with_motion': 0.7376338138105843, 'motion_component': np.float64(15.044010246081827)}, {'ion': 1359, 'force': [4.432460308074951, -3.265843629837036, -9.403403282165527], 'magnitude': 10.896624565124512, 'distance': 5.519796371459961, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.9056182905666778, 'motion_component': np.flo</t>
+          <t>{3045: {'frame': 3045, 'ionic_force': [-7.627856880426407, -3.9306588172912598, -12.917159020900726], 'ionic_force_magnitude': 15.50765219165864, 'motion_vector': [1.7778701782226562, -4.606891632080078, 2.187591552734375], 'cosine_ionic_motion': -0.28309433045404925, 'ionic_motion_component': -4.390128414111872, 'ionic_force_x': -7.627856880426407, 'ionic_force_y': -3.9306588172912598, 'ionic_force_z': -12.917159020900726, 'radial_force': 8.581041855521857, 'axial_force': -12.917159020900726, 'before_closest_residue': None, 'closest_residue': 130, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [-7.494147300720215, -0.09124305844306946, -2.4212799072265625], 'magnitude': 7.876113414764404, 'distance': 6.49251651763916, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': -0.4278520200825079, 'motion_component': -3.3698111144211556}, {'ion': 1307, 'force': [1.882564663887024, -5.34438943862915, -0.9467782378196716], 'magnitude': 5.744818210601807, 'distance': 7.602053165435791, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.8346475560876673, 'motion_component': 4.794898548236267}, {'ion': 1313, 'force': [-0.4650546610355377, 0.3570297062397003, -2.9399447441101074], 'magnitude': 2.997836112976074, 'distance': 10.523618698120117, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5498720949982864, 'motion_component': -1.6484264043733088}, {'ion': 2433, 'force': [-1.5512195825576782, 1.1479439735412598, -6.609156131744385], 'magnitude': 6.885128974914551, 'distance': 6.944052696228027, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6051868537628935, 'motion_component': -4.166789600631844}]}, 3046: {'frame': 3046, 'ionic_force': [-4.8857167065143585, -18.394522786140442, -14.369192890822887], 'ionic_force_magnitude': 23.84748205995401, 'motion_vector': [-0.8094711303710938, 0.4755096435546875, -1.6446151733398438], 'cosine_ionic_motion': 0.41717989236882513, 'ionic_motion_component': 9.948689999039102, 'ionic_force_x': -4.8857167065143585, 'ionic_force_y': -18.394522786140442, 'ionic_force_z': -14.369192890822887, 'radial_force': 19.032306645967886, 'axial_force': -14.369192890822887, 'before_closest_residue': 130, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [-6.388330936431885, -8.717962265014648, -1.3706369400024414], 'magnitude': 10.894598960876465, 'distance': 5.5203094482421875, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': 0.15897644627497726, 'motion_component': 1.7319846067687479}, {'ion': 1307, 'force': [0.800718367099762, -2.2294273376464844, 0.10928446799516678], 'magnitude': 2.3713791370391846, 'distance': 11.832283020019531, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.4204262832769326, 'motion_component': -0.9969901381555366}, {'ion': 1313, 'force': [0.12471722066402435, -1.3755797147750854, -3.6492397785186768], 'magnitude': 3.9018874168395996, 'distance': 9.224263191223145, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.7100456131468871, 'motion_component': 2.7705179963943722}, {'ion': 1460, 'force': [0.05937342345714569, -0.4224264621734619, -1.7580629587173462], 'magnitude': 1.8090755939483643, 'distance': 13.546923637390137, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.7713140753705725, 'motion_component': 1.3953655077247875}, {'ion': 2433, 'force': [0.5178052186965942, -5.649127006530762, -7.70053768157959], 'magnitude': 9.564467430114746, 'distance': 5.8916730880737305, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5277672256931761, 'motion_component': 5.047812483426831}]}, 3047: {'frame': 3047, 'ionic_force': [-5.482337415218353, -11.13136899471283, -11.816646732389927], 'ionic_force_magnitude': 17.13465900532773, 'motion_vector': [-0.13234710693359375, -0.4849433898925781, 0.25323486328125], 'cosine_ionic_motion': 0.3246704946272977, 'ionic_motion_component': 5.563118214529835, 'ionic_force_x': -5.482337415218353, 'ionic_force_y': -11.13136899471283, 'ionic_force_z': -11.816646732389927, 'radial_force': 12.408198871341368, 'axial_force': -11.816646732389927, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [-5.219428062438965, -3.8420631885528564, -1.8072946071624756], 'magnitude': 6.728312969207764, 'distance': 7.024508953094482, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': 0.5535324012756235, 'motion_component': 3.7243391204070377}, {'ion': 1307, 'force': [0.780916154384613, -2.688171625137329, -0.1236976757645607], 'magnitude': 2.802034616470337, 'distance': 10.885096549987793, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.7411646170667333, 'motion_component': 2.076768893614846}, {'ion': 1313, 'force': [-0.18660974502563477, -0.9768067598342896, -3.0291600227355957], 'magnitude': 3.1882259845733643, 'distance': 10.204565048217773, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.1497302620196165, 'motion_component': -0.4773739157492827}, {'ion': 2433, 'force': [-0.8572157621383667, -3.6243274211883545, -6.856494426727295], 'magnitude': 7.80269718170166, 'distance': 6.522989273071289, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.030679655720089183, 'motion_component': 0.23938406446765192}]}, 3048: {'frame': 3048, 'ionic_force': [-4.429650291800499, -10.577412247657776, -9.8163231164217], 'ionic_force_magnitude': 15.095153231767606, 'motion_vector': [0.8934059143066406, 0.363006591796875, 0.44023895263671875], 'cosine_ionic_motion': -0.7573229373147555, 'ionic_motion_component': -11.431905784698568, 'ionic_force_x': -4.429650291800499, 'ionic_force_y': -10.577412247657776, 'ionic_force_z': -9.8163231164217, 'radial_force': 11.467495435558236, 'axial_force': -9.8163231164217, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [-4.9198431968688965, -3.9710214138031006, -1.8163729906082153], 'magnitude': 6.578227519989014, 'distance': 7.104190349578857, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': -0.9516949997528736, 'motion_component': -6.260466360037309}, {'ion': 1307, 'force': [1.057737112045288, -2.743105888366699, -0.21834583580493927], 'magnitude': 2.9480693340301514, 'distance': 10.612071990966797, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.04700579700139751, 'motion_component': -0.13857634721652135}, {'ion': 1313, 'force': [-0.11573232710361481, -0.6885260343551636, -2.368590831756592], 'magnitude': 2.469348907470703, 'distance': 11.59518814086914, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5333248119963518, 'motion_component': -1.3169651037053187}, {'ion': 2433, 'force': [-0.45181187987327576, -3.1747589111328125, -5.413013458251953], 'magnitude': 6.291576862335205, 'distance': 7.264225006103516, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5906146701407322, 'motion_component': -3.7158977529469213}]}, 3049: {'frame': 3049, 'ionic_force': [-5.144243225455284, -12.745068371295929, -11.233862489461899], 'ionic_force_magnitude': 17.751047084152233, 'motion_vector': [-0.10460281372070312, 0.37235260009765625, -0.3997344970703125], 'cosine_ionic_motion': 0.028663380638834744, 'ionic_motion_component': 0.508805019310933, 'ionic_force_x': -5.144243225455284, 'ionic_force_y': -12.745068371295929, 'ionic_force_z': -11.233862489461899, 'radial_force': 13.74408986261551, 'axial_force': -11.233862489461899, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [-6.307946681976318, -6.098640441894531, -1.9738773107528687], 'magnitude': 8.993319511413574, 'distance': 6.075877666473389, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': -0.16432461419422495, 'motion_component': -1.477823780834015}, {'ion': 1307, 'force': [1.0259054899215698, -2.4211580753326416, 0.04042556881904602], 'magnitude': 2.629852056503296, 'distance': 11.235783576965332, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.7007253444328082, 'motion_component': -1.8428041063405833}, {'ion': 1313, 'force': [0.05758988857269287, -0.733098566532135, -2.556490898132324], 'magnitude': 2.660149574279785, 'distance': 11.171616554260254, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.502104509603114, 'motion_component': 1.3356731029582463}, {'ion': 2433, 'force': [0.08020807802677155, -3.492171287536621, -6.743919849395752], 'magnitude': 7.594876289367676, 'distance': 6.611632347106934, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.32834762969437903, 'motion_component': 2.493759686266019}]}, 3050: {'frame': 3050, 'ionic_force': [-8.082814127206802, -15.125333547592163, -8.64464122056961], 'ionic_force_magnitude': 19.205140483038964, 'motion_vector': [-0.5727310180664062, -0.5838508605957031, -0.0329742431640625], 'cosine_ionic_motion': 0.8743827484308434, 'ionic_motion_component': 16.792643519560066, 'ionic_force_x': -8.082814127206802, 'ionic_force_y': -15.125333547592163, 'ionic_force_z': -8.64464122056961, 'radial_force': 17.149565567118334, 'axial_force': -8.64464122056961, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [-8.392095565795898, -9.305026054382324, -0.26266318559646606], 'magnitude': 12.533146858215332, 'distance': 5.146820068359375, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': 0.9989351899041049, 'motion_component': 12.519801422467488}, {'ion': 1307, 'force': [0.8371284604072571, -2.7453901767730713, -0.3088381290435791], 'magnitude': 2.886751174926758, 'distance': 10.724186897277832, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.47976534589531256, 'motion_component': 1.3849631697995441}, {'ion': 1313, 'force': [-0.11458709836006165, -0.5400526523590088, -2.306739091873169], 'magnitude': 2.3718838691711426, 'distance': 11.831024169921875, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.2353907559678917, 'motion_component': 0.5583194983065898}, {'ion': 2433, 'force': [-0.41325992345809937, -2.534864664077759, -5.7664008140563965], 'magnitude': 6.312503337860107, 'distance': 7.252173900604248, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.3690389427126593, 'motion_component': 2.329559633305248}]}, 3051: {'frame': 3051, 'ionic_force': [-4.67364265024662, -11.582442343235016, -10.405707761645317], 'ionic_force_magnitude': 16.256526697832268, 'motion_vector': [-0.0365142822265625, -0.6580581665039062, -0.04845428466796875], 'cosine_ionic_motion': 0.7722879480390109, 'ionic_motion_component': 12.55471964571028, 'ionic_force_x': -4.67364265024662, 'ionic_force_y': -11.582442343235016, 'ionic_force_z': -10.405707761645317, 'radial_force': 12.489832114827152, 'axial_force': -10.405707761645317, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [-4.849881649017334, -4.954220771789551, -1.6263054609298706], 'magnitude': 7.1211323738098145, 'distance': 6.8280158042907715, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': 0.7471442621257792, 'motion_component': 5.320513121167124}, {'ion': 1307, 'force': [0.7434349656105042, -2.424999952316284, -0.24432186782360077], 'magnitude': 2.5481390953063965, 'distance': 11.414515495300293, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.9385651746140502, 'motion_component': 2.3915947333268885}, {'ion': 1313, 'force': [-0.09479077160358429, -0.8810177445411682, -2.8076910972595215], 'magnitude': 2.9441988468170166, 'distance': 10.61904525756836, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.3696753588141691, 'motion_component': 1.088397765406719}, {'ion': 2433, 'force': [-0.47240519523620605, -3.3222038745880127, -5.727389335632324], 'magnitude': 6.638011455535889, 'distance': 7.072126865386963, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5655630955104707, 'motion_component': 3.754214211866548}]}, 3052: {'frame': 3052, 'ionic_force': [-5.209724634885788, -11.401874363422394, -7.101817240938544], 'ionic_force_magnitude': 14.407629155912385, 'motion_vector': [0.28638458251953125, 0.9398269653320312, -0.57830810546875], 'cosine_ionic_motion': -0.4931796418004406, 'ionic_motion_component': -7.105549386306454, 'ionic_force_x': -5.209724634885788, 'ionic_force_y': -11.401874363422394, 'ionic_force_z': -7.101817240938544, 'radial_force': 12.535707788976444, 'axial_force': -7.101817240938544, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [-5.312274932861328, -5.4468512535095215, -0.017082950100302696], 'magnitude': 7.608465194702148, 'distance': 6.605725288391113, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': -0.7644114075375801, 'motion_component': -5.815997726744576}, {'ion': 1307, 'force': [0.7433016300201416, -2.267305374145508, -0.2768886983394623], 'magnitude': 2.4020488262176514, 'distance': 11.756502151489258, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 130, 'cosine_with_motion': -0.6419187203279587, 'motion_component': -1.541920076696405}, {'ion': 1313, 'force': [-0.14602038264274597, -0.7283504605293274, -2.0909371376037598], 'magnitude': 2.2189714908599854, 'distance': 12.231878280639648, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.1908739736332039, 'motion_component': 0.423543905050515}, {'ion': 2433, 'force': [-0.49473094940185547, -2.959367275238037, -4.7169084548950195], 'magnitude': 5.590334415435791, 'distance': 7.7063751220703125, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.030619957291972134, 'motion_component': -0.17117580071300154}]}, 3053: {'frame': 3053, 'ionic_force': [-4.219432383775711, -10.548980951309204, -10.06429785490036], 'ionic_force_magnitude': 15.178099356127948, 'motion_vector': [-1.77386474609375, -1.6370887756347656, 1.1192703247070312], 'cosine_ionic_motion': 0.33402916994198817, 'ionic_motion_component': 5.069927929224444, 'ionic_force_x': -4.219432383775711, 'ionic_force_y': -10.548980951309204, 'ionic_force_z': -10.06429785490036, 'radial_force': 11.361540773695248, 'axial_force': -10.06429785490036, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [-4.823800563812256, -4.440138816833496, -1.7996982336044312], 'magnitude': 6.79873514175415, 'distance': 6.988033771514893, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': 0.7634985619750921, 'motion_component': 5.190824436402412}, {'ion': 1307, 'force': [0.8113200664520264, -2.4498634338378906, -0.3244946599006653], 'magnitude': 2.601032018661499, 'distance': 11.297860145568848, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 130, 'cosine_with_motion': 0.31908654428748695, 'motion_component': 0.8299543378530653}, {'ion': 1313, 'force': [-0.023798733949661255, -0.7062819004058838, -2.4791464805603027], 'magnitude': 2.577899932861328, 'distance': 11.34843635559082, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.2298233006701104, 'motion_component': -0.5924614584764551}, {'ion': 2433, 'force': [-0.1831531524658203, -2.9526968002319336, -5.460958480834961], 'magnitude': 6.210799694061279, 'distance': 7.311311721801758, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.0577042045711351, 'motion_component': -0.35838924755347534}]}, 3054: {'frame': 3054, 'ionic_force': [-4.988561183214188, -11.07318925857544, -6.662068283185363], 'ionic_force_magnitude': 13.852235084805852, 'motion_vector': [1.5704727172851562, 1.5061798095703125, 0.04151153564453125], 'cosine_ionic_motion': -0.822251706294983, 'ionic_motion_component': -11.39002393448084, 'ionic_force_x': -4.988561183214188, 'ionic_force_y': -11.07318925857544, 'ionic_force_z': -6.662068283185363, 'radial_force': 12.14500979970382, 'axial_force': -6.662068283185363, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [-3.5520873069763184, -3.771655559539795, -0.2791522443294525], 'magnitude': 5.188509941101074, 'distance': 7.999221324920654, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': -0.9981049002949264, 'motion_component': -5.1786772419558735}, {'ion': 1307, 'force': [0.37386640906333923, -2.273519277572632, -0.024842804297804832], 'magnitude': 2.3041882514953613, 'distance': 12.003560066223145, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 130, 'cosine_with_motion': -0.5659652843918243, 'motion_component': -1.3040905177746775}, {'ion': 1313, 'force': [-0.4952739477157593, -1.382063388824463, -2.4569201469421387], 'magnitude': 2.8621413707733154, 'distance': 10.770194053649902, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.47541701604638825, 'motion_component': -1.3607106166591176}, {'ion': 2433, 'force': [-1.3150663375854492, -3.64595103263855, -3.901153087615967], 'magnitude': 5.499214172363281, 'distance': 7.769958972930908, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6449186758546064, 'motion_component': -3.5465457642034988}]}, 3055: {'frame': 3055, 'ionic_force': [-5.847180061042309, -12.939044803380966, -12.562161590903997], 'ionic_force_magnitude': 18.958277847054948, 'motion_vector': [-1.2361679077148438, 1.7187881469726562, 1.0966033935546875], 'cosine_ionic_motion': -0.6368513991726591, 'ionic_motion_component': -12.07360577280097, 'ionic_force_x': -5.847180061042309, 'ionic_force_y': -12.939044803380966, 'ionic_force_z': -12.562161590903997, 'radial_force': 14.19888710745144, 'axial_force': -12.562161590903997, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 'SF', 'contributions': [{'ion': 1306, 'force': [-5.2452850341796875, -5.126814842224121, -0.8323266506195068], 'magnitude': 7.381735324859619, 'distance': 6.706405162811279, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': -0.18412155259469762, 'motion_component': -1.3591365284898842}, {'ion': 1307, 'force': [0.7029086351394653, -2.52593994140625, 0.032979581505060196], 'magnitude': 2.6221251487731934, 'distance': 11.252326011657715, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 98, 'cosine_with_motion': -0.827632780295384, 'motion_component': -2.170156805109472}, {'ion': 1313, 'force': [-0.2970026731491089, -1.1441336870193481, -3.2531378269195557], 'magnitude': 3.4612364768981934, 'distance': 9.793848991394043, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.626077286201467, 'motion_component': -2.1670015632897375}, {'ion': 1460, 'force': [-0.07392721623182297, -0.2998761832714081, -1.4589650630950928], 'magnitude': 1.4912981986999512, 'distance': 14.920618057250977, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5692107500329767, 'motion_component': -0.8488629082797575}, {'ion': 2433, 'force': [-0.9338737726211548, -3.842280149459839, -7.050711631774902], 'magnitude': 8.083796501159668, 'distance': 6.408573150634766, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6838925304956538, 'motion_component': -5.528448282595988}]}, 3057: {'frame': 3057, 'ionic_force': [-9.003431349992752, -5.540844574570656, -17.453158974647522], 'ionic_force_magnitude': 20.40528100438464, 'motion_vector': [1.1065635681152344, -1.9793701171875, 0.27787017822265625], 'cosine_ionic_motion': -0.08248170462513246, 'ionic_motion_component': -1.6830623605964803, 'ionic_force_x': -9.003431349992752, 'ionic_force_y': -5.540844574570656, 'ionic_force_z': -17.453158974647522, 'radial_force': 10.5717895681659, 'axial_force': -17.453158974647522, 'before_closest_residue': 'SF', 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [-11.65152359008789, -1.720420479774475, -5.61668586730957], 'magnitude': 13.048563003540039, 'distance': 5.044146537780762, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': -0.3706145430157077, 'motion_component': -4.835987388851706}, {'ion': 1307, 'force': [3.275055408477783, -4.9548420906066895, -1.0855175256729126], 'magnitude': 6.03778076171875, 'distance': 7.415328025817871, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.9518425280821092, 'motion_component': 5.747016491896808}, {'ion': 1313, 'force': [-0.13862550258636475, 0.2216983288526535, -3.2690048217773438], 'magnitude': 3.279444932937622, 'distance': 10.061641693115234, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.20028117554819103, 'motion_component': -0.6568111057233903}, {'ion': 2433, 'force': [-0.4883376657962799, 0.9127196669578552, -7.481950759887695], 'magnitude': 7.553218841552734, 'distance': 6.6298394203186035, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.2564841041419514, 'motion_component': -1.937280621807288}]}, 3058: {'frame': 3058, 'ionic_force': [-6.588992454111576, -12.504871994256973, -18.714533805847168], 'ionic_force_magnitude': 23.452514166359396, 'motion_vector': [-1.3784523010253906, -0.7992706298828125, 1.7841339111328125], 'cosine_ionic_motion': -0.25511064284589696, 'ionic_motion_component': -5.982985965332451, 'ionic_force_x': -6.588992454111576, 'ionic_force_y': -12.504871994256973, 'ionic_force_z': -18.714533805847168, 'radial_force': 14.134590377973169, 'axial_force': -18.714533805847168, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [-10.1950044631958, -6.432916641235352, -4.200505256652832], 'magnitude': 12.765766143798828, 'distance': 5.0997114181518555, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': 0.3831664836802652, 'motion_component': 4.891413600101089}, {'ion': 1307, 'force': [1.875774621963501, -2.822234869003296, -0.4788755178451538], 'magnitude': 3.422405958175659, 'distance': 9.849252700805664, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 130, 'cosine_with_motion': -0.14466313774177342, 'motion_component': -0.4950959698948765}, {'ion': 1313, 'force': [0.3185351490974426, -0.5011558532714844, -3.49147891998291], 'magnitude': 3.541616439819336, 'distance': 9.682071685791016, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7398358992935696, 'motion_component': -2.6202149703753186}, {'ion': 1460, 'force': [0.08552487939596176, -0.14446750283241272, -1.4719749689102173], 'magnitude': 1.481518030166626, 'distance': 14.969785690307617, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7417265424006055, 'motion_component': -1.0988812459595096}, {'ion': 2433, 'force': [1.3261773586273193, -2.6040971279144287, -9.071699142456055], 'magnitude': 9.530781745910645, 'distance': 5.90207576751709, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6988101593540155, 'motion_component': -6.660206849648084}]}, 3059: {'frame': 3059, 'ionic_force': [-6.022938176989555, -14.208095014095306, -16.89050218462944], 'ionic_force_magnitude': 22.878697783361055, 'motion_vector': [-1.1345634460449219, 2.811443328857422, 0.46810150146484375], 'cosine_ionic_motion': -0.5844382974303687, 'ionic_motion_component': -13.371187179931486, 'ionic_force_x': -6.022938176989555, 'ionic_force_y': -14.208095014095306, 'ionic_force_z': -16.89050218462944, 'radial_force': 15.431971624306408, 'axial_force': -16.89050218462944, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 'SF', 'contributions': [{'ion': 1306, 'force': [-6.254308223724365, -3.5317609310150146, 0.3269919455051422], 'magnitude': 7.190036773681641, 'distance': 6.795219421386719, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': -0.12152228533306414, 'motion_component': -0.8737497135220127}, {'ion': 1307, 'force': [1.462602138519287, -3.13942551612854, 0.3486194610595703], 'magnitude': 3.480909824371338, 'distance': 9.766133308410645, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 98, 'cosine_with_motion': -0.9666873695246327, 'motion_component': -3.364951549197073}, {'ion': 1313, 'force': [-0.20075920224189758, -0.7627044320106506, -3.709393262863159], 'magnitude': 3.7923107147216797, 'distance': 9.356578826904297, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.3139972571625627, 'motion_component': -1.1907751680909762}, {'ion': 1460, 'force': [-0.09766055643558502, -0.2889493703842163, -1.8270162343978882], 'magnitude': 1.8523006439208984, 'distance': 13.38792610168457, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.27397514647084603, 'motion_component': -0.5074843378754075}, {'ion': 2433, 'force': [-0.9328123331069946, -6.485254764556885, -12.029704093933105], 'magnitude': 13.698264122009277, 'distance': 4.923072814941406, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5427130449350271, 'motion_component': -7.434226807121489}]}, 3061: {'frame': 3061, 'ionic_force': [-5.298698872327805, -4.543317459523678, -15.510519742965698], 'ionic_force_magnitude': 17.0086497398985, 'motion_vector': [-0.8845176696777344, -3.617359161376953, 1.7931671142578125], 'cosine_ionic_motion': -0.09518324006510809, 'ionic_motion_component': -1.6189383913760973, 'ionic_force_x': -5.298698872327805, 'ionic_force_y': -4.543317459523678, 'ionic_force_z': -15.510519742965698, 'radial_force': 6.979824014802998, 'axial_force': -15.510519742965698, 'before_closest_residue': 'SF', 'closest_residue': 455, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [-7.535388469696045, -0.08941348642110825, -2.3861868381500244], 'magnitude': 7.904679775238037, 'distance': 6.480774402618408, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': 0.08294084820107507, 'motion_component': 0.6556208423691947}, {'ion': 1307, 'force': [3.745265483856201, -5.9981560707092285, -1.080502986907959], 'magnitude': 7.153486728668213, 'distance': 6.812556743621826, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.5562768670438354, 'motion_component': 3.9793193460797696}, {'ion': 1313, 'force': [-0.20985302329063416, 0.3536457419395447, -3.318143844604492], 'magnitude': 3.3435282707214355, 'distance': 9.964753150939941, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5096924092045565, 'motion_component': -1.7041710465112385}, {'ion': 2433, 'force': [-1.2987228631973267, 1.1906063556671143, -8.725686073303223], 'magnitude': 8.901787757873535, 'distance': 6.107035160064697, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.511100406859813, 'motion_component': -4.549707251045189}]}, 3062: {'frame': 3062, 'ionic_force': [-6.907819554209709, -11.125765323638916, -14.435852766036987], 'ionic_force_magnitude': 19.49088171717498, 'motion_vector': [0.18795394897460938, 2.1341514587402344, 0.134765625], 'cosine_ionic_motion': -0.6450252314842391, 'ionic_motion_component': -12.572110491452714, 'ionic_force_x': -6.907819554209709, 'ionic_force_y': -11.125765323638916, 'ionic_force_z': -14.435852766036987, 'radial_force': 13.09582471745129, 'axial_force': -14.435852766036987, 'before_closest_residue': 455, 'closest_residue': 780, 'next_closest_residue': 'SF', 'contributions': [{'ion': 1306, 'force': [-4.487196922302246, -1.7457993030548096, 0.17702478170394897], 'magnitude': 4.8180999755859375, 'distance': 8.301013946533203, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': -0.43946978448725904, 'motion_component': -2.1174094411245683}, {'ion': 1307, 'force': [1.4286413192749023, -4.030808925628662, 0.5166918635368347], 'magnitude': 4.307599067687988, 'distance': 8.779129028320312, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 130, 'cosine_with_motion': -0.8937279278418906, 'motion_component': -3.849821315695113}, {'ion': 1313, 'force': [-0.5085522532463074, -0.7536929845809937, -3.4217631816864014], 'magnitude': 3.5405001640319824, 'distance': 9.683597564697266, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.2848891740816516, 'motion_component': -1.0086501824259444}, {'ion': 1460, 'force': [-0.18697820603847504, -0.31573617458343506, -1.8348346948623657], 'magnitude': 1.8711676597595215, 'distance': 13.320259094238281, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.23806514249066815, 'motion_component': -0.4454598036881149}, {'ion': 2433, 'force': [-3.153733491897583, -4.279727935791016, -9.872971534729004], 'magnitude': 11.213281631469727, 'distance': 5.441300392150879, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.4593454307012366, 'motion_component': -5.15076943727812}]}, 3064: {'frame': 3064, 'ionic_force': [-4.365943253040314, -9.680663853883743, -10.61352539435029], 'ionic_force_magnitude': 15.01411450726209, 'motion_vector': [0.3384208679199219, 0.8003425598144531, 1.3289108276367188], 'cosine_ionic_motion': -0.9786286931020945, 'ionic_motion_component': -14.693243258327097, 'ionic_force_x': -4.365943253040314, 'ionic_force_y': -9.680663853883743, 'ionic_force_z': -10.61352539435029, 'radial_force': 10.61963808896798, 'axial_force': -10.61352539435029, 'before_closest_residue': 'SF', 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [-7.504685878753662, -4.338364124298096, 0.05125337466597557], 'magnitude': 8.668583869934082, 'distance': 6.188636302947998, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': -0.4318404125746951, 'motion_component': -3.7434446856817787}, {'ion': 1307, 'force': [2.084075927734375, -3.0866539478302, -0.5490327477455139], 'magnitude': 3.764603853225708, 'distance': 9.390947341918945, 'befo</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
+        <v>3185</v>
+      </c>
+      <c r="B5" t="n">
+        <v>3631</v>
+      </c>
+      <c r="C5" t="n">
+        <v>2433</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>{3185: {'frame': 3185, 'ionic_force': [10.830740660429, 0.3619977980852127, -26.339956998825073], 'ionic_force_magnitude': 28.48208771068656, 'motion_vector': [3.3021926879882812, 1.7625465393066406, 0.34154510498046875], 'cosine_ionic_motion': 0.2560077544719427, 'ionic_motion_component': 7.291635317485781, 'ionic_force_x': 10.830740660429, 'ionic_force_y': 0.3619977980852127, 'ionic_force_z': -26.339956998825073, 'radial_force': 10.83678853070819, 'axial_force': -26.339956998825073, 'before_closest_residue': None, 'closest_residue': 780, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [6.986976623535156, 8.647163391113281, -13.30506706237793], 'magnitude': 17.33828353881836, 'distance': 4.375885963439941, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.5181762863130486, 'motion_component': 8.984287532274934}, {'ion': 1307, 'force': [2.498210906982422, -7.074841499328613, -3.267333745956421], 'magnitude': 8.183514595031738, 'distance': 6.36940860748291, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.17347977213673554, 'motion_component': -1.4196742329862548}, {'ion': 1313, 'force': [1.0481852293014526, -0.9845649600028992, -6.827840805053711], 'magnitude': 6.9776411056518555, 'distance': 6.8978657722473145, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.023108002613043896, 'motion_component': -0.1612393407807282}, {'ion': 1460, 'force': [0.2973679006099701, -0.2257591336965561, -2.9397153854370117], 'magnitude': 2.963329553604126, 'distance': 10.584712982177734, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.03770713874789775, 'motion_component': -0.11173867455445306}]}, 3186: {'frame': 3186, 'ionic_force': [26.529620349407196, 4.835323363542557, -9.52608323097229], 'ionic_force_magnitude': 28.5997791886076, 'motion_vector': [-1.120147705078125, -0.510986328125, 0.8818283081054688], 'cosine_ionic_motion': -0.937113354825586, 'ionic_motion_component': -26.801235022707043, 'ionic_force_x': 26.529620349407196, 'ionic_force_y': 4.835323363542557, 'ionic_force_z': -9.52608323097229, 'radial_force': 26.966666607382177, 'axial_force': -9.52608323097229, 'before_closest_residue': 780, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [20.750598907470703, 6.123347282409668, -2.4909238815307617], 'magnitude': 21.778141021728516, 'distance': 3.9044389724731445, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.8662286238528618, 'motion_component': -18.86484937355354}, {'ion': 1307, 'force': [1.9073935747146606, -2.2411868572235107, -0.6840906143188477], 'magnitude': 3.0214316844940186, 'distance': 10.482446670532227, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.3484919334053558, 'motion_component': -1.0529445303036908}, {'ion': 1313, 'force': [2.8922908306121826, 0.682626485824585, -4.142235279083252], 'magnitude': 5.0979838371276855, 'distance': 8.069931030273438, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.9379406452351742, 'motion_component': -4.781606164194734}, {'ion': 1460, 'force': [0.9793370366096497, 0.2705364525318146, -2.2088334560394287], 'magnitude': 2.4313035011291504, 'distance': 11.685558319091797, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8644888675281329, 'motion_component': -2.101834725921859}]}, 3187: {'frame': 3187, 'ionic_force': [24.61393254995346, 7.588308960199356, -10.291718065738678], 'ionic_force_magnitude': 27.737115372614944, 'motion_vector': [-4.467868804931641, 3.94091796875, -0.4804229736328125], 'cosine_ionic_motion': -0.4531395888418963, 'ionic_motion_component': -12.568785055606977, 'ionic_force_x': 24.61393254995346, 'ionic_force_y': 7.588308960199356, 'ionic_force_z': -10.291718065738678, 'radial_force': 25.757098214843616, 'axial_force': -10.291718065738678, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 130, 'contributions': [{'ion': 1306, 'force': [18.267154693603516, 8.882265090942383, -0.8097184300422668], 'magnitude': 20.328285217285156, 'distance': 4.0412774085998535, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 1105, 'cosine_with_motion': -0.3804264390643056, 'motion_component': -7.733417511253199}, {'ion': 1307, 'force': [1.5217578411102295, -2.2949981689453125, -0.4252128601074219], 'magnitude': 2.786318302154541, 'distance': 10.915752410888672, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.939085122702101, 'motion_component': -2.6165900339826607}, {'ion': 1313, 'force': [3.834963321685791, 0.7111164927482605, -6.247584819793701], 'magnitude': 7.365116596221924, 'distance': 6.713967323303223, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.257383167032912, 'motion_component': -1.8956571041124768}, {'ion': 1460, 'force': [0.9900566935539246, 0.28992554545402527, -2.809201955795288], 'magnitude': 2.992638349533081, 'distance': 10.532752990722656, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.1079719114881787, 'motion_component': -0.32312089049107406}]}, 3188: {'frame': 3188, 'ionic_force': [11.80595587193966, -1.4899064302444458, -16.767672687768936], 'ionic_force_magnitude': 20.56101317020206, 'motion_vector': [2.9478530883789062, -1.2035942077636719, 0.8451919555664062], 'cosine_ionic_motion': 0.33104627786613133, 'ionic_motion_component': 6.806646879151897, 'ionic_force_x': 11.80595587193966, 'ionic_force_y': -1.4899064302444458, 'ionic_force_z': -16.767672687768936, 'radial_force': 11.89959727138151, 'axial_force': -16.767672687768936, 'before_closest_residue': 455, 'closest_residue': 130, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [0.704689621925354, 5.264189720153809, -0.24574843049049377], 'magnitude': 5.316829204559326, 'distance': 7.902102947235107, 'before_closest_residue': 780, 'closest_residue': 1105, 'next_closest_residue': 780, 'cosine_with_motion': -0.25499213983366775, 'motion_component': -1.355749664960884}, {'ion': 1307, 'force': [11.88012981414795, -11.49898910522461, -8.6984281539917], 'magnitude': 18.682260513305664, 'distance': 4.215550899505615, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.6744395164653703, 'motion_component': 12.600055276058924}, {'ion': 1313, 'force': [-0.5623465180397034, 3.5319478511810303, -5.200526714324951], 'magnitude': 6.311605930328369, 'distance': 7.252689838409424, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.49556723884648435, 'motion_component': -3.127825041783648}, {'ion': 1460, 'force': [-0.21651704609394073, 1.2129451036453247, -2.622969388961792], 'magnitude': 2.897944688796997, 'distance': 10.703454971313477, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.45198706097319374, 'motion_component': -1.3098335379862371}]}, 3189: {'frame': 3189, 'ionic_force': [12.04167953133583, 15.30772179365158, -8.939361959695816], 'ionic_force_magnitude': 21.429899315995037, 'motion_vector': [2.050933837890625, -1.666748046875, -0.683929443359375], 'cosine_ionic_motion': 0.09053688592584529, 'ionic_motion_component': 1.9401963497745927, 'ionic_force_x': 12.04167953133583, 'ionic_force_y': 15.30772179365158, 'ionic_force_z': -8.939361959695816, 'radial_force': 19.476354701206997, 'axial_force': -8.939361959695816, 'before_closest_residue': 130, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [4.522043704986572, 13.012672424316406, 0.44386425614356995], 'magnitude': 13.783161163330078, 'distance': 4.907887935638428, 'before_closest_residue': 1105, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.33801011862514263, 'motion_component': -4.658848022195346}, {'ion': 1307, 'force': [5.291672229766846, -1.454615592956543, -0.7079718708992004], 'magnitude': 5.5334367752075195, 'distance': 7.745893955230713, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.9110284388750086, 'motion_component': 5.041118525031655}, {'ion': 1313, 'force': [1.8297994136810303, 3.0413978099823, -6.2925825119018555], 'magnitude': 7.2246012687683105, 'distance': 6.778944969177246, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.15146603579443732, 'motion_component': 1.0942816903629335}, {'ion': 1460, 'force': [0.39816418290138245, 0.7082671523094177, -2.38267183303833], 'magnitude': 2.517399787902832, 'distance': 11.483993530273438, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.1841759707827572, 'motion_component': 0.4636445661517268}]}, 3190: {'frame': 3190, 'ionic_force': [15.530074954032898, 11.720041185617447, -13.903977543115616], 'ionic_force_magnitude': 23.913661053672072, 'motion_vector': [-0.8215522766113281, -0.8835487365722656, -0.6362762451171875], 'cosine_ionic_motion': -0.4374052493682637, 'ionic_motion_component': -10.459960876489568, 'ionic_force_x': 15.530074954032898, 'ionic_force_y': 11.720041185617447, 'ionic_force_z': -13.903977543115616, 'radial_force': 19.456171089668416, 'axial_force': -13.903977543115616, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [8.8020601272583, 11.90870189666748, -6.9365973472595215], 'magnitude': 16.352670669555664, 'distance': 4.505828857421875, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 1105, 'cosine_with_motion': -0.5980634379987716, 'motion_component': -9.779934223096902}, {'ion': 1307, 'force': [3.2317216396331787, -1.556819200515747, -0.28207412362098694], 'magnitude': 3.5982325077056885, 'distance': 9.605598449707031, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.22413212330142768, 'motion_component': -0.8064794737361263}, {'ion': 1313, 'force': [2.741168975830078, 1.0629887580871582, -4.5104899406433105], 'magnitude': 5.38409423828125, 'distance': 7.852586269378662, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.04375086242833566, 'motion_component': -0.23555877116258728}, {'ion': 1460, 'force': [0.7551242113113403, 0.3051697313785553, -2.174816131591797], 'magnitude': 2.3223190307617188, 'distance': 11.956610679626465, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.15588340078660728, 'motion_component': 0.36201101054708035}]}, 3191: {'frame': 3191, 'ionic_force': [17.29844206571579, 1.1133021712303162, -8.736418187618256], 'ionic_force_magnitude': 19.41135086423247, 'motion_vector': [1.4482460021972656, 0.2650604248046875, 0.5260162353515625], 'cosine_ionic_motion': 0.6837871147111805, 'ionic_motion_component': 13.273231600099901, 'ionic_force_x': 17.29844206571579, 'ionic_force_y': 1.1133021712303162, 'ionic_force_z': -8.736418187618256, 'radial_force': 17.334230286499363, 'axial_force': -8.736418187618256, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [10.922542572021484, 1.8332058191299438, -0.30494749546051025], 'magnitude': 11.079511642456055, 'distance': 5.4740495681762695, 'before_closest_residue': 780, 'closest_residue': 1105, 'next_closest_residue': 'SF', 'cosine_with_motion': 0.9319835102737098, 'motion_component': 10.325921923542372}, {'ion': 1307, 'force': [2.5171878337860107, -1.3357510566711426, -0.5809615254402161], 'magnitude': 2.9082610607147217, 'distance': 10.684454917907715, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.6566780693544112, 'motion_component': 1.9097911877108336}, {'ion': 1313, 'force': [2.9662954807281494, 0.4142634868621826, -5.240616798400879], 'magnitude': 6.036106586456299, 'distance': 7.416356086730957, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.17474385144598134, 'motion_component': 1.0547725824270096}, {'ion': 1460, 'force': [0.8924161791801453, 0.20158392190933228, -2.6098923683166504], 'magnitude': 2.7656068801879883, 'distance': 10.956549644470215, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.006238752915845556, 'motion_component': -0.01725393739331782}]}, 3192: {'frame': 3192, 'ionic_force': [14.277701735496521, 1.8772609233856201, -9.105208367109299], 'ionic_force_magnitude': 17.037655203423625, 'motion_vector': [-1.4279060363769531, -0.3152008056640625, 0.24273681640625], 'cosine_ionic_motion': -0.918206633239828, 'ionic_motion_component': -15.644088022636645, 'ionic_force_x': 14.277701735496521, 'ionic_force_y': 1.8772609233856201, 'ionic_force_z': -9.105208367109299, 'radial_force': 14.400585940241147, 'axial_force': -9.105208367109299, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [7.416618824005127, 2.3804314136505127, -2.2368931770324707], 'magnitude': 8.104096412658691, 'distance': 6.40054178237915, 'before_closest_residue': 1105, 'closest_residue': 'SF', 'next_closest_residue': 1105, 'cosine_with_motion': -0.9892522383075535, 'motion_component': -8.016995571557597}, {'ion': 1307, 'force': [2.5377702713012695, -1.3266432285308838, -0.38498708605766296], 'magnitude': 2.8893728256225586, 'distance': 10.719320297241211, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.7702711774946917, 'motion_component': -2.225600600174946}, {'ion': 1313, 'force': [3.2284295558929443, 0.5756868124008179, -4.195573329925537], 'magnitude': 5.325129985809326, 'distance': 7.895941734313965, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7360294220437638, 'motion_component': -3.919452270043964}, {'ion': 1460, 'force': [1.0948830842971802, 0.24778592586517334, -2.287754774093628], 'magnitude': 2.548330545425415, 'distance': 11.41408634185791, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5815727327514694, 'motion_component': -1.4820395787670382}]}, 3193: {'frame': 3193, 'ionic_force': [24.2664697766304, -1.6357786357402802, -8.331860184669495], 'ionic_force_magnitude': 25.70908830165204, 'motion_vector': [-1.265380859375, 0.5024642944335938, 1.421234130859375], 'cosine_ionic_motion': -0.8571266292121383, 'ionic_motion_component': -22.035944196112233, 'ionic_force_x': 24.2664697766304, 'ionic_force_y': -1.6357786357402802, 'ionic_force_z': -8.331860184669495, 'radial_force': 24.32154039458153, 'axial_force': -8.331860184669495, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [16.86561393737793, 0.2729170322418213, 1.6130274534225464], 'magnitude': 16.94477081298828, 'distance': 4.426405429840088, 'before_closest_residue': 'SF', 'closest_residue': 1105, 'next_closest_residue': 1105, 'cosine_with_motion': -0.5670766966533437, 'motion_component': -9.608984940162713}, {'ion': 1307, 'force': [2.8553409576416016, -2.6237025260925293, -0.7594399452209473], 'magnitude': 3.9513967037200928, 'distance': 9.166293144226074, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.772899017180589, 'motion_component': -3.0540306336895497}, {'ion': 1313, 'force': [3.558159112930298, 0.47408899664878845, -6.336966037750244], 'magnitude': 7.283020973205566, 'distance': 6.751701831817627, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.9258083810288427, 'motion_component': -6.74268190178226}, {'ion': 1460, 'force': [0.9873557686805725, 0.2409178614616394, -2.8484816551208496], 'magnitude': 3.0243611335754395, 'distance': 10.477368354797363, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8696867439300969, 'motion_component': -2.630246830321605}]}, 3194: {'frame': 3194, 'ionic_force': [19.346414268016815, 3.2443795204162598, -13.397719025611877], 'ionic_force_magnitude': 23.75518087894646, 'motion_vector': [1.2636222839355469, 1.3273963928222656, -1.654449462890625], 'cosine_ionic_motion': 0.8681636639582825, 'ionic_motion_component': 20.623384869857894, 'ionic_force_x': 19.346414268016815, 'ionic_force_y': 3.2443795204162598, 'ionic_force_z': -13.397719025611877, 'radial_force': 19.616568086753123, 'axial_force': -13.397719025611877, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [8.542722702026367, 4.372759819030762, 4.92852258682251], 'magnitude': 10.788394927978516, 'distance': 5.547414302825928, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 780, 'cosine_with_motion': 0.31705288259328784, 'motion_component': 3.4204918480876074}, {'ion': 1307, 'force': [3.671895742416382, -4.1611647605896, 0.1399139165878296], 'magnitude': 5.55136775970459, 'distance': 7.73337459564209, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.08135725777908503, 'motion_component': -0.45164407550161195}, {'ion': 1313, 'force': [5.728073596954346, 2.3258800506591797, -12.010092735290527], 'magnitude': 13.507882118225098, 'distance': 4.957644939422607, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.9053912250945034, 'motion_component': 12.229917716004195}, {'ion': 1387, 'force': [0.3024868369102478, 0.18391072750091553, -1.7984228134155273], 'magnitude': 1.832933783531189, 'distance': 13.45846939086914, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.7958791628889741, 'motion_component': 1.4587937625408287}, {'ion': 1460, 'force': [1.1012353897094727, 0.5229936838150024, -4.657639980316162], 'magnitude': 4.814545631408691, 'distance': 8.3040771484375, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.8237175571334348, 'motion_component': 3.965825965203912}]}, 3195: {'frame': 3195, 'ionic_force': [13.184819161891937, 8.239660143852234, -7.467395126819611], 'ionic_force_magnitude': 17.247998306992876, 'motion_vector': [-2.6438636779785156, 0.3204536437988281, -0.75738525390625], 'cosine_ionic_motion': -0.5562117951564536, 'ionic_motion_component': -9.59354010118798, 'ionic_force_x': 13.184819161891937, 'ionic_force_y': 8.239660143852234, 'ionic_force_z': -7.467395126819611, 'radial_force': 15.547715446906654, 'axial_force': -7.467395126819611, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 130, 'contributions': [{'ion': 1306, 'force': [5.561399459838867, 6.935168266296387, 1.1953492164611816], 'magnitude': 8.969647407531738, 'distance': 6.083889961242676, 'before_closest_residue': 1105, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.5390119401823071, 'motion_component': -4.83474729128271}, {'ion': 1307, 'force': [3.3571889400482178, -1.2759623527526855, -0.45971280336380005], 'magnitude': 3.6207916736602783, 'distance': 9.575628280639648, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.891410116498306, 'motion_component': -3.2276104534812227}, {'ion': 1313, 'force': [3.318345785140991, 1.9544174671173096, -5.576297760009766], 'magnitude': 6.776891708374023, 'distance': 6.99928617477417, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.20910020006651614, 'motion_component': -1.4170494408500325}, {'ion': 1460, 'force': [0.9478849768638611, 0.6260367631912231, -2.6267337799072266], 'magnitude': 2.8618416786193848, 'distance': 10.770756721496582, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.039881000971897285, 'motion_component': -0.11413311435657825}]}, 3196: {'frame': 3196, 'ionic_force': [6.619435306638479, 22.22155737876892, -13.786656141281128], 'ionic_force_magnitude': 26.975663544658474, 'motion_vector': [2.318988800048828, -2.4310836791992188, 0.22534942626953125], 'cosine_ionic_motion': -0.4599428152577477, 'ionic_motion_component': -12.407262634176012, 'ionic_force_x': 6.619435306638479, 'ionic_force_y': 22.22155737876892, 'ionic_force_z': -13.786656141281128, 'radial_force': 23.186516256580926, 'axial_force': -13.786656141281128, 'before_closest_residue': 455, 'closest_residue': 130, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [0.034611787647008896, 21.819107055664062, -3.03163743019104], 'magnitude': 22.02874183654785, 'distance': 3.882166862487793, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.72322729482525, 'motion_component': -15.931787191027345}, {'ion': 1307, 'force': [5.983163833618164, -2.2468509674072266, -2.4435293674468994], 'magnitude': 6.8423261642456055, 'distance': 6.965738296508789, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.8153833541846309, 'motion_component': 5.57911868908799}, {'ion': 1313, 'force': [0.49341556429862976, 2.0448687076568604, -5.6436381340026855], 'magnitude': 6.022922515869141, 'distance': 7.424468994140625, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.25140903765843836, 'motion_component': -1.5142172100840625}, {'ion': 1460, 'force': [0.10824412107467651, 0.6044325828552246, -2.667851209640503], 'magnitude': 2.7376058101654053, 'distance': 11.01244068145752, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.19739042068930143, 'motion_component': -0.5403771640603434}]}, 3197: {'frame': 3197, 'ionic_force': [16.769740521907806, 8.663859937340021, -10.408290982246399], 'ionic_force_magnitude': 21.555026962568938, 'motion_vector': [-2.359294891357422, 1.4584197998046875, 2.7145614624023438], 'cosine_ionic_motion': -0.6596524489721276, 'ionic_motion_component': -14.218826323518842, 'ionic_force_x': 16.769740521907806, 'ionic_force_y': 8.663859937340021, 'ionic_force_z': -10.408290982246399, 'radial_force': 18.87555737418003, 'axial_force': -10.408290982246399, 'before_closest_residue': 130, 'closest_residue': 455, 'next_closest_residue': 'SF', 'contributions': [{'ion': 1306, 'force': [11.251453399658203, 10.151823997497559, -1.6383306980133057], 'magnitude': 15.242666244506836, 'distance': 4.667008399963379, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 455, 'cosine_with_motion': -0.2736331120025268, 'motion_component': -4.170898085845295}, {'ion': 1307, 'force': [2.6972978115081787, -1.6630486249923706, -0.5784024000167847], 'magnitude': 3.221132516860962, 'distance': 10.15230655670166, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.8286611706385422, 'motion_component': -2.6692275525959843}, {'ion': 1313, 'force': [2.2362687587738037, 0.05940436199307442, -5.672110557556152], 'magnitude': 6.097315788269043, 'distance': 7.379036903381348, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8699706879091497, 'motion_component': -5.304486381330342}, {'ion': 1460, 'force': [0.5847205519676208, 0.11568020284175873, -2.5194473266601562], 'magnitude': 2.5889949798583984, 'distance': 11.32409381866455, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8011659975708844, 'motion_component': -2.074214723975322}]}, 3199: {'frame': 3199, 'ionic_force': [14.122706681489944, 14.297301888465881, -19.076298475265503], 'ionic_force_magnitude': 27.708642132351915, 'motion_vector': [-0.02933502197265625, -3.176746368408203, 1.2943191528320312], 'cosine_ionic_motion': -0.741947855331392, 'ionic_motion_component': -20.55836760424355, 'ionic_force_x': 14.122706681489944, 'ionic_force_y': 14.297301888465881, 'ionic_force_z': -19.076298475265503, 'radial_force': 20.09636000128707, 'axial_force': -19.076298475265503, 'before_closest_residue': 'SF', 'closest_residue': 455, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [7.464374542236328, 14.71654224395752, -7.845605373382568], 'magnitude': 18.271480560302734, 'distance': 4.262674331665039, 'before_closest_residue': 455, 'closest_residue': 780, 'next_closest_residue': 1105, 'cosine_with_motion': -0.9113801568702047, 'motion_component': -16.652265436172176}, {'ion': 1307, 'force': [5.674992561340332, -3.5322635173797607, -1.162170171737671], 'magnitude': 6.784767150878906, 'distance': 6.995223045349121, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.4103351210578211, 'motion_component': 2.784028260604713}, {'ion': 1313, 'force': [0.8440772891044617, 2.4483911991119385, -7.0417280197143555], 'magnitude': 7.502867221832275, 'distance': 6.652048587799072, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6572728715675435, 'motion_component': -4.931431210428519}, {'ion': 1460, 'force': [0.13926228880882263, 0.6646319627761841, -3.026794910430908], 'magnitude': 3.102034330368042, 'distance': 10.345362663269043, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5669501891312683, 'motion_component': -1.7586989570614022}]}, 3200: {'frame': 3200, 'ionic_force': [23.99060034006834, -11.85288804769516, -7.261751040816307], 'ionic_force_magnitude': 27.72675400992476, 'motion_vector': [-0.7101936340332031, -1.3734970092773438, -0.6399917602539062], 'cosine_ionic_motion': 0.08382402509668414, 'ionic_motion_component': 2.324168123977521, 'ionic_force_x': 23.99060034006834, 'ionic_force_y': -11.85288804769516, 'ionic_force_z': -7.261751040816307, 'radial_force': 26.75892112451625, 'axial_force': -7.261751040816307, 'before_closest_residue': 455, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [20.544967651367188, -4.489597320556641, 7.865688323974609], 'magnitude': 22.45264434814453, 'distance': 3.8453447818756104, 'before_closest_residue': 780, 'closest_residue': 1105, 'next_closest_residue': 130, 'cosine_with_motion': -0.35818913633595006, 'motion_component': -8.042293243506492}, {'ion': 1307, 'force': [1.905739426612854, -3.4375593662261963, -0.18530522286891937], 'magnitude': 3.9348437786102295, 'distance': 9.185552597045898, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.529496981001851, 'motion_component': 2.0834878760571067}, {'ion': 1313, 'force': [1.2463655471801758, -3.3982043266296387, -10.489591598510742], 'magnitude': 11.096519470214844, 'distance': 5.469852924346924, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5652003166871671, 'motion_component': 6.2717565039260705}, {'ion': 1387, 'force': [0.09594348818063736, -0.13932183384895325, -1.5808546543121338], 'magnitude': 1.5898796319961548, 'distance': 14.450634956359863, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.4265788497944352, 'motion_component': 0.6782090140143298}, {'ion': 1460, 'force': [0.19758422672748566, -0.3882052004337311, -2.871687889099121], 'magnitude': 2.9045369625091553, 'distance': 10.691302299499512, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.45894008835435396, 'motion_component': 1.3330083846379597}]}, 3201: {'frame': 3201, 'ionic_force': [3.3897135043516755, -15.518092513084412, -10.52552792429924], 'ionic_force_magnitude': 19.054870531479178, 'motion_vector': [-0.7017936706542969, -0.01294708251953125, -0.8671646118164062], 'cosine_ionic_motion': 0.3269012310977347, 'ionic_motion_component': 6.22906063514849, 'ionic_force_x': 3.3897135043516755, 'ionic_force_y': -15.518092513084412, 'ionic_force_z': -10.52552792429924, 'radial_force': 15.883996754162052, 'axial_force': -10.52552792429924, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [1.4242832660675049, -7.873991966247559, 0.3762785792350769], 'magnitude': 8.010612487792969, 'distance': 6.437780380249023, 'before_closest_residue': 1105, 'closest_residue': 130, 'next_closest_residue': 455, 'cosine_with_motion': -0.13694827961881867, 'motion_component': -1.0970396454494633}, {'ion': 1307, 'force': [1.5798676013946533, -2.8936667442321777, -0.3859957754611969], 'magnitude': 3.3193798065185547, 'distance': 10.000934600830078, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.19889472880136572, 'motion_component': -0.6602071255352406}, {'ion': 1313, 'force': [0.3916058838367462, -3.7393531799316406, -7.343410015106201], 'magnitude': 8.249957084655762, 'distance': 6.343708038330078, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.6672680685827019, 'motion_component': 5.504932773013024}, {'ion': 1460, 'force': [-0.0060432469472289085, -1.0110806226730347, -3.172400712966919], 'magnitude': 3.3296315670013428, 'distance': 9.985526084899902, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.74524006733559, 'motion_component': 2.4813749044541478}]}, 3202: {'frame': 3202, 'ionic_force': [-2.182297945022583, -26.892607748508453, -10.45144271850586], 'ionic_force_magnitude': 28.93453698841915, 'motion_vector': [-0.6875076293945312, -0.4496726989746094, -0.5331268310546875], 'cosine_ionic_motion': 0.6763396079114743, 'ionic_motion_component': 19.569573401847457, 'ionic_force_x': -2.182297945022583, 'ionic_force_y': -26.892607748508453, 'ionic_force_z': -10.45144271850586, 'radial_force': 26.98100768755657, 'axial_force': -10.45144271850586, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [-2.2925589084625244, -21.295202255249023, -2.3005130290985107], 'magnitude': 21.541444778442383, 'distance': 3.9258313179016113, 'before_closest_residue': 130, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': 0.5867615343101018, 'motion_component': 12.63969095104963}, {'ion': 1307, 'force': [0.9534668922424316, -2.877516031265259, -0.7578949928283691], 'magnitude': 3.124676465988159, 'distance': 10.307812690734863, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.34066776310849783, 'motion_component': 1.0644765109163643}, {'ion': 1313, 'force': [-0.6528485417366028, -2.2744596004486084, -5.246335506439209], 'magnitude': 5.755294322967529, 'distance': 7.595130920410156, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.7573262503904421, 'motion_component': 4.358635548107902}, {'ion': 1460, 'force': [-0.19035738706588745, -0.44542986154556274, -2.1466991901397705], 'magnitude': 2.2006728649139404, 'distance': 12.282628059387207, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.6846863323502752, 'motion_component': 1.5067706405058947}]}, 3203: {'frame': 3203, 'ionic_force': [-7.816598609089851, -23.334227353334427, -7.66998678445816], 'ionic_force_magnitude': 25.77623085841855, 'motion_vector': [-1.41168212890625, -0.13762283325195312, 1.837890625], 'cosine_ionic_motion': 0.0024945814596701796, 'ionic_motion_component': 0.0643</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>3320</v>
+      </c>
+      <c r="B6" t="n">
+        <v>3666</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1313</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>{3320: {'frame': 3320, 'ionic_force': [14.295079827308655, -1.2250978574156761, -4.31649112701416], 'ionic_force_magnitude': 14.982732316869418, 'motion_vector': [-0.18167495727539062, 0.760711669921875, 0.7443389892578125], 'cosine_ionic_motion': -0.41676853918356793, 'ionic_motion_component': -6.244331460680102, 'ionic_force_x': 14.295079827308655, 'ionic_force_y': -1.2250978574156761, 'ionic_force_z': -4.31649112701416, 'radial_force': 14.347479640319108, 'axial_force': -4.31649112701416, 'before_closest_residue': None, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [6.963980674743652, -2.6537961959838867, 4.944848537445068], 'magnitude': 8.943778991699219, 'distance': 6.092681884765625, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 130, 'cosine_with_motion': 0.04107998871961835, 'motion_component': 0.36741035270695477}, {'ion': 1307, 'force': [2.457754135131836, -1.7556523084640503, -0.6207482814788818], 'magnitude': 3.0835366249084473, 'distance': 10.376346588134766, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.6740548894571412, 'motion_component': -2.078473018494627}, {'ion': 1387, 'force': [0.3318135738372803, -0.0069795772433280945, -1.9514002799987793], 'magnitude': 1.9794220924377441, 'distance': 12.950896263122559, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7103326722280674, 'motion_component': -1.4060482193826478}, {'ion': 1460, 'force': [1.624815821647644, -0.2846843898296356, -5.312528133392334], 'magnitude': 5.562735557556152, 'distance': 7.725468635559082, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7435987748913293, 'motion_component': -4.1364433416914}, {'ion': 2433, 'force': [2.916715621948242, 3.4760146141052246, -1.3766629695892334], 'magnitude': 4.741846561431885, 'distance': 8.367491722106934, 'before_closest_residue': 780, 'closest_residue': 1105, 'next_closest_residue': 1073, 'cosine_with_motion': 0.21283327257076928, 'motion_component': 1.0092227157837357}]}, 3321: {'frame': 3321, 'ionic_force': [12.688717484474182, 1.7846734374761581, -5.118914902210236], 'ionic_force_magnitude': 13.798257152818387, 'motion_vector': [3.44659423828125, 0.5642127990722656, -0.29720306396484375], 'cosine_ionic_motion': 0.9565169362411797, 'ionic_motion_component': 13.198266657281787, 'ionic_force_x': 12.688717484474182, 'ionic_force_y': 1.7846734374761581, 'ionic_force_z': -5.118914902210236, 'radial_force': 12.813610368636693, 'axial_force': -5.118914902210236, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [4.35039758682251, -0.736777126789093, 5.709558963775635], 'magnitude': 7.215806484222412, 'distance': 6.783074855804443, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 1105, 'cosine_with_motion': 0.5093081050382515, 'motion_component': 3.6750687282516354}, {'ion': 1307, 'force': [3.376248836517334, -2.3066442012786865, -0.3063477873802185], 'magnitude': 4.100428581237793, 'distance': 8.998174667358398, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.7254307926115434, 'motion_component': 2.974576987167009}, {'ion': 1387, 'force': [0.4181758165359497, 0.16234956681728363, -2.319929599761963], 'magnitude': 2.362901210784912, 'distance': 11.853490829467773, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.26833152479280165, 'motion_component': 0.6340408627544847}, {'ion': 1460, 'force': [2.362652540206909, 0.5963982939720154, -7.155970096588135], 'magnitude': 7.559479236602783, 'distance': 6.62709379196167, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.40029079586086974, 'motion_component': 3.0259899505259265}, {'ion': 2433, 'force': [2.1812427043914795, 4.069346904754639, -1.0462263822555542], 'magnitude': 4.734130859375, 'distance': 8.374307632446289, 'before_closest_residue': 1105, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.6101627710360925, 'motion_component': 2.8885903144106857}]}, 3322: {'frame': 3322, 'ionic_force': [11.341214001178741, 1.8453324884176254, -4.039094507694244], 'ionic_force_magnitude': 12.179600627911743, 'motion_vector': [-1.1910209655761719, 1.1273345947265625, 1.091339111328125], 'cosine_ionic_motion': -0.6600153827601511, 'ionic_motion_component': -8.038723770296945, 'ionic_force_x': 11.341214001178741, 'ionic_force_y': 1.8453324884176254, 'ionic_force_z': -4.039094507694244, 'radial_force': 11.490360612850333, 'axial_force': -4.039094507694244, 'before_closest_residue': 780, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [4.151607990264893, 0.16926394402980804, 1.5174075365066528], 'magnitude': 4.423462867736816, 'distance': 8.663389205932617, 'before_closest_residue': 130, 'closest_residue': 1105, 'next_closest_residue': 1105, 'cosine_with_motion': -0.3555124022849969, 'motion_component': -1.5725959538139396}, {'ion': 1307, 'force': [2.0877387523651123, -0.7246052622795105, -0.22269701957702637], 'magnitude': 2.2211034297943115, 'distance': 12.226007461547852, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.81055964865176, 'motion_component': -1.8003367063631615}, {'ion': 1387, 'force': [0.8166144490242004, 0.16744935512542725, -1.7120360136032104], 'magnitude': 1.904196858406067, 'distance': 13.204231262207031, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7070687055580778, 'motion_component': -1.3463980228761798}, {'ion': 1460, 'force': [2.6996209621429443, 0.5092499852180481, -3.1144349575042725], 'magnitude': 4.152949810028076, 'distance': 8.941094398498535, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7383261436332469, 'motion_component': -3.066231583865708}, {'ion': 2433, 'force': [1.5856318473815918, 1.7239744663238525, -0.5073340535163879], 'magnitude': 2.3966026306152344, 'distance': 11.769852638244629, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.10563347096891086, 'motion_component': -0.2531614541572438}]}, 3323: {'frame': 3323, 'ionic_force': [11.9672349691391, 4.672180593013763, -4.230508267879486], 'ionic_force_magnitude': 13.525575200519821, 'motion_vector': [-0.09119033813476562, -1.4596443176269531, 0.58355712890625], 'cosine_ionic_motion': -0.487367887250709, 'ionic_motion_component': -6.59193100932793, 'ionic_force_x': 11.9672349691391, 'ionic_force_y': 4.672180593013763, 'ionic_force_z': -4.230508267879486, 'radial_force': 12.8469445511499, 'axial_force': -4.230508267879486, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [3.659790277481079, 1.3112963438034058, 3.027434825897217], 'magnitude': 4.927364826202393, 'distance': 8.208459854125977, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 1105, 'cosine_with_motion': -0.062005492091044195, 'motion_component': -0.3055236837241404}, {'ion': 1307, 'force': [2.6004390716552734, -0.6885156631469727, -0.16605886816978455], 'magnitude': 2.695164680480957, 'distance': 11.098809242248535, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.15809894751483966, 'motion_component': 0.4261027016091869}, {'ion': 1387, 'force': [0.8393199443817139, 0.3989105820655823, -2.18998122215271], 'magnitude': 2.3789925575256348, 'distance': 11.813334465026855, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5170273796606956, 'motion_component': -1.2300042650106304}, {'ion': 1460, 'force': [3.4794766902923584, 1.5985596179962158, -4.6523637771606445], 'magnitude': 6.02549934387207, 'distance': 7.422881603240967, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5655173853401619, 'motion_component': -3.4075245058578427}, {'ion': 2433, 'force': [1.3882089853286743, 2.0519297122955322, -0.24953922629356384], 'magnitude': 2.4899415969848633, 'distance': 11.547141075134277, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.8333453521952254, 'motion_component': -2.0749813240573336}]}, 3324: {'frame': 3324, 'ionic_force': [16.31632697582245, 2.8348719850182533, -6.47797042876482], 'ionic_force_magnitude': 17.78266363707485, 'motion_vector': [1.4581718444824219, 0.5040359497070312, -1.6050872802734375], 'cosine_ionic_motion': 0.8996778240846612, 'ionic_motion_component': 15.99866812743293, 'ionic_force_x': 16.31632697582245, 'ionic_force_y': 2.8348719850182533, 'ionic_force_z': -6.47797042876482, 'radial_force': 16.560767649882436, 'axial_force': -6.47797042876482, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [4.176307678222656, 1.1397384405136108, 3.9005496501922607], 'magnitude': 5.827077865600586, 'distance': 7.548203945159912, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 1105, 'cosine_with_motion': 0.031104389140727738, 'motion_component': 0.18124769924062178}, {'ion': 1307, 'force': [2.713325262069702, -1.90458083152771, -0.050729237496852875], 'magnitude': 3.315438985824585, 'distance': 10.006875991821289, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.41699078061401385, 'motion_component': 1.3825074850180004}, {'ion': 1316, 'force': [0.5152910947799683, 0.09902171045541763, -1.5304564237594604], 'magnitude': 1.617908239364624, 'distance': 14.32491683959961, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.9044381588025899, 'motion_component': 1.4632979506664054}, {'ion': 1387, 'force': [1.6848300695419312, 0.3395357131958008, -3.116074562072754], 'magnitude': 3.558631420135498, 'distance': 9.658897399902344, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.9629840296835332, 'motion_component': 3.4269052191387033}, {'ion': 1460, 'force': [5.295093536376953, 0.8498631119728088, -5.482320308685303], 'magnitude': 7.6691670417785645, 'distance': 6.579531192779541, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.9926726186717297, 'motion_component': 7.612971853423932}, {'ion': 2433, 'force': [1.9314793348312378, 2.311293840408325, -0.19893954694271088], 'magnitude': 3.018653392791748, 'distance': 10.487269401550293, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 780, 'cosine_with_motion': 0.6399335650787177, 'motion_component': 1.9317376565473425}]}, 3325: {'frame': 3325, 'ionic_force': [13.136695861816406, 2.739805907011032, -4.366748213768005], 'ionic_force_magnitude': 14.111973800160023, 'motion_vector': [-1.0484428405761719, -1.0520210266113281, -0.158599853515625], 'cosine_ionic_motion': -0.7572853651263232, 'ionic_motion_component': -10.68679123190729, 'ionic_force_x': 13.136695861816406, 'ionic_force_y': 2.739805907011032, 'ionic_force_z': -4.366748213768005, 'radial_force': 13.419363419102892, 'axial_force': -4.366748213768005, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [4.4394755363464355, 0.9520545601844788, 1.6842352151870728], 'magnitude': 4.842726230621338, 'distance': 8.27988052368164, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 1105, 'cosine_with_motion': -0.8188536297992145, 'motion_component': -3.965484107521733}, {'ion': 1307, 'force': [2.6720001697540283, -1.5414988994598389, -0.5172479152679443], 'magnitude': 3.1278345584869385, 'distance': 10.302607536315918, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.23495398785767055, 'motion_component': -0.7348972083134715}, {'ion': 1387, 'force': [1.0765461921691895, 0.23434945940971375, -2.0206117630004883], 'magnitude': 2.3014655113220215, 'distance': 12.010658264160156, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.3068244551499629, 'motion_component': -0.7061458862244105}, {'ion': 1460, 'force': [2.5632970333099365, 0.5630773901939392, -3.0066704750061035], 'magnitude': 3.9909415245056152, 'distance': 9.120766639709473, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.47019937350483226, 'motion_component': -1.8765382588053043}, {'ion': 2433, 'force': [2.3853769302368164, 2.5318233966827393, -0.506453275680542], 'magnitude': 3.515202283859253, 'distance': 9.718379974365234, 'before_closest_residue': 1073, 'closest_residue': 780, 'next_closest_residue': 1073, 'cosine_with_motion': -0.9682872249034437, 'motion_component': -3.403725551910478}]}, 3326: {'frame': 3326, 'ionic_force': [13.417050004005432, 2.1709354370832443, -3.8333840072155], 'ionic_force_magnitude': 14.121792535961626, 'motion_vector': [0.80645751953125, 0.5555877685546875, -0.410614013671875], 'cosine_ionic_motion': 0.906934222177686, 'ionic_motion_component': 12.80753692935701, 'ionic_force_x': 13.417050004005432, 'ionic_force_y': 2.1709354370832443, 'ionic_force_z': -3.8333840072155, 'radial_force': 13.591548531420766, 'axial_force': -3.8333840072155, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [5.361866474151611, 1.3586233854293823, 3.1420536041259766], 'magnitude': 6.361443996429443, 'distance': 7.224223613739014, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 780, 'cosine_with_motion': 0.5608614287527562, 'motion_component': 3.567888600576474}, {'ion': 1307, 'force': [2.534034490585327, -1.4627076387405396, -0.48265519738197327], 'magnitude': 2.9654343128204346, 'distance': 10.580955505371094, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.4538269625285481, 'motion_component': 1.3457940323652586}, {'ion': 1387, 'force': [0.7306075096130371, 0.05163702368736267, -1.8644970655441284], 'magnitude': 2.0031981468200684, 'distance': 12.873809814453125, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.6503710687869672, 'motion_component': 1.3028221533939597}, {'ion': 1460, 'force': [2.9076755046844482, 0.214521124958992, -4.017284393310547], 'magnitude': 4.963785648345947, 'distance': 8.178290367126465, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.7804168984028671, 'motion_component': 3.873822364127798}, {'ion': 2433, 'force': [1.8828660249710083, 2.008861541748047, -0.6110009551048279], 'magnitude': 2.820289134979248, 'distance': 10.849812507629395, 'before_closest_residue': 780, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.9634508776201375, 'motion_component': 2.7172101317688018}]}, 3327: {'frame': 3327, 'ionic_force': [21.70894306898117, 0.4854571521282196, -6.7340773940086365], 'ionic_force_magnitude': 22.734592060719194, 'motion_vector': [-0.40179443359375, 0.5124359130859375, 0.6054840087890625], 'cosine_ionic_motion': -0.6208785499721065, 'ionic_motion_component': -14.115420552866697, 'ionic_force_x': 21.70894306898117, 'ionic_force_y': 0.4854571521282196, 'ionic_force_z': -6.7340773940086365, 'radial_force': 21.714370306753498, 'axial_force': -6.7340773940086365, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [14.490052223205566, -0.3445451557636261, -0.7261050343513489], 'magnitude': 14.512324333190918, 'distance': 4.783001899719238, 'before_closest_residue': 1105, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.49893008150847756, 'motion_component': -7.240635089633331}, {'ion': 1307, 'force': [2.2564868927001953, -1.2306782007217407, -0.5171406269073486], 'magnitude': 2.62178111076355, 'distance': 11.25306510925293, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.7937460924658793, 'motion_component': -2.0810285370827515}, {'ion': 1387, 'force': [0.7123898863792419, 0.10276107490062714, -1.644201397895813], 'magnitude': 1.7948418855667114, 'distance': 13.600533485412598, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7701518053219849, 'motion_component': -1.382300725170892}, {'ion': 1460, 'force': [2.544466972351074, 0.2279723435640335, -3.2194597721099854], 'magnitude': 4.109890937805176, 'distance': 8.987810134887695, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7812058518484315, 'motion_component': -3.2106709714302584}, {'ion': 2433, 'force': [1.7055470943450928, 1.7299470901489258, -0.6271705627441406], 'magnitude': 2.508974075317383, 'distance': 11.503260612487793, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.0800267830802497, 'motion_component': -0.20078512136664983}]}, 3328: {'frame': 3328, 'ionic_force': [13.955669224262238, 4.043034732341766, -8.50230523943901], 'ionic_force_magnitude': 16.834370428635996, 'motion_vector': [-1.1094818115234375, 0.8973617553710938, 1.1634902954101562], 'cosine_ionic_motion': -0.7016568818364415, 'ionic_motion_component': -11.811951862636331, 'ionic_force_x': 13.955669224262238, 'ionic_force_y': 4.043034732341766, 'ionic_force_z': -8.50230523943901, 'radial_force': 14.529515936325684, 'axial_force': -8.50230523943901, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [5.705695152282715, 2.9352493286132812, -1.6938565969467163], 'magnitude': 6.636248588562012, 'distance': 7.073066234588623, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 1105, 'cosine_with_motion': -0.4638195022348238, 'motion_component': -3.0780215391998595}, {'ion': 1307, 'force': [2.587146282196045, -1.5906908512115479, -0.39483076333999634], 'magnitude': 3.0625994205474854, 'distance': 10.411755561828613, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.8436581708710822, 'motion_component': -2.58378694130705}, {'ion': 1387, 'force': [0.7809037566184998, 0.18411484360694885, -1.7854108810424805], 'magnitude': 1.9573965072631836, 'distance': 13.023557662963867, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7709661628922033, 'motion_component': -1.5090864508773922}, {'ion': 1460, 'force': [3.093663454055786, 0.4853256046772003, -4.167239665985107], 'magnitude': 5.21269416809082, 'distance': 7.9806437492370605, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8174437983446711, 'motion_component': -4.261084555910353}, {'ion': 2433, 'force': [1.788260579109192, 2.029035806655884, -0.4609673321247101], 'magnitude': 2.7436022758483887, 'distance': 11.000399589538574, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.1384938768402133, 'motion_component': -0.3799721065212349}]}, 3329: {'frame': 3329, 'ionic_force': [22.60821044445038, 6.519129231572151, -6.981471963226795], 'ionic_force_magnitude': 24.543251133698966, 'motion_vector': [0.8754844665527344, -1.0129776000976562, 0.6521530151367188], 'cosine_ionic_motion': 0.2362819368794032, 'ionic_motion_component': 5.799126915188, 'ionic_force_x': 22.60821044445038, 'ionic_force_y': 6.519129231572151, 'ionic_force_z': -6.981471963226795, 'radial_force': 23.529348172834997, 'axial_force': -6.981471963226795, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [12.494484901428223, 2.5334689617156982, 1.6158926486968994], 'magnitude': 12.850748062133789, 'distance': 5.082821369171143, 'before_closest_residue': 780, 'closest_residue': 1105, 'next_closest_residue': 130, 'cosine_with_motion': 0.4925345760540134, 'motion_component': 6.329437772286681}, {'ion': 1307, 'force': [3.9902992248535156, -1.354427695274353, 0.10097753256559372], 'magnitude': 4.215110778808594, 'distance': 8.874921798706055, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.7855641559571375, 'motion_component': 3.3112399291110663}, {'ion': 1316, 'force': [0.37819957733154297, 0.24994249641895294, -1.4104505777359009], 'magnitude': 1.4815117120742798, 'distance': 14.969817161560059, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.38158253503441575, 'motion_component': -0.5653190013484792}, {'ion': 1387, 'force': [0.9713860750198364, 0.7008095979690552, -2.4578428268432617], 'magnitude': 2.734175682067871, 'distance': 11.019346237182617, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.35913446296586105, 'motion_component': -0.9819366955576072}, {'ion': 1460, 'force': [3.2983713150024414, 2.064893960952759, -4.52915096282959], 'magnitude': 5.971285343170166, 'distance': 7.456501483917236, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.2426363541558891, 'motion_component': -1.4488509092765014}, {'ion': 2433, 'force': [1.4754693508148193, 2.324441909790039, -0.3008977770805359], 'magnitude': 2.7695810794830322, 'distance': 10.948685646057129, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1105, 'cosine_with_motion': -0.3052609156370647, 'motion_component': -0.8454448625147428}]}, 3330: {'frame': 3330, 'ionic_force': [14.08597069978714, 0.9935656264424324, -8.829362889751792], 'ionic_force_magnitude': 16.654110370963554, 'motion_vector': [1.0237197875976562, -1.2902107238769531, 0.8571853637695312], 'cosine_ionic_motion': 0.18012324317505612, 'ionic_motion_component': 2.9997923722132924, 'ionic_force_x': 14.08597069978714, 'ionic_force_y': 0.9935656264424324, 'ionic_force_z': -8.829362889751792, 'radial_force': 14.120968210760541, 'axial_force': -8.829362889751792, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [2.8815765380859375, -0.5539013743400574, 0.1647612750530243], 'magnitude': 2.9389514923095703, 'distance': 10.628520965576172, 'before_closest_residue': 1105, 'closest_residue': 130, 'next_closest_residue': 1105, 'cosine_with_motion': 0.6974414307672064, 'motion_component': 2.0497465908190193}, {'ion': 1307, 'force': [2.641782283782959, -1.9233834743499756, 0.02791181392967701], 'magnitude': 3.267904043197632, 'distance': 10.07939338684082, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.8586513054862651, 'motion_component': 2.8059900542559966}, {'ion': 1316, 'force': [0.5562570691108704, 0.11473546177148819, -1.4796452522277832], 'magnitude': 1.5849088430404663, 'distance': 14.47327709197998, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.28779764622325893, 'motion_component': -0.4561330512855037}, {'ion': 1387, 'force': [1.3070932626724243, 0.29501739144325256, -2.6750640869140625], 'magnitude': 2.9919052124023438, 'distance': 10.53404426574707, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.24041965554896735, 'motion_component': -0.7193127855523347}, {'ion': 1460, 'force': [4.905503273010254, 1.0822356939315796, -4.953392505645752], 'magnitude': 7.054877281188965, 'distance': 6.8600029945373535, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.04736466428845592, 'motion_component': -0.33415189509761234}, {'ion': 2433, 'force': [1.7937582731246948, 1.978861927986145, 0.0860658660531044], 'magnitude': 2.672240734100342, 'distance': 11.146313667297363, 'before_closest_residue': 1073, 'closest_residue': 1105, 'next_closest_residue': 780, 'cosine_with_motion': -0.12960900139424755, 'motion_component': -0.3463464546020445}]}, 3331: {'frame': 3331, 'ionic_force': [19.05224919319153, 0.7009375113993883, -4.944461226463318], 'ionic_force_magnitude': 19.69586782892171, 'motion_vector': [-1.5520782470703125, 0.7276382446289062, -2.8383560180664062], 'cosine_ionic_motion': -0.23008541103372485, 'ionic_motion_component': -4.531731845083369, 'ionic_force_x': 19.05224919319153, 'ionic_force_y': 0.7009375113993883, 'ionic_force_z': -4.944461226463318, 'radial_force': 19.06513867545563, 'axial_force': -4.944461226463318, 'before_closest_residue': 455, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [4.111640453338623, 0.03262225165963173, 1.5308387279510498], 'magnitude': 4.387495994567871, 'distance': 8.698826789855957, 'before_closest_residue': 130, 'closest_residue': 1105, 'next_closest_residue': 780, 'cosine_with_motion': -0.7356891080593785, 'motion_component': -3.2278328084017662}, {'ion': 1307, 'force': [2.2052574157714844, -1.7059963941574097, 0.4966766834259033], 'magnitude': 2.8320083618164062, 'distance': 10.827340126037598, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.646809959823399, 'motion_component': -1.831771252770979}, {'ion': 1316, 'force': [0.7236177921295166, -0.01991807110607624, -1.514197587966919], 'magnitude': 1.6783366203308105, 'distance': 14.064668655395508, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5678690160279444, 'motion_component': 0.9530753588752279}, {'ion': 1387, 'force': [2.3421452045440674, -0.13869722187519073, -2.969356060028076], 'magnitude': 3.784435987472534, 'distance': 9.366308212280273, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.3739069185928592, 'motion_component': 1.4150268355639988}, {'ion': 1460, 'force': [6.530500888824463, -0.4096313416957855, -3.7830898761749268], 'magnitude': 7.558241367340088, 'distance': 6.627636432647705, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.01212381215447484, 'motion_component': 0.09163469545941672}, {'ion': 2433, 'force': [3.139087438583374, 2.9425582885742188, 1.2946668863296509], 'magnitude': 4.4931817054748535, 'distance': 8.595913887023926, 'before_closest_residue': 1105, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.42995467800748755, 'motion_component': -1.931864480817218}]}, 3332: {'frame': 3332, 'ionic_force': [25.86655467748642, 2.08726741746068, -8.532694309949875], 'ionic_force_magnitude': 27.31743414639154, 'motion_vector': [0.7343177795410156, 1.0062751770019531, 2.0959930419921875], 'cosine_ionic_motion': 0.0481961128799673, 'ionic_motion_component': 1.3165941397105598, 'ionic_force_x': 25.86655467748642, 'ionic_force_y': 2.08726741746068, 'ionic_force_z': -8.532694309949875, 'radial_force': 25.9506326735089, 'axial_force': -8.532694309949875, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [17.00419807434082, 0.02684025838971138, -1.553012490272522], 'magnitude': 17.07499122619629, 'distance': 4.409494400024414, 'before_closest_residue': 1105, 'closest_residue': 780, 'next_closest_residue': 1105, 'cosine_with_motion': 0.22238171756220773, 'motion_component': 3.7971658434937154}, {'ion': 1307, 'force': [2.9414384365081787, -1.9116371870040894, -0.5534630417823792], 'magnitude': 3.5514416694641113, 'distance': 9.668668746948242, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.10667628466503244, 'motion_component': -0.378854605769849}, {'ion': 1387, 'force': [0.6480094790458679, 0.07161861658096313, -1.956294298171997], 'magnitude': 2.06207013130188, 'distance': 12.688705444335938, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7065626176169941, 'motion_component': -1.4569816124307788}, {'ion': 1460, 'force': [2.506962299346924, 0.3197813332080841, -4.0640716552734375], 'magnitude': 4.785791397094727, 'distance': 8.328987121582031, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5446592892584318, 'motion_component': -2.606625695022325}, {'ion': 2433, 'force': [2.765946388244629, 3.5806643962860107, -0.4058528244495392], 'magnitude': 4.542723178863525, 'distance': 8.54891300201416, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.43187531744995167, 'motion_component': 1.9618899948423572}]}, 3333: {'frame': 3333, 'ionic_force': [17.867564380168915, 6.708176806569099, -8.539877261966467], 'ionic_force_magnitude': 20.908825806274354, 'motion_vector': [-0.58197021484375, -0.06623077392578125, -0.9650726318359375], 'cosine_ionic_motion': -0.11019542926066928, 'ionic_motion_component': -2.3040570350589618, 'ionic_force_x': 17.867564380168915, 'ionic_force_y': 6.708176806569099, 'ionic_force_z': -8.539877261966467, 'radial_force': 19.085321400167004, 'axial_force': -8.539877261966467, 'before_closest_residue': 780, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [3.417433023452759, 0.4562065303325653, 1.5878288745880127], 'magnitude': 3.7958099842071533, 'distance': 9.352265357971191, 'before_closest_residue': 780, 'closest_residue': 1105, 'next_closest_residue': 130, 'cosine_with_motion': -0.8287792619441003, 'motion_component': -3.145888593574688}, {'ion': 1307, 'force': [3.311511516571045, -1.642639398574829, 0.06691984832286835], 'magnitude': 3.69714093208313, 'distance': 9.476240158081055, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.4511513397508429, 'motion_component': -1.6679700794212264}, {'ion': 1316, 'force': [0.6237956881523132, 0.15656648576259613, -1.627447485923767], 'magnitude': 1.7499197721481323, 'distance': 13.773996353149414, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.6060249544382219, 'motion_component': 1.06049509096636}, {'ion': 1387, 'force': [1.9665889739990234, 0.6323477029800415, -3.3439724445343018], 'magnitude': 3.9305837154388428, 'distance': 9.190528869628906, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.4599211400015446, 'motion_component': 1.8077584950588932}, {'ion': 1460, 'force': [5.7677435874938965, 2.1759836673736572, -5.206416130065918], 'magnitude': 8.068985939025879, 'distance': 6.414451599121094, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.16728169529424516, 'motion_component': 1.3497937077936975}, {'ion': 2433, 'force': [2.780491590499878, 4.929711818695068, -0.01678992435336113], 'magnitude': 5.659811973571777, 'distance': 7.658928871154785, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.30182028666503474, 'motion_component': -1.7082461370083915}]}, 3334: {'frame': 3334, 'ionic_force': [20.401569843292236, 2.299112319946289, -6.255825400352478], 'ionic_force_magnitude': 21.462649439669725, 'motion_vector': [0.17787933349609375, -0.084075927734375, 0.6251068115234375], 'cosine_ionic_motion': -0.03375978607508399, 'ionic_motion_component': -0.7245744536877712, 'ionic_force_x': 20.401569843292236, 'ionic_force_y': 2.299112319946289, 'ionic_force_z': -6.255825400352478, 'radial_force': 20.530707964667464, 'axial_force': -6.255825400352478, 'befor</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>4333</v>
+      </c>
+      <c r="B7" t="n">
+        <v>5131</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1460</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>{4333: {'frame': 4333, 'ionic_force': [10.218847453594208, 2.7001716569066048, -15.040524646639824], 'ionic_force_magnitude': 18.382958192379444, 'motion_vector': [-1.0914764404296875, 2.8184471130371094, 0.5848388671875], 'cosine_ionic_motion': -0.21804746967951605, 'ionic_motion_component': -4.008357519072668, 'ionic_force_x': 10.218847453594208, 'ionic_force_y': 2.7001716569066048, 'ionic_force_z': -15.040524646639824, 'radial_force': 10.569568120627757, 'axial_force': -15.040524646639824, 'before_closest_residue': None, 'closest_residue': 780, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [1.9004194736480713, 6.339089393615723, 1.1476751565933228], 'magnitude': 6.716607093811035, 'distance': 7.030627250671387, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.7962185690975874, 'motion_component': 5.347887048097485}, {'ion': 1307, 'force': [2.6483633518218994, -3.5226809978485107, -0.1344403475522995], 'magnitude': 4.409215927124023, 'distance': 8.677374839782715, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.950204056050085, 'motion_component': -4.189654747068637}, {'ion': 1308, 'force': [0.17358297109603882, -0.07655664533376694, -1.6345635652542114], 'magnitude': 1.6455363035202026, 'distance': 14.20415210723877, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.2687048108516073, 'motion_component': -0.4421635449013345}, {'ion': 1316, 'force': [0.8972761631011963, -0.14553450047969818, -3.8930156230926514], 'magnitude': 3.9977312088012695, 'distance': 9.113018035888672, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.2979077327293967, 'motion_component': -1.190955063856654}, {'ion': 1387, 'force': [4.599205493927002, 0.10585440695285797, -10.526180267333984], 'magnitude': 11.487574577331543, 'distance': 5.375945568084717, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.30759072151122985, 'motion_component': -3.5334713216154103}]}, 4334: {'frame': 4334, 'ionic_force': [10.631327830255032, 4.420680075883865, -15.498867347836494], 'ionic_force_magnitude': 19.307574493796572, 'motion_vector': [0.5448684692382812, -2.2713394165039062, -1.4224014282226562], 'cosine_ionic_motion': 0.33705827245975817, 'ionic_motion_component': 6.507777704267163, 'ionic_force_x': 10.631327830255032, 'ionic_force_y': 4.420680075883865, 'ionic_force_z': -15.498867347836494, 'radial_force': 11.513797973200317, 'axial_force': -15.498867347836494, 'before_closest_residue': 780, 'closest_residue': 455, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [-0.03820937126874924, 3.2988882064819336, 0.14286993443965912], 'magnitude': 3.302201509475708, 'distance': 10.0269136428833, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.8545091731447452, 'motion_component': -2.8217615285027273}, {'ion': 1307, 'force': [6.774117946624756, -6.534855365753174, 0.375784695148468], 'magnitude': 9.41988468170166, 'distance': 5.936715602874756, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.6986941979729787, 'motion_component': 6.581618599362891}, {'ion': 1308, 'force': [0.18028856813907623, 0.2747263014316559, -1.6901415586471558], 'magnitude': 1.721789002418518, 'distance': 13.886061668395996, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.39889620431807066, 'motion_component': 0.6868150546000797}, {'ion': 1316, 'force': [0.8013342618942261, 1.1461530923843384, -3.9313461780548096], 'magnitude': 4.172683238983154, 'distance': 8.919927597045898, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.3001616454276057, 'motion_component': 1.2524794981272755}, {'ion': 1387, 'force': [2.9137964248657227, 6.235767841339111, -10.396034240722656], 'magnitude': 12.468061447143555, 'distance': 5.160236358642578, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.06485580436767582, 'motion_component': 0.8086261068832242}]}, 4335: {'frame': 4335, 'ionic_force': [9.905854746699333, 2.9460261538624763, -22.515233606100082], 'ionic_force_magnitude': 24.773792053280943, 'motion_vector': [-2.4897499084472656, -1.9592094421386719, -2.6416397094726562], 'cosine_ionic_motion': 0.28419239569134447, 'ionic_motion_component': 7.040523313981103, 'ionic_force_x': 9.905854746699333, 'ionic_force_y': 2.9460261538624763, 'ionic_force_z': -22.515233606100082, 'radial_force': 10.334651825869484, 'axial_force': -22.515233606100082, 'before_closest_residue': 455, 'closest_residue': 780, 'next_closest_residue': 1105, 'contributions': [{'ion': 1306, 'force': [-0.3307041525840759, 4.825318336486816, 0.4242839515209198], 'magnitude': 4.8552117347717285, 'distance': 8.269227981567383, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.4868868079242441, 'motion_component': -2.3639384514328228}, {'ion': 1307, 'force': [3.035064935684204, -3.5079329013824463, -0.3104632496833801], 'magnitude': 4.649043083190918, 'distance': 8.450594902038574, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.007110203163725899, 'motion_component': 0.0330556394959487}, {'ion': 1308, 'force': [0.17067889869213104, -0.07447502017021179, -1.5542986392974854], 'magnitude': 1.565414309501648, 'distance': 14.563118934631348, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5926381165473805, 'motion_component': 0.9277242097333298}, {'ion': 1316, 'force': [0.7298926711082458, 0.04116610437631607, -3.5585622787475586], 'magnitude': 3.632878065109253, 'distance': 9.559685707092285, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5006490876675077, 'motion_component': 1.8187971175178699}, {'ion': 1387, 'force': [6.300922393798828, 1.661949634552002, -17.516193389892578], 'magnitude': 18.68905258178711, 'distance': 4.214784622192383, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.3544794253429433, 'motion_component': 6.624885037317597}]}, 4336: {'frame': 4336, 'ionic_force': [-1.1519034951925278, -1.205802470445633, -12.496924042701721], 'ionic_force_magnitude': 12.607694150360162, 'motion_vector': [0.6896553039550781, 0.1011199951171875, 0.940399169921875], 'cosine_ionic_motion': -0.858411585680705, 'ionic_motion_component': -10.822590727388015, 'ionic_force_x': -1.1519034951925278, 'ionic_force_y': -1.205802470445633, 'ionic_force_z': -12.496924042701721, 'radial_force': 1.667585458070906, 'axial_force': -12.496924042701721, 'before_closest_residue': 780, 'closest_residue': 1105, 'next_closest_residue': 1105, 'contributions': [{'ion': 1306, 'force': [-1.9411698579788208, 3.975846767425537, -1.9185880422592163], 'magnitude': 4.8224968910217285, 'distance': 8.297228813171387, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.4855515710260739, 'motion_component': -2.341571029680189}, {'ion': 1307, 'force': [1.3281068801879883, -3.4387872219085693, -1.5431928634643555], 'magnitude': 3.996319532394409, 'distance': 9.114627838134766, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.18876178886234163, 'motion_component': -0.7543524202958736}, {'ion': 1316, 'force': [-0.19560758769512177, -0.3452792465686798, -2.427891969680786], 'magnitude': 2.4601097106933594, 'distance': 11.616941452026367, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8518276766603495, 'motion_component': -2.0955894897212177}, {'ion': 1387, 'force': [-0.3432329297065735, -1.397582769393921, -6.607251167297363], 'magnitude': 6.762160301208496, 'distance': 7.006906032562256, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8327335038641387, 'motion_component': -5.631077594624198}]}, 4337: {'frame': 4337, 'ionic_force': [-0.19163120537996292, 0.32513704895973206, -11.826547503471375], 'ionic_force_magnitude': 11.832567873092747, 'motion_vector': [-1.2149238586425781, 0.8994140625, 1.17535400390625], 'cosine_ionic_motion': -0.590332298049414, 'ionic_motion_component': -6.985146984348509, 'ionic_force_x': -0.19163120537996292, 'ionic_force_y': 0.32513704895973206, 'ionic_force_z': -11.826547503471375, 'radial_force': 0.3774077628793832, 'axial_force': -11.826547503471375, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [-1.3619964122772217, 5.054660320281982, -2.5555646419525146], 'magnitude': 5.825421333312988, 'distance': 7.549276828765869, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.2866344016779324, 'motion_component': 1.6697662102834132}, {'ion': 1307, 'force': [1.334238886833191, -3.2292449474334717, -0.951119065284729], 'magnitude': 3.621166229248047, 'distance': 9.575133323669434, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.8138875931739362, 'motion_component': -2.9472221492752126}, {'ion': 1316, 'force': [-0.0917414203286171, -0.38027724623680115, -2.686659812927246], 'magnitude': 2.714989423751831, 'distance': 11.058213233947754, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6517738113728772, 'motion_component': -1.7695590827597387}, {'ion': 1387, 'force': [-0.07213225960731506, -1.1200010776519775, -5.633203983306885], 'magnitude': 5.743917942047119, 'distance': 7.602648735046387, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6856177321457585, 'motion_component': -3.9381319494534495}]}, 4338: {'frame': 4338, 'ionic_force': [-1.9880583882331848, -1.188404381275177, -12.07487940788269], 'ionic_force_magnitude': 12.295014999721138, 'motion_vector': [1.5186386108398438, 5.265224456787109, -0.11255645751953125], 'cosine_ionic_motion': -0.11748555094438694, 'ionic_motion_component': -1.4444866111117394, 'ionic_force_x': -1.9880583882331848, 'ionic_force_y': -1.188404381275177, 'ionic_force_z': -12.07487940788269, 'radial_force': 2.3161781296908845, 'axial_force': -12.07487940788269, 'before_closest_residue': 1105, 'closest_residue': 780, 'next_closest_residue': 130, 'contributions': [{'ion': 1306, 'force': [-1.6397868394851685, 7.1292724609375, -0.15652811527252197], 'magnitude': 7.317098140716553, 'distance': 6.735961437225342, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.8743170953983076, 'motion_component': 6.397464145557997}, {'ion': 1307, 'force': [2.079728841781616, -7.2433953285217285, -1.8075493574142456], 'magnitude': 7.749792098999023, 'distance': 6.5452165603637695, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.81871410957672, 'motion_component': -6.344864404083127}, {'ion': 1316, 'force': [-0.5445583462715149, -0.3111899495124817, -2.85630202293396], 'magnitude': 2.92435359954834, 'distance': 10.65501594543457, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.13376092719612437, 'motion_component': -0.39116425460121373}, {'ion': 1387, 'force': [-1.8834420442581177, -0.7630915641784668, -7.254499912261963], 'magnitude': 7.533752918243408, 'distance': 6.638399124145508, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.14679564559442262, 'motion_component': -1.10592210987212}]}, 4339: {'frame': 4339, 'ionic_force': [7.982106583658606, -1.4821966588497162, -13.919581286609173], 'ionic_force_magnitude': 16.114145203606412, 'motion_vector': [-0.3119239807128906, 0.11574172973632812, 2.2965164184570312], 'cosine_ionic_motion': -0.9260598449343778, 'ionic_motion_component': -14.922662808501801, 'ionic_force_x': 7.982106583658606, 'ionic_force_y': -1.4821966588497162, 'ionic_force_z': -13.919581286609173, 'radial_force': 8.118554825114586, 'axial_force': -13.919581286609173, 'before_closest_residue': 780, 'closest_residue': 130, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-0.076982282102108, 2.2683990001678467, -0.11256872862577438], 'magnitude': 2.2724947929382324, 'distance': 12.086974143981934, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.005318317242196725, 'motion_component': 0.012085847573630737}, {'ion': 1307, 'force': [8.069611549377441, -11.067646980285645, -4.958900451660156], 'magnitude': 14.567159652709961, 'distance': 4.773991107940674, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.44925909704251427, 'motion_component': -6.544428893052576}, {'ion': 1308, 'force': [0.015117759816348553, 0.40834537148475647, -1.4295883178710938], 'magnitude': 1.4868414402008057, 'distance': 14.942962646484375, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.9392277961859843, 'motion_component': -1.3964827394725436}, {'ion': 1316, 'force': [-0.007704783696681261, 1.2880055904388428, -2.648350715637207], 'magnitude': 2.944958209991455, 'distance': 10.61767578125, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8678253609626467, 'motion_component': -2.5557094833582963}, {'ion': 1387, 'force': [-0.017935659736394882, 5.620700359344482, -4.770173072814941], 'magnitude': 7.37205171585083, 'distance': 6.710808753967285, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6020206998732269, 'motion_component': -4.438127686965383}]}, 4340: {'frame': 4340, 'ionic_force': [7.449656866490841, 0.12455254793167114, -8.714410305023193], 'ionic_force_magnitude': 11.465332429979727, 'motion_vector': [0.09852218627929688, -2.540813446044922, -1.569000244140625], 'cosine_ionic_motion': 0.41131931779600295, 'ionic_motion_component': 4.71591271340365, 'ionic_force_x': 7.449656866490841, 'ionic_force_y': 0.12455254793167114, 'ionic_force_z': -8.714410305023193, 'radial_force': 7.450698005264366, 'axial_force': -8.714410305023193, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 130, 'contributions': [{'ion': 1306, 'force': [-0.06719008833169937, 2.7485055923461914, 0.42278754711151123], 'magnitude': 2.781644582748413, 'distance': 10.924919128417969, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.9208647724106859, 'motion_component': -2.5615185427617937}, {'ion': 1307, 'force': [8.1783447265625, -13.644166946411133, 1.9067336320877075], 'magnitude': 16.0213680267334, 'distance': 4.552177906036377, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.6785424206437897, 'motion_component': 10.871178135618344}, {'ion': 1308, 'force': [-0.11230937391519547, 0.5389495491981506, -1.9288716316223145], 'magnitude': 2.0058977603912354, 'distance': 12.865143775939941, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.27463385257681466, 'motion_component': 0.5508874269489278}, {'ion': 1316, 'force': [-0.09320607036352158, 2.1498072147369385, -3.7819480895996094], 'magnitude': 4.351263046264648, 'distance': 8.734969139099121, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.03556952269342487, 'motion_component': 0.15477234838873555}, {'ion': 1387, 'force': [-0.4559823274612427, 8.331457138061523, -5.333111763000488], 'magnitude': 9.902685165405273, 'distance': 5.790186405181885, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.43416573845546347, 'motion_component': -4.299406738489893}]}, 4341: {'frame': 4341, 'ionic_force': [11.73270659148693, 0.9782168567180634, -18.562486216425896], 'ionic_force_magnitude': 21.981337691680405, 'motion_vector': [-0.7720985412597656, -0.6841316223144531, -3.7374649047851562], 'cosine_ionic_motion': 0.6998839156992859, 'ionic_motion_component': 15.384384695961584, 'ionic_force_x': 11.73270659148693, 'ionic_force_y': 0.9782168567180634, 'ionic_force_z': -18.562486216425896, 'radial_force': 11.773415484925701, 'axial_force': -18.562486216425896, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 130, 'contributions': [{'ion': 1306, 'force': [-0.5007864832878113, 3.0563981533050537, -0.13875077664852142], 'magnitude': 3.10025954246521, 'distance': 10.348323822021484, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.09864462923496593, 'motion_component': -0.3058239422923039}, {'ion': 1307, 'force': [13.399417877197266, -12.055536270141602, -0.6212299466133118], 'magnitude': 18.035140991210938, 'distance': 4.290513515472412, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.003199490799020054, 'motion_component': 0.05770326502439005}, {'ion': 1308, 'force': [-0.09177793562412262, 0.24030449986457825, -1.6979613304138184], 'magnitude': 1.717335820198059, 'distance': 13.904053688049316, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.9390324383797626, 'motion_component': 1.6126339887252703}, {'ion': 1316, 'force': [-0.13407957553863525, 0.977773129940033, -3.8091092109680176], 'magnitude': 3.9348864555358887, 'distance': 9.185503005981445, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.8960829730796381, 'motion_component': 3.5259846615014645}, {'ion': 1387, 'force': [-0.9400672912597656, 8.75927734375, -12.295434951782227], 'magnitude': 15.125685691833496, 'distance': 4.685020446777344, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.6937792513859733, 'motion_component': 10.493887334066017}]}, 4342: {'frame': 4342, 'ionic_force': [0.36002762615680695, -0.6625969856977463, -12.154103636741638], 'ionic_force_magnitude': 12.17747469181144, 'motion_vector': [-2.657154083251953, -1.6822662353515625, 5.648590087890625], 'cosine_ionic_motion': -0.8700258456677054, 'ionic_motion_component': -10.594717716840329, 'ionic_force_x': 0.36002762615680695, 'ionic_force_y': -0.6625969856977463, 'ionic_force_z': -12.154103636741638, 'radial_force': 0.7540919420414496, 'axial_force': -12.154103636741638, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 'SF', 'contributions': [{'ion': 1306, 'force': [-0.24011437594890594, 2.6392462253570557, -1.151229977607727], 'magnitude': 2.8893954753875732, 'distance': 10.719278335571289, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.5516407721175797, 'motion_component': -1.593908331880192}, {'ion': 1307, 'force': [1.9842231273651123, -4.65313720703125, -3.5916688442230225], 'magnitude': 6.203943252563477, 'distance': 7.315350532531738, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.4421073504431153, 'motion_component': -2.742808931226641}, {'ion': 1316, 'force': [-0.2974294424057007, 0.23622436821460724, -2.1497864723205566], 'magnitude': 2.183082342147827, 'distance': 12.332013130187988, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.832544475446919, 'motion_component': -1.8175130650926032}, {'ion': 1387, 'force': [-1.0866516828536987, 1.1150696277618408, -5.261418342590332], 'magnitude': 5.4869585037231445, 'distance': 7.778631687164307, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8092803195561473, 'motion_component': -4.440487642549986}]}, 4344: {'frame': 4344, 'ionic_force': [9.202361762523651, 8.81113064289093, -18.928253769874573], 'ionic_force_magnitude': 22.81662279986282, 'motion_vector': [1.4634857177734375, -1.2306327819824219, 0.8022537231445312], 'cosine_ionic_motion': -0.2654885973717331, 'ionic_motion_component': -6.057553183895485, 'ionic_force_x': 9.202361762523651, 'ionic_force_y': 8.81113064289093, 'ionic_force_z': -18.928253769874573, 'radial_force': 12.74046644414752, 'axial_force': -18.928253769874573, 'before_closest_residue': 'SF', 'closest_residue': 130, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [-0.3357532024383545, 1.7316968441009521, -0.49725770950317383], 'magnitude': 1.8326945304870605, 'distance': 13.459346771240234, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.795038428889301, 'motion_component': -1.4570626149438795}, {'ion': 1307, 'force': [10.69202995300293, 3.909050941467285, -13.227506637573242], 'magnitude': 17.45185089111328, 'distance': 4.361624717712402, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.006223300153679032, 'motion_component': 0.10860810920331687}, {'ion': 1316, 'force': [-0.2957773804664612, 0.846617579460144, -1.985202670097351], 'magnitude': 2.1783652305603027, 'distance': 12.345357894897461, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6790620152713646, 'motion_component': -1.4792451065752275}, {'ion': 1387, 'force': [-0.8581376075744629, 2.323765277862549, -3.2182867527008057], 'magnitude': 4.061237812042236, 'distance': 9.041485786437988, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7952878508257138, 'motion_component': -3.2298533141553847}]}, 4345: {'frame': 4345, 'ionic_force': [14.981032002717257, 2.010621815919876, -19.484798073768616], 'ionic_force_magnitude': 24.66031783916478, 'motion_vector': [-1.1395187377929688, 0.0416717529296875, -1.0085220336914062], 'cosine_ionic_motion': 0.07094999718166918, 'ionic_motion_component': 1.7496494811878074, 'ionic_force_x': 14.981032002717257, 'ionic_force_y': 2.010621815919876, 'ionic_force_z': -19.484798073768616, 'radial_force': 15.115353781936154, 'axial_force': -19.484798073768616, 'before_closest_residue': 130, 'closest_residue': 455, 'next_closest_residue': 130, 'contributions': [{'ion': 1306, 'force': [-0.47127556800842285, 3.423821449279785, -0.9305918216705322], 'magnitude': 3.579197406768799, 'distance': 9.631107330322266, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.2970005326814845, 'motion_component': 1.0630235795107588}, {'ion': 1307, 'force': [15.362360000610352, -7.023677349090576, -8.83127212524414], 'magnitude': 19.061100006103516, 'distance': 4.17344856262207, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.30644178089015933, 'motion_component': -5.8411172885114535}, {'ion': 1308, 'force': [-0.04955724999308586, 0.3378300964832306, -1.4625250101089478], 'magnitude': 1.5018537044525146, 'distance': 14.868091583251953, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.6760140450308809, 'motion_component': 1.0152741867035733}, {'ion': 1316, 'force': [-0.044318169355392456, 1.0932285785675049, -2.809373140335083], 'magnitude': 3.014911413192749, 'distance': 10.493775367736816, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.6382689866249723, 'motion_component': 1.9243243929068639}, {'ion': 1387, 'force': [0.18382298946380615, 4.179419040679932, -5.451035976409912], 'magnitude': 6.871326446533203, 'distance': 6.951023101806641, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5221909782986967, 'motion_component': 3.5881446979568086}]}, 4346: {'frame': 4346, 'ionic_force': [2.747163772583008, -0.8378102779388428, -11.040866374969482], 'ionic_force_magnitude': 11.40831123195472, 'motion_vector': [-4.582515716552734, 0.4224891662597656, 2.309173583984375], 'cosine_ionic_motion': -0.6543868084884226, 'ionic_motion_component': -7.465448377321473, 'ionic_force_x': 2.747163772583008, 'ionic_force_y': -0.8378102779388428, 'ionic_force_z': -11.040866374969482, 'radial_force': 2.8720784904337946, 'axial_force': -11.040866374969482, 'before_closest_residue': 455, 'closest_residue': 130, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-0.3646623194217682, 2.5122485160827637, -1.0865371227264404], 'magnitude': 2.7613282203674316, 'distance': 10.965034484863281, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.015717597638865644, 'motion_component': 0.043401447602082754}, {'ion': 1307, 'force': [4.082198143005371, -7.544401168823242, -3.096256732940674], 'magnitude': 9.119711875915527, 'distance': 6.033627510070801, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.618540265813115, 'motion_component': -5.640908727462971}, {'ion': 1316, 'force': [-0.26130351424217224, 0.9197101593017578, -2.4406163692474365], 'magnitude': 2.6212124824523926, 'distance': 11.25428581237793, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.30007228847047807, 'motion_component': -0.7865532102811734}, {'ion': 1387, 'force': [-0.7090685367584229, 3.274632215499878, -4.417456150054932], 'magnitude': 5.544358730316162, 'distance': 7.7382612228393555, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.1950429042251414, 'motion_component': -1.0813878190443305}]}, 4347: {'frame': 4347, 'ionic_force': [-15.417576730251312, -4.030454456806183, -6.167419657111168], 'ionic_force_magnitude': 17.087518854078752, 'motion_vector': [-0.36487579345703125, -0.39484405517578125, 1.3642425537109375], 'cosine_ionic_motion': -0.04777051448418554, 'ionic_motion_component': -0.8162795669175625, 'ionic_force_x': -15.417576730251312, 'ionic_force_y': -4.030454456806183, 'ionic_force_z': -6.167419657111168, 'radial_force': 15.93569061451607, 'axial_force': -6.167419657111168, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-2.907095432281494, 2.6085305213928223, 0.1315348893404007], 'magnitude': 3.9080605506896973, 'distance': 9.216975212097168, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.03668227380280444, 'motion_component': 0.1433565447774372}, {'ion': 1307, 'force': [-7.185686111450195, -11.091068267822266, -0.7672844529151917], 'magnitude': 13.23762035369873, 'distance': 5.007997035980225, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.30675139512678784, 'motion_component': 4.060658662473141}, {'ion': 1308, 'force': [-0.5734414458274841, 0.4193485379219055, -1.335965633392334], 'magnitude': 1.5131069421768188, 'distance': 14.812700271606445, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8017682373028415, 'motion_component': -1.213161044334834}, {'ion': 1316, 'force': [-1.3264715671539307, 1.0629514455795288, -2.074846029281616], 'magnitude': 2.6822338104248047, 'distance': 11.125530242919922, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7033365199731868, 'motion_component': -1.8865130497748017}, {'ion': 1387, 'force': [-3.424882173538208, 2.969783306121826, -2.1208584308624268], 'magnitude': 5.004745006561279, 'distance': 8.144756317138672, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.3837599886865634, 'motion_component': -1.9206208369105298}]}, 4348: {'frame': 4348, 'ionic_force': [-21.16736936569214, -8.308469772338867, 1.6546272039413452], 'ionic_force_magnitude': 22.799692695418802, 'motion_vector': [1.2287940979003906, -3.6073760986328125, -4.4157257080078125], 'cosine_ionic_motion': -0.025152521750439555, 'ionic_motion_component': -0.5734697664248593, 'ionic_force_x': -21.16736936569214, 'ionic_force_y': -8.308469772338867, 'ionic_force_z': 1.6546272039413452, 'radial_force': 22.739573342996362, 'axial_force': 1.6546272039413452, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 1105, 'contributions': [{'ion': 1306, 'force': [-2.4971795082092285, 1.165833592414856, 1.1946948766708374], 'magnitude': 3.003726005554199, 'distance': 10.513296127319336, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.7162920626954248, 'motion_component': -2.1515450239539433}, {'ion': 1307, 'force': [-13.858606338500977, -12.73878288269043, 4.691383361816406], 'magnitude': 19.399656295776367, 'distance': 4.136871337890625, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.07254097291058273, 'motion_component': 1.407269890282521}, {'ion': 1316, 'force': [-1.6572506427764893, 1.0221670866012573, -2.0923280715942383], 'magnitude': 2.858170986175537, 'distance': 10.777670860290527, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.2108659991227886, 'motion_component': 0.602691103493072}, {'ion': 1387, 'force': [-3.1543328762054443, 2.242312431335449, -2.13912296295166], 'magnitude': 4.421948432922363, 'distance': 8.664873123168945, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.09766865255972287, 'motion_component': -0.43188574558306664}]}, 4349: {'frame': 4349, 'ionic_force': [-8.915342390537262, -7.096782431006432, -8.744169890880585], 'ionic_force_magnitude': 14.3634312716055, 'motion_vector': [3.6558074951171875, 0.5428085327148438, 1.3375320434570312], 'cosine_ionic_motion': -0.8527251143535519, 'ionic_motion_component': -12.248058573589184, 'ionic_force_x': -8.915342390537262, 'ionic_force_y': -7.096782431006432, 'ionic_force_z': -8.744169890880585, 'radial_force': 11.395071338677623, 'axial_force': -8.744169890880585, 'before_closest_residue': 98, 'closest_residue': 1105, 'next_closest_residue': 130, 'contributions': [{'ion': 1306, 'force': [-4.382460594177246, 0.3038478493690491, -0.8590322136878967], 'magnitude': 4.476183891296387, 'distance': 8.61221981048584, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 455, 'cosine_with_motion': -0.9665783516939179, 'motion_component': -4.326582284552656}, {'ion': 1307, 'force': [-1.7179875373840332, -7.742946624755859, -2.696408987045288], 'magnitude': 8.377071380615234, 'distance': 6.295394420623779, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.4279350922163116, 'motion_component': -3.584842816880311}, {'ion': 1316, 'force': [-0.7681282162666321, 0.059397414326667786, -1.9104300737380981], 'magnitude': 2.0599253177642822, 'distance': 12.69530963897705, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.658453806185171, 'motion_component': -1.356365627793785}, {'ion': 1387, 'force': [-2.0467660427093506, 0.28291893005371094, -3.2782986164093018], 'magnitude': 3.875117540359497, 'distance': 9.25606918334961, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.769078047461971, 'motion_component': -2.9802678535875486}]}, 4350: {'frame': 4350, 'ionic_force': [-6.837312012910843, -2.323559030890465, -14.161073744297028], 'ionic_force_magnitude': 15.896030061727556, 'motion_vector': [-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>4408</v>
+      </c>
+      <c r="B8" t="n">
+        <v>4416</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1387</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>{4408: {'frame': 4408, 'ionic_force': [9.049361620098352, -12.949827790260315, -9.676596252247691], 'ionic_force_magnitude': 18.52634611999143, 'motion_vector': [0.9472541809082031, 6.171745300292969, -2.0280227661132812], 'cosine_ionic_motion': -0.4252876635747381, 'ionic_motion_component': -7.879026455948069, 'ionic_force_x': 9.049361620098352, 'ionic_force_y': -12.949827790260315, 'ionic_force_z': -9.676596252247691, 'radial_force': 15.798385535513033, 'axial_force': -9.676596252247691, 'before_closest_residue': None, 'closest_residue': 780, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [-1.5873969793319702, -6.355767250061035, -0.6117986440658569], 'magnitude': 6.5795063972473145, 'distance': 7.103499889373779, 'before_closest_residue': 130, 'closest_residue': 455, 'next_closest_residue': 98, 'cosine_with_motion': -0.9142022563738115, 'motion_component': -6.014999570318558}, {'ion': 1307, 'force': [1.3527055978775024, -2.772169589996338, -0.023000208660960197], 'magnitude': 3.0846824645996094, 'distance': 10.374420166015625, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.7792661138721038, 'motion_component': -2.4037884879717932}, {'ion': 1308, 'force': [0.0392477847635746, -0.5659531354904175, -1.739326000213623], 'magnitude': 1.8295077085494995, 'distance': 13.471064567565918, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.00596555141577959, 'motion_component': 0.010914022006728752}, {'ion': 1316, 'force': [0.1305760145187378, -2.5276927947998047, -4.4630842208862305], 'magnitude': 5.130828380584717, 'distance': 8.044059753417969, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.190751381479075, 'motion_component': -0.9787126361579297}, {'ion': 1460, 'force': [9.114229202270508, -0.7282450199127197, -2.8393871784210205], 'magnitude': 9.574007987976074, 'distance': 5.888736724853516, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.157463841084995, 'motion_component': 1.5075601164077739}]}, 4409: {'frame': 4409, 'ionic_force': [8.281869903206825, -9.407124474644661, -19.244575142860413], 'ionic_force_magnitude': 22.96599730915909, 'motion_vector': [1.2028884887695312, 0.22224044799804688, -0.367950439453125], 'cosine_ionic_motion': 0.5096920959417545, 'ionic_motion_component': 11.705587303897989, 'ionic_force_x': 8.281869903206825, 'ionic_force_y': -9.407124474644661, 'ionic_force_z': -19.244575142860413, 'radial_force': 12.53329006985403, 'axial_force': -19.244575142860413, 'before_closest_residue': 780, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [4.004691123962402, -8.651683807373047, -11.288216590881348], 'magnitude': 14.775419235229492, 'distance': 4.740226745605469, 'before_closest_residue': 455, 'closest_residue': 98, 'next_closest_residue': 130, 'cosine_with_motion': 0.3734221781025008, 'motion_component': 5.517469282820457}, {'ion': 1307, 'force': [1.8958126306533813, -4.239731788635254, -1.8980571031570435], 'magnitude': 5.017175674438477, 'distance': 8.134659767150879, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.31777827517979385, 'motion_component': 1.5943494380754615}, {'ion': 1308, 'force': [0.11879675090312958, 0.2119782418012619, -1.456363558769226], 'magnitude': 1.4764965772628784, 'distance': 14.995219230651855, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.38486557312870256, 'motion_component': 0.5682527165054461}, {'ion': 1316, 'force': [0.3882765471935272, 1.0418009757995605, -3.5045788288116455], 'magnitude': 3.6767079830169678, 'distance': 9.502534866333008, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.4233068597611323, 'motion_component': 1.5563756601938152}, {'ion': 1460, 'force': [1.8742928504943848, 2.2305119037628174, -1.09735906124115], 'magnitude': 3.1132545471191406, 'distance': 10.326704025268555, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.7931057531386033, 'motion_component': 2.469140102033048}]}, 4410: {'frame': 4410, 'ionic_force': [15.673005670309067, -6.354610577225685, -18.238948702812195], 'ionic_force_magnitude': 24.8733478268114, 'motion_vector': [-0.20865249633789062, -4.049587249755859, 2.408935546875], 'cosine_ionic_motion': -0.18303666953777947, 'ionic_motion_component': -4.552734746474323, 'ionic_force_x': 15.673005670309067, 'ionic_force_y': -6.354610577225685, 'ionic_force_z': -18.238948702812195, 'radial_force': 16.9122494757418, 'axial_force': -18.238948702812195, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [10.753595352172852, -6.403841495513916, -11.053228378295898], 'magnitude': 16.69799041748047, 'distance': 4.458994388580322, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 455, 'cosine_with_motion': -0.03729673389609892, 'motion_component': -0.6227804744865466}, {'ion': 1307, 'force': [2.1814122200012207, -2.955780029296875, -1.1102296113967896], 'magnitude': 3.8376822471618652, 'distance': 9.301104545593262, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.4883864011670867, 'motion_component': 1.8742717970166183}, {'ion': 1308, 'force': [0.2570955455303192, 0.21237300336360931, -1.531499981880188], 'magnitude': 1.5673840045928955, 'distance': 14.55396556854248, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6226418300254172, 'motion_component': -0.9759188427346958}, {'ion': 1316, 'force': [1.0977156162261963, 1.1136078834533691, -3.712677240371704], 'magnitude': 4.0285325050354, 'distance': 9.078113555908203, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7200942571398282, 'motion_component': -2.900923142959339}, {'ion': 1460, 'force': [1.383186936378479, 1.6790300607681274, -0.8313134908676147], 'magnitude': 2.3288259506225586, 'distance': 11.939895629882812, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.8276203568856679, 'motion_component': -1.9273837390999855}]}, 4411: {'frame': 4411, 'ionic_force': [8.995075047016144, -8.02235746383667, -9.743937104940414], 'ionic_force_magnitude': 15.498835591232748, 'motion_vector': [-2.447307586669922, -1.137054443359375, 2.16204833984375], 'cosine_ionic_motion': -0.6336468893149177, 'ionic_motion_component': -9.820788960387965, 'ionic_force_x': 8.995075047016144, 'ionic_force_y': -8.02235746383667, 'ionic_force_z': -9.743937104940414, 'radial_force': 12.052783677600308, 'axial_force': -9.743937104940414, 'before_closest_residue': 455, 'closest_residue': 780, 'next_closest_residue': 'SF', 'contributions': [{'ion': 1306, 'force': [1.557535171508789, -6.21755838394165, 0.962909996509552], 'magnitude': 6.481600284576416, 'distance': 7.156948566436768, 'before_closest_residue': 130, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': 0.2382523481492783, 'motion_component': 1.5442565147768939}, {'ion': 1307, 'force': [1.0693477392196655, -2.452256441116333, -0.23202911019325256], 'magnitude': 2.685312509536743, 'distance': 11.11915111541748, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.03557547900048474, 'motion_component': -0.09553128193571503}, {'ion': 1308, 'force': [0.3361741900444031, -0.34610939025878906, -2.0818889141082764], 'magnitude': 2.1370694637298584, 'distance': 12.464065551757812, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6671931374770188, 'motion_component': -1.4258381357650443}, {'ion': 1316, 'force': [2.108905553817749, -1.8903121948242188, -7.310626983642578], 'magnitude': 7.840027332305908, 'distance': 6.50744104385376, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6941344152193054, 'motion_component': -5.442032838588133}, {'ion': 1460, 'force': [3.923112392425537, 2.8838789463043213, -1.0823020935058594], 'magnitude': 4.987879753112793, 'distance': 8.158514022827148, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.8824677491173122, 'motion_component': -4.401643196460441}]}, 4414: {'frame': 4414, 'ionic_force': [1.0051689818501472, 3.150031417608261, -16.299150347709656], 'ionic_force_magnitude': 16.631156444193426, 'motion_vector': [-0.04938507080078125, -0.9767036437988281, 0.471405029296875], 'cosine_ionic_motion': -0.598700230282273, 'ionic_motion_component': -9.957077192999114, 'ionic_force_x': 1.0051689818501472, 'ionic_force_y': 3.150031417608261, 'ionic_force_z': -16.299150347709656, 'radial_force': 3.3065182010678202, 'axial_force': -16.299150347709656, 'before_closest_residue': 'SF', 'closest_residue': 130, 'next_closest_residue': 130, 'contributions': [{'ion': 1306, 'force': [-0.07259159535169601, 3.9749860763549805, -9.200763702392578], 'magnitude': 10.022965431213379, 'distance': 5.7553391456604, 'before_closest_residue': 455, 'closest_residue': 1105, 'next_closest_residue': 'SF', 'cosine_with_motion': -0.7550632585559086, 'motion_component': -7.567972958430358}, {'ion': 1307, 'force': [0.6202806830406189, -2.786587715148926, -3.157846212387085], 'magnitude': 4.256971836090088, 'distance': 8.831177711486816, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.260176184204433, 'motion_component': 1.1075627713267258}, {'ion': 1316, 'force': [-0.3398584723472595, 0.2946309745311737, -2.221829891204834], 'magnitude': 2.2669007778167725, 'distance': 12.10187816619873, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5356952746826692, 'motion_component': -1.2143680491908284}, {'ion': 1460, 'force': [0.7973383665084839, 1.6670020818710327, -1.7187105417251587], 'magnitude': 2.5236105918884277, 'distance': 11.469853401184082, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.9043784954636804, 'motion_component': -2.2822991356094935}]}, 4415: {'frame': 4415, 'ionic_force': [-1.2431654334068298, -0.5947210304439068, -11.592971801757812], 'ionic_force_magnitude': 11.674594151199504, 'motion_vector': [-1.1576690673828125, 0.13907241821289062, -4.969749450683594], 'cosine_ionic_motion': 0.9895183826105229, 'ionic_motion_component': 11.552225522129204, 'ionic_force_x': -1.2431654334068298, 'ionic_force_y': -0.5947210304439068, 'ionic_force_z': -11.592971801757812, 'radial_force': 1.3780977464860225, 'axial_force': -11.592971801757812, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 130, 'contributions': [{'ion': 1306, 'force': [-1.8574953079223633, 0.8867517709732056, -4.2414045333862305], 'magnitude': 4.714459419250488, 'distance': 8.39176082611084, 'before_closest_residue': 1105, 'closest_residue': 'SF', 'next_closest_residue': 455, 'cosine_with_motion': 0.9703526311906902, 'motion_component': 4.574688341109766}, {'ion': 1307, 'force': [0.4999687671661377, -3.111016035079956, -3.033966064453125], 'magnitude': 4.374167442321777, 'distance': 8.712069511413574, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.6299753051365686, 'motion_component': 2.75561738317462}, {'ion': 1316, 'force': [-0.3461155891418457, 0.052372146397829056, -2.328737497329712], 'magnitude': 2.35490083694458, 'distance': 11.873608589172363, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.9966853552791446, 'motion_component': 2.3470950127604313}, {'ion': 1460, 'force': [0.46047669649124146, 1.5771710872650146, -1.9888637065887451], 'magnitude': 2.5797455310821533, 'distance': 11.344376564025879, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.7267480067537534, 'motion_component': 1.874824819083032}]}, 4416: {'frame': 4416, 'ionic_force': [-0.9943284774199128, -0.28250962495803833, -4.419668912887573], 'ionic_force_magnitude': 4.5389397560164815, 'motion_vector': [2.0530242919921875, -1.0973854064941406, -5.364692687988281], 'cosine_ionic_motion': 0.8280229965304783, 'ionic_motion_component': 3.758346497848085, 'ionic_force_x': -0.9943284774199128, 'ionic_force_y': -0.28250962495803833, 'ionic_force_z': -4.419668912887573, 'radial_force': 1.0336831280436638, 'axial_force': -4.419668912887573, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': None, 'contributions': [{'ion': 1306, 'force': [-1.0510830879211426, -0.1106332540512085, -1.631767988204956], 'magnitude': 1.9441404342651367, 'distance': 13.067882537841797, 'before_closest_residue': 'SF', 'closest_residue': 455, 'next_closest_residue': 780, 'cosine_with_motion': 0.5908387561172265, 'motion_component': 1.1486735331909976}, {'ion': 1307, 'force': [-0.013370522297918797, -0.8900471329689026, -1.4354690313339233], 'magnitude': 1.6890630722045898, 'distance': 14.019938468933105, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.8757279544678656, 'motion_component': 1.4791597356584902}, {'ion': 1460, 'force': [0.07012513279914856, 0.7181707620620728, -1.3524318933486938], 'magnitude': 1.5328923463821411, 'distance': 14.71679401397705, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.7375033161043688, 'motion_component': 1.1305131545959268}]}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>4857</v>
+      </c>
+      <c r="B9" t="n">
+        <v>4995</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1316</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>{4857: {'frame': 4857, 'ionic_force': [-24.356317825615406, 5.643100440502167, 5.592016190290451], 'ionic_force_magnitude': 25.619239756020416, 'motion_vector': [0.9804725646972656, -0.3909263610839844, 0.2857513427734375], 'cosine_ionic_motion': -0.8741209137903592, 'ionic_motion_component': -22.394313266146863, 'ionic_force_x': -24.356317825615406, 'ionic_force_y': 5.643100440502167, 'ionic_force_z': 5.592016190290451, 'radial_force': 25.001495967321368, 'axial_force': 5.592016190290451, 'before_closest_residue': None, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-0.837573766708374, 2.762312173843384, 3.2253456115722656], 'magnitude': 4.328366279602051, 'distance': 8.758042335510254, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 780, 'cosine_with_motion': -0.20692848187702942, 'motion_component': -0.8956622160151397}, {'ion': 1307, 'force': [0.08748745173215866, 2.7204031944274902, -0.2865326702594757], 'magnitude': 2.7368502616882324, 'distance': 11.013960838317871, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.35403881111452956, 'motion_component': -0.9689511617937128}, {'ion': 1308, 'force': [-1.2521235942840576, 1.593077540397644, -2.4381844997406006], 'magnitude': 3.1702449321746826, 'distance': 10.233463287353516, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7347405368026476, 'motion_component': -2.329307494535591}, {'ion': 1320, 'force': [-0.6172628998756409, 0.6778424382209778, -1.6455979347229004], 'magnitude': 1.8837400674819946, 'distance': 13.275734901428223, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6507174342681865, 'motion_component': -1.2257824654629097}, {'ion': 1460, 'force': [-21.736845016479492, -2.110534906387329, 6.736985683441162], 'magnitude': 22.854578018188477, 'distance': 3.8113815784454346, 'before_closest_residue': 455, 'closest_residue': 130, 'next_closest_residue': 130, 'cosine_with_motion': -0.7427224759895918, 'motion_component': -16.9746092376122}]}, 4858: {'frame': 4858, 'ionic_force': [-9.28166988492012, 11.450447499752045, 3.758600100874901], 'ionic_force_magnitude': 15.211483113605581, 'motion_vector': [-0.14766693115234375, 1.5113677978515625, -0.5906982421875], 'cosine_ionic_motion': 0.6639413357690161, 'ionic_motion_component': 10.099532417475123, 'ionic_force_x': -9.28166988492012, 'ionic_force_y': 11.450447499752045, 'ionic_force_z': 3.758600100874901, 'radial_force': 14.73981491733227, 'axial_force': 3.758600100874901, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-2.1441845893859863, 4.504876136779785, 0.23799630999565125], 'magnitude': 4.994805335998535, 'distance': 8.15285587310791, 'before_closest_residue': 130, 'closest_residue': 780, 'next_closest_residue': 'SF', 'cosine_with_motion': 0.8582062346597942, 'motion_component': 4.2865729479768}, {'ion': 1307, 'force': [1.3651424646377563, 3.7462639808654785, -0.13131223618984222], 'magnitude': 3.9894046783447266, 'distance': 9.122523307800293, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.8519472145823831, 'motion_component': 3.3987623080768814}, {'ion': 1308, 'force': [-1.0608267784118652, 1.5705699920654297, -2.8913075923919678], 'magnitude': 3.4571235179901123, 'distance': 9.799673080444336, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.7523887522231089, 'motion_component': 2.6011008640142848}, {'ion': 1320, 'force': [-0.4662999212741852, 0.6704815030097961, -1.7270715236663818], 'magnitude': 1.9104337692260742, 'distance': 13.182660102844238, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.6753826513946052, 'motion_component': 1.2902738108900658}, {'ion': 1460, 'force': [-6.97550106048584, 0.9582558870315552, 8.270295143127441], 'magnitude': 10.861567497253418, 'distance': 5.5286970138549805, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 130, 'cosine_with_motion': -0.1360003780017847, 'motion_component': -1.4771773018897036}]}, 4859: {'frame': 4859, 'ionic_force': [-11.826732784509659, 21.502933859825134, 4.421850718557835], 'ionic_force_magnitude': 24.93592863146308, 'motion_vector': [-0.5728759765625, -0.2980232238769531, -0.14586639404296875], 'cosine_ionic_motion': -0.016847408767662636, 'ionic_motion_component': -0.4201057826555209, 'ionic_force_x': -11.826732784509659, 'ionic_force_y': 21.502933859825134, 'ionic_force_z': 4.421850718557835, 'radial_force': 24.540737008822898, 'axial_force': 4.421850718557835, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-3.3123834133148193, 5.30451774597168, 0.07961202412843704], 'magnitude': 6.254289150238037, 'distance': 7.285847187042236, 'before_closest_residue': 780, 'closest_residue': 'SF', 'next_closest_residue': 780, 'cosine_with_motion': 0.07368709651645064, 'motion_component': 0.4608603946693295}, {'ion': 1307, 'force': [1.019066572189331, 3.0403809547424316, -0.13036009669303894], 'magnitude': 3.209268808364868, 'distance': 10.17105484008789, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.6923038402744626, 'motion_component': -2.2217891743240976}, {'ion': 1308, 'force': [-0.8318650126457214, 1.5506973266601562, -2.159569263458252], 'magnitude': 2.785749673843384, 'distance': 10.916866302490234, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.1786205972552863, 'motion_component': 0.49759226274005286}, {'ion': 1320, 'force': [-0.4241594970226288, 0.7252730131149292, -1.4648845195770264], 'magnitude': 1.6887328624725342, 'distance': 14.021308898925781, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.2151362361665056, 'motion_component': 0.36330764449495057}, {'ion': 1460, 'force': [-8.27739143371582, 10.882064819335938, 8.097052574157715], 'magnitude': 15.890148162841797, 'distance': 4.570935249328613, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 1105, 'cosine_with_motion': 0.030202565824339556, 'motion_component': 0.47992324150436616}]}, 4860: {'frame': 4860, 'ionic_force': [-4.794602394104004, 12.35471922159195, -2.0622036159038544], 'ionic_force_magnitude': 13.411934346520205, 'motion_vector': [0.6911888122558594, -0.11594009399414062, 0.5926361083984375], 'cosine_ionic_motion': -0.48485910190545994, 'ionic_motion_component': -6.502898442068778, 'ionic_force_x': -4.794602394104004, 'ionic_force_y': 12.35471922159195, 'ionic_force_z': -2.0622036159038544, 'radial_force': 13.25244502580265, 'axial_force': -2.0622036159038544, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-2.5619351863861084, 2.5342040061950684, 0.6784204840660095], 'magnitude': 3.66687273979187, 'distance': 9.515270233154297, 'before_closest_residue': 'SF', 'closest_residue': 780, 'next_closest_residue': 455, 'cosine_with_motion': -0.49398834488022203, 'motion_component': -1.8113924298092634}, {'ion': 1307, 'force': [0.7434799671173096, 3.142179489135742, -0.4046603739261627], 'magnitude': 3.2541980743408203, 'distance': 10.100597381591797, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.03021174737720038, 'motion_component': -0.09831500695590556}, {'ion': 1308, 'force': [-0.9280287027359009, 1.4536443948745728, -2.190319776535034], 'magnitude': 2.7877984046936035, 'distance': 10.912854194641113, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8238689283199169, 'motion_component': -2.2967804955902}, {'ion': 1320, 'force': [-0.4511340856552124, 0.7071818709373474, -1.4634768962860107], 'magnitude': 1.6868292093276978, 'distance': 14.029218673706055, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8145641030190202, 'motion_component': -1.3740305233741053}, {'ion': 1460, 'force': [-1.5969843864440918, 4.517509460449219, 1.3178329467773438], 'magnitude': 4.969399929046631, 'distance': 8.173669815063477, 'before_closest_residue': 130, 'closest_residue': 1105, 'next_closest_residue': 780, 'cosine_with_motion': -0.18561192477866056, 'motion_component': -0.9223798648451975}]}, 4861: {'frame': 4861, 'ionic_force': [-6.5610339641571045, 14.756245732307434, 0.32843945175409317], 'ionic_force_magnitude': 16.152455765750698, 'motion_vector': [0.4648017883300781, 0.24734878540039062, -0.2841033935546875], 'cosine_ionic_motion': 0.05246958628210433, 'ionic_motion_component': 0.8475126714689298, 'ionic_force_x': -6.5610339641571045, 'ionic_force_y': 14.756245732307434, 'ionic_force_z': 0.32843945175409317, 'radial_force': 16.14911622321991, 'axial_force': 0.32843945175409317, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-4.193318843841553, 3.516507863998413, 3.0015461444854736], 'magnitude': 6.2417168617248535, 'distance': 7.293181419372559, 'before_closest_residue': 780, 'closest_residue': 455, 'next_closest_residue': 780, 'cosine_with_motion': -0.5173703735538827, 'motion_component': -3.229279399255646}, {'ion': 1307, 'force': [0.5813269019126892, 2.4661834239959717, -0.11614765971899033], 'magnitude': 2.536432981491089, 'distance': 11.440825462341309, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.6017869355737689, 'motion_component': 1.5263921905233118}, {'ion': 1308, 'force': [-0.8082016706466675, 1.8407821655273438, -2.506990909576416], 'magnitude': 3.2135140895843506, 'distance': 10.164334297180176, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.41189868486252534, 'motion_component': 1.3236421976845847}, {'ion': 1320, 'force': [-0.4184555411338806, 0.7065335512161255, -1.485287070274353], 'magnitude': 1.6971659660339355, 'distance': 13.986430168151855, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.39614474603532723, 'motion_component': 0.672323388035597}, {'ion': 1460, 'force': [-1.7223848104476929, 6.22623872756958, 1.435318946838379], 'magnitude': 6.617612838745117, 'distance': 7.0830183029174805, 'before_closest_residue': 1105, 'closest_residue': 780, 'next_closest_residue': 1105, 'cosine_with_motion': 0.0837816523417639, 'motion_component': 0.554434531374163}]}, 4862: {'frame': 4862, 'ionic_force': [-3.6536727249622345, 22.094812095165253, -0.211676687002182], 'ionic_force_magnitude': 22.395866871403168, 'motion_vector': [-0.7869873046875, 0.3434638977050781, -0.23621368408203125], 'cosine_ionic_motion': 0.5271561819114349, 'ionic_motion_component': 11.806119670525685, 'ionic_force_x': -3.6536727249622345, 'ionic_force_y': 22.094812095165253, 'ionic_force_z': -0.211676687002182, 'radial_force': 22.394866507791328, 'axial_force': -0.211676687002182, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-1.5576599836349487, 2.6959004402160645, 1.676754355430603], 'magnitude': 3.5363383293151855, 'distance': 9.68929386138916, 'before_closest_residue': 455, 'closest_residue': 780, 'next_closest_residue': 1105, 'cosine_with_motion': 0.5574892571033411, 'motion_component': 1.9714706436235507}, {'ion': 1307, 'force': [0.7250994443893433, 2.6796772480010986, -0.3156937062740326], 'magnitude': 2.793940305709839, 'distance': 10.900853157043457, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.1705249007816293, 'motion_component': 0.47643637639311986}, {'ion': 1308, 'force': [-0.5865727663040161, 1.652468204498291, -2.294264078140259], 'magnitude': 2.8876230716705322, 'distance': 10.722567558288574, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.6109457566715136, 'motion_component': 1.7641810025489164}, {'ion': 1320, 'force': [-0.32260993123054504, 0.7156185507774353, -1.465861201286316], 'magnitude': 1.6628097295761108, 'distance': 14.130182266235352, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5712511650610931, 'motion_component': 0.9498819854370506}, {'ion': 1460, 'force': [-1.9119294881820679, 14.351147651672363, 2.1873879432678223], 'magnitude': 14.642252922058105, 'distance': 4.761733531951904, 'before_closest_residue': 780, 'closest_residue': 1105, 'next_closest_residue': 1105, 'cosine_with_motion': 0.45376553288560995, 'motion_component': 6.644149834145949}]}, 4863: {'frame': 4863, 'ionic_force': [-0.5461589097976685, 16.03918308019638, -1.5026157051324844], 'ionic_force_magnitude': 16.118670459815228, 'motion_vector': [1.4510307312011719, -0.018299102783203125, -1.9164810180664062], 'cosine_ionic_motion': 0.046292848970694904, 'ionic_motion_component': 0.7461791772046277, 'ionic_force_x': -0.5461589097976685, 'ionic_force_y': 16.03918308019638, 'ionic_force_z': -1.5026157051324844, 'radial_force': 16.048479162674862, 'axial_force': -1.5026157051324844, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 130, 'contributions': [{'ion': 1306, 'force': [2.4124746322631836, 4.2648186683654785, 1.696656584739685], 'magnitude': 5.185301780700684, 'distance': 8.00169563293457, 'before_closest_residue': 780, 'closest_residue': 1105, 'next_closest_residue': 1105, 'cosine_with_motion': 0.01371224371523597, 'motion_component': 0.07110212325467757}, {'ion': 1307, 'force': [0.740688681602478, 2.5558183193206787, -0.2357446402311325], 'magnitude': 2.6714046001434326, 'distance': 11.148056983947754, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.23043333330765023, 'motion_component': 0.6155806667175762}, {'ion': 1308, 'force': [-0.7104681134223938, 1.5558724403381348, -1.9979960918426514], 'magnitude': 2.630112648010254, 'distance': 11.235227584838867, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.4380751251609181, 'motion_component': 1.1521869135222806}, {'ion': 1320, 'force': [-0.3768095374107361, 0.7196657061576843, -1.397373080253601], 'magnitude': 1.6163402795791626, 'distance': 14.331863403320312, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5451289495529077, 'motion_component': 0.8811138419875748}, {'ion': 1460, 'force': [-2.6120445728302, 6.943007946014404, 0.43184152245521545], 'magnitude': 7.430654048919678, 'distance': 6.684293746948242, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 455, 'cosine_with_motion': -0.2656299511950648, 'motion_component': -1.9738043384000463}]}, 4864: {'frame': 4864, 'ionic_force': [-0.0066828131675720215, 12.786956429481506, -2.553470253944397], 'ionic_force_magnitude': 13.039421372408713, 'motion_vector': [-1.0789031982421875, -0.15365219116210938, 2.0991592407226562], 'cosine_ionic_motion': -0.23727350748459608, 'ionic_motion_component': -3.093909244601021, 'ionic_force_x': -0.0066828131675720215, 'ionic_force_y': 12.786956429481506, 'ionic_force_z': -2.553470253944397, 'radial_force': 12.786958175791858, 'axial_force': -2.553470253944397, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [2.984558343887329, 4.312427520751953, 0.5002753138542175], 'magnitude': 5.268291473388672, 'distance': 7.938421249389648, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 1105, 'cosine_with_motion': -0.22731887570885118, 'motion_component': -1.1975820940089648}, {'ion': 1307, 'force': [0.9359217882156372, 2.3722565174102783, -0.6875678896903992], 'magnitude': 2.641268730163574, 'distance': 11.211475372314453, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.451023395229303, 'motion_component': -1.1912739627321258}, {'ion': 1308, 'force': [-0.32004624605178833, 1.0951236486434937, -1.809603214263916], 'magnitude': 2.139249563217163, 'distance': 12.457712173461914, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7157728839742278, 'motion_component': -1.5312169138518108}, {'ion': 1460, 'force': [-3.60711669921875, 5.007148742675781, -0.5565744638442993], 'magnitude': 6.196176528930664, 'distance': 7.319933891296387, 'before_closest_residue': 1105, 'closest_residue': 455, 'next_closest_residue': 780, 'cosine_with_motion': 0.13333443679738946, 'motion_component': 0.8261637182101396}]}, 4865: {'frame': 4865, 'ionic_force': [-0.5236209034919739, 12.514497458934784, -1.6652111858129501], 'ionic_force_magnitude': 12.635654070669057, 'motion_vector': [3.705402374267578, -1.9471969604492188, -2.8583602905273438], 'cosine_ionic_motion': -0.336453391402117, 'ionic_motion_component': -4.251308664660569, 'ionic_force_x': -0.5236209034919739, 'ionic_force_y': 12.514497458934784, 'ionic_force_z': -1.6652111858129501, 'radial_force': 12.525447117778228, 'axial_force': -1.6652111858129501, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [2.304857015609741, 4.980421543121338, 1.5797655582427979], 'magnitude': 5.7107462882995605, 'distance': 7.624697208404541, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 1105, 'cosine_with_motion': -0.19598413987510246, 'motion_component': -1.119215710669991}, {'ion': 1307, 'force': [0.3401249349117279, 2.030419111251831, -0.1505231112241745], 'magnitude': 2.0642054080963135, 'distance': 12.682141304016113, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.2162962895753994, 'motion_component': -0.44647996958638897}, {'ion': 1308, 'force': [-0.8212441205978394, 1.7357362508773804, -2.2392847537994385], 'magnitude': 2.949850559234619, 'distance': 10.608867645263672, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.0014832429453785205, 'motion_component': -0.004375345063333924}, {'ion': 1320, 'force': [-0.41535165905952454, 0.8550887703895569, -1.5833065509796143], 'magnitude': 1.8467683792114258, 'distance': 13.407963752746582, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.14118443913662393, 'motion_component': 0.26073495759911935}, {'ion': 1460, 'force': [-1.932007074356079, 2.9128317832946777, 0.7281376719474792], 'magnitude': 3.5703535079956055, 'distance': 9.643028259277344, 'before_closest_residue': 455, 'closest_residue': 780, 'next_closest_residue': 455, 'cosine_with_motion': -0.8240002960827033, 'motion_component': -2.9419724204515667}]}, 4866: {'frame': 4866, 'ionic_force': [-1.7787259072065353, 16.205128252506256, -4.119738966226578], 'ionic_force_magnitude': 16.814942660710734, 'motion_vector': [-0.006435394287109375, 0.24068450927734375, 0.5570297241210938], 'cosine_ionic_motion': 0.15846346228410718, 'ionic_motion_component': 2.6645540321249603, 'ionic_force_x': -1.7787259072065353, 'ionic_force_y': 16.205128252506256, 'ionic_force_z': -4.119738966226578, 'radial_force': 16.302455260884607, 'axial_force': -4.119738966226578, 'before_closest_residue': 98, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [4.388768196105957, 2.6268601417541504, -0.013402372598648071], 'magnitude': 5.114866733551025, 'distance': 8.056601524353027, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 1105, 'cosine_with_motion': 0.19218926722432111, 'motion_component': 0.9830224595071845}, {'ion': 1307, 'force': [1.5909762382507324, 2.1847963333129883, -1.0358966588974], 'magnitude': 2.8944122791290283, 'distance': 10.70998477935791, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.034966850579650224, 'motion_component': -0.10120848080482325}, {'ion': 1308, 'force': [0.049068644642829895, 0.7890864014625549, -2.0871825218200684], 'magnitude': 2.2319042682647705, 'distance': 12.196389198303223, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7184098472140821, 'motion_component': -1.603421891308001}, {'ion': 1460, 'force': [-7.807538986206055, 10.604385375976562, -0.9832574129104614], 'magnitude': 13.205204963684082, 'distance': 5.0141401290893555, 'before_closest_residue': 780, 'closest_residue': 455, 'next_closest_residue': 'SF', 'cosine_with_motion': 0.25642628453809563, 'motion_component': 3.386161754441588}]}, 4867: {'frame': 4867, 'ionic_force': [5.378923777490854, 8.464651763439178, -4.732402980327606], 'ionic_force_magnitude': 11.089580174585695, 'motion_vector': [-0.9177093505859375, 0.6418495178222656, 2.0229339599609375], 'cosine_ionic_motion': -0.3539779082731976, 'ionic_motion_component': -3.9254663938277656, 'ionic_force_x': 5.378923777490854, 'ionic_force_y': 8.464651763439178, 'ionic_force_z': -4.732402980327606, 'radial_force': 10.029115139450264, 'axial_force': -4.732402980327606, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [3.6623687744140625, 2.4839608669281006, 0.24527764320373535], 'magnitude': 4.432061195373535, 'distance': 8.65498161315918, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 1105, 'cosine_with_motion': -0.12397397560583501, 'motion_component': -0.5494602648538489}, {'ion': 1307, 'force': [1.5931791067123413, 1.9242557287216187, -0.7641410231590271], 'magnitude': 2.6124494075775146, 'distance': 11.27314567565918, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.2934810663419785, 'motion_component': -0.7667044026091752}, {'ion': 1308, 'force': [0.09774009138345718, 0.9288542866706848, -2.069882869720459], 'magnitude': 2.270845413208008, 'distance': 12.091362953186035, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7009982594382919, 'motion_component': -1.5918586226891804}, {'ion': 1460, 'force': [0.02563580498099327, 3.1275808811187744, -2.1436567306518555], 'magnitude': 3.7917916774749756, 'distance': 9.357219696044922, 'before_closest_residue': 455, 'closest_residue': 'SF', 'next_closest_residue': 'SF', 'cosine_with_motion': -0.2683278059184076, 'motion_component': -1.0174431206508086}]}, 4868: {'frame': 4868, 'ionic_force': [5.495622593909502, 13.52440232038498, -5.167728379368782], 'ionic_force_magnitude': 15.486017642417199, 'motion_vector': [0.3851051330566406, 2.4810562133789062, 0.2808074951171875], 'cosine_ionic_motion': 0.8746522569128867, 'ionic_motion_component': 13.544880281532985, 'ionic_force_x': 5.495622593909502, 'ionic_force_y': 13.52440232038498, 'ionic_force_z': -5.167728379368782, 'radial_force': 14.59833298080035, 'axial_force': -5.167728379368782, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [5.109704494476318, 4.990457057952881, 0.5856501460075378], 'magnitude': 7.166360855102539, 'distance': 6.8064351081848145, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 130, 'cosine_with_motion': 0.8016372440955264, 'motion_component': 5.7448217580309375}, {'ion': 1307, 'force': [1.5923055410385132, 2.200728178024292, -0.21902848780155182], 'magnitude': 2.7251815795898438, 'distance': 11.037514686584473, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.8731838929208929, 'motion_component': 2.37958470645049}, {'ion': 1308, 'force': [-0.13308840990066528, 1.483996033668518, -2.676917314529419], 'magnitude': 3.0636322498321533, 'distance': 10.40999984741211, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.37195321146052107, 'motion_component': 1.1395278843755534}, {'ion': 1320, 'force': [-0.05506179854273796, 0.6272523999214172, -1.598051905632019], 'magnitude': 1.7176283597946167, 'distance': 13.90286922454834, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.25033097015726313, 'motion_component': 0.4299755799140038}, {'ion': 1460, 'force': [-1.0182372331619263, 4.221968650817871, -1.25938081741333], 'magnitude': 4.5219316482543945, 'distance': 8.568544387817383, 'before_closest_residue': 'SF', 'closest_residue': 'SF', 'next_closest_residue': 'SF', 'cosine_with_motion': 0.851620709199047, 'motion_component': 3.8509706902766823}]}, 4869: {'frame': 4869, 'ionic_force': [1.516260078176856, 9.671549260616302, -2.2401423305273056], 'ionic_force_magnitude': 10.042716135897745, 'motion_vector': [-0.0664825439453125, -0.035305023193359375, -0.05754852294921875], 'cosine_ionic_motion': -0.32928576536765514, 'ionic_motion_component': -3.306923469179189, 'ionic_force_x': 1.516260078176856, 'ionic_force_y': 9.671549260616302, 'ionic_force_z': -2.2401423305273056, 'radial_force': 9.78968384194304, 'axial_force': -2.2401423305273056, 'before_closest_residue': 455, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [0.575779914855957, 3.006566047668457, 1.7751314640045166], 'magnitude': 3.538651466369629, 'distance': 9.686126708984375, 'before_closest_residue': 1105, 'closest_residue': 130, 'next_closest_residue': 130, 'cosine_with_motion': -0.735409965892542, 'motion_component': -2.602359494273699}, {'ion': 1307, 'force': [0.8862696886062622, 1.4997901916503906, -0.13419704139232635], 'magnitude': 1.7472416162490845, 'distance': 13.78454875946045, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.6290806353560883, 'motion_component': -1.0991558949241158}, {'ion': 1308, 'force': [-0.011133236810564995, 1.6809277534484863, -1.8282040357589722], 'magnitude': 2.4835402965545654, 'distance': 11.562012672424316, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.19804797994433204, 'motion_component': 0.49186012500856546}, {'ion': 1320, 'force': [0.029794860631227493, 0.8571366667747498, -1.3412694931030273], 'magnitude': 1.5920348167419434, 'distance': 14.440850257873535, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.2979502960962926, 'motion_component': 0.47434724454418253}, {'ion': 1460, 'force': [0.035548850893974304, 2.6271286010742188, -0.7116032242774963], 'magnitude': 2.7220301628112793, 'distance': 11.043903350830078, 'before_closest_residue': 'SF', 'closest_residue': 'SF', 'next_closest_residue': 'SF', 'cosine_with_motion': -0.20999599232849375, 'motion_component': -0.5716154000736449}]}, 4870: {'frame': 4870, 'ionic_force': [2.109794482588768, 14.001262068748474, 0.36937230825424194], 'ionic_force_magnitude': 14.164145162297718, 'motion_vector': [-0.150634765625, -2.8217086791992188, -4.534019470214844], 'cosine_ionic_motion': -0.5484226447158912, 'ionic_motion_component': -7.76793795004711, 'ionic_force_x': 2.109794482588768, 'ionic_force_y': 14.001262068748474, 'ionic_force_z': 0.36937230825424194, 'radial_force': 14.15932810116839, 'axial_force': 0.36937230825424194, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 130, 'contributions': [{'ion': 1306, 'force': [1.2838693857192993, 7.539500713348389, 4.284053325653076], 'magnitude': 8.766157150268555, 'distance': 6.154098033905029, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 455, 'cosine_with_motion': -0.8731376834641819, 'motion_component': -7.654061814393759}, {'ion': 1307, 'force': [0.9159259796142578, 1.6046597957611084, -0.13191652297973633], 'magnitude': 1.8523647785186768, 'distance': 13.387694358825684, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.4110399846012579, 'motion_component': -0.7613960074133352}, {'ion': 1308, 'force': [-0.0317416787147522, 1.5285658836364746, -1.7929517030715942], 'magnitude': 2.3563101291656494, 'distance': 11.870057106018066, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.30352157353261566, 'motion_component': 0.7151909310539509}, {'ion': 1320, 'force': [-0.024010654538869858, 0.8109053373336792, -1.3013789653778076], 'magnitude': 1.5335354804992676, 'distance': 14.71370792388916, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.44135347987078855, 'motion_component': 0.6768312379802743}, {'ion': 1460, 'force': [-0.03424854949116707, 2.5176303386688232, -0.688433825969696], 'magnitude': 2.6102828979492188, 'distance': 11.277822494506836, 'before_closest_residue': 'SF', 'closest_residue': 'SF', 'next_closest_residue': 'SF', 'cosine_with_motion': -0.28521913588366826, 'motion_component': -0.7445026222250654}]}, 4871: {'frame': 4871, 'ionic_force': [-8.979765210300684, 10.853928327560425, -14.876065850257874], 'ionic_force_magnitude': 20.4875884025708, 'motion_vector': [-0.12489700317382812, -0.5373611450195312, 0.7347412109375], 'cosine_ionic_motion': -0.830903443944247, 'ionic_motion_component': -17.02320776180829, 'ionic_force_x': -8.979765210300684, 'ionic_force_y': 10.853928327560425, 'ionic_force_z': -14.876065850257874, 'radial_force': 14.087013287845835, 'axial_force': -14.876065850257874, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 130, 'contributions': [{'ion': 1306, 'force': [-8.6154203414917, 6.36574125289917, -8.871593475341797], 'magnitude': 13.908748626708984, 'distance': 4.885679721832275, 'before_closest_residue': 130, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': -0.6935362226386466, 'motion_component': -9.64622127814738}, {'ion': 1307, 'force': [1.0734245777130127, 1.7163671255111694, -0.9967178106307983], 'magnitude': 2.256458044052124, 'distance': 12.129849433898926, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.8627577007666385, 'motion_component': -1.9467765392489866}, {'ion': 1308, 'force': [-0.03414252772927284, 0.5607947111129761, -1.570929765701294], 'magnitude': 1.6683754920959473, 'distance': 14.106593132019043, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.9467690197126633, 'motion_component': -1.579566219617024}, {'ion': 1460, 'force': [-1.4036269187927246, 2.2110252380371094, -3.4368247985839844], 'magnitude': 4.3209452629089355, 'distance': 8.765560150146484, 'before_closest_residue': 'SF', 'closest_residue': 'SF', 'next_closest_residue': 'SF', 'cosine_with_motion': -0.8911577797428331, 'motion_component': -3.8506437663609603}]}, 4872: {'frame': 4872, 'ionic_force': [-12.953509864215448, 10.026119828224182, -15.728052258491516], 'ionic_force_magnitude': 22.708767568013837, 'motion_vector': [1.6905479431152344, -0.46477508544921875, 1.652435302734375], 'cosine_ionic_motion': -0.9604613279560743, 'ionic_motion_component': -21.8108930546204, 'ionic_force_x': -12.953509864215448, 'ionic_force_y': 10.026119828224182, 'ionic_force_z': -15.728052258491516, 'radial_force': 16.380369245295938, 'axial_force': -15.728052258491516, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [-12.665992736816406, 4.810243606567383, -8.359336853027344], 'magnitude': 15.919934272766113, 'distance': 4.566657066345215, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 98, 'cosine_with_motion': -0.9766974277304483, 'motion_component': -15.548959496090902}, {'ion': 1307, 'force': [1.279715895652771, 1.9624840021133423, -1.071542501449585], 'magnitude': 2.57628</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>4992</v>
+      </c>
+      <c r="B10" t="n">
+        <v>5269</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1308</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>{4992: {'frame': 4992, 'ionic_force': [-19.95671159029007, -2.516607314348221, 0.35591466911137104], 'ionic_force_magnitude': 20.117910555630214, 'motion_vector': [1.30914306640625, -2.567424774169922, 0.49839019775390625], 'cosine_ionic_motion': -0.3312020802294139, 'ionic_motion_component': -6.663093825894011, 'ionic_force_x': -19.95671159029007, 'ionic_force_y': -2.516607314348221, 'ionic_force_z': 0.35591466911137104, 'radial_force': 20.114761988963455, 'axial_force': 0.35591466911137104, 'before_closest_residue': None, 'closest_residue': 1073, 'next_closest_residue': 1073, 'contributions': [{'ion': 1306, 'force': [-1.3452452421188354, -1.3558294773101807, -0.08520316332578659], 'magnitude': 1.9118623733520508, 'distance': 13.177733421325684, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.29998483611445825, 'motion_component': 0.5735297346601306}, {'ion': 1307, 'force': [-8.701690673828125, 2.1244421005249023, 0.4665580689907074], 'magnitude': 8.969411849975586, 'distance': 6.083970069885254, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 'SF', 'cosine_with_motion': -0.6333103158005003, 'motion_component': -5.680421133112911}, {'ion': 1309, 'force': [-0.8666126132011414, -0.2845568358898163, -1.5572242736816406], 'magnitude': 1.8046987056732178, 'distance': 13.56334114074707, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.2235692216062886, 'motion_component': -0.4034750869979291}, {'ion': 1316, 'force': [-3.8274505138397217, -1.5964282751083374, 4.4594645500183105], 'magnitude': 6.089727878570557, 'distance': 7.383633136749268, 'before_closest_residue': 780, 'closest_residue': 130, 'next_closest_residue': 130, 'cosine_with_motion': 0.073584092113622, 'motion_component': 0.44810709179433417}, {'ion': 1320, 'force': [-3.069931983947754, -1.0022555589675903, -2.9554810523986816], 'magnitude': 4.377655506134033, 'distance': 8.708598136901855, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.22796719378171773, 'motion_component': -0.9979618179615599}, {'ion': 1460, 'force': [-2.145780563354492, -0.4019792675971985, 0.027800539508461952], 'magnitude': 2.1832852363586426, 'distance': 12.331439971923828, 'before_closest_residue': 455, 'closest_residue': 423, 'next_closest_residue': 130, 'cosine_with_motion': -0.27613096677313564, 'motion_component': -0.602872663331882}]}, 4993: {'frame': 4993, 'ionic_force': [-11.465587615966797, -15.185635328292847, -2.6171058416366577], 'ionic_force_magnitude': 19.207094071973398, 'motion_vector': [-1.2147407531738281, 0.47171783447265625, 0.3584442138671875], 'cosine_ionic_motion': 0.2244448562089598, 'ionic_motion_component': 4.310933467176033, 'ionic_force_x': -11.465587615966797, 'ionic_force_y': -15.185635328292847, 'ionic_force_z': -2.6171058416366577, 'radial_force': 19.02795889482913, 'axial_force': -2.6171058416366577, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'contributions': [{'ion': 1307, 'force': [-4.743855953216553, -8.147418975830078, -2.642191171646118], 'magnitude': 9.791107177734375, 'distance': 5.823085308074951, 'before_closest_residue': 780, 'closest_residue': 'SF', 'next_closest_residue': 'SF', 'cosine_with_motion': 0.07346829407524873, 'motion_component': 0.7193359403088735}, {'ion': 1309, 'force': [-0.767593502998352, -0.664334774017334, -1.574743628501892], 'magnitude': 1.873594880104065, 'distance': 13.311628341674805, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.02155868336146814, 'motion_component': 0.040392239910257643}, {'ion': 1316, 'force': [-0.9619420766830444, -1.5705485343933105, 2.251835346221924], 'magnitude': 2.9090750217437744, 'distance': 10.68295955657959, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 1105, 'cosine_with_motion': 0.31406873477619174, 'motion_component': 0.9136495223597336}, {'ion': 1320, 'force': [-2.390256643295288, -2.211256742477417, -2.6654586791992188], 'magnitude': 4.2080464363098145, 'distance': 8.882369041442871, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.15913419023094658, 'motion_component': 0.6696440311311278}, {'ion': 1460, 'force': [-2.6019394397735596, -2.592076301574707, 2.0134522914886475], 'magnitude': 4.18842887878418, 'distance': 8.903144836425781, 'before_closest_residue': 423, 'closest_residue': 130, 'next_closest_residue': 780, 'cosine_with_motion': 0.46984474326150344, 'motion_component': 1.9679114067019796}]}, 4994: {'frame': 4994, 'ionic_force': [-15.226321399211884, -15.62778353691101, -3.6030957102775574], 'ionic_force_magnitude': 22.114492540550533, 'motion_vector': [0.4574928283691406, 1.3063774108886719, 0.06430816650390625], 'cosine_ionic_motion': -0.9011274603866004, 'ionic_motion_component': -19.92797650080472, 'ionic_force_x': -15.226321399211884, 'ionic_force_y': -15.62778353691101, 'ionic_force_z': -3.6030957102775574, 'radial_force': 21.81899359797891, 'axial_force': -3.6030957102775574, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'contributions': [{'ion': 1306, 'force': [-0.8425669074058533, -1.2280627489089966, -0.028977513313293457], 'magnitude': 1.4895961284637451, 'distance': 14.929139137268066, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.964909033799051, 'motion_component': -1.4373248190602443}, {'ion': 1307, 'force': [-5.873695373535156, -9.419403076171875, -2.7254559993743896], 'magnitude': 11.430378913879395, 'distance': 5.389379024505615, 'before_closest_residue': 'SF', 'closest_residue': 'SF', 'next_closest_residue': 780, 'cosine_with_motion': -0.9576418833241156, 'motion_component': -10.946209587772444}, {'ion': 1309, 'force': [-0.9202994108200073, -0.567900538444519, -1.5354427099227905], 'magnitude': 1.8780431747436523, 'distance': 13.295854568481445, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.4848207257917492, 'motion_component': -0.9105142778132502}, {'ion': 1316, 'force': [-1.8541682958602905, -1.3925756216049194, 2.6088037490844727], 'magnitude': 3.490424633026123, 'distance': 9.752813339233398, 'before_closest_residue': 130, 'closest_residue': 1105, 'next_closest_residue': 130, 'cosine_with_motion': -0.5168421163071228, 'motion_component': -1.8039984403479077}, {'ion': 1320, 'force': [-2.610811948776245, -1.7711108922958374, -2.3384480476379395], 'magnitude': 3.927023410797119, 'distance': 9.194694519042969, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6723389238516795, 'motion_component': -2.640290627803788}, {'ion': 1460, 'force': [-3.124779462814331, -1.2487306594848633, 0.41642481088638306], 'magnitude': 3.3907203674316406, 'distance': 9.89516544342041, 'before_closest_residue': 130, 'closest_residue': 780, 'next_closest_residue': 423, 'cosine_with_motion': -0.6457740657600884, 'motion_component': -2.189639274119873}]}, 4995: {'frame': 4995, 'ionic_force': [-16.513193786144257, -9.016636848449707, -1.008799159899354], 'ionic_force_magnitude': 18.841522890164374, 'motion_vector': [0.29911041259765625, -1.0097732543945312, -0.8112640380859375], 'cosine_ionic_motion': 0.19897691775147616, 'ionic_motion_component': 3.749028150428792, 'ionic_force_x': -16.513193786144257, 'ionic_force_y': -9.016636848449707, 'ionic_force_z': -1.008799159899354, 'radial_force': 18.814497311264375, 'axial_force': -1.008799159899354, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'contributions': [{'ion': 1306, 'force': [-1.3241117000579834, -1.5251678228378296, 0.027443215250968933], 'magnitude': 2.0199410915374756, 'distance': 12.820343971252441, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.41774291685847037, 'motion_component': 0.8438160626594282}, {'ion': 1307, 'force': [-7.239418983459473, -4.05126953125, 1.7257643938064575], 'magnitude': 8.473502159118652, 'distance': 6.259469985961914, 'before_closest_residue': 'SF', 'closest_residue': 780, 'next_closest_residue': 1073, 'cosine_with_motion': 0.046644447777078414, 'motion_component': 0.39524181776226897}, {'ion': 1309, 'force': [-0.9697037935256958, -0.4882330298423767, -1.6673376560211182], 'magnitude': 1.989651083946228, 'distance': 12.917562484741211, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5881295353879933, 'motion_component': 1.1701726210799208}, {'ion': 1316, 'force': [-0.7669690251350403, -0.3876888155937195, 1.759548544883728], 'magnitude': 1.9582020044326782, 'distance': 13.020878791809082, 'before_closest_residue': 1105, 'closest_residue': 130, 'next_closest_residue': None, 'cosine_with_motion': -0.48608984963177254, 'motion_component': -0.9518621296608849}, {'ion': 1320, 'force': [-3.7609140872955322, -1.9077779054641724, -2.8672845363616943], 'magnitude': 5.099550247192383, 'distance': 8.06869125366211, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.461351578304799, 'motion_component': 2.3526855188822395}, {'ion': 1460, 'force': [-2.4520761966705322, -0.6564997434616089, 0.013066878542304039], 'magnitude': 2.5384721755981445, 'distance': 11.43622875213623, 'before_closest_residue': 780, 'closest_residue': 423, 'next_closest_residue': 455, 'cosine_with_motion': -0.02404027018762123, 'motion_component': -0.061025553861092874}]}, 4996: {'frame': 4996, 'ionic_force': [-3.4634814858436584, -24.222798764705658, -7.885996222496033], 'ionic_force_magnitude': 25.708532054931286, 'motion_vector': [-0.20244598388671875, 1.0721435546875, 1.0912857055664062], 'cosine_ionic_motion': -0.8538624943495546, 'ionic_motion_component': -21.951551306489108, 'ionic_force_x': -3.4634814858436584, 'ionic_force_y': -24.222798764705658, 'ionic_force_z': -7.885996222496033, 'radial_force': 24.469157811379773, 'axial_force': -7.885996222496033, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'contributions': [{'ion': 1306, 'force': [-1.1426242589950562, -1.551206111907959, -0.044628992676734924], 'magnitude': 1.9271279573440552, 'distance': 13.125436782836914, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.4978323819676272, 'motion_component': -0.9593867248527452}, {'ion': 1307, 'force': [3.4352829456329346, -19.294559478759766, -3.6758644580841064], 'magnitude': 19.939739227294922, 'distance': 4.0804619789123535, 'before_closest_residue': 780, 'closest_residue': 1073, 'next_closest_residue': 1105, 'cosine_with_motion': -0.8252532786161767, 'motion_component': -16.45533462281747}, {'ion': 1309, 'force': [-0.8596774935722351, -0.5392806529998779, -1.5933207273483276], 'magnitude': 1.889057993888855, 'distance': 13.257035255432129, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7350984190555, 'motion_component': -1.3886435159335724}, {'ion': 1320, 'force': [-2.712550401687622, -1.9728121757507324, -2.712400197982788], 'magnitude': 4.313587188720703, 'distance': 8.773033142089844, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6799253774807416, 'motion_component': -2.9329172369528784}, {'ion': 1460, 'force': [-2.1839122772216797, -0.864940345287323, 0.14021815359592438], 'magnitude': 2.353137493133545, 'distance': 11.878056526184082, 'before_closest_residue': 423, 'closest_residue': 455, 'next_closest_residue': 780, 'cosine_with_motion': -0.09148190274176744, 'motion_component': -0.21526948954107716}]}, 4997: {'frame': 4997, 'ionic_force': [-12.324485659599304, -21.485591620206833, 0.6895290873944759], 'ionic_force_magnitude': 24.77900410440932, 'motion_vector': [-0.3025016784667969, -0.6528167724609375, -0.76025390625], 'cosine_ionic_motion': 0.6643024147055198, 'ionic_motion_component': 16.460752260557097, 'ionic_force_x': -12.324485659599304, 'ionic_force_y': -21.485591620206833, 'ionic_force_z': 0.6895290873944759, 'radial_force': 24.76940843144969, 'axial_force': 0.6895290873944759, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'contributions': [{'ion': 1306, 'force': [-1.535698652267456, -1.5813456773757935, -0.031177494674921036], 'magnitude': 2.2045400142669678, 'distance': 12.2718505859375, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 455, 'cosine_with_motion': 0.6589519030785869, 'motion_component': 1.4526858174288506}, {'ion': 1307, 'force': [-4.548783779144287, -17.15741729736328, 5.0139594078063965], 'magnitude': 18.444732666015625, 'distance': 4.242607593536377, 'before_closest_residue': 1073, 'closest_residue': 1105, 'next_closest_residue': 98, 'cosine_with_motion': 0.4539732335482293, 'motion_component': 8.373415274994159}, {'ion': 1309, 'force': [-1.0400985479354858, -0.5203492045402527, -1.7408907413482666], 'magnitude': 2.093625783920288, 'distance': 12.592719078063965, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.9025147840163484, 'motion_component': 1.889528208024867}, {'ion': 1320, 'force': [-3.253243923187256, -1.7816591262817383, -2.824697256088257], 'magnitude': 4.662276268005371, 'distance': 8.438592910766602, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.8800268431847608, 'motion_component': 4.102928252537652}, {'ion': 1460, 'force': [-1.9466607570648193, -0.4448203146457672, 0.2723351716995239], 'magnitude': 2.0153212547302246, 'distance': 12.835030555725098, 'before_closest_residue': 455, 'closest_residue': 780, 'next_closest_residue': 455, 'cosine_with_motion': 0.31865627031193433, 'motion_component': 0.6421947467171396}]}, 4998: {'frame': 4998, 'ionic_force': [-8.595291793346405, -8.897465407848358, -3.6955340802669525], 'ionic_force_magnitude': 12.91127041909667, 'motion_vector': [1.2956390380859375, -1.7068977355957031, 0.36876678466796875], 'cosine_ionic_motion': 0.09574013357122195, 'ionic_motion_component': 1.236126754498482, 'ionic_force_x': -8.595291793346405, 'ionic_force_y': -8.897465407848358, 'ionic_force_z': -3.6955340802669525, 'radial_force': 12.371092582978521, 'axial_force': -3.6955340802669525, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'contributions': [{'ion': 1306, 'force': [-1.212032675743103, -1.8853203058242798, 0.2718568742275238], 'magnitude': 2.2577338218688965, 'distance': 12.126421928405762, 'before_closest_residue': 423, 'closest_residue': 455, 'next_closest_residue': 130, 'cosine_with_motion': 0.35604776507517333, 'motion_component': 0.8038610823790502}, {'ion': 1307, 'force': [-1.4655177593231201, -4.378549098968506, 0.14790880680084229], 'magnitude': 4.619665622711182, 'distance': 8.477420806884766, 'before_closest_residue': 1105, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.5604186394119793, 'motion_component': 2.588946787382456}, {'ion': 1309, 'force': [-0.8881041407585144, -0.46092355251312256, -1.5887774229049683], 'magnitude': 1.8776030540466309, 'distance': 13.297412872314453, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.23263898336225206, 'motion_component': -0.4368036629911547}, {'ion': 1320, 'force': [-3.2808942794799805, -1.594046950340271, -2.6922800540924072], 'magnitude': 4.533610820770264, 'distance': 8.557500839233398, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.2559131491847294, 'motion_component': -1.160210559338669}, {'ion': 1460, 'force': [-1.748742938041687, -0.578625500202179, 0.16575771570205688], 'magnitude': 1.8494282960891724, 'distance': 13.39831829071045, 'before_closest_residue': 780, 'closest_residue': 455, 'next_closest_residue': 780, 'cosine_with_motion': -0.3026160485951843, 'motion_component': -0.5596666774590444}]}, 4999: {'frame': 4999, 'ionic_force': [-13.94003438949585, -13.628098368644714, 0.2862973641604185], 'ionic_force_magnitude': 19.496963612483583, 'motion_vector': [-0.551971435546875, 1.3257789611816406, 0.19469451904296875], 'cosine_ionic_motion': -0.3651526840154556, 'ionic_motion_component': -7.119368593250053, 'ionic_force_x': -13.94003438949585, 'ionic_force_y': -13.628098368644714, 'ionic_force_z': 0.2862973641604185, 'radial_force': 19.494861474906244, 'axial_force': 0.2862973641604185, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'contributions': [{'ion': 1306, 'force': [-1.312923789024353, -3.71425461769104, 1.741175651550293], 'magnitude': 4.307104587554932, 'distance': 8.779632568359375, 'before_closest_residue': 455, 'closest_residue': 130, 'next_closest_residue': 130, 'cosine_with_motion': -0.6184868912974, 'motion_component': -2.6638876523400654}, {'ion': 1307, 'force': [-0.6792678236961365, -3.1243350505828857, -0.02229972369968891], 'magnitude': 3.1974008083343506, 'distance': 10.189913749694824, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.8139339513431172, 'motion_component': -2.6024730272623255}, {'ion': 1309, 'force': [-0.7131099104881287, -0.7815901041030884, -1.624629020690918], 'magnitude': 1.938769817352295, 'distance': 13.085969924926758, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.34128113473276755, 'motion_component': -0.6616655531706854}, {'ion': 1320, 'force': [-2.2887518405914307, -2.6869468688964844, -2.5399811267852783], 'magnitude': 4.348513603210449, 'distance': 8.737730026245117, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.44327089905166983, 'motion_component': -1.9275696379600227}, {'ion': 1460, 'force': [-8.9459810256958, -3.320971727371216, 2.7320315837860107], 'magnitude': 9.925896644592285, 'distance': 5.783412456512451, 'before_closest_residue': 455, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.07417239319387016, 'motion_component': 0.7362275165773262}]}, 5000: {'frame': 5000, 'ionic_force': [-10.132799685001373, -11.112239122390747, -2.420377552509308], 'ionic_force_magnitude': 15.231996430745589, 'motion_vector': [-0.7812538146972656, 0.4613761901855469, -0.36583709716796875], 'cosine_ionic_motion': 0.2466097732420178, 'ionic_motion_component': 3.7563591858093943, 'ionic_force_x': -10.132799685001373, 'ionic_force_y': -11.112239122390747, 'ionic_force_z': -2.420377552509308, 'radial_force': 15.038466935481004, 'axial_force': -2.420377552509308, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'contributions': [{'ion': 1306, 'force': [-0.8784706592559814, -1.9305158853530884, 0.7727431654930115], 'magnitude': 2.257373332977295, 'distance': 12.127389907836914, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 455, 'cosine_with_motion': -0.22056165872803313, 'motion_component': -0.497890002691399}, {'ion': 1307, 'force': [-0.2424018383026123, -4.398298740386963, 0.5005394816398621], 'magnitude': 4.43332052230835, 'distance': 8.653753280639648, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.46644297210597535, 'motion_component': -2.0678911681111494}, {'ion': 1309, 'force': [-0.9397225975990295, -0.6545020341873169, -1.707296371459961], 'magnitude': 2.055799722671509, 'distance': 12.70804214477539, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.525454039767896, 'motion_component': 1.080228253059616}, {'ion': 1320, 'force': [-3.7437233924865723, -2.7520456314086914, -2.9792110919952393], 'magnitude': 5.519503593444824, 'distance': 7.755664825439453, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5083565310182332, 'motion_component': 2.805875644879151}, {'ion': 1460, 'force': [-4.328481197357178, -1.3768768310546875, 0.9928472638130188], 'magnitude': 4.649439334869385, 'distance': 8.450234413146973, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.523942040511297, 'motion_component': 2.436036667233086}]}, 5001: {'frame': 5001, 'ionic_force': [-8.440096318721771, -11.586323291063309, -2.215720146894455], 'ionic_force_magnitude': 14.504741605547162, 'motion_vector': [-0.016719818115234375, -0.3343772888183594, 0.31487274169921875], 'cosine_ionic_motion': 0.49766852568352266, 'ionic_motion_component': 7.218553370253107, 'ionic_force_x': -8.440096318721771, 'ionic_force_y': -11.586323291063309, 'ionic_force_z': -2.215720146894455, 'radial_force': 14.33450777928342, 'axial_force': -2.215720146894455, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'contributions': [{'ion': 1306, 'force': [-1.3881559371948242, -1.5592139959335327, 0.5130171179771423], 'magnitude': 2.149723529815674, 'distance': 12.427327156066895, 'before_closest_residue': 130, 'closest_residue': 455, 'next_closest_residue': 130, 'cosine_with_motion': 0.7146767039613597, 'motion_component': 1.5363574097926822}, {'ion': 1307, 'force': [-0.7212875485420227, -6.880537509918213, -0.3214363157749176], 'magnitude': 6.925704002380371, 'distance': 6.923681735992432, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.6947861646970184, 'motion_component': 4.811883197724699}, {'ion': 1309, 'force': [-0.9957014322280884, -0.4937232434749603, -1.515923261642456], 'magnitude': 1.8796827793121338, 'distance': 13.290054321289062, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.3421508167823267, 'motion_component': -0.6431349952876526}, {'ion': 1320, 'force': [-2.770164966583252, -1.6772152185440063, -2.3731327056884766], 'magnitude': 4.014800548553467, 'distance': 9.09362506866455, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.07592411220123893, 'motion_component': -0.3048201694466055}, {'ion': 1460, 'force': [-2.564786434173584, -0.9756333231925964, 1.481755018234253], 'magnitude': 3.1185874938964844, 'distance': 10.317870140075684, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.5830420678716011, 'motion_component': 1.8182676836329943}]}, 5002: {'frame': 5002, 'ionic_force': [-9.872247964143753, -10.693543076515198, -0.6216448545455933], 'ionic_force_magnitude': 14.567071967969735, 'motion_vector': [1.8620643615722656, -2.09149169921875, 0.0738525390625], 'cosine_ionic_motion': 0.09647517585558846, 'ionic_motion_component': 1.4053608298108933, 'ionic_force_x': -9.872247964143753, 'ionic_force_y': -10.693543076515198, 'ionic_force_z': -0.6216448545455933, 'radial_force': 14.553801681857102, 'axial_force': -0.6216448545455933, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'contributions': [{'ion': 1306, 'force': [-1.6060184240341187, -2.4026525020599365, 0.7531222701072693], 'magnitude': 2.9865076541900635, 'distance': 10.543559074401855, 'before_closest_residue': 455, 'closest_residue': 130, 'next_closest_residue': 130, 'cosine_with_motion': 0.2498493852032241, 'motion_component': 0.7461770765906097}, {'ion': 1307, 'force': [-0.4021822512149811, -4.678164482116699, 0.464477002620697], 'magnitude': 4.7183380126953125, 'distance': 8.388311386108398, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 130, 'cosine_with_motion': 0.6862030828318468, 'motion_component': 3.23773800062905}, {'ion': 1309, 'force': [-1.0093481540679932, -0.5549268126487732, -1.643075942993164], 'magnitude': 2.0065956115722656, 'distance': 12.862906455993652, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.14947363285212528, 'motion_component': -0.299933138318341}, {'ion': 1320, 'force': [-3.4694180488586426, -2.0770719051361084, -2.471514940261841], 'magnitude': 4.739142894744873, 'distance': 8.369877815246582, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.17314703360432673, 'motion_component': -0.8205685344170597}, {'ion': 1460, 'force': [-3.3852810859680176, -0.9807273745536804, 2.2753467559814453], 'magnitude': 4.195135116577148, 'distance': 8.896026611328125, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 1105, 'cosine_with_motion': -0.34755786630106694, 'motion_component': -1.4580521448367174}]}, 5003: {'frame': 5003, 'ionic_force': [-6.47410349547863, -13.501843988895416, 0.07296353578567505], 'ionic_force_magnitude': 14.973948405420469, 'motion_vector': [-0.707275390625, -0.40502166748046875, -0.429779052734375], 'cosine_ionic_motion': 0.7259607803572045, 'ionic_motion_component': 10.870499269427562, 'ionic_force_x': -6.47410349547863, 'ionic_force_y': -13.501843988895416, 'ionic_force_z': 0.07296353578567505, 'radial_force': 14.973770639709954, 'axial_force': 0.07296353578567505, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'contributions': [{'ion': 1306, 'force': [-1.46103036403656, -4.1621856689453125, 0.9036324620246887], 'magnitude': 4.502771377563477, 'distance': 8.58675479888916, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 130, 'cosine_with_motion': 0.5617807033865024, 'motion_component': 2.5295701225316485}, {'ion': 1307, 'force': [0.11960072815418243, -2.6055352687835693, 0.605388879776001], 'magnitude': 2.6776134967803955, 'distance': 11.135125160217285, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 130, 'cosine_with_motion': 0.2879913075521765, 'motion_component': 0.7711294135987297}, {'ion': 1309, 'force': [-0.6637636423110962, -0.8726678490638733, -1.511733055114746], 'magnitude': 1.8674763441085815, 'distance': 13.333417892456055, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.8558256065889733, 'motion_component': 1.5982341395508683}, {'ion': 1320, 'force': [-2.242825746536255, -3.0832972526550293, -2.36020565032959], 'magnitude': 4.484145164489746, 'distance': 8.604570388793945, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.9316849689159826, 'motion_component': 4.17781086980186}, {'ion': 1460, 'force': [-2.2260844707489014, -2.778157949447632, 2.4358808994293213], 'magnitude': 4.313598155975342, 'distance': 8.773021697998047, 'before_closest_residue': 780, 'closest_residue': 1105, 'next_closest_residue': 780, 'cosine_with_motion': 0.41583722061378225, 'motion_component': 1.793754685761428}]}, 5004: {'frame': 5004, 'ionic_force': [-5.378649363294244, -8.704846262931824, -1.6704208105802536], 'ionic_force_magnitude': 10.36795655464293, 'motion_vector': [-0.6747245788574219, 2.4837417602539062, -0.2197113037109375], 'cosine_ionic_motion': -0.6580799962279065, 'ionic_motion_component': -6.822944810370518, 'ionic_force_x': -5.378649363294244, 'ionic_force_y': -8.704846262931824, 'ionic_force_z': -1.6704208105802536, 'radial_force': 10.23250787610465, 'axial_force': -1.6704208105802536, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'contributions': [{'ion': 1306, 'force': [-0.679743230342865, -1.729952335357666, 0.21382690966129303], 'magnitude': 1.8709644079208374, 'distance': 13.320982933044434, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 'SF', 'cosine_with_motion': -0.8038812309290956, 'motion_component': -1.504033187031456}, {'ion': 1307, 'force': [0.01817171834409237, -2.3790934085845947, 0.4441870450973511], 'magnitude': 2.4202723503112793, 'distance': 11.712158203125, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 130, 'cosine_with_motion': -0.962740313188367, 'motion_component': -2.3300936689444516}, {'ion': 1309, 'force': [-0.6875178813934326, -0.8340977430343628, -1.441748857498169], 'magnitude': 1.8019543886184692, 'distance': 13.573665618896484, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.27736274933035654, 'motion_component': -0.4997950258276198}, {'ion': 1320, 'force': [-2.1348366737365723, -2.760021209716797, -1.877365231513977], 'magnitude': 3.9622902870178223, 'distance': 9.15368366241455, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.48873895636195097, 'motion_component': -1.936525656408099}, {'ion': 1460, 'force': [-1.8947232961654663, -1.0016815662384033, 0.9906793236732483], 'magnitude': 2.3610990047454834, 'distance': 11.858014106750488, 'before_closest_residue': 1105, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.23399998864807015, 'motion_component': -0.552497107667592}]}, 5005: {'frame': 5005, 'ionic_force': [-15.396269142627716, -9.154443114995956, -4.018658101558685], 'ionic_force_magnitude': 18.357520126508113, 'motion_vector': [1.9760818481445312, -2.551136016845703, 1.67626953125], 'cosine_ionic_motion': -0.20682385342436435, 'ionic_motion_component': -3.7967730518797325, 'ionic_force_x': -15.396269142627716, 'ionic_force_y': -9.154443114995956, 'ionic_force_z': -4.018658101558685, 'radial_force': 17.912256481468972, 'axial_force': -4.018658101558685, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'contributions': [{'ion': 1306, 'force': [-9.041532516479492, -2.8369057178497314, -1.7358170747756958], 'magnitude': 9.63381576538086, 'distance': 5.870429515838623, 'before_closest_residue': 130, 'closest_residue': 'SF', 'next_closest_residue': 780, 'cosine_with_motion': -0.3864805182232081, 'motion_component': -3.723282089699737}, {'ion': 1307, 'force': [-0.49104100465774536, -3.2770609855651855, 0.7138523459434509], 'magnitude': 3.3896660804748535, 'distance': 9.89670467376709, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 98, 'cosine_with_motion': 0.696615409710498, 'motion_component': 2.3612935232982935}, {'ion': 1309, 'force': [-0.8727691173553467, -0.5728297829627991, -1.483247995376587], 'magnitude': 1.8138039112091064, 'distance': 13.529254913330078, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.4168848729684455, 'motion_component': -0.7561473993155872}, {'ion': 1320, 'force': [-3.1719272136688232, -2.036134958267212, -2.4662981033325195], 'magnitude': 4.504396915435791, 'distance': 8.585206031799316, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.31793913100847976, 'motion_component': -1.4321241320576232}, {'ion': 1460, 'force': [-1.8189992904663086, -0.43151167035102844, 0.952852725982666], 'magnitude': 2.098306179046631, 'distance': 12.578666687011719, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.11748188627750467, 'motion_component': -0.24651297452992438}]}, 5006: {'frame': 5006, 'ionic_force': [-9.796686068177223, -15.417952418327332, 4.106213748455048], 'ionic_force_magnitude': 18.722961999646973, 'motion_vector': [-2.692249298095703, 2.7754745483398438, -1.560882568359375], 'cosine_ionic_motion': -0.2923741660247024, 'ionic_motion_component': -5.474110400158978, 'ionic_force_x': -9.796686068177223, 'ionic_force_y': -15.417952418327332, 'ionic_force_z': 4.106213748455048, 'radial_force': 18.26713756153994, 'axial_force': 4.106213748455048, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'contributions': [{'ion': 1306, 'force': [-5.318778038024902, -7.265165328979492, 6.092695236206055], 'magnitude': 10.871658325195312, 'distance': 5.526130676269531, 'before_closest_residue': 'SF', 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.338707949884267, 'motion_component': -3.682317221195376}, {'ion': 1307, 'force': [0.1557546108</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>5173</v>
+      </c>
+      <c r="B11" t="n">
+        <v>5400</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1320</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>{5173: {'frame': 5173, 'ionic_force': [-0.03178515285253525, 10.060459554195404, -0.028999194502830505], 'ionic_force_magnitude': 10.06055155997052, 'motion_vector': [-0.32863616943359375, 0.4364585876464844, -0.3377685546875], 'cosine_ionic_motion': 0.6826207059370479, 'ionic_motion_component': 6.867540807983145, 'ionic_force_x': -0.03178515285253525, 'ionic_force_y': 10.060459554195404, 'ionic_force_z': -0.028999194502830505, 'radial_force': 10.060509765292386, 'axial_force': -0.028999194502830505, 'before_closest_residue': None, 'closest_residue': 130, 'next_closest_residue': 130, 'contributions': [{'ion': 1306, 'force': [-1.142738938331604, 1.9904721975326538, -0.18408028781414032], 'magnitude': 2.3025457859039307, 'distance': 12.007840156555176, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.8833599908585629, 'motion_component': 2.0339768831825404}, {'ion': 1307, 'force': [0.9537079930305481, 3.515716075897217, 5.352444171905518], 'magnitude': 6.474447727203369, 'distance': 7.160901069641113, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 130, 'cosine_with_motion': -0.14111211941911425, 'motion_component': -0.9136230812118349}, {'ion': 1308, 'force': [0.7354629039764404, 2.4643869400024414, -0.565873920917511], 'magnitude': 2.633310079574585, 'distance': 11.22840404510498, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.6060114431838383, 'motion_component': 1.5958160407950677}, {'ion': 1309, 'force': [-0.48083266615867615, 1.5299593210220337, -3.0795645713806152], 'magnitude': 3.4721310138702393, 'distance': 9.778471946716309, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.8366618689570267, 'motion_component': 2.904999593045128}, {'ion': 1403, 'force': [-0.09738444536924362, 0.5599250197410583, -1.5519245862960815], 'magnitude': 1.652715802192688, 'distance': 14.173266410827637, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.7541353633832589, 'motion_component': 1.246371467798952}]}, 5174: {'frame': 5174, 'ionic_force': [-0.6643470674753189, 10.092601358890533, -2.0427508652210236], 'ionic_force_magnitude': 10.318662234655388, 'motion_vector': [-2.1065216064453125, -0.9170722961425781, 2.1868057250976562], 'cosine_ionic_motion': -0.37652310142994416, 'ionic_motion_component': -3.8852147072004852, 'ionic_force_x': -0.6643470674753189, 'ionic_force_y': 10.092601358890533, 'ionic_force_z': -2.0427508652210236, 'radial_force': 10.114443099624522, 'axial_force': -2.0427508652210236, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-0.6169819831848145, 2.007314682006836, -0.35312172770500183], 'magnitude': 2.1294772624969482, 'distance': 12.4862642288208, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.1944484357255886, 'motion_component': -0.41407354740905694}, {'ion': 1307, 'force': [0.5131598114967346, 2.890629529953003, 4.478611946105957], 'magnitude': 5.3550944328308105, 'distance': 7.873819828033447, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 130, 'cosine_with_motion': 0.3568898842478798, 'motion_component': 1.9111790539570173}, {'ion': 1308, 'force': [0.4955497980117798, 2.235003709793091, -0.6512793898582458], 'magnitude': 2.3801209926605225, 'distance': 11.81053352355957, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.5984301635066598, 'motion_component': -1.4243362059982232}, {'ion': 1309, 'force': [-0.8381993174552917, 2.3942766189575195, -3.879767417907715], 'magnitude': 4.635486602783203, 'distance': 8.462942123413086, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6062927398856023, 'motion_component': -2.8104617289922547}, {'ion': 1403, 'force': [-0.2178753763437271, 0.5653768181800842, -1.637194275856018], 'magnitude': 1.7457164525985718, 'distance': 13.790569305419922, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6573360244306076, 'motion_component': -1.147522273230206}]}, 5175: {'frame': 5175, 'ionic_force': [-4.48947374522686, 8.996800035238266, -3.1096643209457397], 'ionic_force_magnitude': 10.524628144124973, 'motion_vector': [0.8205947875976562, 1.4489250183105469, -0.349456787109375], 'cosine_ionic_motion': 0.5829208355145403, 'ionic_motion_component': 6.135025031253175, 'ionic_force_x': -4.48947374522686, 'ionic_force_y': 8.996800035238266, 'ionic_force_z': -3.1096643209457397, 'radial_force': 10.05473944879451, 'axial_force': -3.1096643209457397, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-1.0581152439117432, 1.6551977396011353, 0.1323573887348175], 'magnitude': 1.9689606428146362, 'distance': 12.98525619506836, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.4428939790755767, 'motion_component': 0.8720408015903445}, {'ion': 1307, 'force': [-0.3703985810279846, 0.40683475136756897, 2.9235332012176514], 'magnitude': 2.974853992462158, 'distance': 10.564190864562988, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 130, 'cosine_with_motion': -0.14543511396598727, 'motion_component': -0.4326482227258275}, {'ion': 1308, 'force': [0.23377586901187897, 3.548218250274658, -0.4093410074710846], 'magnitude': 3.5793943405151367, 'distance': 9.630842208862305, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.8991608912132001, 'motion_component': 3.218451420795778}, {'ion': 1309, 'force': [-2.680544376373291, 2.8133533000946045, -3.845205307006836], 'magnitude': 5.466797828674316, 'distance': 7.792961597442627, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.34623075238245715, 'motion_component': 1.892773534790706}, {'ion': 1403, 'force': [-0.6141914129257202, 0.5731959939002991, -1.911008596420288], 'magnitude': 2.087519645690918, 'distance': 12.611123085021973, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.2799529169991263, 'motion_component': 0.5844072358015922}]}, 5176: {'frame': 5176, 'ionic_force': [-1.6972591429948807, 9.394513070583344, -1.1074041053652763], 'ionic_force_magnitude': 9.610614355202319, 'motion_vector': [-0.2884254455566406, 1.5469932556152344, -1.362060546875], 'cosine_ionic_motion': 0.8264716526834646, 'ionic_motion_component': 7.94290032944749, 'ionic_force_x': -1.6972591429948807, 'ionic_force_y': 9.394513070583344, 'ionic_force_z': -1.1074041053652763, 'radial_force': 9.546599626665035, 'axial_force': -1.1074041053652763, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-0.5284325480461121, 1.4004030227661133, 0.022839702665805817], 'magnitude': 1.4969606399536133, 'distance': 14.89237117767334, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.7342917700181234, 'motion_component': 1.099205897200822}, {'ion': 1307, 'force': [-0.19438980519771576, 2.0637528896331787, 3.8672609329223633], 'magnitude': 4.387775421142578, 'distance': 8.6985502243042, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 130, 'cosine_with_motion': -0.22106392007030384, 'motion_component': -0.9699787685514543}, {'ion': 1308, 'force': [0.5721141695976257, 2.9097232818603516, -0.24224546551704407], 'magnitude': 2.9753129482269287, 'distance': 10.563375473022461, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.7535516993446264, 'motion_component': 2.242052118813529}, {'ion': 1309, 'force': [-1.1644694805145264, 2.285262107849121, -3.060650587081909], 'magnitude': 3.99324369430542, 'distance': 9.11813735961914, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.9673941460377422, 'motion_component': 3.863040438722315}, {'ion': 1403, 'force': [-0.3820814788341522, 0.7353717684745789, -1.6946086883544922], 'magnitude': 1.8863871097564697, 'distance': 13.266416549682617, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.905742166955266, 'motion_component': 1.708580390070872}]}, 5177: {'frame': 5177, 'ionic_force': [-1.3824736773967743, 8.549700021743774, -0.875838428735733], 'ionic_force_magnitude': 8.70492371498744, 'motion_vector': [1.0473556518554688, -0.16293716430664062, -0.0436553955078125], 'cosine_ionic_motion': -0.30350618160509957, 'ionic_motion_component': -2.641998157899516, 'ionic_force_x': -1.3824736773967743, 'ionic_force_y': 8.549700021743774, 'ionic_force_z': -0.875838428735733, 'radial_force': 8.660750771757634, 'axial_force': -0.875838428735733, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1307, 'force': [-0.45594823360443115, 2.804142475128174, 3.031407594680786], 'magnitude': 4.154580116271973, 'distance': 8.939340591430664, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 130, 'cosine_with_motion': -0.24204226476245888, 'motion_component': -1.0055839768415815}, {'ion': 1308, 'force': [0.689740777015686, 2.4730772972106934, -0.39926019310951233], 'magnitude': 2.5983190536499023, 'distance': 11.303756713867188, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.12221501182130788, 'motion_component': 0.3175536045510019}, {'ion': 1309, 'force': [-1.2035044431686401, 2.5528600215911865, -2.146219491958618], 'magnitude': 3.5456700325012207, 'distance': 9.676535606384277, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.42078615680419346, 'motion_component': -1.4919688284648274}, {'ion': 1403, 'force': [-0.41276177763938904, 0.7196202278137207, -1.3617663383483887], 'magnitude': 1.594563603401184, 'distance': 14.429394721984863, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.2897338193037402, 'motion_component': -0.46199900587296655}]}, 5178: {'frame': 5178, 'ionic_force': [-1.344180654734373, 9.261112630367279, -1.605331540107727], 'ionic_force_magnitude': 9.494846925494645, 'motion_vector': [-0.499969482421875, -1.2579994201660156, 0.6877059936523438], 'cosine_ionic_motion': -0.838081190111417, 'ionic_motion_component': -7.957452611244281, 'ionic_force_x': -1.344180654734373, 'ionic_force_y': 9.261112630367279, 'ionic_force_z': -1.605331540107727, 'radial_force': 9.358153064836591, 'axial_force': -1.605331540107727, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-0.6633750796318054, 1.5338643789291382, -0.1830899715423584], 'magnitude': 1.681168794631958, 'distance': 14.052817344665527, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 780, 'cosine_with_motion': -0.6753160374592341, 'motion_component': -1.135320218736478}, {'ion': 1307, 'force': [0.008810419589281082, 2.18619704246521, 2.864572048187256], 'magnitude': 3.603513479232788, 'distance': 9.598557472229004, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': None, 'cosine_with_motion': -0.14340799999121803, 'motion_component': -0.5167726362489959}, {'ion': 1308, 'force': [0.52821284532547, 2.203639030456543, -0.34880292415618896], 'magnitude': 2.2927489280700684, 'distance': 12.033468246459961, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.9410791659335338, 'motion_component': -2.1576581707824296}, {'ion': 1309, 'force': [-0.9532740116119385, 2.5756494998931885, -2.5336785316467285], 'magnitude': 3.7366065979003906, 'distance': 9.426063537597656, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.794204453800667, 'motion_component': -2.9676295725849258}, {'ion': 1403, 'force': [-0.26455482840538025, 0.7617626786231995, -1.404332160949707], 'magnitude': 1.6193888187408447, 'distance': 14.318366050720215, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7287143440952004, 'motion_component': -1.1800719301357088}]}, 5179: {'frame': 5179, 'ionic_force': [-2.9875034540891647, 9.438717722892761, -3.671563595533371], 'ionic_force_magnitude': 10.559116836965606, 'motion_vector': [0.006259918212890625, 2.1265487670898438, -1.1589584350585938], 'cosine_ionic_motion': 0.9505575012028823, 'ionic_motion_component': 10.037047715455309, 'ionic_force_x': -2.9875034540891647, 'ionic_force_y': 9.438717722892761, 'ionic_force_z': -3.671563595533371, 'radial_force': 9.90023076198957, 'axial_force': -3.671563595533371, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-0.7968317866325378, 2.22175669670105, 0.06649583578109741], 'magnitude': 2.3612635135650635, 'distance': 11.857600212097168, 'before_closest_residue': 748, 'closest_residue': 780, 'next_closest_residue': 748, 'cosine_with_motion': 0.8118365588407953, 'motion_component': 1.9169600507336204}, {'ion': 1307, 'force': [-0.160544291138649, 0.86920565366745, 1.6906518936157227], 'magnitude': 1.9077726602554321, 'distance': 13.191850662231445, 'before_closest_residue': 130, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.02423879128922786, 'motion_component': -0.04624210486356184}, {'ion': 1308, 'force': [0.29383471608161926, 2.3622288703918457, -0.319489985704422], 'magnitude': 2.401777982711792, 'distance': 11.75716495513916, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.9275760945020237, 'motion_component': 2.2278319278088166}, {'ion': 1309, 'force': [-1.8343040943145752, 3.2689404487609863, -3.492114543914795], 'magnitude': 5.123036861419678, 'distance': 8.050174713134766, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.885550252509541, 'motion_component': 4.53670662706779}, {'ion': 1403, 'force': [-0.489657998085022, 0.7165860533714294, -1.6171067953109741], 'magnitude': 1.8352915048599243, 'distance': 13.449821472167969, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.7637974619760005, 'motion_component': 1.4017909947725329}]}, 5180: {'frame': 5180, 'ionic_force': [-0.47080206871032715, 4.05627167224884, -2.3710789382457733], 'ionic_force_magnitude': 4.721970965432023, 'motion_vector': [0.3277015686035156, -0.06797409057617188, 1.3685455322265625], 'cosine_ionic_motion': -0.552400466844324, 'ionic_motion_component': -2.6084189657299928, 'ionic_force_x': -0.47080206871032715, 'ionic_force_y': 4.05627167224884, 'ionic_force_z': -2.3710789382457733, 'radial_force': 4.083502720335855, 'axial_force': -2.3710789382457733, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1308, 'force': [0.32464051246643066, 1.7187424898147583, -0.2759523093700409], 'magnitude': 1.770767331123352, 'distance': 13.69267463684082, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.15556355057782062, 'motion_component': -0.27546685084777156}, {'ion': 1309, 'force': [-0.7954425811767578, 2.337529182434082, -2.0951266288757324], 'magnitude': 3.238259792327881, 'distance': 10.125423431396484, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7204338815501123, 'motion_component': -2.332952148085589}]}, 5181: {'frame': 5181, 'ionic_force': [-0.8457868248224258, 6.44456821680069, -2.367974877357483], 'ionic_force_magnitude': 6.917739506069667, 'motion_vector': [-0.3796195983886719, -1.8383750915527344, -0.54205322265625], 'cosine_ionic_motion': -0.7578190826587865, 'ionic_motion_component': -5.242395006562162, 'ionic_force_x': -0.8457868248224258, 'ionic_force_y': 6.44456821680069, 'ionic_force_z': -2.367974877357483, 'radial_force': 6.4998319096758825, 'axial_force': -2.367974877357483, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1307, 'force': [-0.15910173952579498, 1.1764719486236572, 1.3695497512817383], 'magnitude': 1.8124750852584839, 'distance': 13.534213066101074, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8033078924738504, 'motion_component': -1.455975584328685}, {'ion': 1308, 'force': [0.3693566620349884, 1.7314714193344116, -0.16969358921051025], 'magnitude': 1.7785425186157227, 'distance': 13.662712097167969, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.9298734282283851, 'motion_component': -1.6538194403953677}, {'ion': 1309, 'force': [-0.789997935295105, 2.699798583984375, -2.170147180557251], 'magnitude': 3.5528225898742676, 'distance': 9.666790008544922, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5023273269637426, 'motion_component': -1.7846798437849252}, {'ion': 1403, 'force': [-0.2660438120365143, 0.8368262648582458, -1.39768385887146], 'magnitude': 1.6506295204162598, 'distance': 14.182221412658691, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.21078027551344006, 'motion_component': -0.3479201363469171}]}, 5182: {'frame': 5182, 'ionic_force': [-2.513504236936569, 7.566243886947632, -3.646450847387314], 'ionic_force_magnitude': 8.767117764024967, 'motion_vector': [3.399822235107422, 1.0570564270019531, -0.6069412231445312], 'cosine_ionic_motion': 0.052603579491658066, 'ionic_motion_component': 0.46118177621261486, 'ionic_force_x': -2.513504236936569, 'ionic_force_y': 7.566243886947632, 'ionic_force_z': -3.646450847387314, 'radial_force': 7.972813186439934, 'axial_force': -3.646450847387314, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [-0.7537117600440979, 1.4613643884658813, -0.11885979771614075], 'magnitude': 1.648573637008667, 'distance': 14.191061019897461, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.15881261849617107, 'motion_component': -0.26181429164471703}, {'ion': 1307, 'force': [-0.25020793080329895, 0.5931304693222046, 1.390986442565918], 'magnitude': 1.5327266454696655, 'distance': 14.717589378356934, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.19291528115268364, 'motion_component': -0.2956863965203489}, {'ion': 1308, 'force': [0.24988240003585815, 2.1664843559265137, -0.3289939761161804], 'magnitude': 2.2055232524871826, 'distance': 12.26911449432373, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.4192119235928302, 'motion_component': 0.9245816354512906}, {'ion': 1309, 'force': [-1.407989263534546, 2.6396069526672363, -3.090088129043579], 'magnitude': 4.301000118255615, 'distance': 8.785860061645508, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.00780209540420473, 'motion_component': -0.033556814397886825}, {'ion': 1403, 'force': [-0.3514776825904846, 0.7056577205657959, -1.4994953870773315], 'magnitude': 1.694100260734558, 'distance': 13.999079704284668, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.07535424101003572, 'motion_component': 0.12765764161992088}]}, 5183: {'frame': 5183, 'ionic_force': [0.7419249042868614, 5.625347793102264, -1.300440564751625], 'ionic_force_magnitude': 5.8211799507843, 'motion_vector': [-0.3704338073730469, 0.2990570068359375, 0.07714080810546875], 'cosine_ionic_motion': 0.46558880640952865, 'ionic_motion_component': 2.710276225180741, 'ionic_force_x': 0.7419249042868614, 'ionic_force_y': 5.625347793102264, 'ionic_force_z': -1.300440564751625, 'radial_force': 5.674062949682669, 'axial_force': -1.300440564751625, 'before_closest_residue': 98, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [-0.26556774973869324, 1.5205553770065308, -0.20820355415344238], 'magnitude': 1.5575505495071411, 'distance': 14.599836349487305, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.7149221828031384, 'motion_component': 1.1135274134201563}, {'ion': 1307, 'force': [0.10141553729772568, 0.7528913617134094, 1.3469141721725464], 'magnitude': 1.5463855266571045, 'distance': 14.652446746826172, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.39083826640936153, 'motion_component': 0.604386651568277}, {'ion': 1308, 'force': [0.6261655688285828, 1.4340345859527588, -0.20961131155490875], 'magnitude': 1.5787575244903564, 'distance': 14.501446723937988, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.23736511913737168, 'motion_component': 0.37474197496300743}, {'ion': 1309, 'force': [0.2799115478992462, 1.9178664684295654, -2.2295398712158203], 'magnitude': 2.954219102859497, 'distance': 10.601020812988281, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.20906377391369516, 'motion_component': 0.6176201873585594}]}, 5184: {'frame': 5184, 'ionic_force': [0.4307818403467536, 6.582498788833618, -4.181024253368378], 'ionic_force_magnitude': 7.8099825291880896, 'motion_vector': [-0.18041229248046875, 0.4036216735839844, 0.16362762451171875], 'cosine_ionic_motion': 0.5146979813853528, 'ionic_motion_component': 4.019782242427982, 'ionic_force_x': 0.4307818403467536, 'ionic_force_y': 6.582498788833618, 'ionic_force_z': -4.181024253368378, 'radial_force': 6.596579666688532, 'axial_force': -4.181024253368378, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [-0.2947106957435608, 1.6236279010772705, -0.13380694389343262], 'magnitude': 1.6555743217468262, 'distance': 14.161026000976562, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.8797408980647319, 'motion_component': 1.4564764190388058}, {'ion': 1308, 'force': [0.5973078608512878, 1.5048673152923584, -0.26393312215805054], 'magnitude': 1.6404459476470947, 'distance': 14.22617244720459, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.5902359183247087, 'motion_component': 0.9682501389175825}, {'ion': 1309, 'force': [0.1381777822971344, 2.6733298301696777, -2.3793797492980957], 'magnitude': 3.581512689590454, 'distance': 9.6279935836792, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.3937215782895846, 'motion_component': 1.410118846732325}, {'ion': 1403, 'force': [-0.009993107058107853, 0.7806737422943115, -1.4039044380187988], 'magnitude': 1.6063930988311768, 'distance': 14.376167297363281, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.1151254858041788, 'motion_component': 0.18493679439559696}]}, 5185: {'frame': 5185, 'ionic_force': [0.11261998489499092, 6.809355080127716, -3.9867260307073593], 'ionic_force_magnitude': 7.891386716679048, 'motion_vector': [-0.11819076538085938, -0.16250991821289062, 0.146270751953125], 'cosine_ionic_motion': -0.8682999722634465, 'ionic_motion_component': -6.852090867212548, 'ionic_force_x': 0.11261998489499092, 'ionic_force_y': 6.809355080127716, 'ionic_force_z': -3.9867260307073593, 'radial_force': 6.810286327920353, 'axial_force': -3.9867260307073593, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-0.6213038563728333, 1.6895768642425537, -0.13035066425800323], 'magnitude': 1.8049044609069824, 'distance': 13.562568664550781, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.4908801225802014, 'motion_component': -0.8859916747134058}, {'ion': 1308, 'force': [0.8244546055793762, 1.679525375366211, -0.2533508837223053], 'magnitude': 1.8880459070205688, 'distance': 13.260587692260742, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.8682598275267359, 'motion_component': -1.6393144610569834}, {'ion': 1309, 'force': [-0.028522875159978867, 2.627678871154785, -2.242663860321045], 'magnitude': 3.454714298248291, 'distance': 9.803089141845703, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8754357746797629, 'motion_component': -3.024380502198848}, {'ion': 1403, 'force': [-0.06200788915157318, 0.8125739693641663, -1.3603606224060059], 'magnitude': 1.5857813358306885, 'distance': 14.469295501708984, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8213012027582747, 'motion_component': -1.302404121518519}]}, 5186: {'frame': 5186, 'ionic_force': [0.2758752889931202, 6.846363365650177, -3.949508366174996], 'ionic_force_magnitude': 7.908692359934109, 'motion_vector': [0.29323577880859375, 0.5634040832519531, 0.6587371826171875], 'cosine_ionic_motion': 0.1846734597098065, 'ionic_motion_component': 1.460525579889546, 'ionic_force_x': 0.2758752889931202, 'ionic_force_y': 6.846363365650177, 'ionic_force_z': -3.949508366174996, 'radial_force': 6.851919330347801, 'axial_force': -3.949508366174996, 'before_closest_residue': 455, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-0.3327000141143799, 1.484390139579773, 0.015022787265479565], 'magnitude': 1.521291971206665, 'distance': 14.772797584533691, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.5377898382174252, 'motion_component': 0.8181353292022178}, {'ion': 1308, 'force': [0.7067315578460693, 1.7726627588272095, -0.21329709887504578], 'magnitude': 1.920233964920044, 'distance': 13.148977279663086, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.6063586115181139, 'motion_component': 1.1643503887190967}, {'ion': 1309, 'force': [-0.05736168473958969, 2.774033784866333, -2.3771002292633057], 'magnitude': 3.6536500453948975, 'distance': 9.532472610473633, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.005923090307569401, 'motion_component': -0.021640899696546034}, {'ion': 1403, 'force': [-0.04079456999897957, 0.8152766823768616, -1.374133825302124], 'magnitude': 1.598306655883789, 'distance': 14.41248893737793, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.31303085430443395, 'motion_component': -0.5003192851393142}]}, 5187: {'frame': 5187, 'ionic_force': [-0.016629517078399658, 7.088494658470154, -3.625397428870201], 'ionic_force_magnitude': 7.961817605374844, 'motion_vector': [-0.44336700439453125, -0.58660888671875, -0.7073516845703125], 'cosine_ionic_motion': -0.19528123302760486, 'ionic_motion_component': -1.5547935591184918, 'ionic_force_x': -0.016629517078399658, 'ionic_force_y': 7.088494658470154, 'ionic_force_z': -3.625397428870201, 'radial_force': 7.088514164759648, 'axial_force': -3.625397428870201, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 130, 'contributions': [{'ion': 1306, 'force': [-0.464724063873291, 1.453264594078064, 0.03563608229160309], 'magnitude': 1.5261770486831665, 'distance': 14.749135971069336, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.4313343020519969, 'motion_component': -0.6582925096112762}, {'ion': 1308, 'force': [0.5526303648948669, 1.42279052734375, -0.1382688283920288], 'magnitude': 1.5325963497161865, 'distance': 14.718214988708496, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.6278833176374604, 'motion_component': -0.962291660716259}, {'ion': 1309, 'force': [-0.0501912422478199, 3.1493821144104004, -2.052255630493164], 'magnitude': 3.7593722343444824, 'distance': 9.397479057312012, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.09738347942390585, 'motion_component': -0.36610075432767797}, {'ion': 1403, 'force': [-0.054344575852155685, 1.0630574226379395, -1.4705090522766113], 'magnitude': 1.8153350353240967, 'distance': 13.523548126220703, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.23791276105627682, 'motion_component': 0.43189137043733694}]}, 5188: {'frame': 5188, 'ionic_force': [0.0713690547272563, 6.948368489742279, -4.33288237452507], 'ionic_force_magnitude': 8.188943025976311, 'motion_vector': [0.09778976440429688, 0.3133354187011719, -0.27387237548828125], 'cosine_ionic_motion': 0.9628964307048866, 'ionic_motion_component': 7.885104010958264, 'ionic_force_x': 0.0713690547272563, 'ionic_force_y': 6.948368489742279, 'ionic_force_z': -4.33288237452507, 'radial_force': 6.948735007986422, 'axial_force': -4.33288237452507, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-0.5290773510932922, 1.6023163795471191, -0.10008007287979126], 'magnitude': 1.6903717517852783, 'distance': 14.014510154724121, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.6611149119204682, 'motion_component': 1.1175299689312546}, {'ion': 1308, 'force': [0.7558067440986633, 2.0558364391326904, -0.4618763029575348], 'magnitude': 2.238534450531006, 'distance': 12.178313255310059, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.8825643705961469, 'motion_component': 1.975650853246151}, {'ion': 1309, 'force': [-0.012659800238907337, 2.442432165145874, -2.3873846530914307], 'magnitude': 3.4154415130615234, 'distance': 9.859289169311523, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.9711197726701742, 'motion_component': 3.3168027721633653}, {'ion': 1403, 'force': [-0.14270053803920746, 0.8477835059165955, -1.3835413455963135], 'magnitude': 1.6288913488388062, 'distance': 14.276540756225586, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.9055977262933529, 'motion_component': 1.4751202866299886}]}, 5189: {'frame': 5189, 'ionic_force': [-0.3013307675719261, 6.295839011669159, -3.964147448539734], 'ionic_force_magnitude': 7.445995842471634, 'motion_vector': [-0.000904083251953125, -0.1085205078125, 0.5684127807617188], 'cosine_ionic_motion': -0.6814411885396898, 'ionic_motion_component': -5.074008256755459, 'ionic_force_x': -0.3013307675719261, 'ionic_force_y': 6.295839011669159, 'ionic_force_z': -3.964147448539734, 'radial_force': 6.30304601699375, 'axial_force': -3.964147448539734, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 130, 'contributions': [{'ion': 1306, 'force': [-0.6288329362869263, 1.568109154701233, -0.1296226680278778], 'magnitude': 1.6944613456726074, 'distance': 13.997588157653809, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.2481081375513412, 'motion_component': -0.42040964620464205}, {'ion': 1308, 'force': [0.5216655135154724, 1.448395848274231, -0.2568974792957306], 'magnitude': 1.5607632398605347, 'distance': 14.58480167388916, 'before_closes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>5213</v>
+      </c>
+      <c r="B12" t="n">
+        <v>5677</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1309</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>{5213: {'frame': 5213, 'ionic_force': [8.349748060107231, 9.205024123191833, -18.89620530605316], 'ionic_force_magnitude': 22.61674903128917, 'motion_vector': [-0.08104324340820312, -3.535572052001953, 0.40856170654296875], 'cosine_ionic_motion': -0.5084941210523158, 'ionic_motion_component': -11.500483919726202, 'ionic_force_x': 8.349748060107231, 'ionic_force_y': 9.205024123191833, 'ionic_force_z': -18.89620530605316, 'radial_force': 12.427822084975631, 'axial_force': -18.89620530605316, 'before_closest_residue': None, 'closest_residue': 130, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [-0.7094604969024658, 2.2941157817840576, -1.2060950994491577], 'magnitude': 2.687185764312744, 'distance': 11.115274429321289, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.8933602894883115, 'motion_component': -2.400624964861471}, {'ion': 1308, 'force': [4.778199672698975, 9.435524940490723, -10.170702934265137], 'magnitude': 14.673224449157715, 'distance': 4.756705284118652, 'before_closest_residue': 780, 'closest_residue': 1105, 'next_closest_residue': 423, 'cosine_with_motion': -0.7255885946159099, 'motion_component': -10.646724441459995}, {'ion': 1320, 'force': [4.232130527496338, -3.0712902545928955, -4.9525957107543945], 'magnitude': 7.202219009399414, 'distance': 6.789470195770264, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.33121377374106037, 'motion_component': 2.3854740970482444}, {'ion': 1403, 'force': [0.04887835681438446, 0.5466736555099487, -2.5668115615844727], 'magnitude': 2.624835729598999, 'distance': 11.246515274047852, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.31949001303026325, 'motion_component': -0.8386088114752297}]}, 5214: {'frame': 5214, 'ionic_force': [-0.392241433262825, -3.0962782502174377, -10.358314990997314], 'ionic_force_magnitude': 10.818293848729445, 'motion_vector': [-2.800647735595703, -0.17963790893554688, 2.6386032104492188], 'cosine_ionic_motion': -0.6161574107543613, 'ionic_motion_component': -6.665771926612968, 'ionic_force_x': -0.392241433262825, 'ionic_force_y': -3.0962782502174377, 'ionic_force_z': -10.358314990997314, 'radial_force': 3.121024246098968, 'axial_force': -10.358314990997314, 'before_closest_residue': 130, 'closest_residue': 780, 'next_closest_residue': 1105, 'contributions': [{'ion': 1306, 'force': [-1.26851487159729, 3.9690990447998047, -2.3935248851776123], 'magnitude': 4.805397033691406, 'distance': 8.311978340148926, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.18777962040059085, 'motion_component': -0.9023555904444934}, {'ion': 1308, 'force': [-1.3250770568847656, -3.1238503456115723, -2.5353305339813232], 'magnitude': 4.2358198165893555, 'distance': 8.85319995880127, 'before_closest_residue': 1105, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.14816259756217112, 'motion_component': -0.6275900945759094}, {'ion': 1320, 'force': [2.0835518836975098, -3.640300989151001, -2.173349618911743], 'magnitude': 4.724026679992676, 'distance': 8.383258819580078, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.5998743875613214, 'motion_component': -2.8338226264943356}, {'ion': 1403, 'force': [0.11779861152172089, -0.3012259602546692, -3.2561099529266357], 'magnitude': 3.272134780883789, 'distance': 10.072875022888184, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7035172793829035, 'motion_component': -2.302003315099296}]}, 5215: {'frame': 5215, 'ionic_force': [-7.000141829252243, -6.792514324188232, -8.448651671409607], 'ionic_force_magnitude': 12.904260983828621, 'motion_vector': [0.9844284057617188, -0.2884941101074219, -5.571617126464844], 'cosine_ionic_motion': 0.5764379053583872, 'ionic_motion_component': 7.438505171716131, 'ionic_force_x': -7.000141829252243, 'ionic_force_y': -6.792514324188232, 'ionic_force_z': -8.448651671409607, 'radial_force': 9.753985671198684, 'axial_force': -8.448651671409607, 'before_closest_residue': 780, 'closest_residue': 1105, 'next_closest_residue': 1105, 'contributions': [{'ion': 1306, 'force': [-3.8426830768585205, 2.8841068744659424, -1.3305236101150513], 'magnitude': 4.98543643951416, 'distance': 8.160512924194336, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.0990755866994647, 'motion_component': 0.49393506282470323}, {'ion': 1308, 'force': [-2.1365599632263184, -3.032615900039673, -0.8023586273193359], 'magnitude': 3.7954483032226562, 'distance': 9.352710723876953, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.15077678582865442, 'motion_component': 0.5722654804066467}, {'ion': 1320, 'force': [0.5601136684417725, -6.005922317504883, -0.8906189203262329], 'magnitude': 6.097379207611084, 'distance': 7.378998756408691, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.20977316123691703, 'motion_component': 1.2790664955624322}, {'ion': 1403, 'force': [-1.2336101531982422, -0.5227363109588623, -3.747150182723999], 'magnitude': 3.9794700145721436, 'distance': 9.133903503417969, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.8788779690915066, 'motion_component': 3.4974685416808162}, {'ion': 1469, 'force': [-0.34740230441093445, -0.11534667015075684, -1.6780003309249878], 'magnitude': 1.7174626588821411, 'distance': 13.903539657592773, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.9291435751757805, 'motion_component': 1.5957694874407418}]}, 5216: {'frame': 5216, 'ionic_force': [-1.1580060422420502, -1.9418916404247284, -7.661372423171997], 'ionic_force_magnitude': 7.988025321915354, 'motion_vector': [0.49591064453125, 1.3578147888183594, -0.21898651123046875], 'cosine_ionic_motion': -0.13128610401620075, 'ionic_motion_component': -1.0487167232970247, 'ionic_force_x': -1.1580060422420502, 'ionic_force_y': -1.9418916404247284, 'ionic_force_z': -7.661372423171997, 'radial_force': 2.2609558016512707, 'axial_force': -7.661372423171997, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 130, 'contributions': [{'ion': 1306, 'force': [-1.4940450191497803, 1.5567138195037842, -2.294883966445923], 'magnitude': 3.1499240398406982, 'distance': 10.266419410705566, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.4072191966841656, 'motion_component': 1.2827094981918563}, {'ion': 1308, 'force': [-0.5920225381851196, -1.5384231805801392, -1.2295265197753906], 'magnitude': 2.0564465522766113, 'distance': 12.706043243408203, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.7028663925785696, 'motion_component': -1.4454071028631574}, {'ion': 1320, 'force': [1.186414122581482, -1.7023833990097046, -2.2223496437072754], 'magnitude': 3.0404810905456543, 'distance': 10.449557304382324, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.2781600982653527, 'motion_component': -0.8457405365038682}, {'ion': 1403, 'force': [-0.2583526074886322, -0.2577988803386688, -1.9146122932434082], 'magnitude': 1.9490886926651, 'distance': 13.051283836364746, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.020665348923662074, 'motion_component': -0.04027859703741399}]}, 5217: {'frame': 5217, 'ionic_force': [-1.6522649973630905, -0.9567364044487476, -8.501810789108276], 'ionic_force_magnitude': 8.713559023895268, 'motion_vector': [1.0223388671875, -0.4985237121582031, 2.0433120727539062], 'cosine_ionic_motion': -0.9120070943707188, 'ionic_motion_component': -7.946827647010481, 'ionic_force_x': -1.6522649973630905, 'ionic_force_y': -0.9567364044487476, 'ionic_force_z': -8.501810789108276, 'radial_force': 1.9092732044180507, 'axial_force': -8.501810789108276, 'before_closest_residue': 1105, 'closest_residue': 130, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [-1.082576036453247, 1.5340907573699951, -1.8062469959259033], 'magnitude': 2.6053662300109863, 'distance': 11.288458824157715, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.9129267309902062, 'motion_component': -2.3785085357285993}, {'ion': 1308, 'force': [-1.6062496900558472, -1.6342322826385498, -2.415165901184082], 'magnitude': 3.329231023788452, 'distance': 9.986126899719238, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.7401330330015188, 'motion_component': -2.4640738930936728}, {'ion': 1320, 'force': [1.2217909097671509, -0.8660487532615662, -2.349320888519287], 'magnitude': 2.7860584259033203, 'distance': 10.916261672973633, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 1105, 'cosine_with_motion': -0.47880292106144073, 'motion_component': -1.333972960252149}, {'ion': 1403, 'force': [-0.18523018062114716, 0.009453874081373215, -1.931077003479004], 'magnitude': 1.939963459968567, 'distance': 13.08194351196289, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.912528632425414, 'motion_component': -1.7702721473163905}]}, 5218: {'frame': 5218, 'ionic_force': [2.5373760387301445, -1.672971323132515, -10.462154865264893], 'ionic_force_magnitude': 10.894668174604103, 'motion_vector': [-0.7376747131347656, 0.12036895751953125, 5.263938903808594], 'cosine_ionic_motion': -0.9865544437351113, 'ionic_motion_component': -10.748183300675171, 'ionic_force_x': 2.5373760387301445, 'ionic_force_y': -1.672971323132515, 'ionic_force_z': -10.462154865264893, 'radial_force': 3.0392614579771906, 'axial_force': -10.462154865264893, 'before_closest_residue': 130, 'closest_residue': 780, 'next_closest_residue': 'SF', 'contributions': [{'ion': 1306, 'force': [-1.6688743829727173, 2.59674072265625, -2.762474775314331], 'magnitude': 4.142399311065674, 'distance': 8.952473640441895, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.5901659535800505, 'motion_component': -2.444702962503534}, {'ion': 1308, 'force': [-1.0178943872451782, -2.646784543991089, -2.161548376083374], 'magnitude': 3.5656511783599854, 'distance': 9.649384498596191, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.5773913926795388, 'motion_component': -2.0587763371135157}, {'ion': 1320, 'force': [5.3220672607421875, -1.4583486318588257, -2.8955790996551514], 'magnitude': 6.231818199157715, 'distance': 7.298971652984619, 'before_closest_residue': 98, 'closest_residue': 1105, 'next_closest_residue': 780, 'cosine_with_motion': -0.5838190835985204, 'motion_component': -3.6382544330410886}, {'ion': 1403, 'force': [-0.09792245179414749, -0.1645788699388504, -2.642552614212036], 'magnitude': 2.6494827270507812, 'distance': 11.194082260131836, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.9837579542078188, 'motion_component': -2.606449820321628}]}, 5221: {'frame': 5221, 'ionic_force': [-15.416450023651123, -5.343946605920792, 0.2550990181043744], 'ionic_force_magnitude': 16.31838754803007, 'motion_vector': [0.09583663940429688, 4.582389831542969, -4.5017547607421875], 'cosine_ionic_motion': -0.2586308283145971, 'ionic_motion_component': -4.220438088305625, 'ionic_force_x': -15.416450023651123, 'ionic_force_y': -5.343946605920792, 'ionic_force_z': 0.2550990181043744, 'radial_force': 16.31639349423349, 'axial_force': 0.2550990181043744, 'before_closest_residue': 'SF', 'closest_residue': 1073, 'next_closest_residue': 130, 'contributions': [{'ion': 1306, 'force': [-4.9202728271484375, 2.8619911670684814, 0.1428222358226776], 'magnitude': 5.6938982009887695, 'distance': 7.635969638824463, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.3280550325105419, 'motion_component': 1.8679119479651973}, {'ion': 1308, 'force': [-0.9717339277267456, -2.528850793838501, 0.010465134866535664], 'magnitude': 2.709144353866577, 'distance': 11.070137023925781, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.6738649628328864, 'motion_component': -1.825597403703803}, {'ion': 1320, 'force': [-6.512366771697998, -3.0620293617248535, 8.233292579650879], 'magnitude': 10.934991836547852, 'distance': 5.510104179382324, 'before_closest_residue': 130, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.7362136948005549, 'motion_component': -8.050490911518978}, {'ion': 1403, 'force': [-2.5566587448120117, -2.16740083694458, -6.0023908615112305], 'magnitude': 6.874796390533447, 'distance': 6.9492692947387695, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.3813827954446882, 'motion_component': 2.6219290923979797}, {'ion': 1469, 'force': [-0.4554177522659302, -0.4476567804813385, -2.1290900707244873], 'magnitude': 2.22279691696167, 'distance': 12.221348762512207, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5244785240319814, 'motion_component': 1.1658092836760383}]}, 5222: {'frame': 5222, 'ionic_force': [-11.94608449935913, 3.242609441280365, -10.622156023979187], 'ionic_force_magnitude': 16.31115107686353, 'motion_vector': [-3.9730682373046875, -1.5599021911621094, 2.0731430053710938], 'cosine_ionic_motion': 0.2633525663991598, 'ionic_motion_component': 4.29558349701643, 'ionic_force_x': -11.94608449935913, 'ionic_force_y': 3.242609441280365, 'ionic_force_z': -10.622156023979187, 'radial_force': 12.378346046807266, 'axial_force': -10.622156023979187, 'before_closest_residue': 1073, 'closest_residue': 130, 'next_closest_residue': 1105, 'contributions': [{'ion': 1306, 'force': [-1.2669048309326172, 1.7904175519943237, -0.7504638433456421], 'magnitude': 2.3181540966033936, 'distance': 11.967347145080566, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.06225492238107728, 'motion_component': 0.1443165090675862}, {'ion': 1308, 'force': [-2.3145053386688232, -2.909573793411255, -2.4544501304626465], 'magnitude': 4.454983711242676, 'distance': 8.632686614990234, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.4089915671206331, 'motion_component': 1.822050778624856}, {'ion': 1320, 'force': [-7.233617305755615, 3.4570906162261963, -3.964205026626587], 'magnitude': 8.943802833557129, 'distance': 6.0926737785339355, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.356471846835402, 'motion_component': 3.1882140577431386}, {'ion': 1403, 'force': [-1.1310570240020752, 0.9046750664710999, -3.4530370235443115], 'magnitude': 3.74448823928833, 'distance': 9.4161376953125, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.22940328619630437, 'motion_component': -0.8589978912641101}]}, 5223: {'frame': 5223, 'ionic_force': [-10.693952560424805, 0.50745789706707, -4.039891541004181], 'ionic_force_magnitude': 11.442851853667822, 'motion_vector': [1.1881523132324219, 0.9744796752929688, 2.5615386962890625], 'cosine_ionic_motion': -0.660012129402739, 'ionic_motion_component': -7.552421018379379, 'ionic_force_x': -10.693952560424805, 'ionic_force_y': 0.50745789706707, 'ionic_force_z': -4.039891541004181, 'radial_force': 10.705985936937894, 'axial_force': -4.039891541004181, 'before_closest_residue': 130, 'closest_residue': 1105, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-1.6322910785675049, 1.243991732597351, -0.25848662853240967], 'magnitude': 2.068502902984619, 'distance': 12.668959617614746, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.22484641609739942, 'motion_component': -0.46509550102333463}, {'ion': 1308, 'force': [-2.0935752391815186, -1.8744561672210693, -0.5705388188362122], 'magnitude': 2.8674304485321045, 'distance': 10.760255813598633, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.6742965102789934, 'motion_component': -1.933498388602409}, {'ion': 1320, 'force': [-4.028995990753174, 0.7997772693634033, 0.7936450242996216], 'magnitude': 4.183578014373779, 'distance': 8.908306121826172, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.15801994549859863, 'motion_component': -0.6610887659741991}, {'ion': 1403, 'force': [-2.2542738914489746, 0.2554945647716522, -2.6964259147644043], 'magnitude': 3.523881435394287, 'distance': 9.706404685974121, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.886971707792664, 'motion_component': -3.125583209489937}, {'ion': 1469, 'force': [-0.6848163604736328, 0.08265049755573273, -1.3080852031707764], 'magnitude': 1.4788141250610352, 'distance': 14.983464241027832, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.9244940953963866, 'motion_component': -1.367155000136628}]}, 5224: {'frame': 5224, 'ionic_force': [-13.356659054756165, 2.8882558345794678, -2.429133066907525], 'ionic_force_magnitude': 13.879591144112485, 'motion_vector': [0.0398406982421875, 2.6087303161621094, -0.5442276000976562], 'cosine_ionic_motion': 0.22503772707378417, 'ionic_motion_component': 3.1234316437844973, 'ionic_force_x': -13.356659054756165, 'ionic_force_y': 2.8882558345794678, 'ionic_force_z': -2.429133066907525, 'radial_force': 13.66537093792123, 'axial_force': -2.429133066907525, 'before_closest_residue': 1105, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-1.5037639141082764, 1.3657737970352173, 0.1421593874692917], 'magnitude': 2.0363824367523193, 'distance': 12.768485069274902, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.6311843126097167, 'motion_component': 1.2853326232558475}, {'ion': 1308, 'force': [-3.0808727741241455, -2.469778537750244, 0.02193385921418667], 'magnitude': 3.948678731918335, 'distance': 9.16944694519043, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 455, 'cosine_with_motion': -0.6250168030414615, 'motion_component': -2.4679905922540377}, {'ion': 1320, 'force': [-3.7092082500457764, 2.256039619445801, 2.863736867904663], 'magnitude': 5.2008585929870605, 'distance': 7.989719390869141, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 'SF', 'cosine_with_motion': 0.3014942239922375, 'motion_component': 1.5680288067766102}, {'ion': 1403, 'force': [-4.130849361419678, 1.4701601266860962, -3.665073871612549], 'magnitude': 5.714722633361816, 'distance': 7.622044086456299, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.3719633106605391, 'motion_component': 2.125667116136732}, {'ion': 1469, 'force': [-0.9319647550582886, 0.26606082916259766, -1.7918893098831177], 'magnitude': 2.0372073650360107, 'distance': 12.765899658203125, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.3006044973620889, 'motion_component': 0.6123937048573254}]}, 5225: {'frame': 5225, 'ionic_force': [-13.915466248989105, 5.79730761051178, -5.813826458645053], 'ionic_force_magnitude': 16.157028023398794, 'motion_vector': [1.9323806762695312, 0.8050422668457031, -0.5858154296875], 'cosine_ionic_motion': -0.5357630139396757, 'ionic_motion_component': -8.65633803012394, 'ionic_force_x': -13.915466248989105, 'ionic_force_y': 5.79730761051178, 'ionic_force_z': -5.813826458645053, 'radial_force': 15.074779482886399, 'axial_force': -5.813826458645053, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-1.1882764101028442, 1.3025888204574585, 0.0017900298116728663], 'magnitude': 1.76316237449646, 'distance': 13.722172737121582, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.3257746846152665, 'motion_component': -0.5743936763948767}, {'ion': 1308, 'force': [-5.498988151550293, -1.1754382848739624, 0.6942658424377441], 'magnitude': 5.665909767150879, 'distance': 7.654806613922119, 'before_closest_residue': 423, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': -0.9726077449400174, 'motion_component': -5.510707500471813}, {'ion': 1320, 'force': [-4.546165466308594, 3.720468282699585, -2.5248541831970215], 'magnitude': 6.394090175628662, 'distance': 7.2057576179504395, 'before_closest_residue': 780, 'closest_residue': 'SF', 'next_closest_residue': 'SF', 'cosine_with_motion': -0.3101345317109207, 'motion_component': -1.983028263270576}, {'ion': 1403, 'force': [-2.0169267654418945, 1.4461729526519775, -2.5027101039886475], 'magnitude': 3.524623155593872, 'distance': 9.70538330078125, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.16538079293163058, 'motion_component': -0.5829049549384706}, {'ion': 1469, 'force': [-0.6651094555854797, 0.5035158395767212, -1.4823180437088013], 'magnitude': 1.7009308338165283, 'distance': 13.970943450927734, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.0031178895486980596, 'motion_component': -0.005303314350566524}]}, 5226: {'frame': 5226, 'ionic_force': [-9.706894367933273, 11.867905139923096, -8.138043537735939], 'ionic_force_magnitude': 17.35795850042606, 'motion_vector': [-0.0262298583984375, 0.5780372619628906, 0.1553192138671875], 'cosine_ionic_motion': 0.5625994574730244, 'ionic_motion_component': 9.765578035178974, 'ionic_force_x': -9.706894367933273, 'ionic_force_y': 11.867905139923096, 'ionic_force_z': -8.138043537735939, 'radial_force': 15.332024350372906, 'axial_force': -8.138043537735939, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-1.0723364353179932, 1.5610697269439697, -0.06959237158298492], 'magnitude': 1.8951747417449951, 'distance': 13.235623359680176, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.8099804945886041, 'motion_component': 1.5350545574107208}, {'ion': 1308, 'force': [-3.372286558151245, 1.1184394359588623, 0.5709807872772217], 'magnitude': 3.5985054969787598, 'distance': 9.605234146118164, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': 0.382035810311084, 'motion_component': 1.374757997942818}, {'ion': 1320, 'force': [-3.445181369781494, 6.423120021820068, -3.7658469676971436], 'magnitude': 8.204105377197266, 'distance': 6.361410617828369, 'before_closest_residue': 'SF', 'closest_residue': 'SF', 'next_closest_residue': 'SF', 'cosine_with_motion': 0.6547561796468672, 'motion_component': 5.371688847001148}, {'ion': 1403, 'force': [-1.4268732070922852, 2.1184980869293213, -3.1947760581970215], 'magnitude': 4.090305328369141, 'distance': 9.009303092956543, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.31249432221731166, 'motion_component': 1.278197102482256}, {'ion': 1469, 'force': [-0.39021679759025574, 0.646777868270874, -1.6788089275360107], 'magnitude': 1.8409210443496704, 'distance': 13.429241180419922, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.11183524775394986, 'motion_component': 0.20587985755624938}]}, 5227: {'frame': 5227, 'ionic_force': [-8.839239090681076, 11.614094018936157, -6.965418614447117], 'ionic_force_magnitude': 16.172086570922115, 'motion_vector': [-1.3651809692382812, -0.9860496520996094, 0.14288330078125], 'cosine_ionic_motion': -0.013908562817473859, 'ionic_motion_component': -0.22493048196129564, 'ionic_force_x': -8.839239090681076, 'ionic_force_y': 11.614094018936157, 'ionic_force_z': -6.965418614447117, 'radial_force': 14.595181656386227, 'axial_force': -6.965418614447117, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-0.8923192024230957, 1.3975685834884644, -0.07134971767663956], 'magnitude': 1.6596753597259521, 'distance': 14.143518447875977, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.06063771765795272, 'motion_component': -0.10063892563123056}, {'ion': 1308, 'force': [-3.113513946533203, 1.471713900566101, 0.5079912543296814], 'magnitude': 3.4810869693756104, 'distance': 9.765885353088379, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': 0.4881399211648226, 'motion_component': 1.6992574855999774}, {'ion': 1320, 'force': [-3.006080389022827, 5.83809232711792, -2.921882152557373], 'magnitude': 7.1872968673706055, 'distance': 6.796514511108398, 'before_closest_residue': 'SF', 'closest_residue': 'SF', 'next_closest_residue': 'SF', 'cosine_with_motion': -0.17043338293533036, 'motion_component': -1.2249553237593886}, {'ion': 1403, 'force': [-1.393346905708313, 2.2208824157714844, -2.820758104324341], 'magnitude': 3.851027250289917, 'distance': 9.284975051879883, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.10613156239445612, 'motion_component': -0.40871553483142975}, {'ion': 1469, 'force': [-0.4339786469936371, 0.6858367919921875, -1.6594198942184448], 'magnitude': 1.8472638130187988, 'distance': 13.40616512298584, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.10278906205083915, 'motion_component': -0.1898785247648629}]}, 5228: {'frame': 5228, 'ionic_force': [-10.743721067905426, 8.693426668643951, -6.970459129661322], 'ionic_force_magnitude': 15.478711513117739, 'motion_vector': [0.7691383361816406, -0.3768424987792969, -0.10305023193359375], 'cosine_ionic_motion': -0.8103878506468886, 'ionic_motion_component': -12.543759753898733, 'ionic_force_x': -10.743721067905426, 'ionic_force_y': 8.693426668643951, 'ionic_force_z': -6.970459129661322, 'radial_force': 13.820391080864708, 'axial_force': -6.970459129661322, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-0.8692330718040466, 1.303725004196167, 0.019824136048555374], 'magnitude': 1.5670539140701294, 'distance': 14.555498123168945, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.8594881308442263, 'motion_component': -1.346864252275051}, {'ion': 1308, 'force': [-2.4451513290405273, 0.9452031254768372, 0.08026061952114105], 'magnitude': 2.622711658477783, 'distance': 11.251069068908691, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': -0.9923019662020579, 'motion_component': -2.6025218019028573}, {'ion': 1320, 'force': [-5.125226974487305, 4.3977861404418945, -2.9678163528442383], 'magnitude': 7.3767476081848145, 'distance': 6.708672046661377, 'before_closest_residue': 'SF', 'closest_residue': 'SF', 'next_closest_residue': 'SF', 'cosine_with_motion': -0.8318170866945936, 'motion_component': -6.136104879864973}, {'ion': 1403, 'force': [-1.7134193181991577, 1.530916690826416, -2.4926624298095703], 'magnitude': 3.3901147842407227, 'distance': 9.896049499511719, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.560051014426819, 'motion_component': -1.8986371754413724}, {'ion': 1469, 'force': [-0.5906903743743896, 0.5157957077026367, -1.6100651025772095], 'magnitude': 1.790885329246521, 'distance': 13.615549087524414, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.3124889054191626, 'motion_component': -0.5596317703114053}]}, 5229: {'frame': 5229, 'ionic_force': [-10.3910593688488, 9.424004197120667, -7.209954544901848], 'ionic_force_magnitude': 15.772425763142435, 'motion_vector': [-2.0034332275390625, -4.632930755615234, 0.2904510498046875], 'cosine_ionic_motion': -0.3127150604223023, 'ionic_motion_component': -4.932275075527364, 'ionic_force_x': -10.3910593688488, 'ionic_force_y': 9.424004197120667, 'ionic_force_z': -7.209954544901848, 'radial_force': 14.02804226947896, 'axial_force': -7.209954544901848, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 1105, 'contributions': [{'ion': 1306, 'force': [-0.9774071574211121, 1.5085536241531372, -0.06464840471744537], 'magnitude': 1.7986767292022705, 'distance': 13.586027145385742, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.5552746684783254, 'motion_component': -0.9987596597597498}, {'ion': 1308, 'force': [-3.0030407905578613, 0.9390349388122559, 0.19887909293174744], 'magnitude': 3.152712106704712, 'distance': 10.261878967285156, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': 0.10813634399926765, 'motion_component': 0.3409227587045228}, {'ion': 1320, 'force': [-4.218984603881836, 4.771722316741943, -2.8418822288513184], 'magnitude': 6.974629878997803, 'distance': 6.899354457855225, 'before_closest_residue': 'SF', 'closest_residue': 'SF', 'next_closest_residue': 'SF', 'cosine_with_motion': -0.41062905962600516, 'motion_component': -2.8639856380834434}, {'ion': 1403, 'force': [-1.7074979543685913, 1.6937834024429321, -2.7924537658691406], 'magnitude': 3.685410261154175, 'distance': 9.49130916595459, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.28108048830992605, 'motion_component': -1.0358969432865663}, {'ion': 1469, 'force': [-0.4841288626194, 0.510909914970398, -1.709849238395691], 'magnitude': 1.8490521907806396, 'distance': 13.399681091308594, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.20256639275756702, 'motion_component': -0.37455583836772854}]}, 5230: {'frame': 5230, 'ionic_force': [-15.662788987159729, -0.7856491804122925, -5.916200011968613], 'ionic_force_magnitude': 16.761313375526154, 'motion_vector': [5.115959167480469, 0.8695487976074219, -4.300270080566406], 'cosine_ionic_motion': -0.49017623311192193, 'ionic_motion_component': -8.215997452423883, 'ionic_force_x': -15.662788987159729, 'ionic_force_y': -0.7856491804122925, 'ionic_force_z': -5.916200011968613, 'radial_force': 15.682480782420065, 'axial_force': -5.916200011968613, 'before_closest_residue': 98, 'closest_residue': 1105, 'next_closest_residue': 130, 'contributions': [{'ion': 1306, 'force': [-2.190549612045288, 1.3503695726394653, -0.047841042280197144], 'magnitude': 2.573770523071289, 'distance': 11.357536315917969, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.5665165463387223, 'motion_component': -1.458083548777168}, {'ion': 1308, 'force': [-3.4431419372558594, -1.4593416452407837, 1.5944634675979614], 'magnitude': 4.065368175506592, 'distance': 9.03689193725586, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': -0.9394801019205968, 'motion_component': -3.819332482993259}, {'ion': 1320, 'force': [-6.761546611785889, -0.46857988834381104, -2.9621737003326416], 'magnitude': 7.396793365478516, 'distance': 6.699575424194336, 'before_closest_residue': 'SF', 'closest_residue': 'SF', 'next_closest_residue': 'SF', 'cosine_with_motion': -0.44655252950108015, 'motion_component': -3.3030568067030313}, {'ion': 1403, 'force': [-2.4797613620758057, -0.12971417605876923, -2.8303792476654053], 'magnitude': 3.7652475833892822, 'distance': 9.390144</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>5293</v>
+      </c>
+      <c r="B13" t="n">
+        <v>5331</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1403</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>{5293: {'frame': 5293, 'ionic_force': [-7.19414022564888, -9.335815489292145, -6.3991100788116455], 'ionic_force_magnitude': 13.411253268697719, 'motion_vector': [3.6029815673828125, -0.9414405822753906, -2.305633544921875], 'cosine_ionic_motion': -0.04047029908956818, 'ionic_motion_component': -0.5427574309501456, 'ionic_force_x': -7.19414022564888, 'ionic_force_y': -9.335815489292145, 'ionic_force_z': -6.3991100788116455, 'radial_force': 11.786140353669918, 'axial_force': -6.3991100788116455, 'before_closest_residue': None, 'closest_residue': 1105, 'next_closest_residue': 1105, 'contributions': [{'ion': 1306, 'force': [-2.7549750804901123, 2.149670362472534, -0.8896871209144592], 'magnitude': 3.6058998107910156, 'distance': 9.595380783081055, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.6267500552568542, 'motion_component': -2.2599979134049164}, {'ion': 1309, 'force': [-0.4600997269153595, -6.4237165451049805, -1.8560487031936646], 'magnitude': 6.702293872833252, 'distance': 7.038130283355713, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.2953168585098998, 'motion_component': 1.9793003634343174}, {'ion': 1320, 'force': [-2.2913060188293457, -4.553028583526611, 0.9146720767021179], 'magnitude': 5.178492069244385, 'distance': 8.00695514678955, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 423, 'cosine_with_motion': -0.26797402199208176, 'motion_component': -1.387701281697467}, {'ion': 1469, 'force': [-1.280375599861145, -0.43071743845939636, -2.963862419128418], 'magnitude': 3.2572009563446045, 'distance': 10.095939636230469, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.18406364306654752, 'motion_component': 0.5995323182463634}, {'ion': 2436, 'force': [-0.4073837995529175, -0.0780232846736908, -1.6041839122772217], 'magnitude': 1.656941533088684, 'distance': 14.155181884765625, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.3175182671968274, 'motion_component': 0.5261092018864266}]}, 5294: {'frame': 5294, 'ionic_force': [-3.9219388999044895, -4.9589075446128845, -9.572859406471252], 'ionic_force_magnitude': 11.472227594790288, 'motion_vector': [-1.1986160278320312, 0.10608673095703125, 0.8895950317382812], 'cosine_ionic_motion': -0.2528709329394575, 'ionic_motion_component': -2.9009928947884087, 'ionic_force_x': -3.9219388999044895, 'ionic_force_y': -4.9589075446128845, 'ionic_force_z': -9.572859406471252, 'radial_force': 6.322370502477898, 'axial_force': -9.572859406471252, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 1105, 'contributions': [{'ion': 1306, 'force': [-4.087786674499512, 1.854230284690857, -3.7001771926879883], 'magnitude': 5.817171096801758, 'distance': 7.554628372192383, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.20732159310216006, 'motion_component': 1.206025206449235}, {'ion': 1309, 'force': [1.4283074140548706, -3.2946081161499023, -1.909952163696289], 'magnitude': 4.067237377166748, 'distance': 9.034814834594727, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.6178726576783165, 'motion_component': -2.5130349266499294}, {'ion': 1320, 'force': [-1.2332184314727783, -2.8408944606781006, -1.2032557725906372], 'magnitude': 3.3225491046905518, 'distance': 9.996163368225098, 'before_closest_residue': 130, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.021392684254919057, 'motion_component': 0.0710782469366329}, {'ion': 1469, 'force': [-0.029241207987070084, -0.6776352524757385, -2.759474277496338], 'magnitude': 2.841609239578247, 'distance': 10.809033393859863, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.585957106898025, 'motion_component': -1.665061108476534}]}, 5295: {'frame': 5295, 'ionic_force': [-4.847121506929398, -6.3855297565460205, -10.225951194763184], 'ionic_force_magnitude': 12.993831421576576, 'motion_vector': [1.4610366821289062, 0.4837226867675781, -0.33788299560546875], 'cosine_ionic_motion': -0.3279972204302937, 'ionic_motion_component': -4.2619405890169295, 'ionic_force_x': -4.847121506929398, 'ionic_force_y': -6.3855297565460205, 'ionic_force_z': -10.225951194763184, 'radial_force': 8.016830868533537, 'axial_force': -10.225951194763184, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 1105, 'contributions': [{'ion': 1306, 'force': [-3.9522693157196045, 1.6182080507278442, -3.028805732727051], 'magnitude': 5.235713481903076, 'distance': 7.963080883026123, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.48101160257019815, 'motion_component': -2.518438865528612}, {'ion': 1309, 'force': [1.2909294366836548, -4.2322163581848145, -2.066220760345459], 'magnitude': 4.883382320404053, 'distance': 8.245342254638672, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.06979078553032043, 'motion_component': 0.340815084300246}, {'ion': 1320, 'force': [-1.8195945024490356, -3.148383855819702, -1.8783209323883057], 'magnitude': 4.09283971786499, 'distance': 9.006513595581055, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 455, 'cosine_with_motion': -0.5499726823402922, 'motion_component': -2.2509498785102373}, {'ion': 1469, 'force': [-0.36618712544441223, -0.6231375932693481, -3.252603769302368], 'magnitude': 3.331940174102783, 'distance': 9.98206615447998, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.05001077294285725, 'motion_component': 0.16663289920801638}]}, 5296: {'frame': 5296, 'ionic_force': [-3.5437815007171594, -4.856745570898056, -10.527804255485535], 'ionic_force_magnitude': 12.123573207065744, 'motion_vector': [-0.4652824401855469, 0.103912353515625, -2.422882080078125], 'cosine_ionic_motion': 0.8902564047286571, 'ionic_motion_component': 10.793088695787025, 'ionic_force_x': -3.5437815007171594, 'ionic_force_y': -4.856745570898056, 'ionic_force_z': -10.527804255485535, 'radial_force': 6.012184699862692, 'axial_force': -10.527804255485535, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 1105, 'contributions': [{'ion': 1306, 'force': [-3.8624563217163086, 3.411072015762329, -3.2963201999664307], 'magnitude': 6.1171650886535645, 'distance': 7.367055416107178, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.6711642842303779, 'motion_component': 4.105622688348834}, {'ion': 1309, 'force': [2.060899019241333, -4.070521354675293, -2.4136157035827637], 'magnitude': 5.161587715148926, 'distance': 8.020055770874023, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.350394413188984, 'motion_component': 1.808591562717023}, {'ion': 1320, 'force': [-1.741642713546753, -3.7549068927764893, -1.5699185132980347], 'magnitude': 4.426882743835449, 'distance': 8.660042762756348, 'before_closest_residue': 423, 'closest_residue': 455, 'next_closest_residue': 423, 'cosine_with_motion': 0.3863979687561965, 'motion_component': 1.7105384314382377}, {'ion': 1469, 'force': [-0.000581484695430845, -0.4423893392086029, -3.2479498386383057], 'magnitude': 3.2779393196105957, 'distance': 10.063952445983887, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.9665632598820196, 'motion_component': 3.1683358083492243}]}, 5297: {'frame': 5297, 'ionic_force': [-0.009639695286750793, -1.7626727223396301, -9.943647146224976], 'ionic_force_magnitude': 10.098674498092981, 'motion_vector': [0.11940383911132812, -0.8824501037597656, 1.4705276489257812], 'cosine_ionic_motion': -0.7527271372165049, 'ionic_motion_component': -7.6015463446308535, 'ionic_force_x': -0.009639695286750793, 'ionic_force_y': -1.7626727223396301, 'ionic_force_z': -9.943647146224976, 'radial_force': 1.7626990808999203, 'axial_force': -9.943647146224976, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 1105, 'contributions': [{'ion': 1306, 'force': [-2.068286657333374, 2.263288974761963, -3.181971549987793], 'magnitude': 4.418736457824707, 'distance': 8.668022155761719, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.911401759394988, 'motion_component': -4.027243949037029}, {'ion': 1309, 'force': [2.703697919845581, -1.9296005964279175, -3.2435293197631836], 'magnitude': 4.642609596252441, 'distance': 8.45644760131836, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 1105, 'cosine_with_motion': -0.34381617958818117, 'motion_component': -1.5962042757614867}, {'ion': 1320, 'force': [-0.5463349223136902, -1.8209863901138306, -1.1804895401000977], 'magnitude': 2.2378625869750977, 'distance': 12.18014144897461, 'before_closest_residue': 455, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.050490734426634716, 'motion_component': -0.1129913241681777}, {'ion': 1469, 'force': [-0.09871603548526764, -0.27537471055984497, -2.3376567363739014], 'magnitude': 2.3558895587921143, 'distance': 11.871116638183594, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7916784499341073, 'motion_component': -1.8651069085584862}]}, 5298: {'frame': 5298, 'ionic_force': [-0.9545583575963974, -6.526641249656677, -10.410386621952057], 'ionic_force_magnitude': 12.324137993316027, 'motion_vector': [-0.8501853942871094, 0.7801551818847656, 2.5111923217773438], 'cosine_ionic_motion': -0.8932328782438211, 'ionic_motion_component': -11.008325251643704, 'ionic_force_x': -0.9545583575963974, 'ionic_force_y': -6.526641249656677, 'ionic_force_z': -10.410386621952057, 'radial_force': 6.596076686923614, 'axial_force': -10.410386621952057, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 1105, 'contributions': [{'ion': 1306, 'force': [-3.5949900150299072, 2.179809331893921, -3.1837265491485596], 'magnitude': 5.273674011230469, 'distance': 7.934369087219238, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.22216736785251526, 'motion_component': -1.1716382549161608}, {'ion': 1309, 'force': [3.2287416458129883, -6.1072096824646, -3.8306076526641846], 'magnitude': 7.899135589599609, 'distance': 6.483048439025879, 'before_closest_residue': 98, 'closest_residue': 1105, 'next_closest_residue': 1073, 'cosine_with_motion': -0.7846489917489425, 'motion_component': -6.19804851018975}, {'ion': 1320, 'force': [-0.4978197515010834, -2.0856738090515137, -0.9577496647834778], 'magnitude': 2.3484344482421875, 'distance': 11.889945030212402, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.5560732892391631, 'motion_component': -1.3059016451634013}, {'ion': 1469, 'force': [-0.09049023687839508, -0.5135670900344849, -2.438302755355835], 'magnitude': 2.493443489074707, 'distance': 11.539029121398926, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.9355482454164143, 'motion_component': -2.3327365935457256}]}, 5299: {'frame': 5299, 'ionic_force': [2.9334011897444725, -1.9908200800418854, -12.94955426454544], 'ionic_force_magnitude': 13.426062817576092, 'motion_vector': [-0.3539390563964844, 2.2585983276367188, 2.1390380859375], 'cosine_ionic_motion': -0.790642145551316, 'ionic_motion_component': -10.615211112395107, 'ionic_force_x': 2.9334011897444725, 'ionic_force_y': -1.9908200800418854, 'ionic_force_z': -12.94955426454544, 'radial_force': 3.5451667282502055, 'axial_force': -12.94955426454544, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 'SF', 'contributions': [{'ion': 1306, 'force': [-5.214995384216309, 3.869166851043701, -2.5838310718536377], 'magnitude': 6.988763332366943, 'distance': 6.892374515533447, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.23115378997793093, 'motion_component': 1.6154791161662985}, {'ion': 1309, 'force': [9.771367073059082, -2.351778030395508, -4.5568013191223145], 'magnitude': 11.03516674041748, 'distance': 5.485037326812744, 'before_closest_residue': 1105, 'closest_residue': 1073, 'next_closest_residue': 1105, 'cosine_with_motion': -0.5359722734248957, 'motion_component': -5.914543591356164}, {'ion': 1320, 'force': [-1.1783761978149414, -2.824215888977051, -0.5681673884391785], 'magnitude': 3.11248779296875, 'distance': 10.32797622680664, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 455, 'cosine_with_motion': -0.7365107631581589, 'motion_component': -2.2923807326295993}, {'ion': 1469, 'force': [-0.3746396005153656, -0.5283625721931458, -3.711301326751709], 'magnitude': 3.767396926879883, 'distance': 9.387465476989746, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7629798072189766, 'motion_component': -2.8744477578251457}, {'ion': 2436, 'force': [-0.06995470076799393, -0.1556304395198822, -1.529453158378601], 'magnitude': 1.5389416217803955, 'distance': 14.687841415405273, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7468235204612907, 'motion_component': -1.1493178342881796}]}, 5302: {'frame': 5302, 'ionic_force': [-6.390175463631749, -3.4052871465682983, -11.440962880849838], 'ionic_force_magnitude': 13.539791528955249, 'motion_vector': [-1.703094482421875, 1.6502799987792969, -1.0469818115234375], 'cosine_ionic_motion': 0.4912288202597912, 'ionic_motion_component': 6.651135819332201, 'ionic_force_x': -6.390175463631749, 'ionic_force_y': -3.4052871465682983, 'ionic_force_z': -11.440962880849838, 'radial_force': 7.240878607364199, 'axial_force': -11.440962880849838, 'before_closest_residue': 'SF', 'closest_residue': 1105, 'next_closest_residue': 1105, 'contributions': [{'ion': 1306, 'force': [-15.774862289428711, 7.403421878814697, -5.208380699157715], 'magnitude': 18.18747329711914, 'distance': 4.272507667541504, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.9446234981448682, 'motion_component': 17.18031413779147}, {'ion': 1309, 'force': [9.655634880065918, -6.011810302734375, 0.029120855033397675], 'magnitude': 11.374268531799316, 'distance': 5.402655601501465, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 'SF', 'cosine_with_motion': -0.8952160799916463, 'motion_component': -10.182428538158979}, {'ion': 1320, 'force': [-0.391956627368927, -2.144749641418457, -0.11846282333135605], 'magnitude': 2.1834867000579834, 'distance': 12.33087158203125, 'before_closest_residue': 423, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': -0.4854638859897166, 'motion_component': -1.0600039710206126}, {'ion': 1469, 'force': [0.1119040995836258, -2.1314122676849365, -4.249485492706299], 'magnitude': 4.755372524261475, 'distance': 8.355583190917969, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.06011979097258749, 'motion_component': 0.2858920014635995}, {'ion': 2436, 'force': [0.009104473516345024, -0.520736813545227, -1.8937547206878662], 'magnitude': 1.9640663862228394, 'distance': 13.001425743103027, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.21759044093186494, 'motion_component': 0.42736206507377106}]}, 5303: {'frame': 5303, 'ionic_force': [0.2442486435174942, -4.38072469830513, -19.32172292470932], 'ionic_force_magnitude': 19.813616102605764, 'motion_vector': [2.9986648559570312, -0.3383674621582031, -0.0259552001953125], 'cosine_ionic_motion': 0.045426446406585275, 'ionic_motion_component': 0.9000621700056757, 'ionic_force_x': 0.2442486435174942, 'ionic_force_y': -4.38072469830513, 'ionic_force_z': -19.32172292470932, 'radial_force': 4.387528493605564, 'axial_force': -19.32172292470932, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [-4.38976526260376, 3.0124411582946777, -1.014961838722229], 'magnitude': 5.419869899749756, 'distance': 7.826626777648926, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.8655110961920905, 'motion_component': -4.6909574261108125}, {'ion': 1309, 'force': [6.351526737213135, -4.161134243011475, -12.593794822692871], 'magnitude': 14.705801963806152, 'distance': 4.751433849334717, 'before_closest_residue': 1105, 'closest_residue': 'SF', 'next_closest_residue': 1105, 'cosine_with_motion': 0.46825843997322103, 'motion_component': 6.886115674686596}, {'ion': 1320, 'force': [-0.7893285751342773, -2.2547266483306885, -0.49746209383010864], 'magnitude': 2.440143585205078, 'distance': 11.664371490478516, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': -0.21606729356545698, 'motion_component': -0.5272352060481691}, {'ion': 1469, 'force': [-0.7389268279075623, -0.7736309766769409, -3.6220219135284424], 'magnitude': 3.7767128944396973, 'distance': 9.375880241394043, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.16319631554447808, 'motion_component': -0.6163456335657835}, {'ion': 2436, 'force': [-0.1892574280500412, -0.20367398858070374, -1.593482255935669], 'magnitude': 1.6175559759140015, 'distance': 14.326476097106934, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.093669258529189, 'motion_component': -0.15151526404247218}]}, 5304: {'frame': 5304, 'ionic_force': [5.99651138484478, -0.8443090319633484, -13.91120171546936], 'ionic_force_magnitude': 15.172097406044612, 'motion_vector': [-1.4822731018066406, 2.659027099609375, -2.7203369140625], 'cosine_ionic_motion': 0.4312047220637964, 'ionic_motion_component': 6.542280045098313, 'ionic_force_x': 5.99651138484478, 'ionic_force_y': -0.8443090319633484, 'ionic_force_z': -13.91120171546936, 'radial_force': 6.055659050014949, 'axial_force': -13.91120171546936, 'before_closest_residue': 1105, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [-5.513181209564209, 9.734850883483887, -3.1628122329711914], 'magnitude': 11.62608528137207, 'distance': 5.343825817108154, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.8987944896174224, 'motion_component': 10.449461812861117}, {'ion': 1309, 'force': [10.475059509277344, -6.060859680175781, -4.418924331665039], 'magnitude': 12.883625030517578, 'distance': 5.076332092285156, 'before_closest_residue': 'SF', 'closest_residue': 1105, 'next_closest_residue': 780, 'cosine_with_motion': -0.3730478564218393, 'motion_component': -4.806208557360378}, {'ion': 1320, 'force': [-0.10482928156852722, -3.094301462173462, -0.409082293510437], 'magnitude': 3.122985601425171, 'distance': 10.310602188110352, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': -0.5458528017668542, 'motion_component': -1.7046904380766525}, {'ion': 1469, 'force': [0.9543324708938599, -1.1745716333389282, -4.332919597625732], 'magnitude': 4.589614391326904, 'distance': 8.50512981414795, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.3868788436129706, 'motion_component': 1.7756247490290527}, {'ion': 2436, 'force': [0.18512989580631256, -0.24942713975906372, -1.5874632596969604], 'magnitude': 1.6175681352615356, 'distance': 14.326422691345215, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5119368498997857, 'motion_component': 0.8280927206379406}]}, 5305: {'frame': 5305, 'ionic_force': [-9.088852025568485, 12.996454022824764, -18.47400403022766], 'ionic_force_magnitude': 24.347564009956855, 'motion_vector': [3.7210350036621094, 0.5313720703125, 4.7978057861328125], 'cosine_ionic_motion': -0.778655237347414, 'ionic_motion_component': -18.95835823300431, 'ionic_force_x': -9.088852025568485, 'ionic_force_y': 12.996454022824764, 'ionic_force_z': -18.47400403022766, 'radial_force': 15.85922596818894, 'axial_force': -18.47400403022766, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 423, 'contributions': [{'ion': 1306, 'force': [-1.5247687101364136, 2.842219114303589, -1.7802704572677612], 'magnitude': 3.684086322784424, 'distance': 9.493014335632324, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.5658156977839071, 'motion_component': -2.08451387191859}, {'ion': 1309, 'force': [-6.675297737121582, 13.578149795532227, -11.790082931518555], 'magnitude': 19.181549072265625, 'distance': 4.160324573516846, 'before_closest_residue': 1105, 'closest_residue': 780, 'next_closest_residue': 1105, 'cosine_with_motion': -0.6346004901054394, 'motion_component': -12.17262015225235}, {'ion': 1320, 'force': [-0.9775453209877014, -3.548858880996704, -1.993395209312439], 'magnitude': 4.186121940612793, 'distance': 8.905597686767578, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 98, 'cosine_with_motion': -0.5913323316384337, 'motion_component': -2.4753893727261147}, {'ion': 1469, 'force': [0.08875974267721176, 0.12494399398565292, -2.9102554321289062], 'magnitude': 2.91428804397583, 'distance': 10.673399925231934, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7637664263245683, 'motion_component': -2.2258355180118463}]}, 5306: {'frame': 5306, 'ionic_force': [17.38727957010269, 2.2386045455932617, -4.978819995420054], 'ionic_force_magnitude': 18.22409091579758, 'motion_vector': [-1.9650535583496094, -1.8321075439453125, -0.7120208740234375], 'cosine_ionic_motion': -0.6855274194985111, 'ionic_motion_component': -12.493114018212973, 'ionic_force_x': 17.38727957010269, 'ionic_force_y': 2.2386045455932617, 'ionic_force_z': -4.978819995420054, 'radial_force': 17.530796934550956, 'axial_force': -4.978819995420054, 'before_closest_residue': 780, 'closest_residue': 423, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [-0.08853501081466675, 6.812282085418701, 0.0004690892528742552], 'magnitude': 6.812857627868652, 'distance': 6.98078727722168, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.6499496001958854, 'motion_component': -4.4280139398283245}, {'ion': 1309, 'force': [4.468284606933594, 4.662998676300049, 3.70725679397583], 'magnitude': 7.44666862487793, 'distance': 6.677102088928223, 'before_closest_residue': 780, 'closest_residue': 1105, 'next_closest_residue': 1105, 'cosine_with_motion': -0.9645342433791801, 'motion_component': -7.182567102252463}, {'ion': 1320, 'force': [7.873488903045654, -10.533976554870605, 0.34959670901298523], 'magnitude': 13.155938148498535, 'distance': 5.023519992828369, 'before_closest_residue': 455, 'closest_residue': 98, 'next_closest_residue': 455, 'cosine_with_motion': 0.09786899057282514, 'motion_component': 1.2875583823797827}, {'ion': 1469, 'force': [4.469884872436523, 1.055068850517273, -6.895050525665283], 'magnitude': 8.2846097946167, 'distance': 6.330427169799805, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.25219732116268007, 'motion_component': -2.0893564481400375}, {'ion': 2436, 'force': [0.6641561985015869, 0.24223148822784424, -2.14109206199646], 'magnitude': 2.2547848224639893, 'distance': 12.13434886932373, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.03580609982653162, 'motion_component': -0.08073505180798435}]}, 5307: {'frame': 5307, 'ionic_force': [3.0109886080026627, 10.63396979868412, -2.637856215238571], 'ionic_force_magnitude': 11.362466787151483, 'motion_vector': [-1.8429718017578125, 0.5340690612792969, 3.6442413330078125], 'cosine_ionic_motion': -0.20264017499624698, 'ionic_motion_component': -2.3024922581374208, 'ionic_force_x': 3.0109886080026627, 'ionic_force_y': 10.63396979868412, 'ionic_force_z': -2.637856215238571, 'radial_force': 11.052029952766496, 'axial_force': -2.637856215238571, 'before_closest_residue': 423, 'closest_residue': 780, 'next_closest_residue': 'SF', 'contributions': [{'ion': 1306, 'force': [-2.994255304336548, 7.662434101104736, -1.3457634449005127], 'magnitude': 8.336038589477539, 'distance': 6.310869216918945, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.13708150785158865, 'motion_component': 1.1427167481169676}, {'ion': 1309, 'force': [5.069587707519531, 8.484151840209961, 7.271227836608887], 'magnitude': 12.269975662231445, 'distance': 5.201722621917725, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 1105, 'cosine_with_motion': 0.4291373195283767, 'motion_component': 5.265504527085966}, {'ion': 1320, 'force': [-0.18250830471515656, -4.807651519775391, -0.49011465907096863], 'magnitude': 4.836014270782471, 'distance': 8.285624504089355, 'before_closest_residue': 98, 'closest_residue': 455, 'next_closest_residue': 423, 'cosine_with_motion': -0.2017022843551575, 'motion_component': -0.975435141621853}, {'ion': 1469, 'force': [0.850151538848877, -0.5294232368469238, -5.994930744171143], 'magnitude': 6.078012943267822, 'distance': 7.390745162963867, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.9466319012710269, 'motion_component': -5.753640939993872}, {'ion': 2436, 'force': [0.26801297068595886, -0.17554138600826263, -2.078275203704834], 'magnitude': 2.102825164794922, 'distance': 12.565143585205078, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.942369072941603, 'motion_component': -1.9816373740599276}]}, 5319: {'frame': 5319, 'ionic_force': [-1.0818994492292404, -4.203714609146118, -11.860607624053955], 'ionic_force_magnitude': 12.629953924902411, 'motion_vector': [-0.37534332275390625, 2.9748268127441406, 1.076873779296875], 'cosine_ionic_motion': -0.6181108593164678, 'ionic_motion_component': -7.806711673648825, 'ionic_force_x': -1.0818994492292404, 'ionic_force_y': -4.203714609146118, 'ionic_force_z': -11.860607624053955, 'radial_force': 4.340705349754926, 'axial_force': -11.860607624053955, 'before_closest_residue': 'SF', 'closest_residue': 780, 'next_closest_residue': 1105, 'contributions': [{'ion': 1306, 'force': [-5.016157627105713, 3.5561301708221436, -4.3967204093933105], 'magnitude': 7.559037685394287, 'distance': 6.627286911010742, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.3208522915447733, 'motion_component': 2.425334536935946}, {'ion': 1309, 'force': [-0.5297877788543701, -1.9051895141601562, -0.5782485008239746], 'magnitude': 2.0602896213531494, 'distance': 12.69418716430664, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.928019348194915, 'motion_component': -1.911988672116065}, {'ion': 1320, 'force': [4.629401683807373, -4.809083938598633, -4.047743797302246], 'magnitude': 7.806591987609863, 'distance': 6.521361827850342, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 1105, 'cosine_with_motion': -0.8203338325197492, 'motion_component': -6.4040115065710275}, {'ion': 1469, 'force': [-0.16535572707653046, -1.0455713272094727, -2.837894916534424], 'magnitude': 3.028895854949951, 'distance': 10.469522476196289, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6325889031253409, 'motion_component': -1.9160458411847072}]}, 5320: {'frame': 5320, 'ionic_force': [8.028144970536232, 0.7072750627994537, -13.924635171890259], 'ionic_force_magnitude': 16.088716989015854, 'motion_vector': [2.132244110107422, -0.18821334838867188, -5.501701354980469], 'cosine_ionic_motion': 0.9854204000835611, 'ionic_motion_component': 15.85414993214719, 'ionic_force_x': 8.028144970536232, 'ionic_force_y': 0.7072750627994537, 'ionic_force_z': -13.924635171890259, 'radial_force': 8.05924001891023, 'axial_force': -13.924635171890259, 'before_closest_residue': 780, 'closest_residue': 1105, 'next_closest_residue': 130, 'contributions': [{'ion': 1306, 'force': [-3.2315402030944824, 3.8009941577911377, -1.959601640701294], 'magnitude': 5.360079288482666, 'distance': 7.870157718658447, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.1003483208085931, 'motion_component': 0.5378749305689388}, {'ion': 1309, 'force': [-1.0903435945510864, -3.212728977203369, -0.8711439371109009], 'magnitude': 3.5027658939361572, 'distance': 9.735616683959961, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.14858877414098715, 'motion_component': 0.5204716793931627}, {'ion': 1320, 'force': [13.06535816192627, 0.526891827583313, -5.3541388511657715], 'magnitude': 14.129684448242188, 'distance': 4.84733247756958, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 1105, 'cosine_with_motion': 0.6859328826384599, 'motion_component': 9.692015648645212}, {'ion': 1469, 'force': [-0.6009418368339539, -0.342739462852478, -4.116855621337891], 'magnitude': 4.1745781898498535, 'distance': 8.917902946472168, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.8696858990365816, 'motion_component': 3.63057163764374}, {'ion': 2436, 'force': [-0.11438755691051483, -0.06514248251914978, -1.6228951215744019], 'magnitude': 1.6282249689102173, 'distance': 14.279461860656738, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.9047987658167145, 'motion_component': 1.4732159652510708}]}, 5321: {'frame': 5321, 'ionic_force': [1.2822358161211014, 0.02604774385690689, -8.487277030944824], 'ionic_force_magnitude': 8.583628520218438, 'motion_vector': [-0.4481773376464844, -0.15670394897460938, 0.02079010009765625], 'cosine_ionic_motion': -0.1851317969355534, 'ionic_motion_component': -1.5891025721753047, 'ionic_force_x': 1.2822358161211014, 'ionic_force_y': 0.02604774385690689, 'ionic_force_z': -8.487277030944824, 'radial_force': 1.2825003598844649, 'axial_force': -8.487277030944824, 'before_closest_residue': 1105, 'closest_residue': 130, 'next_closest_residue': 1105, 'contributions': [{'ion': 1306, 'force': [-0.8649483323097229, 1.5502290725708008, -2.8214263916015625], 'magnitude': 3.333435535430908, 'distance': 9.979826927185059, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.05432825060791179, 'motion_component': 0.1810997228602922}, {'ion': 1309, 'force': [-0.149215430021286, -1.4748518466949463, -1.3792165517807007], 'magnitude': 2.0247695446014404, 'distance': 12.805048942565918, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.27988222322103423, 'motion_component': 0.56669698798355}, {'ion': 1320, 'force': [2.1659634113311768, 0.05920436233282089, -2.643592596054077], 'magnitude': 3.4181110858917236, 'distance': 9.855438232421875, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 1073, 'cosine_with_motion': -0.6371356173177156, 'motion_component': -2.1778004168818765}, {'ion': 1469, 'force': [0.13043616712093353, -0.1085338443517685, -1.6430414915084839], 'magnitude': 1.651780366897583, 'distance': 14.177278518676758, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.09631962227384024, 'motion_component': -0.15909886543356633}]}, 5322: {'frame': 5322, 'ionic_force': [0.05070401728153229, -0.26690953969955444, -7.58734929561615], 'ionic_force_magnitude</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>5347</v>
+      </c>
+      <c r="B14" t="n">
+        <v>5886</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1469</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>{5347: {'frame': 5347, 'ionic_force': [-1.5767408609390259, -7.108273267745972, -12.609045714139938], 'ionic_force_magnitude': 14.560277964818443, 'motion_vector': [3.316211700439453, -1.65020751953125, -0.9902801513671875], 'cosine_ionic_motion': 0.340118482876991, 'ionic_motion_component': 4.952219651661331, 'ionic_force_x': -1.5767408609390259, 'ionic_force_y': -7.108273267745972, 'ionic_force_z': -12.609045714139938, 'radial_force': 7.281048042109511, 'axial_force': -12.609045714139938, 'before_closest_residue': None, 'closest_residue': 130, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [-2.2620508670806885, 2.0216140747070312, -0.8754827976226807], 'magnitude': 3.1575732231140137, 'distance': 10.253976821899414, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.8235514697076532, 'motion_component': -2.6004239462711567}, {'ion': 1309, 'force': [-3.900376081466675, -0.4288240671157837, -0.44240328669548035], 'magnitude': 3.948739528656006, 'distance': 9.169376373291016, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': -0.7786338398051467, 'motion_component': -3.0746222669723364}, {'ion': 1320, 'force': [5.2017621994018555, -9.052448272705078, -8.116565704345703], 'magnitude': 13.224363327026367, 'distance': 5.010506629943848, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.793340665917229, 'motion_component': 10.491425302286757}, {'ion': 2436, 'force': [-0.6160761117935181, 0.3513849973678589, -3.174593925476074], 'magnitude': 3.2528553009033203, 'distance': 10.102682113647461, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.04176044234126463, 'motion_component': 0.13584067736087846}]}, 5348: {'frame': 5348, 'ionic_force': [-6.454585552215576, -0.6436145454645157, -10.31672191619873], 'ionic_force_magnitude': 12.186495206997735, 'motion_vector': [1.4751319885253906, 0.6213607788085938, -1.0232925415039062], 'cosine_ionic_motion': 0.027459638819205618, 'ionic_motion_component': 0.3346367568561382, 'ionic_force_x': -6.454585552215576, 'ionic_force_y': -0.6436145454645157, 'ionic_force_z': -10.31672191619873, 'radial_force': 6.4865949722488105, 'axial_force': -10.31672191619873, 'before_closest_residue': 130, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [-3.4947903156280518, 3.541504383087158, -3.898306131362915], 'magnitude': 6.320806980133057, 'distance': 7.247408866882324, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.0861393042315145, 'motion_component': 0.5444699322082869}, {'ion': 1309, 'force': [-6.009511947631836, -2.5683140754699707, -1.4689178466796875], 'magnitude': 6.6983723640441895, 'distance': 7.04019021987915, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': -0.7039018768949364, 'motion_component': -4.714996792595642}, {'ion': 1320, 'force': [2.708761215209961, -1.4557560682296753, -2.3566243648529053], 'magnitude': 3.874311685562134, 'distance': 9.25703239440918, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.7476143142621089, 'motion_component': 2.8964909137275363}, {'ion': 2436, 'force': [0.3409554958343506, -0.1610487848520279, -2.5928735733032227], 'magnitude': 2.6201491355895996, 'distance': 11.256568908691406, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.6139624104715719, 'motion_component': 1.6086729895284697}]}, 5349: {'frame': 5349, 'ionic_force': [-8.160462379455566, -2.827123999595642, -15.069315671920776], 'ionic_force_magnitude': 17.368651391964672, 'motion_vector': [-0.10723876953125, -1.5981407165527344, 3.5609359741210938], 'cosine_ionic_motion': -0.7117284220392917, 'ionic_motion_component': -12.361762848153562, 'ionic_force_x': -8.160462379455566, 'ionic_force_y': -2.827123999595642, 'ionic_force_z': -15.069315671920776, 'radial_force': 8.636305712259105, 'axial_force': -15.069315671920776, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [-0.7823565006256104, 3.8195178508758545, -4.267391204833984], 'magnitude': 5.780261993408203, 'distance': 7.578710079193115, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.9400336360373088, 'motion_component': -5.433640478541244}, {'ion': 1309, 'force': [-10.252406120300293, -4.798220634460449, -6.5559773445129395], 'magnitude': 13.08111572265625, 'distance': 5.037866592407227, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': -0.28541032674556904, 'motion_component': -3.733485544288841}, {'ion': 1320, 'force': [2.3740317821502686, -1.7368981838226318, -2.094464063644409], 'magnitude': 3.61104154586792, 'distance': 9.588546752929688, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 130, 'cosine_with_motion': -0.35015323973539414, 'motion_component': -1.2644179383602139}, {'ion': 2436, 'force': [0.5002684593200684, -0.11152303218841553, -2.1514830589294434], 'magnitude': 2.2116928100585938, 'distance': 12.25199031829834, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.872733684797831, 'motion_component': -1.9302188522429757}]}, 5350: {'frame': 5350, 'ionic_force': [-2.6436456441879272, -5.840722948312759, -5.4077256843447685], 'ionic_force_magnitude': 8.387276311658225, 'motion_vector': [2.5827255249023438, 0.7509269714355469, 2.464935302734375], 'cosine_ionic_motion': -0.8020869676506136, 'ionic_motion_component': -6.7273250236657685, 'ionic_force_x': -2.6436456441879272, 'ionic_force_y': -5.840722948312759, 'ionic_force_z': -5.4077256843447685, 'radial_force': 6.4111548765398805, 'axial_force': -5.4077256843447685, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 748, 'contributions': [{'ion': 1306, 'force': [-2.4985830783843994, 10.913158416748047, -2.3083724975585938], 'magnitude': 11.43103313446045, 'distance': 5.389224529266357, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 780, 'cosine_with_motion': -0.09467071712865942, 'motion_component': -1.0821841420227116}, {'ion': 1309, 'force': [-7.1796159744262695, -10.836474418640137, 3.318307876586914], 'magnitude': 13.415931701660156, 'distance': 4.974605083465576, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': -0.3779898179059257, 'motion_component': -5.07108568105761}, {'ion': 1320, 'force': [5.264742851257324, -4.707367897033691, -0.06457030028104782], 'magnitude': 7.062648296356201, 'distance': 6.856228351593018, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 98, 'cosine_with_motion': 0.3843443305678448, 'motion_component': 2.714488781801923}, {'ion': 2434, 'force': [0.3296545743942261, -0.23305991291999817, -1.7742886543273926], 'magnitude': 1.8196399211883545, 'distance': 13.50754165649414, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5569081574761272, 'motion_component': -1.0133722924457365}, {'ion': 2436, 'force': [1.4401559829711914, -0.97697913646698, -4.578802108764648], 'magnitude': 4.8983635902404785, 'distance': 8.232723236083984, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.4644758616720765, 'motion_component': -2.2751716672537476}]}, 5351: {'frame': 5351, 'ionic_force': [11.309775292873383, -1.0368304997682571, 9.539171248674393], 'ionic_force_magnitude': 14.831784207305441, 'motion_vector': [-4.924442291259766, -0.13016128540039062, 1.0756683349609375], 'cosine_ionic_motion': -0.6057121873694583, 'ionic_motion_component': -8.983792454798767, 'ionic_force_x': 11.309775292873383, 'ionic_force_y': -1.0368304997682571, 'ionic_force_z': 9.539171248674393, 'radial_force': 11.357201885171316, 'axial_force': 9.539171248674393, 'before_closest_residue': 780, 'closest_residue': 748, 'next_closest_residue': 'SF', 'contributions': [{'ion': 1306, 'force': [4.731605052947998, 9.634112358093262, 3.1262471675872803], 'magnitude': 11.179339408874512, 'distance': 5.449554443359375, 'before_closest_residue': 748, 'closest_residue': 780, 'next_closest_residue': 748, 'cosine_with_motion': -0.3759469247346106, 'motion_component': -4.2028382551803}, {'ion': 1309, 'force': [-0.7276131510734558, -8.576908111572266, 12.734542846679688], 'magnitude': 15.370795249938965, 'distance': 4.647515773773193, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 130, 'cosine_with_motion': 0.23737887367365, 'motion_component': 3.648702129922416}, {'ion': 1320, 'force': [2.105349540710449, -1.2945811748504639, 0.18129947781562805], 'magnitude': 2.478165864944458, 'distance': 11.574542999267578, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.8006204730018646, 'motion_component': -1.984070416350552}, {'ion': 2434, 'force': [1.0735446214675903, -0.11892910301685333, -2.175081729888916], 'magnitude': 2.428502082824707, 'distance': 11.692296028137207, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6215390624157976, 'motion_component': -1.5094089525808843}, {'ion': 2436, 'force': [4.126889228820801, -0.680524468421936, -4.327836513519287], 'magnitude': 6.018678665161133, 'distance': 7.427085876464844, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8201429451411554, 'motion_component': -4.93617713739299}]}, 5356: {'frame': 5356, 'ionic_force': [7.467401668429375, -6.617893993854523, -8.658861584961414], 'ionic_force_magnitude': 13.211150310971338, 'motion_vector': [-5.566600799560547, -5.137775421142578, 0.14322662353515625], 'cosine_ionic_motion': -0.08798602614629404, 'ionic_motion_component': -1.1623966166837447, 'ionic_force_x': 7.467401668429375, 'ionic_force_y': -6.617893993854523, 'ionic_force_z': -8.658861584961414, 'radial_force': 9.977906022385538, 'axial_force': -8.658861584961414, 'before_closest_residue': 'SF', 'closest_residue': 130, 'next_closest_residue': 1073, 'contributions': [{'ion': 1306, 'force': [-1.726586937904358, 2.723762273788452, 0.031108908355236053], 'magnitude': 3.225050687789917, 'distance': 10.146138191223145, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.1791871882714379, 'motion_component': -0.5778877426540897}, {'ion': 1309, 'force': [-5.083637714385986, 1.7815605401992798, 4.272593021392822], 'magnitude': 6.875491142272949, 'distance': 6.948917865753174, 'before_closest_residue': 455, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.37927224489761086, 'motion_component': 2.6076830443856958}, {'ion': 1320, 'force': [15.738530158996582, -14.13753890991211, -3.5142836570739746], 'magnitude': 21.44577980041504, 'distance': 3.934577465057373, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.09525757946206342, 'motion_component': -2.042873198654397}, {'ion': 2434, 'force': [-0.2095593959093094, 0.4638260006904602, -2.334017753601074], 'magnitude': 2.3888676166534424, 'distance': 11.788891792297363, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.08568202920856213, 'motion_component': -0.20468302640401867}, {'ion': 2436, 'force': [-1.2513444423675537, 2.5504961013793945, -7.114262104034424], 'magnitude': 7.660523414611816, 'distance': 6.583241939544678, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.12331218202884321, 'motion_component': -0.9446358543236686}]}, 5357: {'frame': 5357, 'ionic_force': [-8.905019342899323, -7.153529971837997, -3.628664266318083], 'ionic_force_magnitude': 11.984972461922863, 'motion_vector': [1.0815353393554688, -1.1651802062988281, 1.2048263549804688], 'cosine_ionic_motion': -0.23708065434814912, 'ionic_motion_component': -2.84140511361722, 'ionic_force_x': -8.905019342899323, 'ionic_force_y': -7.153529971837997, 'ionic_force_z': -3.628664266318083, 'radial_force': 11.42244984910836, 'axial_force': -3.628664266318083, 'before_closest_residue': 130, 'closest_residue': 1073, 'next_closest_residue': 1073, 'contributions': [{'ion': 1306, 'force': [-2.544297695159912, 0.6225996017456055, -0.04454083368182182], 'magnitude': 2.6197452545166016, 'distance': 11.257436752319336, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.6756708779650437, 'motion_component': -1.7700855391522772}, {'ion': 1309, 'force': [-1.7606245279312134, -0.44900551438331604, 1.1280972957611084], 'magnitude': 2.13869309425354, 'distance': 12.459333419799805, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 1105, 'cosine_with_motion': -0.005120338601344486, 'motion_component': -0.010950832851939651}, {'ion': 1320, 'force': [-1.3347965478897095, -6.032811641693115, -0.6402768492698669], 'magnitude': 6.211799621582031, 'distance': 7.310723304748535, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.38853205719115985, 'motion_component': 2.4134832243306086}, {'ion': 2434, 'force': [-0.9485629200935364, -0.36116552352905273, -1.7239831686019897], 'magnitude': 2.000582456588745, 'distance': 12.882223129272461, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6721193525377495, 'motion_component': -1.344630176815933}, {'ion': 2436, 'force': [-2.316737651824951, -0.9331468939781189, -2.3479607105255127], 'magnitude': 3.427966594696045, 'distance': 9.84126091003418, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6211325241080135, 'motion_component': -2.129221633842434}]}, 5358: {'frame': 5358, 'ionic_force': [-11.324523270130157, -9.701948136091232, -1.8851598501205444], 'ionic_force_magnitude': 15.030850028911543, 'motion_vector': [-0.13986587524414062, 0.56707763671875, 0.13983154296875], 'cosine_ionic_motion': -0.463206567748584, 'ionic_motion_component': -6.96238845223582, 'ionic_force_x': -11.324523270130157, 'ionic_force_y': -9.701948136091232, 'ionic_force_z': -1.8851598501205444, 'radial_force': 14.912163656932, 'axial_force': -1.8851598501205444, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'contributions': [{'ion': 1306, 'force': [-2.950573682785034, 0.41228511929512024, 0.27555233240127563], 'magnitude': 2.9919545650482178, 'distance': 10.533956527709961, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.3812197736169768, 'motion_component': 1.1405923085798113}, {'ion': 1309, 'force': [-2.585419178009033, -2.5263538360595703, 2.679021120071411], 'magnitude': 4.499334335327148, 'distance': 8.590034484863281, 'before_closest_residue': 780, 'closest_residue': 1105, 'next_closest_residue': 780, 'cosine_with_motion': -0.2577219996351968, 'motion_component': -1.1595774628844175}, {'ion': 1320, 'force': [-1.769490361213684, -4.937245845794678, 0.018840014934539795], 'magnitude': 5.244792461395264, 'distance': 7.956185340881348, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.8094466141356852, 'motion_component': -4.245379473738665}, {'ion': 2434, 'force': [-0.9104146361351013, -0.6412608623504639, -1.7891393899917603], 'magnitude': 2.107389450073242, 'distance': 12.551528930664062, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.3843774113266263, 'motion_component': -0.8100328801187882}, {'ion': 2436, 'force': [-3.1086254119873047, -2.0093727111816406, -3.0694339275360107], 'magnitude': 4.808591842651367, 'distance': 8.309216499328613, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.39262866442624267, 'motion_component': -1.887990983593486}]}, 5359: {'frame': 5359, 'ionic_force': [-10.53284615278244, -8.8823823928833, -3.6715437918901443], 'ionic_force_magnitude': 14.25895504121372, 'motion_vector': [-0.3754844665527344, 0.34723663330078125, 0.0055084228515625], 'cosine_ionic_motion': 0.11660758817000877, 'ionic_motion_component': 1.66270235718052, 'ionic_force_x': -10.53284615278244, 'ionic_force_y': -8.8823823928833, 'ionic_force_z': -3.6715437918901443, 'radial_force': 13.778155357361417, 'axial_force': -3.6715437918901443, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'contributions': [{'ion': 1306, 'force': [-3.0441882610321045, 0.7864692211151123, 0.17377707362174988], 'magnitude': 3.1489386558532715, 'distance': 10.268025398254395, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.8798769350281354, 'motion_component': 2.7706784675866705}, {'ion': 1309, 'force': [-3.55322265625, -1.968692660331726, 0.8038131594657898], 'magnitude': 4.140924453735352, 'distance': 8.95406723022461, 'before_closest_residue': 1105, 'closest_residue': 780, 'next_closest_residue': 455, 'cosine_with_motion': 0.3092681448214228, 'motion_component': 1.2806561095230804}, {'ion': 1320, 'force': [-0.5556600689888, -5.521777629852295, -0.23913930356502533], 'magnitude': 5.554815292358398, 'distance': 7.730974197387695, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.6018995063443169, 'motion_component': -3.3434406354042325}, {'ion': 2434, 'force': [-0.9361525774002075, -0.5566215515136719, -1.8760818243026733], 'magnitude': 2.169306993484497, 'distance': 12.37110710144043, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.133298819524226, 'motion_component': 0.2891660423462572}, {'ion': 2436, 'force': [-2.443622589111328, -1.6217597723007202, -2.5339128971099854], 'magnitude': 3.8758368492126465, 'distance': 9.255210876464844, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.1717416192223846, 'motion_component': 0.6656424831540266}]}, 5360: {'frame': 5360, 'ionic_force': [-9.028356164693832, -11.008867591619492, -3.8418196588754654], 'ionic_force_magnitude': 14.746727059849487, 'motion_vector': [0.4962959289550781, -1.1936683654785156, -0.0410003662109375], 'cosine_ionic_motion': 0.462310699916301, 'ionic_motion_component': 6.817569708513672, 'ionic_force_x': -9.028356164693832, 'ionic_force_y': -11.008867591619492, 'ionic_force_z': -3.8418196588754654, 'radial_force': 14.23749910224317, 'axial_force': -3.8418196588754654, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'contributions': [{'ion': 1306, 'force': [-3.037724494934082, 1.0906109809875488, 0.26996007561683655], 'magnitude': 3.2388393878936768, 'distance': 10.124517440795898, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.67330393731189, 'motion_component': -2.1807233413795872}, {'ion': 1309, 'force': [-1.7648735046386719, -0.8681292533874512, 0.4014160633087158], 'magnitude': 2.0073769092559814, 'distance': 12.860404014587402, 'before_closest_residue': 780, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': 0.05542519617332915, 'motion_component': 0.11125925468247111}, {'ion': 1320, 'force': [-0.222377210855484, -9.145050048828125, 0.049248531460762024], 'magnitude': 9.147886276245117, 'distance': 6.024328708648682, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 1105, 'cosine_with_motion': 0.9131206022804962, 'motion_component': 8.35312313240585}, {'ion': 2434, 'force': [-0.8280560374259949, -0.4974512755870819, -1.6552377939224243], 'magnitude': 1.91649329662323, 'distance': 13.161803245544434, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.10113794630997673, 'motion_component': 0.1938302006527346}, {'ion': 2436, 'force': [-3.1753249168395996, -1.5888479948043823, -2.9072065353393555], 'magnitude': 4.589005947113037, 'distance': 8.505693435668945, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.074107570812104, 'motion_component': 0.340080087499274}]}, 5361: {'frame': 5361, 'ionic_force': [-7.815921291708946, -18.790564686059952, -0.12370511889457703], 'ionic_force_magnitude': 20.351639978528347, 'motion_vector': [-0.574737548828125, 0.9560508728027344, -0.38732147216796875], 'cosine_ionic_motion': -0.5586194842637767, 'ionic_motion_component': -11.368822628727566, 'ionic_force_x': -7.815921291708946, 'ionic_force_y': -18.790564686059952, 'ionic_force_z': -0.12370511889457703, 'radial_force': 20.351264011338277, 'axial_force': -0.12370511889457703, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'contributions': [{'ion': 1306, 'force': [-2.695746898651123, 0.2362404763698578, 0.13357296586036682], 'magnitude': 2.7093729972839355, 'distance': 11.069668769836426, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.5386975741727908, 'motion_component': 1.4595327211185432}, {'ion': 1309, 'force': [-1.4405096769332886, -0.9803712368011475, 0.35021817684173584], 'magnitude': 1.7773150205612183, 'distance': 13.667428970336914, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': -0.1167459297738805, 'motion_component': -0.2074942939315676}, {'ion': 1320, 'force': [0.1950037032365799, -15.115640640258789, 4.1602349281311035], 'magnitude': 15.678908348083496, 'distance': 4.601624011993408, 'before_closest_residue': 98, 'closest_residue': 1105, 'next_closest_residue': 1105, 'cosine_with_motion': -0.8736388570428829, 'motion_component': -13.69770373827267}, {'ion': 2434, 'force': [-0.9663851857185364, -0.6437287330627441, -2.0172598361968994], 'magnitude': 2.3275790214538574, 'distance': 11.943093299865723, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.2624381036375999, 'motion_component': 0.6108454331708925}, {'ion': 2436, 'force': [-2.908283233642578, -2.287064552307129, -2.750471353530884], 'magnitude': 4.610191822052002, 'distance': 8.486127853393555, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.10107972759484486, 'motion_component': 0.4659969298493891}]}, 5362: {'frame': 5362, 'ionic_force': [-5.433648765087128, -16.242994844913483, 4.414413258433342], 'ionic_force_magnitude': 17.68746632082874, 'motion_vector': [0.4037361145019531, -0.2184600830078125, -0.226226806640625], 'cosine_ionic_motion': 0.039331868497438374, 'ionic_motion_component': 0.6956810993837061, 'ionic_force_x': -5.433648765087128, 'ionic_force_y': -16.242994844913483, 'ionic_force_z': 4.414413258433342, 'radial_force': 17.127738333890406, 'axial_force': 4.414413258433342, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'contributions': [{'ion': 1306, 'force': [-3.100250244140625, 0.8727033138275146, 0.33708640933036804], 'magnitude': 3.2383313179016113, 'distance': 10.125311851501465, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.9163193481452945, 'motion_component': -2.9673456667900666}, {'ion': 1309, 'force': [-1.5750622749328613, -0.9575368165969849, 0.24507339298725128], 'magnitude': 1.8595050573349, 'distance': 13.361966133117676, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 423, 'cosine_with_motion': -0.5066735521869951, 'motion_component': -0.9421620101963059}, {'ion': 1320, 'force': [3.2834606170654297, -13.994690895080566, 8.046475410461426], 'magnitude': 16.473562240600586, 'distance': 4.489265441894531, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 1105, 'cosine_with_motion': 0.3039632998783835, 'motion_component': 5.007358344099799}, {'ion': 2434, 'force': [-0.9333657622337341, -0.5060002207756042, -1.6682040691375732], 'magnitude': 1.977400541305542, 'distance': 12.957514762878418, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.1097857354681624, 'motion_component': 0.2170903667758015}, {'ion': 2436, 'force': [-3.108431100845337, -1.6574702262878418, -2.54601788520813], 'magnitude': 4.346465110778809, 'distance': 8.739789009094238, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.14247442357158616, 'motion_component': -0.6192601042226045}]}, 5363: {'frame': 5363, 'ionic_force': [-7.829004019498825, -12.926209926605225, 2.645269814878702], 'ionic_force_magnitude': 15.342022663179213, 'motion_vector': [-0.16725540161132812, -0.3708457946777344, 0.30941009521484375], 'cosine_ionic_motion': 0.8826822518738041, 'ionic_motion_component': 13.542131112633966, 'ionic_force_x': -7.829004019498825, 'ionic_force_y': -12.926209926605225, 'ionic_force_z': 2.645269814878702, 'radial_force': 15.112253538238306, 'axial_force': 2.645269814878702, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'contributions': [{'ion': 1306, 'force': [-3.2139596939086914, 0.8764947652816772, 0.03317352011799812], 'magnitude': 3.331498146057129, 'distance': 9.982728004455566, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.13082922569889527, 'motion_component': 0.4358573341147805}, {'ion': 1309, 'force': [-1.4222971200942993, -1.290872573852539, 0.12278829514980316], 'magnitude': 1.924670934677124, 'distance': 13.133811950683594, 'before_closest_residue': 455, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.7670795510974251, 'motion_component': 1.476375688362606}, {'ion': 1320, 'force': [0.3337534964084625, -10.261008262634277, 7.174679279327393], 'magnitude': 12.525003433227539, 'distance': 5.148492813110352, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 1105, 'cosine_with_motion': 0.9324657304241323, 'motion_component': 11.679136241201018}, {'ion': 2434, 'force': [-0.8723053932189941, -0.5652945041656494, -1.9188066720962524], 'magnitude': 2.182267904281616, 'distance': 12.334314346313477, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.2135258965253157, 'motion_component': -0.4659707309890351}, {'ion': 2436, 'force': [-2.6541953086853027, -1.685529351234436, -2.7665646076202393], 'magnitude': 4.188035488128662, 'distance': 8.903563499450684, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.09950545026923256, 'motion_component': 0.41673236184657725}]}, 5364: {'frame': 5364, 'ionic_force': [-8.431658707559109, -11.04861706495285, 2.1248207800090313], 'ionic_force_magnitude': 14.059860275119481, 'motion_vector': [0.7199592590332031, 0.047824859619140625, -0.00384521484375], 'cosine_ionic_motion': -0.6512600568590633, 'ionic_motion_component': -9.1566254022048, 'ionic_force_x': -8.431658707559109, 'ionic_force_y': -11.04861706495285, 'ionic_force_z': 2.1248207800090313, 'radial_force': 13.898374279343779, 'axial_force': 2.1248207800090313, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'contributions': [{'ion': 1306, 'force': [-3.066877841949463, 0.6862186789512634, 0.2053302526473999], 'magnitude': 3.149412155151367, 'distance': 10.267253875732422, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 780, 'cosine_with_motion': -0.9575443821834538, 'motion_component': -3.015701819420745}, {'ion': 1309, 'force': [-1.2786661386489868, -1.378605604171753, 0.06221873685717583], 'magnitude': 1.8813323974609375, 'distance': 13.284226417541504, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.7269007740173844, 'motion_component': -1.3675419927947812}, {'ion': 1320, 'force': [-0.05913498252630234, -7.958459854125977, 6.173501968383789], 'magnitude': 10.072373390197754, 'distance': 5.741206169128418, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 1105, 'cosine_with_motion': -0.061494054302821094, 'motion_component': -0.6193910793836221}, {'ion': 2434, 'force': [-0.9266603589057922, -0.606224775314331, -1.7449246644973755], 'magnitude': 2.0666325092315674, 'distance': 12.674692153930664, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.462342170077388, 'motion_component': -0.9554913652822146}, {'ion': 2436, 'force': [-3.1003193855285645, -1.7915455102920532, -2.571305513381958], 'magnitude': 4.408313274383545, 'distance': 8.678262710571289, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7255607242424008, 'motion_component': -3.198499114070995}]}, 5365: {'frame': 5365, 'ionic_force': [-8.391353130340576, -13.809379696846008, 1.3839904889464378], 'ionic_force_magnitude': 16.218175132956034, 'motion_vector': [-0.7137031555175781, 0.053272247314453125, -0.5380477905273438], 'cosine_ionic_motion': 0.31048079975389636, 'ionic_motion_component': 5.035431985828944, 'ionic_force_x': -8.391353130340576, 'ionic_force_y': -13.809379696846008, 'ionic_force_z': 1.3839904889464378, 'radial_force': 16.159015284655787, 'axial_force': 1.3839904889464378, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'contributions': [{'ion': 1306, 'force': [-3.618155002593994, 1.0749030113220215, 0.35524982213974], 'magnitude': 3.7911295890808105, 'distance': 9.358036041259766, 'before_closest_residue': 748, 'closest_residue': 780, 'next_closest_residue': 748, 'cosine_with_motion': 0.7212868613666649, 'motion_component': 2.734492055708021}, {'ion': 1309, 'force': [-0.9053996205329895, -1.410875916481018, 0.084062360227108], 'magnitude': 1.6785070896148682, 'distance': 14.06395435333252, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.3498541792620414, 'motion_component': 0.5872326946989048}, {'ion': 1320, 'force': [0.3944142460823059, -10.42065715789795, 5.925753593444824], 'magnitude': 11.994174003601074, 'distance': 5.261188507080078, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 1105, 'cosine_with_motion': -0.37478686319241056, 'motion_component': -4.495258911100009}, {'ion': 2434, 'force': [-0.8353512287139893, -0.7200510501861572, -1.9241082668304443], 'magnitude': 2.217764139175415, 'distance': 12.235208511352539, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.8022675846631492, 'motion_component': 1.7792402857389131}, {'ion': 2436, 'force': [-3.426861524581909, -2.3326985836029053, -3.05696702003479], 'magnitude': 5.150719165802002, 'distance': 8.028512954711914, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.8600207886859776, 'motion_component': 4.429725728516766}]}, 5366: {'frame': 5366, 'ionic_force': [-9.92858612537384, -13.66172307729721, 7.323934718966484], 'ionic_force_magnitude': 18.408137321777122, 'motion_vector': [0.0323638916015625, -0.11964035034179688, 0.4410858154296875], 'cosine_ionic_motion': 0.5387287868758152, 'ionic_motion_component': 9.916993488004406, 'ionic_force_x': -9.92858612537384, 'ionic_force_y': -13.66172307729721, 'ionic_force_z': 7.323934718966484, 'radial_force': 16.88844279055121, 'axial_force': 7.323934718966484, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'contributions': [{'ion': 1306, 'force': [-2.773057222366333, 0.35567569732666016, -0.231277197599411], 'magnitude': 2.805323600769043, 'distance': 10.878714561462402, 'before_cl</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>5415</v>
+      </c>
+      <c r="B15" t="n">
+        <v>5433</v>
+      </c>
+      <c r="C15" t="n">
+        <v>2436</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>{5415: {'frame': 5415, 'ionic_force': [-3.694307893514633, 14.67146983742714, -7.464431181550026], 'ionic_force_magnitude': 16.87061560426042, 'motion_vector': [-0.3487205505371094, 3.4752159118652344, 0.6145477294921875], 'cosine_ionic_motion': 0.7970690893810838, 'ionic_motion_component': 13.447046216986154, 'ionic_force_x': -3.694307893514633, 'ionic_force_y': 14.67146983742714, 'ionic_force_z': -7.464431181550026, 'radial_force': 15.129439447732981, 'axial_force': -7.464431181550026, 'before_closest_residue': None, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-2.831329822540283, 2.6498525142669678, -0.15361477434635162], 'magnitude': 3.880946397781372, 'distance': 9.249115943908691, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.7339741185017447, 'motion_component': 2.8485141609403417}, {'ion': 1309, 'force': [-1.2417367696762085, 2.2549033164978027, 3.7121427059173584], 'magnitude': 4.517355442047119, 'distance': 8.572882652282715, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.6585883074501265, 'motion_component': 2.9750776534110397}, {'ion': 1469, 'force': [3.919631004333496, 7.311126232147217, -1.3659437894821167], 'magnitude': 8.407251358032227, 'distance': 6.284084796905518, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.7781850453014673, 'motion_component': 6.542397326645556}, {'ion': 2434, 'force': [-3.1615939140319824, 2.1154823303222656, -7.686925411224365], 'magnitude': 8.576698303222656, 'distance': 6.221698760986328, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.12264335860419856, 'motion_component': 1.0518751575718213}, {'ion': 2444, 'force': [-0.37927839159965515, 0.34010544419288635, -1.9700899124145508], 'magnitude': 2.0348901748657227, 'distance': 12.773165702819824, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.014340683672517583, 'motion_component': 0.0291817164848438}]}, 5416: {'frame': 5416, 'ionic_force': [-4.081433027982712, 10.87008786201477, -3.291440822184086], 'ionic_force_magnitude': 12.068574413565539, 'motion_vector': [-2.1743736267089844, -0.24370956420898438, 0.42597198486328125], 'cosine_ionic_motion': 0.17929564223551642, 'ionic_motion_component': 2.1638428003473544, 'ionic_force_x': -4.081433027982712, 'ionic_force_y': 10.87008786201477, 'ionic_force_z': -3.291440822184086, 'radial_force': 11.611068240684359, 'axial_force': -3.291440822184086, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-1.1908079385757446, 1.3305332660675049, 0.07573240250349045], 'magnitude': 1.7871983051300049, 'distance': 13.629586219787598, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.5766515859184972, 'motion_component': 1.0305907262945522}, {'ion': 1309, 'force': [-1.7372729778289795, 1.9497443437576294, 1.9252551794052124], 'magnitude': 3.244414806365967, 'distance': 10.115814208984375, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 130, 'cosine_with_motion': 0.57002217966702, 'motion_component': 1.849388441445887}, {'ion': 1469, 'force': [1.0098694562911987, 3.874903678894043, -0.12357929348945618], 'magnitude': 4.0062432289123535, 'distance': 9.103331565856934, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.35753160520772975, 'motion_component': -1.432358656018975}, {'ion': 2434, 'force': [-1.7631807327270508, 3.0347986221313477, -3.503937005996704], 'magnitude': 4.959474086761475, 'distance': 8.181844711303711, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.14487779028910183, 'motion_component': 0.7185176510370184}, {'ion': 2444, 'force': [-0.4000408351421356, 0.6801079511642456, -1.6649121046066284], 'magnitude': 1.8424201011657715, 'distance': 13.423776626586914, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.0012458317985159255, 'motion_component': -0.00229534554213906}]}, 5417: {'frame': 5417, 'ionic_force': [-5.814258098602295, 10.77547174692154, -1.0274325460195541], 'ionic_force_magnitude': 12.287066624808661, 'motion_vector': [0.7505950927734375, 1.0793838500976562, -1.4337081909179688], 'cosine_ionic_motion': 0.365659235567866, 'ionic_motion_component': 4.492879389398975, 'ionic_force_x': -5.814258098602295, 'ionic_force_y': 10.77547174692154, 'ionic_force_z': -1.0274325460195541, 'radial_force': 12.244034817243321, 'axial_force': -1.0274325460195541, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-1.2127642631530762, 1.3744667768478394, 0.10965488851070404], 'magnitude': 1.836295247077942, 'distance': 13.446145057678223, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.11647925335625721, 'motion_component': 0.21389030055099933}, {'ion': 1309, 'force': [-1.6386932134628296, 1.689590573310852, 3.3819234371185303], 'magnitude': 4.120368480682373, 'distance': 8.976375579833984, 'before_closest_residue': 780, 'closest_residue': 130, 'next_closest_residue': 130, 'cosine_with_motion': -0.5308672048478624, 'motion_component': -2.187368593057652}, {'ion': 1469, 'force': [0.2765955328941345, 4.555323600769043, -0.1436668336391449], 'magnitude': 4.56597375869751, 'distance': 8.527118682861328, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.6001537030888063, 'motion_component': 2.7402861903056674}, {'ion': 2434, 'force': [-2.509505271911621, 2.4902234077453613, -2.8283956050872803], 'magnitude': 4.527543544769287, 'distance': 8.563232421875, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5517515902465349, 'motion_component': 2.4980793799438032}, {'ion': 2444, 'force': [-0.7298908829689026, 0.6658673882484436, -1.5469484329223633], 'magnitude': 1.8355298042297363, 'distance': 13.448948860168457, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.669012387353238, 'motion_component': 1.227992153000633}]}, 5418: {'frame': 5418, 'ionic_force': [-3.0948960185050964, 8.432614922523499, -0.9114571809768677], 'ionic_force_magnitude': 9.028739114055682, 'motion_vector': [0.6279106140136719, 0.4439239501953125, -0.27136993408203125], 'cosine_ionic_motion': 0.278089260161465, 'ionic_motion_component': 2.510795380418626, 'ionic_force_x': -3.0948960185050964, 'ionic_force_y': 8.432614922523499, 'ionic_force_z': -0.9114571809768677, 'radial_force': 8.982615198088176, 'axial_force': -0.9114571809768677, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-1.2676705121994019, 1.2841308116912842, -0.15775233507156372], 'magnitude': 1.8113162517547607, 'distance': 13.538542747497559, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.12397442968086314, 'motion_component': -0.22455688916636163}, {'ion': 1309, 'force': [-1.2601678371429443, 2.125608205795288, 2.1942358016967773], 'magnitude': 3.3046791553497314, 'distance': 10.023154258728027, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 780, 'cosine_with_motion': -0.1644300780964941, 'motion_component': -0.5433886430388242}, {'ion': 1469, 'force': [0.4336826205253601, 3.54756498336792, -0.8087297081947327], 'magnitude': 3.6643335819244385, 'distance': 9.518566131591797, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.6916117806805393, 'motion_component': 2.5342963743771456}, {'ion': 2434, 'force': [-1.0007402896881104, 1.4753109216690063, -2.1392109394073486], 'magnitude': 2.784644842147827, 'distance': 10.919032096862793, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.26733916725288576, 'motion_component': 0.7444446326850809}]}, 5419: {'frame': 5419, 'ionic_force': [-3.6241090893745422, 8.350408673286438, -1.4899036781862378], 'ionic_force_magnitude': 9.224061181109839, 'motion_vector': [-0.07321548461914062, -1.4095268249511719, 1.3923492431640625], 'cosine_ionic_motion': -0.7425320583510501, 'ionic_motion_component': -6.849161135165507, 'ionic_force_x': -3.6241090893745422, 'ionic_force_y': 8.350408673286438, 'ionic_force_z': -1.4899036781862378, 'radial_force': 9.102938630057029, 'axial_force': -1.4899036781862378, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-1.068015694618225, 1.3272424936294556, 0.00673897098749876], 'magnitude': 1.7036066055297852, 'distance': 13.959966659545898, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.5279510651796915, 'motion_component': -0.899420938797942}, {'ion': 1309, 'force': [-2.2032456398010254, 2.115774631500244, 1.356068730354309], 'magnitude': 3.3421125411987305, 'distance': 9.966863632202148, 'before_closest_residue': 130, 'closest_residue': 780, 'next_closest_residue': 423, 'cosine_with_motion': -0.14077735077576017, 'motion_component': -0.4704937454166113}, {'ion': 1469, 'force': [0.5705264210700989, 3.1289117336273193, -0.7028989195823669], 'magnitude': 3.257246732711792, 'distance': 10.095869064331055, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.8409491019474874, 'motion_component': -2.7391786691732083}, {'ion': 2434, 'force': [-0.9233741760253906, 1.778479814529419, -2.1498124599456787], 'magnitude': 2.9389290809631348, 'distance': 10.628561973571777, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.9323354010550714, 'motion_component': -2.7400675900062055}]}, 5420: {'frame': 5420, 'ionic_force': [-4.995375692844391, 9.29425859451294, -4.6483332216739655], 'ionic_force_magnitude': 11.530135423057965, 'motion_vector': [1.37384033203125, 0.6198310852050781, 1.271148681640625], 'cosine_ionic_motion': -0.3083860954873238, 'ionic_motion_component': -3.5557334435569286, 'ionic_force_x': -4.995375692844391, 'ionic_force_y': 9.29425859451294, 'ionic_force_z': -4.6483332216739655, 'radial_force': 10.551635945877692, 'axial_force': -4.6483332216739655, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-0.9783754944801331, 1.3178855180740356, 0.07299147546291351], 'magnitude': 1.6429754495620728, 'distance': 14.215216636657715, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.1341246890559753, 'motion_component': -0.2203635825066144}, {'ion': 1309, 'force': [-2.296131134033203, 1.0717114210128784, 0.202259823679924], 'magnitude': 2.5419859886169434, 'distance': 11.428321838378906, 'before_closest_residue': 780, 'closest_residue': 423, 'next_closest_residue': 455, 'cosine_with_motion': -0.44556351398937477, 'motion_component': -1.132616194223882}, {'ion': 1469, 'force': [0.5067126154899597, 4.24498176574707, -0.2817506194114685], 'magnitude': 4.2843918800354, 'distance': 8.802873611450195, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.3514901901202061, 'motion_component': 1.505921613751351}, {'ion': 2434, 'force': [-1.693018913269043, 2.0171566009521484, -2.944333791732788], 'magnitude': 3.9502322673797607, 'distance': 9.167643547058105, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6186448965736641, 'motion_component': -2.4437910563266314}, {'ion': 2444, 'force': [-0.5345627665519714, 0.6425232887268066, -1.6975001096725464], 'magnitude': 1.8921153545379639, 'distance': 13.246319770812988, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6685027957609565, 'motion_component': -1.2648843400024923}]}, 5421: {'frame': 5421, 'ionic_force': [-5.303912997245789, 10.99374771118164, -2.734027996659279], 'ionic_force_magnitude': 12.508752571938622, 'motion_vector': [-0.43817138671875, 0.11849594116210938, -1.432342529296875], 'cosine_ionic_motion': 0.4013204451655481, 'ionic_motion_component': 5.020018150636102, 'ionic_force_x': -5.303912997245789, 'ionic_force_y': 10.99374771118164, 'ionic_force_z': -2.734027996659279, 'radial_force': 12.206309098964534, 'axial_force': -2.734027996659279, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-0.9376237988471985, 1.6168675422668457, 0.2334917038679123], 'magnitude': 1.883591651916504, 'distance': 13.276257514953613, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.0946907895215011, 'motion_component': 0.17835877819294144}, {'ion': 1309, 'force': [-3.586841344833374, 1.4117411375045776, 1.6100742816925049], 'magnitude': 4.177413463592529, 'distance': 8.914875984191895, 'before_closest_residue': 423, 'closest_residue': 455, 'next_closest_residue': 780, 'cosine_with_motion': -0.09037177139810013, 'motion_component': -0.377520252610303}, {'ion': 1469, 'force': [1.202595829963684, 3.48968505859375, 0.13294559717178345], 'magnitude': 3.6934826374053955, 'distance': 9.480932235717773, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.05475204072792799, 'motion_component': -0.2022257049529017}, {'ion': 2434, 'force': [-1.507516622543335, 3.459397077560425, -2.9776651859283447], 'magnitude': 4.806924819946289, 'distance': 8.310657501220703, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.7387225120534889, 'motion_component': 3.550983443186361}, {'ion': 2444, 'force': [-0.4745270609855652, 1.0160568952560425, -1.7328743934631348], 'magnitude': 2.0640740394592285, 'distance': 12.682544708251953, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.906179644664221, 'motion_component': 1.8704217850621294}]}, 5422: {'frame': 5422, 'ionic_force': [-4.211169719696045, 10.116018772125244, -4.300447233021259], 'ionic_force_magnitude': 11.771220523381396, 'motion_vector': [0.1480560302734375, -0.8996047973632812, 0.5749053955078125], 'cosine_ionic_motion': -0.961287586761805, 'ionic_motion_component': -11.315528170162334, 'ionic_force_x': -4.211169719696045, 'ionic_force_y': 10.116018772125244, 'ionic_force_z': -4.300447233021259, 'radial_force': 10.957544716133956, 'axial_force': -4.300447233021259, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-0.8739737868309021, 1.613553762435913, -0.04794659465551376], 'magnitude': 1.8356701135635376, 'distance': 13.448433876037598, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.8129816312037785, 'motion_component': -1.4923660909049268}, {'ion': 1309, 'force': [-2.566864252090454, 1.8449293375015259, 0.5315044522285461], 'magnitude': 3.205472469329834, 'distance': 10.17707633972168, 'before_closest_residue': 455, 'closest_residue': 780, 'next_closest_residue': 423, 'cosine_with_motion': -0.501938957417652, 'motion_component': -1.6089514764139317}, {'ion': 1469, 'force': [1.0937838554382324, 3.111398458480835, -0.23599140346050262], 'magnitude': 3.3064868450164795, 'distance': 10.020413398742676, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1105, 'cosine_with_motion': -0.7780253814588048, 'motion_component': -2.572530709600221}, {'ion': 2434, 'force': [-1.3929810523986816, 2.763676643371582, -2.991767168045044], 'magnitude': 4.304529666900635, 'distance': 8.782258033752441, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.9510453856970562, 'motion_component': -4.093803070234479}, {'ion': 2444, 'force': [-0.4711344838142395, 0.7824605703353882, -1.5562465190887451], 'magnitude': 1.8044710159301758, 'distance': 13.564197540283203, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8578010229664738, 'motion_component': -1.5478770422136625}]}, 5423: {'frame': 5423, 'ionic_force': [-8.426977157592773, 12.587924428284168, -3.720699816942215], 'ionic_force_magnitude': 15.598506100091043, 'motion_vector': [-0.2519950866699219, 0.5466041564941406, 0.0637054443359375], 'cosine_ionic_motion': 0.9286137775832735, 'ionic_motion_component': 14.484987674261278, 'ionic_force_x': -8.426977157592773, 'ionic_force_y': 12.587924428284168, 'ionic_force_z': -3.720699816942215, 'radial_force': 15.148260145204256, 'axial_force': -3.720699816942215, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-1.232452630996704, 1.7019360065460205, 0.152567058801651], 'magnitude': 2.106846570968628, 'distance': 12.553146362304688, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.9807032353494604, 'motion_component': 2.0661912233645827}, {'ion': 1309, 'force': [-7.53367280960083, -0.03545748442411423, 1.090088963508606], 'magnitude': 7.612212181091309, 'distance': 6.604099273681641, 'before_closest_residue': 780, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.4229142947215601, 'motion_component': 3.219313426221046}, {'ion': 1469, 'force': [3.078547954559326, 6.243687152862549, 0.9668325781822205], 'magnitude': 7.0282182693481445, 'distance': 6.873001575469971, 'before_closest_residue': 1073, 'closest_residue': 1105, 'next_closest_residue': 1073, 'cosine_with_motion': 0.6343949704708078, 'motion_component': 4.45866631981975}, {'ion': 2434, 'force': [-2.2350199222564697, 3.7992143630981445, -4.083253383636475], 'magnitude': 6.008519172668457, 'distance': 7.4333624839782715, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.654372414694982, 'motion_component': 3.931809165797851}, {'ion': 2444, 'force': [-0.5043797492980957, 0.8785443902015686, -1.8469350337982178], 'magnitude': 2.106515645980835, 'distance': 12.554132461547852, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.3840500646571, 'motion_component': 0.8090074727170524}]}, 5424: {'frame': 5424, 'ionic_force': [-10.658977925777435, 9.611903131008148, -3.6862301863729954], 'ionic_force_magnitude': 14.818595925694929, 'motion_vector': [-1.8115425109863281, -1.1403274536132812, 0.10491180419921875], 'cosine_ionic_motion': 0.2506981698617583, 'ionic_motion_component': 3.714994878492627, 'ionic_force_x': -10.658977925777435, 'ionic_force_y': 9.611903131008148, 'ionic_force_z': -3.6862301863729954, 'radial_force': 14.352786914815354, 'axial_force': -3.6862301863729954, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-0.8292531967163086, 1.547203540802002, 0.13406047224998474], 'magnitude': 1.7605317831039429, 'distance': 13.732420921325684, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.06573620778867038, 'motion_component': -0.1157306777328101}, {'ion': 1309, 'force': [-8.29712200164795, 0.1777876615524292, 0.9536499381065369], 'magnitude': 8.353639602661133, 'distance': 6.30421781539917, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.8338212823493995, 'motion_component': 6.965442263992603}, {'ion': 1469, 'force': [0.7835202217102051, 3.773498058319092, -0.03277162089943886], 'magnitude': 3.854123115539551, 'distance': 9.281245231628418, 'before_closest_residue': 1105, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.6932081742710833, 'motion_component': -2.671709695405911}, {'ion': 2434, 'force': [-1.8014920949935913, 3.1987240314483643, -3.0620651245117188], 'magnitude': 4.7805280685424805, 'distance': 8.33357048034668, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.06884699269022612, 'motion_component': -0.3291250055472901}, {'ion': 2444, 'force': [-0.5146308541297913, 0.914689838886261, -1.6791038513183594], 'magnitude': 1.9801243543624878, 'distance': 12.948599815368652, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.06761305818944655, 'motion_component': -0.13388225810879462}]}, 5425: {'frame': 5425, 'ionic_force': [-8.817112369462848, 4.628080368041992, -5.053674541413784], 'ionic_force_magnitude': 11.16692548552753, 'motion_vector': [0.7701644897460938, 1.122161865234375, -0.6427230834960938], 'cosine_ionic_motion': 0.09822379400640156, 'ionic_motion_component': 1.096857788575292, 'ionic_force_x': -8.817112369462848, 'ionic_force_y': 4.628080368041992, 'ionic_force_z': -5.053674541413784, 'radial_force': 9.957941475465221, 'axial_force': -5.053674541413784, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-1.4571207761764526, 1.3220487833023071, 0.14216242730617523], 'magnitude': 1.972618579864502, 'distance': 12.973211288452148, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.09092287495943208, 'motion_component': 0.17935615330719656}, {'ion': 1309, 'force': [-4.172080993652344, -2.511462926864624, -0.10490787774324417], 'magnitude': 4.87080192565918, 'distance': 8.255983352661133, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.8135006963141567, 'motion_component': -3.9624007676868804}, {'ion': 1469, 'force': [0.024452881887555122, 2.9648444652557373, -0.17231887578964233], 'magnitude': 2.9699485301971436, 'distance': 10.572911262512207, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.77325275445924, 'motion_component': 2.2965209036455843}, {'ion': 2434, 'force': [-2.4676637649536133, 2.1257126331329346, -3.127074718475342], 'magnitude': 4.515153884887695, 'distance': 8.574973106384277, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.36708742493103036, 'motion_component': 1.6574562268455113}, {'ion': 2444, 'force': [-0.7446997165679932, 0.7269374132156372, -1.791535496711731], 'magnitude': 2.0718626976013184, 'distance': 12.658683776855469, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.4469046351630615, 'motion_component': 0.9259250504055956}]}, 5426: {'frame': 5426, 'ionic_force': [-6.718421280384064, 6.112494587898254, -4.578008808195591], 'ionic_force_magnitude': 10.17142759084089, 'motion_vector': [0.9683570861816406, -1.1876640319824219, -1.7886962890625], 'cosine_ionic_motion': -0.23277867905907038, 'ionic_motion_component': -2.367691478740925, 'ionic_force_x': -6.718421280384064, 'ionic_force_y': 6.112494587898254, 'ionic_force_z': -4.578008808195591, 'radial_force': 9.082938653750938, 'axial_force': -4.578008808195591, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 130, 'contributions': [{'ion': 1306, 'force': [-1.0048154592514038, 1.347147822380066, 0.03903442621231079], 'magnitude': 1.681066632270813, 'distance': 14.053243637084961, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.6674565924882243, 'motion_component': -1.1220390114394014}, {'ion': 1309, 'force': [-3.82336688041687, -1.281545877456665, 0.038811035454273224], 'magnitude': 4.032617092132568, 'distance': 9.073514938354492, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 455, 'cosine_with_motion': -0.23686059447804464, 'motion_component': -0.9551680765469284}, {'ion': 1469, 'force': [0.3030494451522827, 3.1069347858428955, -0.22176901996135712], 'magnitude': 3.129547119140625, 'distance': 10.299788475036621, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.40697035549176575, 'motion_component': -1.2736328422891834}, {'ion': 2434, 'force': [-1.6431152820587158, 2.2570924758911133, -2.791811227798462], 'magnitude': 3.948227882385254, 'distance': 9.169970512390137, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.07762936310697147, 'motion_component': 0.306498423729046}, {'ion': 2444, 'force': [-0.5501731038093567, 0.6828653812408447, -1.642274022102356], 'magnitude': 1.8617355823516846, 'distance': 13.353959083557129, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.3634511718692843, 'motion_component': 0.6766499945516973}]}, 5427: {'frame': 5427, 'ionic_force': [-9.343294322490692, 4.070650577545166, -8.845907121896744], 'ionic_force_magnitude': 13.495088652186734, 'motion_vector': [1.9277992248535156, -0.47090911865234375, 1.2962722778320312], 'cosine_ionic_motion': -0.9814844580478329, 'ionic_motion_component': -13.245219772098956, 'ionic_force_x': -9.343294322490692, 'ionic_force_y': 4.070650577545166, 'ionic_force_z': -8.845907121896744, 'radial_force': 10.191533001524137, 'axial_force': -8.845907121896744, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 98, 'contributions': [{'ion': 1306, 'force': [-1.3020676374435425, 1.8560971021652222, -0.37471261620521545], 'magnitude': 2.298017978668213, 'distance': 12.019664764404297, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.7104564841892261, 'motion_component': -1.632641696377048}, {'ion': 1309, 'force': [-7.151926517486572, -4.424306392669678, -2.266660690307617], 'magnitude': 8.709896087646484, 'distance': 6.1739420890808105, 'before_closest_residue': 423, 'closest_residue': 455, 'next_closest_residue': 423, 'cosine_with_motion': -0.7092263629987502, 'motion_component': -6.17728795671141}, {'ion': 1469, 'force': [1.0913169384002686, 4.217013835906982, -1.362021803855896], 'magnitude': 4.563910484313965, 'distance': 8.529046058654785, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.1522963508158204, 'motion_component': -0.6950669595563213}, {'ion': 2434, 'force': [-1.582262396812439, 1.9491033554077148, -3.3685457706451416], 'magnitude': 4.2011494636535645, 'distance': 8.889656066894531, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8369729709418179, 'motion_component': -3.516248744739322}, {'ion': 2444, 'force': [-0.398354709148407, 0.4727426767349243, -1.4739662408828735], 'magnitude': 1.5983580350875854, 'distance': 14.412257194519043, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7657695663854323, 'motion_component': -1.2239739834485697}]}, 5428: {'frame': 5428, 'ionic_force': [-5.052740648388863, 4.340230464935303, -10.841399222612381], 'ionic_force_magnitude': 12.724139485744958, 'motion_vector': [0.24727249145507812, -2.330799102783203, -4.778404235839844], 'cosine_ionic_motion': 0.5971344145129348, 'ionic_motion_component': 7.598021582001231, 'ionic_force_x': -5.052740648388863, 'ionic_force_y': 4.340230464935303, 'ionic_force_z': -10.841399222612381, 'radial_force': 6.660914993349909, 'axial_force': -10.841399222612381, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 130, 'contributions': [{'ion': 1306, 'force': [-1.0390822887420654, 2.3038768768310547, -0.21337798237800598], 'magnitude': 2.5363497734069824, 'distance': 11.441012382507324, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.34129400365784895, 'motion_component': -0.8656410130242884}, {'ion': 1309, 'force': [-4.697807788848877, -6.503828525543213, -1.5563700199127197], 'magnitude': 8.172605514526367, 'distance': 6.373658657073975, 'before_closest_residue': 455, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.49277885349233314, 'motion_component': 4.027286881652531}, {'ion': 1469, 'force': [2.3175904750823975, 4.2220258712768555, -0.8517012596130371], 'magnitude': 4.891024589538574, 'distance': 8.238897323608398, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.19967505294610755, 'motion_component': -0.9766156258850804}, {'ion': 2434, 'force': [-1.4328304529190063, 3.6519341468811035, -6.213566780090332], 'magnitude': 7.3483357429504395, 'distance': 6.7216291427612305, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5324640438268261, 'motion_component': 3.91272456724384}, {'ion': 2444, 'force': [-0.20061059296131134, 0.666222095489502, -2.006383180618286], 'magnitude': 2.123598337173462, 'distance': 12.503536224365234, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.7064737784360602, 'motion_component': 1.5002665511818145}]}, 5429: {'frame': 5429, 'ionic_force': [-1.4938891232013702, 2.3611837029457092, -9.631623983383179], 'ionic_force_magnitude': 10.0287124671494, 'motion_vector': [3.7690887451171875, -2.5068588256835938, -3.2027816772460938], 'cosine_ionic_motion': 0.34702650901315546, 'ionic_motion_component': 3.480229077371566, 'ionic_force_x': -1.4938891232013702, 'ionic_force_y': 2.3611837029457092, 'ionic_force_z': -9.631623983383179, 'radial_force': 2.7940818154584828, 'axial_force': -9.631623983383179, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [-1.4194684028625488, 2.385871410369873, -1.6436631679534912], 'magnitude': 3.226282835006714, 'distance': 10.144200325012207, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.3391182227344014, 'motion_component': -1.0940913331980795}, {'ion': 1309, 'force': [-1.8123735189437866, -2.4131195545196533, -2.5620484352111816], 'magnitude': 3.9587795734405518, 'distance': 9.15774154663086, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 455, 'cosine_with_motion': 0.3381963958982721, 'motion_component': 1.3388449937113478}, {'ion': 1469, 'force': [1.9238256216049194, 2.0180952548980713, -2.4386179447174072], 'magnitude': 3.7041423320770264, 'distance': 9.467279434204102, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.4869727291469073, 'motion_component': 1.803816336372222}, {'ion': 2434, 'force': [-0.18587282299995422, 0.3703365921974182, -2.9872944355010986], 'magnitude': 3.0158956050872803, 'distance': 10.492063522338867, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.4747044569942231, 'motion_component': 1.431659057345513}]}, 5430: {'frame': 5430, 'ionic_force': [2.1646444126963615, 0.24572302401065826, -6.06149160861969], 'ionic_force_magnitude': 6.441098179605201, 'motion_vector': [-0.60418701171875, 0.23330307006835938, 2.4262313842773438], 'cosine_ionic_motion': -0.9865399986875489, 'ionic_motion_component': -6.354400989654089, 'ionic_force_x': 2.1646444126963615, 'ionic_force_y': 0.24572302401065826, 'ionic_force_z': -6.06149160861969, 'radial_force': 2.1785465884269075, 'axial_force': -6.06149160861969, 'before_closest_residue': 130, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [-0.31000417470932007, 2.013558864593506, -2.840615749359131], 'magnitude': 3.495657205581665, 'distance': 9.745511054992676, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>5477</v>
+      </c>
+      <c r="B16" t="n">
+        <v>6017</v>
+      </c>
+      <c r="C16" t="n">
+        <v>2434</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>{5477: {'frame': 5477, 'ionic_force': [-0.44713205099105835, -1.720797836780548, -10.73732876777649], 'ionic_force_magnitude': 10.883533494844983, 'motion_vector': [-0.5623664855957031, 0.9072761535644531, 0.3484649658203125], 'cosine_ionic_motion': -0.41334270206300877, 'ionic_motion_component': -4.4986291427524865, 'ionic_force_x': -0.44713205099105835, 'ionic_force_y': -1.720797836780548, 'ionic_force_z': -10.73732876777649, 'radial_force': 1.7779404562842043, 'axial_force': -10.73732876777649, 'before_closest_residue': None, 'closest_residue': 130, 'next_closest_residue': 130, 'contributions': [{'ion': 1306, 'force': [-1.8695889711380005, 2.9205055236816406, -1.3217833042144775], 'magnitude': 3.71104097366333, 'distance': 9.458476066589355, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.7776565697684376, 'motion_component': 2.8859155436734625}, {'ion': 1309, 'force': [-0.14590446650981903, -7.744018077850342, -4.193130970001221], 'magnitude': 8.807579040527344, 'distance': 6.1396098136901855, 'before_closest_residue': 423, 'closest_residue': 130, 'next_closest_residue': 98, 'cosine_with_motion': -0.8498765392041681, 'motion_component': -7.485354932675172}, {'ion': 1469, 'force': [1.5043941736221313, 2.458629608154297, -1.5455207824707031], 'magnitude': 3.270580291748047, 'distance': 10.075268745422363, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.23038555492130164, 'motion_component': 0.753494470362682}, {'ion': 2444, 'force': [0.06396721303462982, 0.6440851092338562, -3.676893711090088], 'magnitude': 3.7334280014038086, 'distance': 9.430074691772461, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.174821671211077, 'motion_component': -0.6526841261401124}]}, 5478: {'frame': 5478, 'ionic_force': [1.7842273004353046, -1.3310573995113373, -13.13483214378357], 'ionic_force_magnitude': 13.322124316556373, 'motion_vector': [5.6822967529296875, -1.4546623229980469, 1.581939697265625], 'cosine_ionic_motion': -0.10754218376397533, 'ionic_motion_component': -1.4326903413776297, 'ionic_force_x': 1.7842273004353046, 'ionic_force_y': -1.3310573995113373, 'ionic_force_z': -13.13483214378357, 'radial_force': 2.226023553427173, 'axial_force': -13.13483214378357, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [-1.9984097480773926, 2.8898801803588867, -1.3281662464141846], 'magnitude': 3.756204843521118, 'distance': 9.401440620422363, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.7739222944329999, 'motion_component': -2.907010643008448}, {'ion': 1309, 'force': [2.848625421524048, -7.680440902709961, -5.491806507110596], 'magnitude': 9.862239837646484, 'distance': 5.802047252655029, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.311636488808021, 'motion_component': 3.073433847690566}, {'ion': 1469, 'force': [1.1187093257904053, 2.1294939517974854, -1.1434855461120605], 'magnitude': 2.663421392440796, 'distance': 11.164752006530762, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.08962698302468124, 'motion_component': 0.23871443615680477}, {'ion': 2443, 'force': [-0.03920864686369896, 0.29816392064094543, -1.4478132724761963], 'magnitude': 1.478716492652893, 'distance': 14.983959197998047, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.3280365163349735, 'motion_component': -0.48507299002336723}, {'ion': 2444, 'force': [-0.14548905193805695, 1.0318454504013062, -3.7235605716705322], 'magnitude': 3.8666231632232666, 'distance': 9.266230583190918, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.34985431505545295, 'motion_component': -1.3527548319276432}]}, 5479: {'frame': 5479, 'ionic_force': [8.564183592796326, 7.061019524931908, -8.43285158276558], 'ionic_force_magnitude': 13.939735404933026, 'motion_vector': [-0.8315162658691406, 0.4536933898925781, 0.4904327392578125], 'cosine_ionic_motion': -0.5416253131713804, 'ionic_motion_component': -7.55011355422303, 'ionic_force_x': 8.564183592796326, 'ionic_force_y': 7.061019524931908, 'ionic_force_z': -8.43285158276558, 'radial_force': 11.099695371612295, 'axial_force': -8.43285158276558, 'before_closest_residue': 130, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [0.8983935117721558, 7.096762180328369, -1.9228250980377197], 'magnitude': 7.407320976257324, 'distance': 6.694813251495361, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.19360576957130374, 'motion_component': 1.434100034401105}, {'ion': 1309, 'force': [2.8427734375, -2.1192972660064697, -0.8717526197433472], 'magnitude': 3.6514017581939697, 'distance': 9.535407066345215, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.963547918868339, 'motion_component': -3.518300505546865}, {'ion': 1469, 'force': [1.5580865144729614, 1.1739774942398071, -0.4098491966724396], 'magnitude': 1.9934475421905518, 'distance': 12.905256271362305, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.4533369941770629, 'motion_component': -0.9037035172938319}, {'ion': 2443, 'force': [0.5962351560592651, 0.1816510409116745, -1.6120604276657104], 'magnitude': 1.7283612489700317, 'distance': 13.859634399414062, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6530594455283119, 'motion_component': -1.1287225779949241}, {'ion': 2444, 'force': [2.6686949729919434, 0.7279260754585266, -3.6163642406463623], 'magnitude': 4.553009986877441, 'distance': 8.539250373840332, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7541136132982074, 'motion_component': -3.433486780340937}]}, 5480: {'frame': 5480, 'ionic_force': [8.845621451735497, 5.174365371465683, -6.945133060216904], 'ionic_force_magnitude': 12.379577904312578, 'motion_vector': [-2.4467201232910156, 2.9426307678222656, 1.0514373779296875], 'cosine_ionic_motion': -0.27922766908566493, 'ionic_motion_component': -3.456720682485602, 'ionic_force_x': 8.845621451735497, 'ionic_force_y': 5.174365371465683, 'ionic_force_z': -6.945133060216904, 'radial_force': 10.247881530581157, 'axial_force': -6.945133060216904, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 423, 'contributions': [{'ion': 1306, 'force': [0.21233676373958588, 5.167843818664551, -0.9647490382194519], 'magnitude': 5.261410236358643, 'distance': 7.943610668182373, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.654805013476343, 'motion_component': 3.4451977799912146}, {'ion': 1309, 'force': [4.6044087409973145, -2.470323085784912, -0.8643374443054199], 'magnitude': 5.296239852905273, 'distance': 7.917448043823242, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.9250340582306482, 'motion_component': -4.899202125768213}, {'ion': 1469, 'force': [1.6390438079833984, 1.4995357990264893, -0.4266315996646881], 'magnitude': 2.2620978355407715, 'distance': 12.11471939086914, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.005154729957164885, 'motion_component': -0.011660503617133777}, {'ion': 2443, 'force': [0.6318773031234741, 0.20215561985969543, -1.57472562789917], 'magnitude': 1.708770513534546, 'distance': 13.938857078552246, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.38439987659516817, 'motion_component': -0.6568511695921728}, {'ion': 2444, 'force': [1.7579548358917236, 0.7751532196998596, -3.114689350128174], 'magnitude': 3.6595845222473145, 'distance': 9.524741172790527, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.36457819253244267, 'motion_component': -1.334204640375063}]}, 5481: {'frame': 5481, 'ionic_force': [10.121144622564316, 6.428409576416016, -5.320772521197796], 'ionic_force_magnitude': 13.11764606838259, 'motion_vector': [1.9404220581054688, -4.451213836669922, 0.8924026489257812], 'cosine_ionic_motion': -0.21189854349301115, 'ionic_motion_component': -2.779610095947095, 'ionic_force_x': 10.121144622564316, 'ionic_force_y': 6.428409576416016, 'ionic_force_z': -5.320772521197796, 'radial_force': 11.990079989433752, 'axial_force': -5.320772521197796, 'before_closest_residue': 455, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1306, 'force': [-0.6012338399887085, 2.818525791168213, -0.07370224595069885], 'magnitude': 2.882880926132202, 'distance': 10.731383323669434, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.9680474829339109, 'motion_component': -2.790765515449601}, {'ion': 1309, 'force': [8.690352439880371, -0.589633584022522, -0.05870877951383591], 'magnitude': 8.710530281066895, 'distance': 6.173717498779297, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.45193035456920416, 'motion_component': 3.9365530964176982}, {'ion': 1469, 'force': [0.9652875065803528, 1.5830146074295044, -0.20551034808158875], 'magnitude': 1.865462303161621, 'distance': 13.34061336517334, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.5816164448618182, 'motion_component': -1.0849835709259943}, {'ion': 2443, 'force': [0.3752489387989044, 0.6354923248291016, -1.8373764753341675], 'magnitude': 1.9800541400909424, 'distance': 12.948829650878906, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.3826061510855403, 'motion_component': -0.757580910428099}, {'ion': 2444, 'force': [0.691489577293396, 1.9810104370117188, -3.145474672317505], 'magnitude': 3.781080722808838, 'distance': 9.370463371276855, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5508565617056489, 'motion_component': -2.0828331023756945}]}, 5482: {'frame': 5482, 'ionic_force': [10.774185962509364, 7.967799760401249, -6.948080446571112], 'ionic_force_magnitude': 15.094526758683356, 'motion_vector': [-3.371776580810547, 2.4830093383789062, -2.777191162109375], 'cosine_ionic_motion': 0.03628633384766448, 'ionic_motion_component': 0.5477250372380891, 'ionic_force_x': 10.774185962509364, 'ionic_force_y': 7.967799760401249, 'ionic_force_z': -6.948080446571112, 'radial_force': 13.400332689026195, 'axial_force': -6.948080446571112, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 130, 'contributions': [{'ion': 1306, 'force': [0.0029737423174083233, 8.807312965393066, 1.0229673385620117], 'magnitude': 8.866522789001465, 'distance': 6.119167804718018, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.4268726062393223, 'motion_component': 3.7848758433912693}, {'ion': 1309, 'force': [2.8360345363616943, -2.8020989894866943, 0.3442707359790802], 'magnitude': 4.001671314239502, 'distance': 9.10853099822998, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.8691628231816363, 'motion_component': -3.4781039011742347}, {'ion': 1469, 'force': [2.137364387512207, 1.547278881072998, -0.054249223321676254], 'magnitude': 2.639193296432495, 'distance': 11.215882301330566, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.24237600744025303, 'motion_component': -0.6396771424608481}, {'ion': 2443, 'force': [0.930376410484314, 0.07820767909288406, -2.1504712104797363], 'magnitude': 2.344406843185425, 'distance': 11.900153160095215, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.25717236860653303, 'motion_component': 0.6029166436709448}, {'ion': 2444, 'force': [4.86743688583374, 0.33709922432899475, -6.110598087310791], 'magnitude': 7.819525718688965, 'distance': 6.515966415405273, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.035515385916932506, 'motion_component': 0.2777134832245567}]}, 5483: {'frame': 5483, 'ionic_force': [13.281899441033602, -1.611535370349884, -14.18665498495102], 'ionic_force_magnitude': 19.500437909792, 'motion_vector': [-1.0512886047363281, -1.1198539733886719, -3.1050186157226562], 'cosine_ionic_motion': 0.47209675845205223, 'ionic_motion_component': 9.206093525608317, 'ionic_force_x': 13.281899441033602, 'ionic_force_y': -1.611535370349884, 'ionic_force_z': -14.18665498495102, 'radial_force': 13.379308614858147, 'axial_force': -14.18665498495102, 'before_closest_residue': 423, 'closest_residue': 130, 'next_closest_residue': 130, 'contributions': [{'ion': 1306, 'force': [-1.4231153726577759, 3.2190465927124023, -0.5271512866020203], 'magnitude': 3.5588490962982178, 'distance': 9.658601760864258, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.038280827770216845, 'motion_component': -0.13623568887828696}, {'ion': 1309, 'force': [12.95172119140625, -9.656329154968262, -6.279929161071777], 'magnitude': 17.332895278930664, 'distance': 4.376565933227539, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.27807920582061574, 'motion_component': 4.819917962997209}, {'ion': 1469, 'force': [1.47786545753479, 2.6548736095428467, -0.7496045827865601], 'magnitude': 3.129592180252075, 'distance': 10.299714088439941, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.20285152649453522, 'motion_component': -0.6348425513631568}, {'ion': 2443, 'force': [0.023254413157701492, 0.36658936738967896, -1.7489255666732788], 'magnitude': 1.7870839834213257, 'distance': 13.630022048950195, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.8069254149980343, 'motion_component': 1.4420434863079719}, {'ion': 2444, 'force': [0.2521737515926361, 1.8042842149734497, -4.881044387817383], 'magnitude': 5.209954738616943, 'distance': 7.982741832733154, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.7130983805644391, 'motion_component': 3.7152102230572357}]}, 5484: {'frame': 5484, 'ionic_force': [2.082847408950329, 0.5381690561771393, -11.26388955116272], 'ionic_force_magnitude': 11.467479543595898, 'motion_vector': [-1.2701416015625, -1.1113739013671875, -2.5788192749023438], 'cosine_ionic_motion': 0.730104621679469, 'ionic_motion_component': 8.372459813794134, 'ionic_force_x': 2.082847408950329, 'ionic_force_y': 0.5381690561771393, 'ionic_force_z': -11.26388955116272, 'radial_force': 2.151250627425287, 'axial_force': -11.26388955116272, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 130, 'contributions': [{'ion': 1306, 'force': [-1.2755056619644165, 2.3901894092559814, -1.6815731525421143], 'magnitude': 3.188668727874756, 'distance': 10.203856468200684, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.3358087175494165, 'motion_component': 1.0707827623608317}, {'ion': 1309, 'force': [2.1952145099639893, -4.486453056335449, -5.257387638092041], 'magnitude': 7.251713752746582, 'distance': 6.766260623931885, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.7049620782123642, 'motion_component': 5.112183207305485}, {'ion': 1469, 'force': [1.2880535125732422, 2.27970814704895, -1.8271305561065674], 'magnitude': 3.1928915977478027, 'distance': 10.19710636138916, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.05510102667779303, 'motion_component': 0.17593160856745982}, {'ion': 2444, 'force': [-0.12491495162248611, 0.35472455620765686, -2.497798204421997], 'magnitude': 2.5259511470794678, 'distance': 11.46453857421875, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.7971501673219711, 'motion_component': 2.0135623682589534}]}, 5485: {'frame': 5485, 'ionic_force': [0.2769479751586914, 0.9982298463582993, -7.456764340400696], 'ionic_force_magnitude': 7.528379469406177, 'motion_vector': [4.385654449462891, -1.0877685546875, 2.3917007446289062], 'cosine_ionic_motion': -0.4600208106524478, 'ionic_motion_component': -3.4632112264154746, 'ionic_force_x': 0.2769479751586914, 'ionic_force_y': 0.9982298463582993, 'ionic_force_z': -7.456764340400696, 'radial_force': 1.0359358122514217, 'axial_force': -7.456764340400696, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 780, 'contributions': [{'ion': 1306, 'force': [-1.2062158584594727, 1.471609354019165, -1.7157915830612183], 'magnitude': 2.562134027481079, 'distance': 11.38329792022705, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.8393462507593696, 'motion_component': -2.1505177159951145}, {'ion': 1309, 'force': [0.5064878463745117, -2.087893009185791, -3.4851157665252686], 'magnitude': 4.094125270843506, 'distance': 9.005099296569824, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.18359875780452614, 'motion_component': -0.7516762541344804}, {'ion': 1469, 'force': [0.7889192700386047, 1.6113115549087524, -1.897242546081543], 'magnitude': 2.611177444458008, 'distance': 11.275890350341797, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.21202473408075306, 'motion_component': -0.5536342103565328}, {'ion': 2436, 'force': [0.3979494571685791, -0.12599879503250122, 1.4812759160995483], 'magnitude': 1.538966417312622, 'distance': 14.687723159790039, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.6895196838728914, 'motion_component': 1.0611476762695622}, {'ion': 2444, 'force': [-0.2101927399635315, 0.129200741648674, -1.8398903608322144], 'magnitude': 1.8563593626022339, 'distance': 13.373282432556152, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5756054760786232, 'motion_component': -1.0685306575260782}]}, 5486: {'frame': 5486, 'ionic_force': [3.3664588928222656, 2.9159571398049593, -8.914527297019958], 'ionic_force_magnitude': 9.965171772104863, 'motion_vector': [-1.728607177734375, 5.325992584228516, 4.6172027587890625], 'cosine_ionic_motion': -0.434840541839197, 'ionic_motion_component': -4.3332606929027495, 'ionic_force_x': 3.3664588928222656, 'ionic_force_y': 2.9159571398049593, 'ionic_force_z': -8.914527297019958, 'radial_force': 4.453745785093894, 'axial_force': -8.914527297019958, 'before_closest_residue': 130, 'closest_residue': 780, 'next_closest_residue': 455, 'contributions': [{'ion': 1306, 'force': [-0.8589418530464172, 4.029123783111572, -3.341933012008667], 'magnitude': 5.304727554321289, 'distance': 7.911111354827881, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.19515705116594398, 'motion_component': 1.035255012450767}, {'ion': 1309, 'force': [2.1206986904144287, -2.4510836601257324, -1.6197460889816284], 'magnitude': 3.623361825942993, 'distance': 9.57223129272461, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.9202215468575357, 'motion_component': -3.334295689758271}, {'ion': 1469, 'force': [1.5200526714324951, 1.3517338037490845, -1.3707325458526611], 'magnitude': 2.4528865814208984, 'distance': 11.634034156799316, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1105, 'cosine_with_motion': -0.098707559429281, 'motion_component': -0.24211843857373339}, {'ion': 2444, 'force': [0.584649384021759, -0.01381678692996502, -2.582115650177002], 'magnitude': 2.6475133895874023, 'distance': 11.19824504852295, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6769000204594124, 'motion_component': -1.7921018533477944}]}, 5487: {'frame': 5487, 'ionic_force': [14.640848532319069, 6.408383667469025, -6.467983774840832], 'ionic_force_magnitude': 17.24113224493674, 'motion_vector': [0.3015022277832031, -3.9131088256835938, 0.8899307250976562], 'cosine_ionic_motion': -0.380757123972371, 'ionic_motion_component': -6.564683927609421, 'ionic_force_x': 14.640848532319069, 'ionic_force_y': 6.408383667469025, 'ionic_force_z': -6.467983774840832, 'radial_force': 15.981921879917733, 'axial_force': -6.467983774840832, 'before_closest_residue': 780, 'closest_residue': 455, 'next_closest_residue': 'SF', 'contributions': [{'ion': 1306, 'force': [-0.8415454030036926, 2.4747672080993652, -0.05607883632183075], 'magnitude': 2.614539384841919, 'distance': 11.268638610839844, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.9492363714774793, 'motion_component': -2.481815886121387}, {'ion': 1309, 'force': [13.761055946350098, -2.1138620376586914, -0.08146259933710098], 'magnitude': 13.922704696655273, 'distance': 4.883230686187744, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 130, 'cosine_with_motion': 0.22038793154140668, 'motion_component': 3.068396117715446}, {'ion': 1469, 'force': [0.9084755182266235, 1.9054216146469116, -0.2553384602069855], 'magnitude': 2.1263012886047363, 'distance': 12.495586395263672, 'before_closest_residue': 1073, 'closest_residue': 1105, 'next_closest_residue': 1073, 'cosine_with_motion': -0.8658976507435727, 'motion_component': -1.8411592612795076}, {'ion': 2443, 'force': [0.1551320105791092, 0.6592459082603455, -1.8346444368362427], 'magnitude': 1.9556562900543213, 'distance': 13.029350280761719, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5292905712008917, 'motion_component': -1.0351104068303}, {'ion': 2444, 'force': [0.6577304601669312, 3.4828109741210938, -4.240459442138672], 'magnitude': 5.526669979095459, 'distance': 7.750635147094727, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7735209358664246, 'motion_component': -4.274994714874654}]}, 5491: {'frame': 5491, 'ionic_force': [-0.4789837822318077, 1.569911241531372, -13.855378150939941], 'ionic_force_magnitude': 13.952259690654829, 'motion_vector': [0.054042816162109375, 6.2353515625, 0.45986175537109375], 'cosine_ionic_motion': 0.03887700197206414, 'ionic_motion_component': 0.5424220275083388, 'ionic_force_x': -0.4789837822318077, 'ionic_force_y': 1.569911241531372, 'ionic_force_z': -13.855378150939941, 'radial_force': 1.6413551626408167, 'axial_force': -13.855378150939941, 'before_closest_residue': 'SF', 'closest_residue': 780, 'next_closest_residue': 130, 'contributions': [{'ion': 1306, 'force': [-4.010654926300049, 4.951197147369385, -4.815889835357666], 'magnitude': 7.987020969390869, 'distance': 6.447281360626221, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.5695160329648224, 'motion_component': 4.5487363932602385}, {'ion': 1309, 'force': [0.08836428076028824, -4.612890720367432, -2.9233412742614746], 'magnitude': 5.461913108825684, 'distance': 7.796445369720459, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.8814617600389186, 'motion_component': -4.814467416335644}, {'ion': 1469, 'force': [3.120267152786255, 1.8323882818222046, -2.4592511653900146], 'magnitude': 4.375114917755127, 'distance': 8.711126327514648, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.3824934866218572, 'motion_component': 1.6734529448831683}, {'ion': 2444, 'force': [0.323039710521698, -0.6007834672927856, -3.656895875930786], 'magnitude': 3.719970941543579, 'distance': 9.44711685180664, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.23260932244380778, 'motion_component': -0.865299891166011}]}, 5492: {'frame': 5492, 'ionic_force': [6.9292623698711395, 0.5161893367767334, -12.308781921863556], 'ionic_force_magnitude': 14.134611449272644, 'motion_vector': [2.7979888916015625, 1.0762748718261719, 3.96209716796875], 'cosine_ionic_motion': -0.41045585284262676, 'ionic_motion_component': -5.801633997010359, 'ionic_force_x': 6.9292623698711395, 'ionic_force_y': 0.5161893367767334, 'ionic_force_z': -12.308781921863556, 'radial_force': 6.9484623062886515, 'axial_force': -12.308781921863556, 'before_closest_residue': 780, 'closest_residue': 130, 'next_closest_residue': 423, 'contributions': [{'ion': 1306, 'force': [-0.46328631043434143, 1.9176650047302246, -0.6137864589691162], 'magnitude': 2.0661091804504395, 'distance': 12.676297187805176, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.1621202431939229, 'motion_component': -0.3349581207391008}, {'ion': 1309, 'force': [6.099052906036377, -4.69687557220459, -7.9687724113464355], 'magnitude': 11.079730033874512, 'distance': 5.473995685577393, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.3553767598406582, 'motion_component': -3.9374786012320016}, {'ion': 1469, 'force': [1.0042378902435303, 1.8420790433883667, -0.7561507821083069], 'magnitude': 2.230137586593628, 'distance': 12.20121955871582, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1105, 'cosine_with_motion': 0.16213359381764256, 'motion_component': 0.36158019590189205}, {'ion': 2444, 'force': [0.28925788402557373, 1.453320860862732, -2.9700722694396973], 'magnitude': 3.3192079067230225, 'distance': 10.001193046569824, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5696472702968612, 'motion_component': -1.8907777069422327}]}, 5493: {'frame': 5493, 'ionic_force': [10.491299332119524, 7.6357075572013855, -3.8044148929184303], 'ionic_force_magnitude': 13.52201775818585, 'motion_vector': [-1.495269775390625, 1.0756874084472656, 0.23244476318359375], 'cosine_ionic_motion': -0.3329221093087497, 'ionic_motion_component': -4.501778674165604, 'ionic_force_x': 10.491299332119524, 'ionic_force_y': 7.6357075572013855, 'ionic_force_z': -3.8044148929184303, 'radial_force': 12.975800228703967, 'axial_force': -3.8044148929184303, 'before_closest_residue': 130, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1306, 'force': [-0.00997841265052557, 2.116476058959961, -0.0016361012822017074], 'magnitude': 2.11650013923645, 'distance': 12.524484634399414, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.5830791569139248, 'motion_component': 1.234087160089051}, {'ion': 1309, 'force': [7.177574157714844, 0.5480061769485474, 0.4017539322376251], 'magnitude': 7.2096662521362305, 'distance': 6.7859625816345215, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.7507798160511517, 'motion_component': -5.412871918936274}, {'ion': 1469, 'force': [0.9419129490852356, 1.280834674835205, -0.03194640204310417], 'magnitude': 1.5902068614959717, 'distance': 14.44914722442627, 'before_closest_residue': 1073, 'closest_residue': 1105, 'next_closest_residue': 1073, 'cosine_with_motion': -0.012891961460507317, 'motion_component': -0.02050088629485819}, {'ion': 2443, 'force': [0.5624699592590332, 0.8197107911109924, -1.5806218385696411], 'magnitude': 1.8672609329223633, 'distance': 13.334186553955078, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.09423761570225872, 'motion_component': -0.17596622429598163}, {'ion': 2444, 'force': [1.8193206787109375, 2.8706798553466797, -2.5919644832611084], 'magnitude': 4.274226188659668, 'distance': 8.813335418701172, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.02960224101162135, 'motion_component': -0.1265266770110891}]}, 5494: {'frame': 5494, 'ionic_force': [7.315649628639221, 9.33461844921112, -4.467438533902168], 'ionic_force_magnitude': 12.673272589807093, 'motion_vector': [0.6881828308105469, 0.4589118957519531, 0.434112548828125], 'cosine_ionic_motion': 0.6232797087657117, 'ionic_motion_component': 7.898993648883442, 'ionic_force_x': 7.315649628639221, 'ionic_force_y': 9.33461844921112, 'ionic_force_z': -4.467438533902168, 'radial_force': 11.859756788457418, 'axial_force': -4.467438533902168, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1306, 'force': [-0.2891250550746918, 2.140397787094116, 0.09338859468698502], 'magnitude': 2.1618549823760986, 'distance': 12.392409324645996, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 780, 'cosine_with_motion': 0.40793231607021746, 'motion_component': 0.8818905523555348}, {'ion': 1309, 'force': [5.270052433013916, 1.1801180839538574, -0.09136883914470673], 'magnitude': 5.401340484619141, 'distance': 7.8400397300720215, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.8182541697057424, 'motion_component': 4.419669416924913}, {'ion': 1469, 'force': [0.786957323551178, 1.485055923461914, -0.08958549052476883], 'magnitude': 1.6830681562423706, 'distance': 14.04488468170166, 'before_closest_residue': 1105, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.7531818377095537, 'motion_component': 1.2676563817786788}, {'ion': 2443, 'force': [0.3067300617694855, 1.0199345350265503, -1.5694105625152588], 'magnitude': 1.8966810703277588, 'distance': 13.230366706848145, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.0012159144470626063, 'motion_component': -0.0023062019846715742}, {'ion': 2444, 'force': [1.2410348653793335, 3.5091121196746826, -2.810462236404419], 'magnitude': 4.663982391357422, 'distance': 8.43704891204834, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.2856107534826452, 'motion_component': 1.332083575267653}]}, 5495: {'frame': 5495, 'ionic_force': [7.954343676567078, 8.369591236114502, -2.939272278919816], 'ionic_force_magnitude': 11.914737190312417, 'motion_vector': [0.6293601989746094, -1.066162109375, -0.34174346923828125], 'cosine_ionic_motion': -0.19033843513047935, 'ionic_motion_component': -2.26783243179499, 'ionic_force_x': 7.954343676567078, 'ionic_force_y': 8.369591236114502, 'ionic_force_z': -2.939272278919816, 'radial_force': 11.546499070479646, 'axial_force': -2.939272278919816, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1306, 'force': [0.2466723620891571, 1.525595784187317, 0.19774486124515533], 'magnitude': 1.5580092668533325, 'distance': 14.597686767578125, 'before_closest_residue': 748, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.769029715873882, 'motion_component': -1.198155400493806}, {'ion': 1309, 'force': [4.939149856567383, 1.1103832721710205, 0.3859111964702606], 'magnitude': 5.077113151550293, 'distance': 8.08650016784668, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.2749294025598821, 'motion_component': 1.3958477346173073}, {'ion': 1469, 'force': [1.0719969272613525, 1.4649080038070679, 0.0071951355785131454], 'magnitude': 1.815264344215393, 'distance': 13.523811340332031, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, '</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>5576</v>
+      </c>
+      <c r="B17" t="n">
+        <v>5582</v>
+      </c>
+      <c r="C17" t="n">
+        <v>2444</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>{5576: {'frame': 5576, 'ionic_force': [-5.12838389724493, -9.299570322036743, -7.61335426568985], 'ionic_force_magnitude': 13.066961878987996, 'motion_vector': [0.9404220581054688, -0.198822021484375, -0.6372222900390625], 'cosine_ionic_motion': 0.12459092668388769, 'ionic_motion_component': 1.6280248894461486, 'ionic_force_x': -5.12838389724493, 'ionic_force_y': -9.299570322036743, 'ionic_force_z': -7.61335426568985, 'radial_force': 10.619902521776162, 'axial_force': -7.61335426568985, 'before_closest_residue': None, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1309, 'force': [6.9591827392578125, -4.298310279846191, -0.8726447224617004], 'magnitude': 8.226007461547852, 'distance': 6.352936267852783, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.838575231832428, 'motion_component': 6.898126405392048}, {'ion': 1380, 'force': [-0.09576242417097092, -0.6451082229614258, -1.4218106269836426], 'magnitude': 1.5642507076263428, 'distance': 14.568533897399902, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5234101473850589, 'motion_component': 0.8187447342328956}, {'ion': 1469, 'force': [-11.656188011169434, -2.1556320190429688, -2.5449581146240234], 'magnitude': 12.123954772949219, 'distance': 5.2329535484313965, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.6373557234813525, 'motion_component': -7.727271987372546}, {'ion': 2443, 'force': [-0.33561620116233826, -2.2005198001861572, -2.7739408016204834], 'magnitude': 3.55663800239563, 'distance': 9.661603927612305, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.46066700205914507, 'motion_component': 1.6384257216959917}]}, 5577: {'frame': 5577, 'ionic_force': [-5.55037547647953, -9.919090867042542, -9.448231399059296], 'ionic_force_magnitude': 14.780531388577412, 'motion_vector': [1.2938232421875, 4.777435302734375, -1.3350448608398438], 'cosine_ionic_motion': -0.5537087550802853, 'ionic_motion_component': -8.184109634594279, 'ionic_force_x': -5.55037547647953, 'ionic_force_y': -9.919090867042542, 'ionic_force_z': -9.448231399059296, 'radial_force': 11.366399234522433, 'axial_force': -9.448231399059296, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1309, 'force': [4.450619697570801, -1.8525863885879517, -2.3408517837524414], 'magnitude': 5.359074592590332, 'distance': 7.8708953857421875, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.001195564678229169, 'motion_component': 0.0064071201351936224}, {'ion': 1469, 'force': [-9.812492370605469, -4.156482219696045, -4.021743297576904], 'magnitude': 11.39016056060791, 'distance': 5.398885250091553, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.4655485963425134, 'motion_component': -5.302673516991831}, {'ion': 2434, 'force': [-0.3545006811618805, -1.8371081352233887, -0.5042237639427185], 'magnitude': 1.9377509355545044, 'distance': 13.089409828186035, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.8619284381256479, 'motion_component': -1.6702026260898677}, {'ion': 2443, 'force': [0.16599787771701813, -2.0729141235351562, -2.5814125537872314], 'magnitude': 3.3148481845855713, 'distance': 10.007767677307129, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.3673291426502491, 'motion_component': -1.2176403718538467}]}, 5578: {'frame': 5578, 'ionic_force': [1.3535993099212646, 2.408291459083557, -11.13271152973175], 'ionic_force_magnitude': 11.470368993538804, 'motion_vector': [-3.8603553771972656, 0.4764251708984375, -2.4455490112304688], 'cosine_ionic_motion': 0.4392217845722206, 'ionic_motion_component': 5.038035939043979, 'ionic_force_x': 1.3535993099212646, 'ionic_force_y': 2.408291459083557, 'ionic_force_z': -11.13271152973175, 'radial_force': 2.762625353484278, 'axial_force': -11.13271152973175, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 1105, 'contributions': [{'ion': 1309, 'force': [3.6393582820892334, 1.2222265005111694, -1.990733027458191], 'magnitude': 4.32455587387085, 'distance': 8.761899948120117, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.4327486833242564, 'motion_component': -1.871445900624309}, {'ion': 1469, 'force': [-2.00545072555542, 5.622910022735596, -3.1680915355682373], 'magnitude': 6.7583842277526855, 'distance': 7.00886344909668, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.5850980689663797, 'motion_component': 3.9543174027435417}, {'ion': 2434, 'force': [-1.0407629013061523, -3.8392817974090576, -2.276965618133545], 'magnitude': 4.583431720733643, 'distance': 8.5108642578125, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.368348936706906, 'motion_component': 1.6883021294440397}, {'ion': 2443, 'force': [0.7604546546936035, -0.5975632667541504, -3.6969213485717773], 'magnitude': 3.8213350772857666, 'distance': 9.320978164672852, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.33152354779450083, 'motion_component': 1.2668625111317056}]}, 5579: {'frame': 5579, 'ionic_force': [-1.6814625263214111, 1.4262338280677795, -10.292737245559692], 'ionic_force_magnitude': 10.526248104898524, 'motion_vector': [2.0666732788085938, -1.3358840942382812, 0.7496261596679688], 'cosine_ionic_motion': -0.4836302150923508, 'ionic_motion_component': -5.090811635087523, 'ionic_force_x': -1.6814625263214111, 'ionic_force_y': 1.4262338280677795, 'ionic_force_z': -10.292737245559692, 'radial_force': 2.20487168781951, 'axial_force': -10.292737245559692, 'before_closest_residue': 780, 'closest_residue': 1105, 'next_closest_residue': 780, 'contributions': [{'ion': 1309, 'force': [2.5060808658599854, 1.78612220287323, -4.071807861328125], 'magnitude': 5.103948593139648, 'distance': 8.065214157104492, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.019736404334987183, 'motion_component': -0.10073359671217474}, {'ion': 1469, 'force': [-2.498354911804199, 1.540704369544983, -2.071153163909912], 'magnitude': 3.592384099960327, 'distance': 9.613414764404297, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.9494373347064944, 'motion_component': -3.4107434696653627}, {'ion': 2434, 'force': [-1.2354334592819214, -1.6161770820617676, -1.6747441291809082], 'magnitude': 2.634974718093872, 'distance': 11.22485637664795, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.2433668646071048, 'motion_component': -0.6412655505220783}, {'ion': 2443, 'force': [-0.4537550210952759, -0.28441566228866577, -2.475032091140747], 'magnitude': 2.5323052406311035, 'distance': 11.450145721435547, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.3704407508345466, 'motion_component': -0.9380690479944036}]}, 5580: {'frame': 5580, 'ionic_force': [-0.7721650202292949, 0.8433377742767334, -11.557860493659973], 'ionic_force_magnitude': 11.614284162654782, 'motion_vector': [-1.6046180725097656, 1.9312629699707031, -1.8199996948242188], 'cosine_ionic_motion': 0.6636535826097525, 'ionic_motion_component': 7.707861293993555, 'ionic_force_x': -0.7721650202292949, 'ionic_force_y': 0.8433377742767334, 'ionic_force_z': -11.557860493659973, 'radial_force': 1.1434410435119695, 'axial_force': -11.557860493659973, 'before_closest_residue': 1105, 'closest_residue': 780, 'next_closest_residue': 1105, 'contributions': [{'ion': 1309, 'force': [3.384483575820923, 0.7182776927947998, -3.0355429649353027], 'magnitude': 4.60273551940918, 'distance': 8.492998123168945, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.10376222845352057, 'motion_component': 0.4775900803784907}, {'ion': 1469, 'force': [-3.7529938220977783, 2.630032777786255, -4.193670749664307], 'magnitude': 6.211997032165527, 'distance': 7.310606479644775, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.9724726226719216, 'motion_component': 6.040997223573072}, {'ion': 2434, 'force': [-0.40012770891189575, -1.974854826927185, -1.4709564447402954], 'magnitude': 2.494767904281616, 'distance': 11.535965919494629, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.06395217211863438, 'motion_component': -0.15954582303928788}, {'ion': 2443, 'force': [-0.0035270650405436754, -0.5301178693771362, -2.8576903343200684], 'magnitude': 2.9064464569091797, 'distance': 10.687788963317871, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.4640786037765659, 'motion_component': 1.3488196484509294}]}, 5581: {'frame': 5581, 'ionic_force': [-1.0563013553619385, 1.5127899050712585, -8.483844637870789], 'ionic_force_magnitude': 8.682161348981825, 'motion_vector': [0.801727294921875, 2.2831573486328125, -1.9393539428710938], 'cosine_ionic_motion': 0.7079269250678751, 'ionic_motion_component': 6.1463357867278585, 'ionic_force_x': -1.0563013553619385, 'ionic_force_y': 1.5127899050712585, 'ionic_force_z': -8.483844637870789, 'radial_force': 1.8450761096022505, 'axial_force': -8.483844637870789, 'before_closest_residue': 780, 'closest_residue': 1105, 'next_closest_residue': 130, 'contributions': [{'ion': 1309, 'force': [1.5847398042678833, 1.608560562133789, -3.1895318031311035], 'magnitude': 3.907938003540039, 'distance': 9.217119216918945, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.9183044697980314, 'motion_component': 3.5886770553587723}, {'ion': 1469, 'force': [-1.8289650678634644, 1.3348606824874878, -1.9141175746917725], 'magnitude': 2.964930534362793, 'distance': 10.581854820251465, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.5757282457888437, 'motion_component': 1.7069941852641575}, {'ion': 2434, 'force': [-0.5441734194755554, -1.361169457435608, -1.2634094953536987], 'magnitude': 1.9352288246154785, 'distance': 13.097936630249023, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 98, 'cosine_with_motion': -0.1822682099252567, 'motion_component': -0.35273069138135327}, {'ion': 2443, 'force': [-0.267902672290802, -0.0694618821144104, -2.116785764694214], 'magnitude': 2.1348018646240234, 'distance': 12.470683097839355, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5637035846568351, 'motion_component': 1.203395432897583}]}, 5582: {'frame': 5582, 'ionic_force': [-0.011387579143047333, 0.7488982081413269, -5.534487962722778], 'ionic_force_magnitude': 5.584938246090046, 'motion_vector': [1.6045913696289062, -2.307353973388672, -3.4020919799804688], 'cosine_ionic_motion': 0.6931398514922855, 'ionic_motion_component': 3.87114326648844, 'ionic_force_x': -0.011387579143047333, 'ionic_force_y': 0.7488982081413269, 'ionic_force_z': -5.534487962722778, 'radial_force': 0.7489847816317962, 'axial_force': -5.534487962722778, 'before_closest_residue': 1105, 'closest_residue': 130, 'next_closest_residue': None, 'contributions': [{'ion': 1306, 'force': [0.44565045833587646, 0.22126013040542603, 1.527474284172058], 'magnitude': 1.606467604637146, 'distance': 14.375834465026855, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7041937092394214, 'motion_component': -1.131264359448302}, {'ion': 1309, 'force': [0.9512708783149719, 0.9681544303894043, -2.003573179244995], 'magnitude': 2.420029878616333, 'distance': 11.71274471282959, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.5720386383493259, 'motion_component': 1.384350614990204}, {'ion': 1469, 'force': [-1.059220314025879, 0.999154806137085, -1.5712475776672363], 'magnitude': 2.1422131061553955, 'distance': 12.449092864990234, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.1418053295081253, 'motion_component': 0.30377723401855405}, {'ion': 2434, 'force': [-0.2705686688423157, -1.578347086906433, -1.934159755706787], 'magnitude': 2.511047840118408, 'distance': 11.498509407043457, 'before_closest_residue': 423, 'closest_residue': 98, 'next_closest_residue': 423, 'cosine_with_motion': 0.8833188285271076, 'motion_component': 2.218055772580776}, {'ion': 2443, 'force': [-0.07851993292570114, 0.13867592811584473, -1.5529817342758179], 'magnitude': 1.5611369609832764, 'distance': 14.58305549621582, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.702195832082078, 'motion_component': 1.096223878320914}]}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>5594</v>
+      </c>
+      <c r="B18" t="n">
+        <v>6202</v>
+      </c>
+      <c r="C18" t="n">
+        <v>2443</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>{5594: {'frame': 5594, 'ionic_force': [-4.9196601659059525, 1.0488449931144714, -6.5911475121974945], 'ionic_force_magnitude': 8.291342321670859, 'motion_vector': [1.2472190856933594, -0.8786392211914062, 1.1838226318359375], 'cosine_ionic_motion': -0.9281191389561603, 'ionic_motion_component': -7.695353496379928, 'ionic_force_x': -4.9196601659059525, 'ionic_force_y': 1.0488449931144714, 'ionic_force_z': -6.5911475121974945, 'radial_force': 5.03022186067206, 'axial_force': -6.5911475121974945, 'before_closest_residue': None, 'closest_residue': 98, 'next_closest_residue': 'SF', 'contributions': [{'ion': 1309, 'force': [2.8878653049468994, 3.550973415374756, 0.24883276224136353], 'magnitude': 4.5837860107421875, 'distance': 8.51053524017334, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.08770757195450159, 'motion_component': 0.4020327582711829}, {'ion': 1380, 'force': [-0.7073386907577515, 1.981725811958313, -4.544967174530029], 'magnitude': 5.008421897888184, 'distance': 8.141765594482422, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8275660510800515, 'motion_component': -4.144800091426141}, {'ion': 1469, 'force': [-1.5927733182907104, 2.366380214691162, 0.28326359391212463], 'magnitude': 2.8665170669555664, 'distance': 10.761969566345215, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.6739140830450312, 'motion_component': -1.9317862597870918}, {'ion': 1476, 'force': [-0.1692715436220169, 0.5136356949806213, -2.323270082473755], 'magnitude': 2.3853843212127686, 'distance': 11.797496795654297, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7408856258182113, 'motion_component': -1.7672969554629239}, {'ion': 2434, 'force': [-5.338141918182373, -7.363870143890381, -0.2550066113471985], 'magnitude': 9.098756790161133, 'distance': 6.040571212768555, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 455, 'cosine_with_motion': -0.02786127094080532, 'motion_component': -0.2535029218473497}]}, 5597: {'frame': 5597, 'ionic_force': [-2.391743592917919, 3.8317089676856995, -11.019856214523315], 'ionic_force_magnitude': 11.909645755272281, 'motion_vector': [1.3422393798828125, -0.8549842834472656, -0.35398101806640625], 'cosine_ionic_motion': -0.13316181833832863, 'ionic_motion_component': -1.585910084537414, 'ionic_force_x': -2.391743592917919, 'ionic_force_y': 3.8317089676856995, 'ionic_force_z': -11.019856214523315, 'radial_force': 4.5169050274836335, 'axial_force': -11.019856214523315, 'before_closest_residue': 'SF', 'closest_residue': 98, 'next_closest_residue': 455, 'contributions': [{'ion': 1309, 'force': [2.360955238342285, 3.685953378677368, -0.3692745864391327], 'magnitude': 4.392804145812988, 'distance': 8.69356918334961, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 'SF', 'cosine_with_motion': 0.02070077484749574, 'motion_component': 0.09093444345478696}, {'ion': 1380, 'force': [-0.3367534875869751, 4.115484714508057, -6.502329349517822], 'magnitude': 7.702655792236328, 'distance': 6.565212726593018, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.13290461052277605, 'motion_component': -1.0237184513445428}, {'ion': 1469, 'force': [-1.0739519596099854, 3.1200692653656006, -0.15641751885414124], 'magnitude': 3.3034331798553467, 'distance': 10.025043487548828, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.7526977822934205, 'motion_component': -2.486486908028081}, {'ion': 1476, 'force': [-0.05223899334669113, 0.661562979221344, -2.2055890560150146], 'magnitude': 2.30326247215271, 'distance': 12.005972862243652, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.0386131363744981, 'motion_component': 0.0889361842241847}, {'ion': 2434, 'force': [-3.2897543907165527, -7.75136137008667, -1.7862457036972046], 'magnitude': 8.60794734954834, 'distance': 6.210395336151123, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.20265278659256922, 'motion_component': 1.7444245546876704}]}, 5598: {'frame': 5598, 'ionic_force': [3.7280571311712265, -0.048622846603393555, -10.82320636510849], 'ionic_force_magnitude': 11.44738267798423, 'motion_vector': [1.0442886352539062, 2.5621337890625, -0.08968353271484375], 'cosine_ionic_motion': 0.14955505651374204, 'ionic_motion_component': 1.7120139633403633, 'ionic_force_x': 3.7280571311712265, 'ionic_force_y': -0.048622846603393555, 'ionic_force_z': -10.82320636510849, 'radial_force': 3.728374197219004, 'axial_force': -10.82320636510849, 'before_closest_residue': 98, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1309, 'force': [7.3780598640441895, 4.05808687210083, -3.189204216003418], 'magnitude': 9.004158020019531, 'distance': 6.0722198486328125, 'before_closest_residue': 1073, 'closest_residue': 'SF', 'next_closest_residue': 'SF', 'cosine_with_motion': 0.7377235610363455, 'motion_component': 6.642579449055013}, {'ion': 1380, 'force': [0.361459881067276, 1.1916948556900024, -3.9953513145446777], 'magnitude': 4.184927940368652, 'distance': 8.906867980957031, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.32707079284715657, 'motion_component': 1.3687677047499784}, {'ion': 1469, 'force': [-1.4546935558319092, 3.4690563678741455, -0.2319532036781311], 'magnitude': 3.768857717514038, 'distance': 9.385645866394043, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.708311737890327, 'motion_component': 2.669526086335598}, {'ion': 1476, 'force': [0.21506913006305695, 0.3528536558151245, -1.9371775388717651], 'magnitude': 1.9807617664337158, 'distance': 12.946516036987305, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.23752247681468455, 'motion_component': 0.470475445232283}, {'ion': 2434, 'force': [-2.7718381881713867, -9.120314598083496, -1.469520092010498], 'magnitude': 9.644827842712402, 'distance': 5.867076873779297, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.9786939015619761, 'motion_component': -9.439334723743546}]}, 5599: {'frame': 5599, 'ionic_force': [-1.9013180434703827, -9.60105836391449, -11.383936129510403], 'ionic_force_magnitude': 15.012972184430726, 'motion_vector': [-3.3165664672851562, 2.1229324340820312, -0.15932464599609375], 'cosine_ionic_motion': -0.20725825176288065, 'ionic_motion_component': -3.1115623687098677, 'ionic_force_x': -1.9013180434703827, 'ionic_force_y': -9.60105836391449, 'ionic_force_z': -11.383936129510403, 'radial_force': 9.787508978780986, 'axial_force': -11.383936129510403, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 98, 'contributions': [{'ion': 1309, 'force': [3.44903564453125, 3.2919468879699707, -1.7546262741088867], 'magnitude': 5.080499172210693, 'distance': 8.083805084228516, 'before_closest_residue': 'SF', 'closest_residue': 'SF', 'next_closest_residue': 'SF', 'cosine_with_motion': -0.2083068570552768, 'motion_component': -1.0583028704620006}, {'ion': 1380, 'force': [0.5980334877967834, 1.709892749786377, -2.676297664642334], 'magnitude': 3.2317094802856445, 'distance': 10.135680198669434, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.16276051846555098, 'motion_component': 0.5259947179221207}, {'ion': 1469, 'force': [-0.6552402973175049, 2.634486198425293, -0.08947023004293442], 'magnitude': 2.716222047805786, 'distance': 11.055704116821289, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.7268021563776397, 'motion_component': 1.9741560530515698}, {'ion': 1476, 'force': [0.27780506014823914, 0.6250635385513306, -1.5681666135787964], 'magnitude': 1.710855484008789, 'distance': 13.930360794067383, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.09721179363021912, 'motion_component': 0.16631533363621465}, {'ion': 2434, 'force': [-5.57095193862915, -17.86244773864746, -5.295375347137451], 'magnitude': 19.445913314819336, 'distance': 4.131947994232178, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 455, 'cosine_with_motion': -0.24271040835726235, 'motion_component': -4.719725562381129}]}, 5600: {'frame': 5600, 'ionic_force': [-18.553392615169287, 5.5990365743637085, -7.359938099980354], 'ionic_force_magnitude': 20.7303226441178, 'motion_vector': [-2.751720428466797, -2.4600486755371094, 0.600830078125], 'cosine_ionic_motion': 0.42384193582320084, 'ionic_motion_component': 8.786380079722424, 'ionic_force_x': -18.553392615169287, 'ionic_force_y': 5.5990365743637085, 'ionic_force_z': -7.359938099980354, 'radial_force': 19.379824253426055, 'axial_force': -7.359938099980354, 'before_closest_residue': 455, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1309, 'force': [-0.036227066069841385, 5.730989933013916, -1.8837703466415405], 'magnitude': 6.032756328582764, 'distance': 7.418415546417236, 'before_closest_residue': 'SF', 'closest_residue': 'SF', 'next_closest_residue': 'SF', 'cosine_with_motion': -0.6706774795430298, 'motion_component': -4.046033798670543}, {'ion': 1380, 'force': [-0.34478411078453064, 1.6263123750686646, -1.8408604860305786], 'magnitude': 2.4804306030273438, 'distance': 11.569257736206055, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.44827028613449765, 'motion_component': -1.1119032798557278}, {'ion': 1469, 'force': [-0.7819127440452576, 1.468832015991211, -0.126841738820076], 'magnitude': 1.6688151359558105, 'distance': 14.104735374450684, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.24644546931116953, 'motion_component': -0.4112719219322474}, {'ion': 1476, 'force': [-0.10772905498743057, 0.7481944561004639, -1.3221204280853271], 'magnitude': 1.5229586362838745, 'distance': 14.7647123336792, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.41060629870047766, 'motion_component': -0.6253363968497498}, {'ion': 2434, 'force': [-17.282739639282227, -3.975292205810547, -2.186345100402832], 'magnitude': 17.86829948425293, 'distance': 4.310497760772705, 'before_closest_residue': 423, 'closest_residue': 455, 'next_closest_residue': 423, 'cosine_with_motion': 0.8384080211694442, 'motion_component': 14.980925987625355}]}, 5601: {'frame': 5601, 'ionic_force': [-9.747690379619598, 9.922138929367065, -7.001989342272282], 'ionic_force_magnitude': 15.572224099976358, 'motion_vector': [-0.6682701110839844, -0.8040084838867188, 0.39972686767578125], 'cosine_ionic_motion': -0.24454050825740734, 'ionic_motion_component': -3.808039596106466, 'ionic_force_x': -9.747690379619598, 'ionic_force_y': 9.922138929367065, 'ionic_force_z': -7.001989342272282, 'radial_force': 13.909216680697368, 'axial_force': -7.001989342272282, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1309, 'force': [-1.464813470840454, 7.521646022796631, -2.570472478866577], 'magnitude': 8.082584381103516, 'distance': 6.409053802490234, 'before_closest_residue': 'SF', 'closest_residue': 'SF', 'next_closest_residue': 'SF', 'cosine_with_motion': -0.6738434349501465, 'motion_component': -5.446396251043808}, {'ion': 1380, 'force': [-1.123779535293579, 1.281681776046753, -2.1522297859191895], 'magnitude': 2.745483875274658, 'distance': 10.99662971496582, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.3709104648523173, 'motion_component': -1.0183286977882204}, {'ion': 1469, 'force': [-1.2938627004623413, 1.2048321962356567, -0.07915589958429337], 'magnitude': 1.769736409187317, 'distance': 13.696661949157715, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.06849944068954568, 'motion_component': -0.1212259543360079}, {'ion': 1476, 'force': [-0.5480816960334778, 0.5199006199836731, -1.4181257486343384], 'magnitude': 1.606788992881775, 'distance': 14.374396324157715, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.3439627835312633, 'motion_component': -0.5526756114863964}, {'ion': 2434, 'force': [-5.317152976989746, -0.6059216856956482, -0.7820054292678833], 'magnitude': 5.408400058746338, 'distance': 7.834921360015869, 'before_closest_residue': 455, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.6158174580254275, 'motion_component': 3.3305870717415047}]}, 5602: {'frame': 5602, 'ionic_force': [-9.748128592967987, 11.87373073399067, -8.434279189445078], 'ionic_force_magnitude': 17.525654283189, 'motion_vector': [1.2005729675292969, 0.9844474792480469, -0.0977783203125], 'cosine_ionic_motion': 0.029724777835226476, 'ionic_motion_component': 0.5209461799847783, 'ionic_force_x': -9.748128592967987, 'ionic_force_y': 11.87373073399067, 'ionic_force_z': -8.434279189445078, 'radial_force': 15.362665543724976, 'axial_force': -8.434279189445078, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1309, 'force': [-2.806483507156372, 9.153647422790527, -4.609921932220459], 'magnitude': 10.626240730285645, 'distance': 5.589580535888672, 'before_closest_residue': 'SF', 'closest_residue': 'SF', 'next_closest_residue': 'SF', 'cosine_with_motion': 0.3685633566753359, 'motion_component': 3.916442934703298}, {'ion': 1380, 'force': [-1.2517857551574707, 1.1912050247192383, -2.192772626876831], 'magnitude': 2.7918074131011963, 'distance': 10.90501594543457, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.02665741311094373, 'motion_component': -0.07442236424890325}, {'ion': 1469, 'force': [-1.356601595878601, 1.2908194065093994, -0.006111637689173222], 'magnitude': 1.872597098350525, 'distance': 13.315174102783203, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.12267176777810217, 'motion_component': -0.22971479932318095}, {'ion': 1476, 'force': [-0.6084700226783752, 0.47949525713920593, -1.4761505126953125], 'magnitude': 1.667084813117981, 'distance': 14.112052917480469, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.04401119431896101, 'motion_component': -0.07337039408029966}, {'ion': 2434, 'force': [-3.724787712097168, -0.24143637716770172, -0.1493224799633026], 'magnitude': 3.7355899810791016, 'distance': 9.427346229553223, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.8079016858035686, 'motion_component': -3.017989412981734}]}, 5603: {'frame': 5603, 'ionic_force': [-17.560770630836487, 16.140983641147614, -9.764761259779334], 'ionic_force_magnitude': 25.773291999919827, 'motion_vector': [-1.2378005981445312, -0.32138824462890625, 0.05432891845703125], 'cosine_ionic_motion': 0.4855662067281127, 'ionic_motion_component': 12.514639631297083, 'ionic_force_x': -17.560770630836487, 'ionic_force_y': 16.140983641147614, 'ionic_force_z': -9.764761259779334, 'radial_force': 23.851876614904835, 'axial_force': -9.764761259779334, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1309, 'force': [-7.167101860046387, 12.286242485046387, -4.010806083679199], 'magnitude': 14.77855396270752, 'distance': 4.739724159240723, 'before_closest_residue': 'SF', 'closest_residue': 'SF', 'next_closest_residue': 'SF', 'cosine_with_motion': 0.24871857187461996, 'motion_component': 3.6757009343113474}, {'ion': 1380, 'force': [-1.6355546712875366, 2.433621406555176, -2.8497138023376465], 'magnitude': 4.0888166427612305, 'distance': 9.010942459106445, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.20779505125123693, 'motion_component': 0.8496358498721843}, {'ion': 1469, 'force': [-1.2709964513778687, 1.487382173538208, -0.02657478116452694], 'magnitude': 1.9566409587860107, 'distance': 13.02607250213623, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.43672253559983204, 'motion_component': 0.8545092104852909}, {'ion': 1476, 'force': [-0.5827058553695679, 0.6906329989433289, -1.6999109983444214], 'magnitude': 1.9251538515090942, 'distance': 13.13216495513916, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.16514870871978457, 'motion_component': 0.3179366770997212}, {'ion': 2434, 'force': [-6.904411792755127, -0.7568954229354858, -1.17775559425354], 'magnitude': 7.044920444488525, 'distance': 6.864849090576172, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.9676272386019888, 'motion_component': 6.816856713678004}]}, 5604: {'frame': 5604, 'ionic_force': [-14.2177032828331, 19.06482544541359, -2.1827616719529033], 'ionic_force_magnitude': 23.882527178238888, 'motion_vector': [0.9648094177246094, 0.07035064697265625, 0.3220977783203125], 'cosine_ionic_motion': -0.5371282190388663, 'ionic_motion_component': -12.827979289394776, 'ionic_force_x': -14.2177032828331, 'ionic_force_y': 19.06482544541359, 'ionic_force_z': -2.1827616719529033, 'radial_force': 23.782570422533652, 'axial_force': -2.1827616719529033, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1309, 'force': [-7.5053019523620605, 15.458601951599121, 1.4540939331054688], 'magnitude': 17.245647430419922, 'distance': 4.387622833251953, 'before_closest_residue': 'SF', 'closest_residue': 'SF', 'next_closest_residue': 'SF', 'cosine_with_motion': -0.3233335147373387, 'motion_component': -5.576095474802756}, {'ion': 1380, 'force': [-1.4976059198379517, 1.5437307357788086, -2.2601349353790283], 'magnitude': 3.1199581623077393, 'distance': 10.315604209899902, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.648929883303207, 'motion_component': -2.0246339891788097}, {'ion': 1469, 'force': [-1.2702255249023438, 1.183520793914795, 0.04746720567345619], 'magnitude': 1.7367923259735107, 'distance': 13.825953483581543, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.6364187952686731, 'motion_component': -1.1053272624682102}, {'ion': 1476, 'force': [-0.6734047532081604, 0.5765787363052368, -1.429139256477356], 'magnitude': 1.6817716360092163, 'distance': 14.050297737121582, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6237018120886582, 'motion_component': -1.0489240501870594}, {'ion': 2434, 'force': [-3.271165132522583, 0.30239322781562805, 0.004951381124556065], 'magnitude': 3.285115957260132, 'distance': 10.052953720092773, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.9354306093367044, 'motion_component': -3.0729981144680583}]}, 5605: {'frame': 5605, 'ionic_force': [-18.65671706199646, 11.948305934667587, -10.66128496825695], 'ionic_force_magnitude': 24.586543136727947, 'motion_vector': [-0.040676116943359375, 0.6826667785644531, -0.5590362548828125], 'cosine_ionic_motion': 0.6849713259002533, 'ionic_motion_component': 16.841077051668314, 'ionic_force_x': -18.65671706199646, 'ionic_force_y': 11.948305934667587, 'ionic_force_z': -10.66128496825695, 'radial_force': 22.154798718106253, 'axial_force': -10.66128496825695, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1309, 'force': [-11.117942810058594, 8.545702934265137, -6.663941860198975], 'magnitude': 15.525650024414062, 'distance': 4.6242804527282715, 'before_closest_residue': 'SF', 'closest_residue': 'SF', 'next_closest_residue': 'SF', 'cosine_with_motion': 0.7300339144435805, 'motion_component': 11.334251141633246}, {'ion': 1380, 'force': [-1.4706867933273315, 1.5739147663116455, -2.449951410293579], 'magnitude': 3.262267589569092, 'distance': 10.08809757232666, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.8689412030578023, 'motion_component': 2.83471864706858}, {'ion': 1469, 'force': [-1.0578231811523438, 1.5526583194732666, 0.06499066203832626], 'magnitude': 1.8798832893371582, 'distance': 13.289344787597656, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.6423665599546077, 'motion_component': 1.2075742205013205}, {'ion': 1476, 'force': [-0.48204028606414795, 0.6503790020942688, -1.660539984703064], 'magnitude': 1.8473626375198364, 'distance': 13.405807495117188, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.8530031608461415, 'motion_component': 1.5758061713531215}, {'ion': 2434, 'force': [-4.528223991394043, -0.37434908747673035, 0.048157624900341034], 'magnitude': 4.54392671585083, 'distance': 8.547780990600586, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 455, 'cosine_with_motion': -0.024488314677508453, 'motion_component': -0.11127310436116833}]}, 5606: {'frame': 5606, 'ionic_force': [-21.41411665081978, 2.977629542350769, -6.465997515246272], 'ionic_force_magnitude': 22.566342049467565, 'motion_vector': [-0.3365478515625, -0.6044425964355469, 0.14295196533203125], 'cosine_ionic_motion': 0.2811967488243754, 'ionic_motion_component': 6.345582017169072, 'ionic_force_x': -21.41411665081978, 'ionic_force_y': 2.977629542350769, 'ionic_force_z': -6.465997515246272, 'radial_force': 21.62014499549892, 'axial_force': -6.465997515246272, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1309, 'force': [-7.701904296875, 6.24114990234375, -5.068641662597656], 'magnitude': 11.133840560913086, 'distance': 5.460677623748779, 'before_closest_residue': 'SF', 'closest_residue': 'SF', 'next_closest_residue': 'SF', 'cosine_with_motion': -0.24219307971669768, 'motion_component': -2.6965391842246618}, {'ion': 1380, 'force': [-1.0523978471755981, 1.6155245304107666, -2.1546742916107178], 'magnitude': 2.891380786895752, 'distance': 10.715598106384277, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.45546704130604865, 'motion_component': -1.3169285881203194}, {'ion': 1469, 'force': [-1.061071753501892, 1.283768892288208, -0.014648376032710075], 'magnitude': 1.6655781269073486, 'distance': 14.11843490600586, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.3577673465268641, 'motion_component': -0.5958894575502764}, {'ion': 1476, 'force': [-0.44619205594062805, 0.6866577863693237, -1.5260471105575562], 'magnitude': 1.7318793535232544, 'distance': 13.845550537109375, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.3948078010148448, 'motion_component': -0.6837594740408859}, {'ion': 2434, 'force': [-11.15255069732666, -6.849471569061279, 2.298013925552368], 'magnitude': 13.288171768188477, 'distance': 4.998462200164795, 'before_closest_residue': 423, 'closest_residue': 455, 'next_closest_residue': 130, 'cosine_with_motion': 0.8758690610119446, 'motion_component': 11.638698756338389}]}, 5607: {'frame': 5607, 'ionic_force': [-23.770193874835968, 13.231722950935364, -0.08699758723378181], 'ionic_force_magnitude': 27.204929290071377, 'motion_vector': [-0.3793296813964844, -0.6377906799316406, 0.31902313232421875], 'cosine_ionic_motion': 0.025025193227587485, 'ionic_motion_component': 0.6808086122268906, 'ionic_force_x': -23.770193874835968, 'ionic_force_y': 13.231722950935364, 'ionic_force_z': -0.08699758723378181, 'radial_force': 27.20479018661234, 'axial_force': -0.08699758723378181, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1309, 'force': [-8.924793243408203, 5.3618340492248535, -5.453948497772217], 'magnitude': 11.753583908081055, 'distance': 5.314762592315674, 'before_closest_residue': 'SF', 'closest_residue': 'SF', 'next_closest_residue': 'SF', 'cosine_with_motion': -0.1868816901934147, 'motion_component': -2.1965297723835135}, {'ion': 1380, 'force': [-1.5038363933563232, 1.5769492387771606, -2.552949905395508], 'magnitude': 3.3564634323120117, 'distance': 9.945533752441406, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.4609719947420178, 'motion_component': -1.5472355919411385}, {'ion': 1469, 'force': [-1.4209312200546265, 1.4332846403121948, 0.041228216141462326], 'magnitude': 2.0186753273010254, 'distance': 12.824362754821777, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.2219976237801517, 'motion_component': -0.44814113030013036}, {'ion': 1476, 'force': [-0.508072555065155, 0.625862717628479, -1.5353832244873047], 'magnitude': 1.7341405153274536, 'distance': 13.836520195007324, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.4970715103472714, 'motion_component': -0.8619918711442516}, {'ion': 2434, 'force': [-11.41256046295166, 4.233792304992676, 9.414055824279785], 'magnitude': 15.388176918029785, 'distance': 4.644890308380127, 'before_closest_residue': 455, 'closest_residue': 130, 'next_closest_residue': 455, 'cosine_with_motion': 0.3726696751642105, 'motion_component': 5.7347067941715295}]}, 5608: {'frame': 5608, 'ionic_force': [-18.901110351085663, 10.239649832248688, -9.298373874276876], 'ionic_force_magnitude': 23.42140384129062, 'motion_vector': [-1.0680618286132812, 0.4606742858886719, 1.07733154296875], 'cosine_ionic_motion': 0.4009149166517778, 'ionic_motion_component': 9.389990168898658, 'ionic_force_x': -18.901110351085663, 'ionic_force_y': 10.239649832248688, 'ionic_force_z': -9.298373874276876, 'radial_force': 21.496567195507943, 'axial_force': -9.298373874276876, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1309, 'force': [-12.437792778015137, 5.437849521636963, -5.057575702667236], 'magnitude': 14.486129760742188, 'distance': 4.78732442855835, 'before_closest_residue': 'SF', 'closest_residue': 'SF', 'next_closest_residue': 130, 'cosine_with_motion': 0.4502448365240324, 'motion_component': 6.522305330380007}, {'ion': 1380, 'force': [-1.8392237424850464, 1.9834181070327759, -2.787628412246704], 'magnitude': 3.8842713832855225, 'distance': 9.245156288146973, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.02031175472901016, 'motion_component': -0.07889636593342786}, {'ion': 1469, 'force': [-1.3467543125152588, 1.3719929456710815, 0.04987660422921181], 'magnitude': 1.9231743812561035, 'distance': 13.138921737670898, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.6966672397713636, 'motion_component': 1.3398125508718068}, {'ion': 1476, 'force': [-0.6551981568336487, 0.6240441799163818, -1.8183751106262207], 'magnitude': 2.031059741973877, 'distance': 12.785204887390137, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.30176468217530766, 'motion_component': -0.6129021072239702}, {'ion': 2434, 'force': [-2.6221413612365723, 0.8223450779914856, 0.3153287470340729], 'magnitude': 2.7660999298095703, 'distance': 10.955573081970215, 'before_closest_residue': 130, 'closest_residue': 455, 'next_closest_residue': 780, 'cosine_with_motion': 0.802455270445704, 'motion_component': 2.2196714879421684}]}, 5609: {'frame': 5609, 'ionic_force': [-12.13606995344162, 7.872880041599274, 1.560283213853836], 'ionic_force_magnitude': 14.54994562779101, 'motion_vector': [1.0545501708984375, 1.109100341796875, -1.9637222290039062], 'cosine_ionic_motion': -0.19683564010415658, 'ionic_motion_component': -2.863947861126918, 'ionic_force_x': -12.13606995344162, 'ionic_force_y': 7.872880041599274, 'ionic_force_z': 1.560283213853836, 'radial_force': 14.466044174695467, 'axial_force': 1.560283213853836, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1309, 'force': [-4.694593906402588, 2.2950472831726074, 4.785083293914795], 'magnitude': 7.0854411125183105, 'distance': 6.845191478729248, 'before_closest_residue': 'SF', 'closest_residue': 130, 'next_closest_residue': 'SF', 'cosine_with_motion': -0.6690258524147681, 'motion_component': -4.740343296502999}, {'ion': 1380, 'force': [-2.6745073795318604, 2.1261026859283447, -2.479200601577759], 'magnitude': 4.221343040466309, 'distance': 8.868368148803711, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.41924361152831724, 'motion_component': 1.769771147065427}, {'ion': 1469, 'force': [-1.283077597618103, 1.198951244354248, 0.1152741014957428], 'magnitude': 1.7598466873168945, 'distance': 13.73509407043457, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.05698592106483147, 'motion_component': -0.10028648381809724}, {'ion': 1476, 'force': [-0.8566756844520569, 0.700995147228241, -1.6807165145874023], 'magnitude': 2.0124850273132324, 'distance': 12.844072341918945, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.6335882762341097, 'motion_component': 1.2750868315675952}, {'ion': 2434, 'force': [-2.6272153854370117, 1.5517836809158325, 0.8198429346084595], 'magnitude': 3.159499406814575, 'distance': 10.250850677490234, 'before_closest_residue': 455, 'closest_residue': 780, 'next_closest_residue': 130, 'cosine_with_motion': -0.3380839767120004, 'motion_component': -1.0681760815864507}]}, 5610: {'frame': 5610, 'ionic_force': [-9.932288229465485, 6.841108322143555, -1.9635789394378662], 'ionic_force_magnitude': 12.219114321418077, 'motion_vector': [-1.6703529357910156, -1.2484626770019531, 1.5174026489257812], 'cosine_ionic_motion': 0.1608859926502964, 'ionic_motion_component': 1.9658843369088004, 'ionic_force_x': -9.932288229465485, 'ionic_force_y': 6.841108322143555, 'ionic_force_z': -1.9635789394378662, 'radial_force': 12.06031146150382, 'axial_force': -1.9635789394378662, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1309, 'force': [-3.3086962699890137, 1.7046713829040527, -0.6709098815917969], 'magnitude': 3.781996250152588, 'distance': 9.369329452514648, 'before_closest_residue': 130, 'closest_residue': 'SF', 'next_closest_residue': 'SF', 'cosine_with_motion': 0.24405238491228257, 'motion_component': 0.9230052034104261}, {'ion': 1380, 'force': [-1.2851455211639404, 1.4375178813934326, -2.0031657218933105], 'magnitude': 2.780418872833252, 'distance': 10.927326202392578, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.3748097210425503, 'motion_component': -1.0421280538444577}, {'ion': 1476, 'force': [-0.5182755589485168, 0.6067698001861572, -1.3568806648254395], 'magnitude': 1.5741360187530518, 'distance': 14.52271842956543, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.4805185316498841, 'motion_component': -0.7564015403241271}, {'ion': 2434, 'force': [-4.820170879364014, 3.092149257659912, 2.0673773288726807], 'magnitude': 6.088470935821533, 'distance': 7.384394645690918, 'before_closest_residue': 780, 'closest_residue': 130, 'next_closest_residue': 130, 'cosine_with_motion': 0.4666867689292263, 'motion_component': 2.8414090212096283}]}, 5611: {'frame': 5611, 'ionic_force': [-7.319891095161438, 3.427933633327484, -1.2991392612457275], 'ionic_forc</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>5689</v>
+      </c>
+      <c r="B19" t="n">
+        <v>6427</v>
+      </c>
+      <c r="C19" t="n">
+        <v>1380</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>{5689: {'frame': 5689, 'ionic_force': [-10.846781343221664, 1.6348312199115753, -4.6059174835681915], 'ionic_force_magnitude': 11.897050663534147, 'motion_vector': [1.6955833435058594, -2.072643280029297, 4.204833984375], 'cosine_ionic_motion': -0.6937842477004733, 'ionic_motion_component': -8.253986344454455, 'ionic_force_x': -10.846781343221664, 'ionic_force_y': 1.6348312199115753, 'ionic_force_z': -4.6059174835681915, 'radial_force': 10.969290707482374, 'axial_force': -4.6059174835681915, 'before_closest_residue': None, 'closest_residue': 130, 'next_closest_residue': 'SF', 'contributions': [{'ion': 1355, 'force': [-0.2695693075656891, 0.3014860451221466, -1.9719277620315552], 'magnitude': 2.0129730701446533, 'distance': 12.842514038085938, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.9340956117594803, 'motion_component': -1.88030930318196}, {'ion': 1469, 'force': [-2.6125478744506836, 2.329728126525879, -0.3506489098072052], 'magnitude': 3.5179531574249268, 'distance': 9.714579582214355, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.6119997277317742, 'motion_component': -2.1529863553754645}, {'ion': 1476, 'force': [-1.3893324136734009, 1.863111972808838, -5.913637638092041], 'magnitude': 6.353939056396484, 'distance': 7.228488922119141, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.9813094185006677, 'motion_component': -6.235180191289949}, {'ion': 2434, 'force': [-0.631294310092926, -5.49688720703125, -1.0274757146835327], 'magnitude': 5.62761116027832, 'distance': 7.680809497833252, 'before_closest_residue': 423, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.2139528837455448, 'motion_component': 1.2040436448136056}, {'ion': 2443, 'force': [-5.944037437438965, 2.637392282485962, 4.657772541046143], 'magnitude': 7.998891353607178, 'distance': 6.442495822906494, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 130, 'cosine_with_motion': 0.10131979104044181, 'motion_component': 0.8104460085251759}]}, 5692: {'frame': 5692, 'ionic_force': [-2.2680077254772186, -15.304942309856415, -10.105775147676468], 'ionic_force_magnitude': 18.48003813541121, 'motion_vector': [5.063621520996094, 4.651702880859375, -0.6800384521484375], 'cosine_ionic_motion': -0.5936836240157243, 'ionic_motion_component': -10.971296012179716, 'ionic_force_x': -2.2680077254772186, 'ionic_force_y': -15.304942309856415, 'ionic_force_z': -10.105775147676468, 'radial_force': 15.472075431268339, 'axial_force': -10.105775147676468, 'before_closest_residue': 'SF', 'closest_residue': 780, 'next_closest_residue': 455, 'contributions': [{'ion': 1355, 'force': [-0.16544833779335022, -0.5105010867118835, -1.7802817821502686], 'magnitude': 1.859405279159546, 'distance': 13.362324714660645, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.1558124509191535, 'motion_component': -0.2897184830593833}, {'ion': 1469, 'force': [-8.14029312133789, 1.124986171722412, -1.0288584232330322], 'magnitude': 8.281818389892578, 'distance': 6.331493854522705, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.6166491039821831, 'motion_component': -5.106975882015757}, {'ion': 1476, 'force': [-0.7527567744255066, -2.250356912612915, -4.554305553436279], 'magnitude': 5.135411262512207, 'distance': 8.040470123291016, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.3151520722030431, 'motion_component': -1.618435477507159}, {'ion': 2434, 'force': [-0.9204217195510864, -2.4938366413116455, -0.17049100995063782], 'magnitude': 2.663731336593628, 'distance': 11.164103507995605, 'before_closest_residue': 98, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.8772231185167029, 'motion_component': -2.336686691254273}, {'ion': 2443, 'force': [7.710912227630615, -11.175233840942383, -2.57183837890625], 'magnitude': 13.818768501281738, 'distance': 4.901560306549072, 'before_closest_residue': 130, 'closest_residue': 1105, 'next_closest_residue': 'SF', 'cosine_with_motion': -0.11719417252773648, 'motion_component': -1.6194791760610485}]}, 5693: {'frame': 5693, 'ionic_force': [14.037217020988464, 0.7251570634543896, -12.502707362174988], 'ionic_force_magnitude': 18.811884696786514, 'motion_vector': [0.5311241149902344, 0.9281234741210938, 2.3688735961914062], 'cosine_ionic_motion': -0.43950603727257137, 'ionic_motion_component': -8.267936896713168, 'ionic_force_x': 14.037217020988464, 'ionic_force_y': 0.7251570634543896, 'ionic_force_z': -12.502707362174988, 'radial_force': 14.055935204069705, 'axial_force': -12.502707362174988, 'before_closest_residue': 780, 'closest_residue': 455, 'next_closest_residue': 423, 'contributions': [{'ion': 1355, 'force': [0.4393165409564972, 0.04694287106394768, -1.5332221984863281], 'magnitude': 1.595610499382019, 'distance': 14.424660682678223, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8090304904701983, 'motion_component': -1.2908975703916323}, {'ion': 1469, 'force': [-0.2973380386829376, 6.702067852020264, -1.863255262374878], 'magnitude': 6.9626030921936035, 'distance': 6.90531063079834, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.09110255835193735, 'motion_component': 0.63431096597406}, {'ion': 1476, 'force': [1.3921409845352173, 0.3217581510543823, -3.227895498275757], 'magnitude': 3.529999256134033, 'distance': 9.697990417480469, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7202940567532118, 'motion_component': -2.5426374261861078}, {'ion': 2434, 'force': [2.518434524536133, -7.808837413787842, -1.8178147077560425], 'magnitude': 8.403862953186035, 'distance': 6.285351276397705, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.4677274978934718, 'motion_component': -3.930717568695087}, {'ion': 2443, 'force': [9.984663009643555, 1.4632256031036377, -4.060519695281982], 'magnitude': 10.877607345581055, 'distance': 5.524619102478027, 'before_closest_residue': 1105, 'closest_residue': 'SF', 'next_closest_residue': 1105, 'cosine_with_motion': -0.10461816669192547, 'motion_component': -1.1379953539395444}]}, 5694: {'frame': 5694, 'ionic_force': [15.186673760414124, -2.523807108402252, -6.381444334983826], 'ionic_force_magnitude': 16.66515808584394, 'motion_vector': [-6.16156005859375, -6.210399627685547, -0.5569686889648438], 'cosine_ionic_motion': -0.5089087171859848, 'ionic_motion_component': -8.481044223168483, 'ionic_force_x': 15.186673760414124, 'ionic_force_y': -2.523807108402252, 'ionic_force_z': -6.381444334983826, 'radial_force': 15.39495573964643, 'axial_force': -6.381444334983826, 'before_closest_residue': 455, 'closest_residue': 423, 'next_closest_residue': 1105, 'contributions': [{'ion': 1355, 'force': [0.7672042846679688, 0.321216881275177, -2.13971209526062], 'magnitude': 2.2956807613372803, 'distance': 12.02578067779541, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.2748099851973862, 'motion_component': -0.6308760194952647}, {'ion': 1469, 'force': [0.36691606044769287, 5.6577959060668945, 0.787419319152832], 'magnitude': 5.724099159240723, 'distance': 7.6157989501953125, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.7540475151744416, 'motion_component': -4.316242741675154}, {'ion': 1476, 'force': [4.058429718017578, 1.9305769205093384, -4.828175067901611], 'magnitude': 6.596154689788818, 'distance': 7.09453010559082, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5933128190732816, 'motion_component': -3.9135829908792417}, {'ion': 2434, 'force': [3.7240912914276123, -11.90422248840332, -1.445675253868103], 'magnitude': 12.556645393371582, 'distance': 5.142002105712891, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.470498550170999, 'motion_component': 5.9078834976516035}, {'ion': 2443, 'force': [6.2700324058532715, 1.4708256721496582, 1.2446987628936768], 'magnitude': 6.559413909912109, 'distance': 7.114371299743652, 'before_closest_residue': 'SF', 'closest_residue': 1105, 'next_closest_residue': 'SF', 'cosine_with_motion': -0.8427926757632486, 'motion_component': -5.528225916871648}]}, 5695: {'frame': 5695, 'ionic_force': [-17.885726302862167, -13.695586919784546, -6.164025843143463], 'ionic_force_magnitude': 23.35516048014249, 'motion_vector': [2.018024444580078, -2.0229759216308594, -1.58453369140625], 'cosine_ionic_motion': 0.01807265163752099, 'ionic_motion_component': 0.4220896792960127, 'ionic_force_x': -17.885726302862167, 'ionic_force_y': -13.695586919784546, 'ionic_force_z': -6.164025843143463, 'radial_force': 22.527057208127943, 'axial_force': -6.164025843143463, 'before_closest_residue': 423, 'closest_residue': 1105, 'next_closest_residue': 780, 'contributions': [{'ion': 1355, 'force': [-0.28277072310447693, -0.719104528427124, -1.999786376953125], 'magnitude': 2.143878698348999, 'distance': 12.444255828857422, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5785769589171919, 'motion_component': 1.240398856016542}, {'ion': 1469, 'force': [-9.842928886413574, 4.126557350158691, -0.23699882626533508], 'magnitude': 10.67557430267334, 'distance': 5.576650142669678, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.7980207558039879, 'motion_component': -8.519330112078663}, {'ion': 1476, 'force': [-1.4224494695663452, -3.3690109252929688, -5.0304341316223145], 'magnitude': 6.219233512878418, 'distance': 7.306352615356445, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5863940567574065, 'motion_component': 3.646921530555055}, {'ion': 2434, 'force': [-1.0529464483261108, -2.425291061401367, -0.3027394115924835], 'magnitude': 2.6612749099731445, 'distance': 11.169254302978516, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 130, 'cosine_with_motion': 0.37504453080532796, 'motion_component': 0.9980965971669695}, {'ion': 2443, 'force': [-5.28463077545166, -11.308737754821777, 1.405932903289795], 'magnitude': 12.561509132385254, 'distance': 5.141005992889404, 'before_closest_residue': 1105, 'closest_residue': 'SF', 'next_closest_residue': 98, 'cosine_with_motion': 0.24328309559108077, 'motion_component': 3.0560029014484797}]}, 5696: {'frame': 5696, 'ionic_force': [-15.213935688138008, -14.176376223564148, -12.65572875738144], 'ionic_force_magnitude': 24.3433964831378, 'motion_vector': [-0.21909713745117188, -0.3765602111816406, 0.164337158203125], 'cosine_ionic_motion': 0.5815461614722945, 'ionic_motion_component': 14.15680878196694, 'ionic_force_x': -15.213935688138008, 'ionic_force_y': -14.176376223564148, 'ionic_force_z': -12.65572875738144, 'radial_force': 20.79503503134424, 'axial_force': -12.65572875738144, 'before_closest_residue': 1105, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1355, 'force': [0.09340129792690277, -0.6584328413009644, -1.331163763999939], 'magnitude': 1.4880372285842896, 'distance': 14.936958312988281, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.012579553778028203, 'motion_component': 0.01871884341876351}, {'ion': 1469, 'force': [-16.17984390258789, -5.707157611846924, -8.072161674499512], 'magnitude': 18.960981369018555, 'distance': 4.184452533721924, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.49469054526340944, 'motion_component': 9.379817903545728}, {'ion': 1476, 'force': [0.16498154401779175, -2.0770199298858643, -2.584268808364868], 'magnitude': 3.319589853286743, 'distance': 10.000617980957031, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.20785866103990283, 'motion_component': 0.6900054763974506}, {'ion': 2434, 'force': [-0.31412482261657715, -3.6910321712493896, -0.3123330771923065], 'magnitude': 3.7175185680389404, 'distance': 9.450231552124023, 'before_closest_residue': 423, 'closest_residue': 130, 'next_closest_residue': 130, 'cosine_with_motion': 0.813063294942147, 'motion_component': 3.0225779550752616}, {'ion': 2443, 'force': [1.0216501951217651, -2.042733669281006, -0.35580143332481384], 'magnitude': 2.3115200996398926, 'distance': 11.98450756072998, 'before_closest_residue': 'SF', 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.45238145992863704, 'motion_component': 1.045688783874306}]}, 5697: {'frame': 5697, 'ionic_force': [-14.388794315978885, -13.769953429698944, -10.123002961277962], 'ionic_force_magnitude': 22.341087893781413, 'motion_vector': [-1.5983009338378906, 3.4348678588867188, 0.1610565185546875], 'cosine_ionic_motion': -0.30608964031464103, 'ionic_motion_component': -6.838375557645334, 'ionic_force_x': -14.388794315978885, 'ionic_force_y': -13.769953429698944, 'ionic_force_z': -10.123002961277962, 'radial_force': 19.916049290048065, 'axial_force': -10.123002961277962, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 1105, 'contributions': [{'ion': 1355, 'force': [0.01840483583509922, -0.6926707625389099, -1.3557699918746948], 'magnitude': 1.5225780010223389, 'distance': 14.766557693481445, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.45500860962911804, 'motion_component': -0.692786103021971}, {'ion': 1469, 'force': [-15.130455017089844, -6.483215808868408, -6.229846477508545], 'magnitude': 17.60038948059082, 'distance': 4.3431806564331055, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.013645146477585305, 'motion_component': 0.24015990551625777}, {'ion': 1476, 'force': [0.08019865304231644, -2.2278919219970703, -2.5778114795684814], 'magnitude': 3.408085346221924, 'distance': 9.86992359161377, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6341951047869588, 'motion_component': -2.1613910932444793}, {'ion': 2434, 'force': [-0.08338899910449982, -2.282119035720825, 0.2655191719532013], 'magnitude': 2.2990262508392334, 'distance': 12.017027854919434, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 455, 'cosine_with_motion': -0.8789782128093423, 'motion_component': -2.0207939367997354}, {'ion': 2443, 'force': [0.7264462113380432, -2.0840559005737305, -0.22509418427944183], 'magnitude': 2.2184860706329346, 'distance': 12.233217239379883, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.9932740707349745, 'motion_component': -2.2035646993996467}]}, 5698: {'frame': 5698, 'ionic_force': [-9.738676965236664, -11.330120891332626, -6.976988285779953], 'ionic_force_magnitude': 16.48914291239402, 'motion_vector': [-2.993671417236328, -2.5537109375, 1.6241912841796875], 'cosine_ionic_motion': 0.6661082666101348, 'ionic_motion_component': 10.98355440326157, 'ionic_force_x': -9.738676965236664, 'ionic_force_y': -11.330120891332626, 'ionic_force_z': -6.976988285779953, 'radial_force': 14.940330265608027, 'axial_force': -6.976988285779953, 'before_closest_residue': 780, 'closest_residue': 1105, 'next_closest_residue': 1073, 'contributions': [{'ion': 1355, 'force': [-0.1521759033203125, -0.4667292535305023, -1.7436898946762085], 'magnitude': 1.8114768266677856, 'distance': 13.537941932678223, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.15362174844894844, 'motion_component': -0.2782822313194284}, {'ion': 1469, 'force': [-6.2060546875, 1.8714954853057861, -0.3370665907859802], 'magnitude': 6.490856647491455, 'distance': 7.151844024658203, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.4796095587467847, 'motion_component': 3.1130770405235584}, {'ion': 1476, 'force': [-0.9171950221061707, -2.0580520629882812, -4.527716159820557], 'magnitude': 5.057374477386475, 'distance': 8.102265357971191, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.030079234334032482, 'motion_component': 0.15212195803306727}, {'ion': 2434, 'force': [-3.975003957748413, -6.597219944000244, 0.32685384154319763], 'magnitude': 7.709137439727783, 'distance': 6.5624518394470215, 'before_closest_residue': 130, 'closest_residue': 455, 'next_closest_residue': 130, 'cosine_with_motion': 0.8921549445409725, 'motion_component': 6.877745132606193}, {'ion': 2443, 'force': [1.5117526054382324, -4.079615116119385, -0.6953694820404053], 'magnitude': 4.4059271812438965, 'distance': 8.680612564086914, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.25395165049253243, 'motion_component': 1.1188924746078683}]}, 5699: {'frame': 5699, 'ionic_force': [-7.502817556262016, -9.551654130220413, -3.1742424368858337], 'ionic_force_magnitude': 12.553970804253016, 'motion_vector': [-0.2769050598144531, -0.16832733154296875, 0.20163726806640625], 'cosine_ionic_motion': 0.635580549251634, 'ionic_motion_component': 7.979059659056109, 'ionic_force_x': -7.502817556262016, 'ionic_force_y': -9.551654130220413, 'ionic_force_z': -3.1742424368858337, 'radial_force': 12.14604330248786, 'axial_force': -3.1742424368858337, 'before_closest_residue': 1105, 'closest_residue': 1073, 'next_closest_residue': 1073, 'contributions': [{'ion': 1355, 'force': [-0.6258348226547241, -0.9120814800262451, -1.6169955730438232], 'magnitude': 1.959141731262207, 'distance': 13.017755508422852, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.001041146067423937, 'motion_component': 0.0020397527652349368}, {'ion': 1469, 'force': [-3.346435785293579, -0.3936164677143097, 0.2601182758808136], 'magnitude': 3.379530668258667, 'distance': 9.91153335571289, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.8104449305357946, 'motion_component': 2.7389235418649394}, {'ion': 1476, 'force': [-2.058412790298462, -2.6242835521698, -2.340930461883545], 'magnitude': 4.074786186218262, 'distance': 9.026442527770996, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.3470317338278969, 'motion_component': 1.414080129720439}, {'ion': 2434, 'force': [-1.4498467445373535, -2.6175620555877686, 0.3526051938533783], 'magnitude': 3.012974739074707, 'distance': 10.497147560119629, 'before_closest_residue': 455, 'closest_residue': 130, 'next_closest_residue': 130, 'cosine_with_motion': 0.7941024342820463, 'motion_component': 2.3926106197890356}, {'ion': 2443, 'force': [-0.022287413477897644, -3.00411057472229, 0.17096012830734253], 'magnitude': 3.0090537071228027, 'distance': 10.503984451293945, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.47569963817289296, 'motion_component': 1.4314057776705322}]}, 5700: {'frame': 5700, 'ionic_force': [-7.085268452763557, -8.294093906879425, -2.452709883451462], 'ionic_force_magnitude': 11.180733811170061, 'motion_vector': [0.4935493469238281, -0.46282196044921875, 0.6883697509765625], 'cosine_ionic_motion': -0.12478037358923734, 'ionic_motion_component': -1.3951361419596175, 'ionic_force_x': -7.085268452763557, 'ionic_force_y': -8.294093906879425, 'ionic_force_z': -2.452709883451462, 'radial_force': 10.908392309770532, 'axial_force': -2.452709883451462, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'contributions': [{'ion': 1355, 'force': [-0.5744865536689758, -0.7606053352355957, -1.4772404432296753], 'magnitude': 1.7580655813217163, 'distance': 13.742049217224121, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5588955682721238, 'motion_component': -0.9825750645518134}, {'ion': 1469, 'force': [-3.6154754161834717, -0.5478944182395935, 0.3197089731693268], 'magnitude': 3.670703649520874, 'distance': 9.510303497314453, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.3699541929998266, 'motion_component': -1.3579921723084798}, {'ion': 1476, 'force': [-1.7856495380401611, -2.236912727355957, -2.2723193168640137], 'magnitude': 3.654552936553955, 'distance': 9.531294822692871, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.3997822563788361, 'motion_component': -1.4610254591911342}, {'ion': 2434, 'force': [-0.9666056632995605, -1.7378770112991333, 0.8489934206008911], 'magnitude': 2.1622519493103027, 'distance': 12.39127254486084, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 780, 'cosine_with_motion': 0.4368284570045849, 'motion_component': 0.9445331170802014}, {'ion': 2443, 'force': [-0.14305128157138824, -3.0108044147491455, 0.12814748287200928], 'magnitude': 3.016923666000366, 'distance': 10.490275382995605, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.48457418995848245, 'motion_component': 1.4619233628143808}]}, 5701: {'frame': 5701, 'ionic_force': [-7.92530158162117, -8.08792930841446, -1.2593768686056137], 'ionic_force_magnitude': 11.393464607165614, 'motion_vector': [0.5581855773925781, 0.4502677917480469, 0.15650177001953125], 'cosine_ionic_motion': -0.9879751759881211, 'ionic_motion_component': -11.256460200378877, 'ionic_force_x': -7.92530158162117, 'ionic_force_y': -8.08792930841446, 'ionic_force_z': -1.2593768686056137, 'radial_force': 11.323648071957933, 'axial_force': -1.2593768686056137, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'contributions': [{'ion': 1355, 'force': [-0.6315168142318726, -1.0191653966903687, -1.574242353439331], 'magnitude': 1.978825569152832, 'distance': 12.952848434448242, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7282307151891029, 'motion_component': -1.441041549650734}, {'ion': 1469, 'force': [-3.8441007137298584, -0.7395055890083313, 0.717881441116333], 'magnitude': 3.979865789413452, 'distance': 9.13344955444336, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.8100171774076058, 'motion_component': -3.223759742268882}, {'ion': 1476, 'force': [-1.9888440370559692, -2.9822001457214355, -2.092775821685791], 'magnitude': 4.150750637054443, 'distance': 8.943463325500488, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.9125854852277061, 'motion_component': -3.787914575494952}, {'ion': 2434, 'force': [-1.2842319011688232, -1.5509859323501587, 1.57150137424469], 'magnitude': 2.554295539855957, 'distance': 11.400751113891602, 'before_closest_residue': 130, 'closest_residue': 780, 'next_closest_residue': 130, 'cosine_with_motion': -0.623623740374531, 'motion_component': -1.592919314496072}, {'ion': 2443, 'force': [-0.1766081154346466, -1.796072244644165, 0.11825849115848541], 'magnitude': 1.8086047172546387, 'distance': 13.548686981201172, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.6694801324993472, 'motion_component': -1.2108249223917582}]}, 5702: {'frame': 5702, 'ionic_force': [-7.804108589887619, -8.228433191776276, -0.8812482059001923], 'ionic_force_magnitude': 11.37487679382443, 'motion_vector': [-0.39960479736328125, -0.060466766357421875, -0.1700592041015625], 'cosine_ionic_motion': 0.755066697342409, 'ionic_motion_component': 8.588790653389824, 'ionic_force_x': -7.804108589887619, 'ionic_force_y': -8.228433191776276, 'ionic_force_z': -0.8812482059001923, 'radial_force': 11.340688853605112, 'axial_force': -0.8812482059001923, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'contributions': [{'ion': 1355, 'force': [-0.5931767225265503, -0.9305346608161926, -1.5677777528762817], 'magnitude': 1.9172064065933228, 'distance': 13.159355163574219, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.6660555764511565, 'motion_component': 1.276966028057073}, {'ion': 1469, 'force': [-4.320357799530029, -0.4477121829986572, 0.8675047755241394], 'magnitude': 4.4292778968811035, 'distance': 8.65770149230957, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.8269179285556999, 'motion_component': 3.662649262649394}, {'ion': 1476, 'force': [-1.978808045387268, -2.9532740116119385, -2.4418883323669434], 'magnitude': 4.312809467315674, 'distance': 8.773823738098145, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.7321725204097072, 'motion_component': 3.1577207300576404}, {'ion': 2434, 'force': [-0.7739160060882568, -1.956164002418518, 2.087541341781616], 'magnitude': 2.963671922683716, 'distance': 10.584100723266602, 'before_closest_residue': 780, 'closest_residue': 130, 'next_closest_residue': 1105, 'cosine_with_motion': 0.05581996945277117, 'motion_component': 0.16543208727818737}, {'ion': 2443, 'force': [-0.13785001635551453, -1.9407483339309692, 0.17337176203727722], 'magnitude': 1.9533469676971436, 'distance': 13.037050247192383, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.16690467565863135, 'motion_component': 0.3260227469765544}]}, 5703: {'frame': 5703, 'ionic_force': [-7.383249953389168, -8.355258643627167, -1.0149785578250885], 'ionic_force_magnitude': 11.196111304777759, 'motion_vector': [-0.3843231201171875, 0.9410591125488281, -0.6316909790039062], 'cosine_ionic_motion': -0.32718268002181145, 'ionic_motion_component': -3.6631737025196873, 'ionic_force_x': -7.383249953389168, 'ionic_force_y': -8.355258643627167, 'ionic_force_z': -1.0149785578250885, 'radial_force': 11.15001017381274, 'axial_force': -1.0149785578250885, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'contributions': [{'ion': 1355, 'force': [-0.60088050365448, -0.9079782366752625, -1.5684553384780884], 'magnitude': 1.9093282222747803, 'distance': 13.18647575378418, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.16071629272356294, 'motion_component': 0.30686014280205853}, {'ion': 1469, 'force': [-3.552804470062256, -0.41763007640838623, 0.6142292618751526], 'magnitude': 3.6296157836914062, 'distance': 9.563981056213379, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.13453440074523831, 'motion_component': 0.48830820908270667}, {'ion': 1476, 'force': [-2.070937156677246, -2.9030516147613525, -2.323512554168701], 'magnitude': 4.256195545196533, 'distance': 8.83198356628418, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.09193349991236771, 'motion_component': -0.39128694689864574}, {'ion': 2434, 'force': [-1.004224419593811, -1.850171685218811, 2.136342763900757], 'magnitude': 2.999260425567627, 'distance': 10.521120071411133, 'before_closest_residue': 130, 'closest_residue': 1105, 'next_closest_residue': 780, 'cosine_with_motion': -0.7534954304754614, 'motion_component': -2.2599289317871296}, {'ion': 2443, 'force': [-0.15440340340137482, -2.2764270305633545, 0.12641730904579163], 'magnitude': 2.285156726837158, 'distance': 12.05344009399414, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.7908105052909971, 'motion_component': -1.8071260334216284}]}, 5704: {'frame': 5704, 'ionic_force': [-9.369131922721863, -6.612637624144554, -1.1421239897608757], 'ionic_force_magnitude': 11.524411331673532, 'motion_vector': [0.2603874206542969, -0.4796562194824219, 0.38088226318359375], 'cosine_ionic_motion': 0.03874520782907011, 'ionic_motion_component': 0.4465157121533816, 'ionic_force_x': -9.369131922721863, 'ionic_force_y': -6.612637624144554, 'ionic_force_z': -1.1421239897608757, 'radial_force': 11.467676719092582, 'axial_force': -1.1421239897608757, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'contributions': [{'ion': 1355, 'force': [-0.6172433495521545, -0.7568070888519287, -1.5594958066940308], 'magnitude': 1.8400471210479736, 'distance': 13.432429313659668, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.3198527868126092, 'motion_component': -0.5885442069841993}, {'ion': 1469, 'force': [-3.870227813720703, 0.14175964891910553, 0.3387364447116852], 'magnitude': 3.887608766555786, 'distance': 9.24118709564209, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.36590838633313716, 'motion_component': -1.4225086309504258}, {'ion': 1476, 'force': [-2.3841171264648438, -2.5097689628601074, -2.422724962234497], 'magnitude': 4.2252278327941895, 'distance': 8.864290237426758, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.12081579075749667, 'motion_component': -0.5104742520899492}, {'ion': 2434, 'force': [-2.1380257606506348, -1.4192434549331665, 2.406752109527588], 'magnitude': 3.518218517303467, 'distance': 9.714213371276855, 'before_closest_residue': 1105, 'closest_residue': 780, 'next_closest_residue': 130, 'cosine_with_motion': 0.444465918681543, 'motion_component': 1.5637282455528023}, {'ion': 2443, 'force': [-0.3595178723335266, -2.068577766418457, 0.09460822492837906], 'magnitude': 2.101717710494995, 'distance': 12.568453788757324, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.6681745362650324, 'motion_component': 1.4043143293516351}]}, 5705: {'frame': 5705, 'ionic_force': [-7.721536681056023, -8.126845806837082, -1.4946873784065247], 'ionic_force_magnitude': 11.309369648400695, 'motion_vector': [-0.3619537353515625, 0.5146217346191406, -0.38831329345703125], 'cosine_ionic_motion': -0.09651394143405095, 'ionic_motion_component': -1.091511839901778, 'ionic_force_x': -7.721536681056023, 'ionic_force_y': -8.126845806837082, 'ionic_force_z': -1.4946873784065247, 'radial_force': 11.210162866122825, 'axial_force': -1.4946873784065247, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'contributions': [{'ion': 1355, 'force': [-0.6187195181846619, -0.849595308303833, -1.482783317565918], 'magnitude': 1.8174906969070435, 'distance': 13.515525817871094, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.2697753721747423, 'motion_component': 0.49031422647946593}, {'ion': 1469, 'force': [-3.246384620666504, -0.28951355814933777, 0.4443724453449249], 'magnitude': 3.2894222736358643, 'distance': 10.046371459960938, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.35094051822464967, 'motion_component': 1.1543915137098413}, {'ion': 1476, 'force': [-2.1111855506896973, -2.8807077407836914, -2.3419687747955322], 'magnitude': 4.270877838134766, 'distance': 8.816789627075195, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.06051771865582957, 'motion_component': 0.2584637958280638}, {'ion': 2434, 'force': [-1.5408753156661987, -2.4781036376953125, 1.7578200101852417], 'magnitude': 3.406644344329834, 'distance': 9.872011184692383, 'before_closest_residue': 780, 'closest_residue': 130, 'next_closest_residue': 455, 'cosine_with_motion': -0.5559020648508023, 'motion_component': -1.8937606151929602}, {'ion': 2443, 'force': [-0.20437167584896088, -1.6289255619049072, 0.127872258424758</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>5891</v>
+      </c>
+      <c r="B20" t="n">
+        <v>6489</v>
+      </c>
+      <c r="C20" t="n">
+        <v>1476</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>{5891: {'frame': 5891, 'ionic_force': [-1.5849148631095886, 7.950932557694614, -11.96000251173973], 'ionic_force_magnitude': 14.448908046670327, 'motion_vector': [-0.0869140625, 0.02236175537109375, -1.756866455078125], 'cosine_ionic_motion': 0.8390809281841389, 'ionic_motion_component': 12.123803175047412, 'ionic_force_x': -1.5849148631095886, 'ionic_force_y': 7.950932557694614, 'ionic_force_z': -11.96000251173973, 'radial_force': 8.10735984524641, 'axial_force': -11.96000251173973, 'before_closest_residue': None, 'closest_residue': 130, 'next_closest_residue': 130, 'contributions': [{'ion': 1355, 'force': [-1.7060837745666504, 0.8367077708244324, -5.490914821624756], 'magnitude': 5.810417175292969, 'distance': 7.559018135070801, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.9601190966229708, 'motion_component': 5.578692453569913}, {'ion': 1380, 'force': [7.263280868530273, 6.749550819396973, -3.8440001010894775], 'magnitude': 10.634284973144531, 'distance': 5.587465763092041, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.3353246454323799, 'motion_component': 3.5659379188627023}, {'ion': 1443, 'force': [-0.4787597060203552, 0.010035867802798748, -2.1720573902130127], 'magnitude': 2.2242178916931152, 'distance': 12.21744441986084, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.9859692911877616, 'motion_component': 2.1930104608552266}, {'ion': 2434, 'force': [-3.879657030105591, -2.270467758178711, -0.30914631485939026], 'magnitude': 4.5058112144470215, 'distance': 8.583858489990234, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.10465668711356463, 'motion_component': 0.47156326582191443}, {'ion': 2443, 'force': [-2.7836952209472656, 2.625105857849121, -0.14388388395309448], 'magnitude': 3.8289480209350586, 'distance': 9.311707496643066, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.08216328848026491, 'motion_component': 0.3145989551665549}]}, 5892: {'frame': 5892, 'ionic_force': [-2.49815434217453, 7.7181031331419945, -11.375910818576813], 'ionic_force_magnitude': 13.972159390851319, 'motion_vector': [1.8442268371582031, 0.5494155883789062, -1.9481353759765625], 'cosine_ionic_motion': 0.5696590418762275, 'ionic_motion_component': 7.959366931534297, 'ionic_force_x': -2.49815434217453, 'ionic_force_y': 7.7181031331419945, 'ionic_force_z': -11.375910818576813, 'radial_force': 8.112329572394216, 'axial_force': -11.375910818576813, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 130, 'contributions': [{'ion': 1355, 'force': [-1.323460340499878, 0.5493678450584412, -3.9731087684631348], 'magnitude': 4.2236175537109375, 'distance': 8.86598014831543, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.4843039886928752, 'motion_component': 2.045514847932078}, {'ion': 1380, 'force': [4.6296796798706055, 6.161921977996826, -3.7464330196380615], 'magnitude': 8.56965446472168, 'distance': 6.224255084991455, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.8191423334410239, 'motion_component': 7.019766713293727}, {'ion': 1443, 'force': [-0.2683507800102234, 0.09991147369146347, -1.5568095445632935], 'magnitude': 1.582924723625183, 'distance': 14.482345581054688, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5981912216623002, 'motion_component': 0.9468916215238075}, {'ion': 2434, 'force': [-3.6428050994873047, -2.0931317806243896, -1.1591386795043945], 'magnitude': 4.358306407928467, 'distance': 8.72790813446045, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.4700724450400846, 'motion_component': -2.048719607946321}, {'ion': 2443, 'force': [-1.8932178020477295, 3.0000336170196533, -0.9404208064079285], 'magnitude': 3.6699955463409424, 'distance': 9.511220932006836, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 780, 'cosine_with_motion': -0.0011135754220507616, 'motion_component': -0.004086816738126942}]}, 5893: {'frame': 5893, 'ionic_force': [-2.40166874229908, 3.821544498205185, -9.344871044158936], 'ionic_force_magnitude': 10.377804677842944, 'motion_vector': [1.5363502502441406, -0.806884765625, 5.4425048828125], 'cosine_ionic_motion': -0.9721669729770439, 'ionic_motion_component': -10.08895895980558, 'ionic_force_x': -2.40166874229908, 'ionic_force_y': 3.821544498205185, 'ionic_force_z': -9.344871044158936, 'radial_force': 4.513559028028632, 'axial_force': -9.344871044158936, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 'SF', 'contributions': [{'ion': 1355, 'force': [-0.15968115627765656, 0.468254417181015, -2.7393507957458496], 'magnitude': 2.7836670875549316, 'distance': 10.92094898223877, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.9767616758619528, 'motion_component': -2.7189794345203118}, {'ion': 1380, 'force': [2.5271170139312744, 2.5101613998413086, -2.471982479095459], 'magnitude': 4.335657596588135, 'distance': 8.750675201416016, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.4682241377097566, 'motion_component': -2.030059606386061}, {'ion': 2434, 'force': [-3.2794134616851807, -2.170670509338379, -2.4210591316223145], 'magnitude': 4.618212699890137, 'distance': 8.478754997253418, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.6240561968776958, 'motion_component': -2.882024381575036}, {'ion': 2443, 'force': [-1.489691138267517, 3.0137991905212402, -1.7124786376953125], 'magnitude': 3.7728965282440186, 'distance': 9.380620956420898, 'before_closest_residue': 748, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.6514611145093603, 'motion_component': -2.457895387573828}]}, 5895: {'frame': 5895, 'ionic_force': [5.1735977828502655, -3.9379420280456543, -22.839519739151], 'ionic_force_magnitude': 23.746940083935648, 'motion_vector': [-0.4307060241699219, 1.0893287658691406, 5.436920166015625], 'cosine_ionic_motion': -0.9895653006108213, 'ionic_motion_component': -23.49914790274694, 'ionic_force_x': 5.1735977828502655, 'ionic_force_y': -3.9379420280456543, 'ionic_force_z': -22.839519739151, 'radial_force': 6.5018075513630444, 'axial_force': -22.839519739151, 'before_closest_residue': 'SF', 'closest_residue': 130, 'next_closest_residue': 'SF', 'contributions': [{'ion': 1355, 'force': [-0.23459890484809875, -0.226188063621521, -2.4711523056030273], 'magnitude': 2.4925472736358643, 'distance': 11.54110336303711, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.9796625124195689, 'motion_component': -2.441855024673414}, {'ion': 1380, 'force': [2.8447628021240234, 1.016716718673706, -3.0548858642578125], 'magnitude': 4.296360492706299, 'distance': 8.790602684020996, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.700017157373819, 'motion_component': -3.0075262584837823}, {'ion': 2434, 'force': [-1.8455193042755127, -1.5154215097427368, -1.5823023319244385], 'magnitude': 2.864633321762085, 'distance': 10.765507698059082, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.5936900479778674, 'motion_component': -1.700704341499744}, {'ion': 2443, 'force': [4.4089531898498535, -3.2130491733551025, -15.731179237365723], 'magnitude': 16.650300979614258, 'distance': 4.4653754234313965, 'before_closest_residue': 780, 'closest_residue': 130, 'next_closest_residue': 130, 'cosine_with_motion': -0.9819078479353249, 'motion_component': -16.349062107802858}]}, 5897: {'frame': 5897, 'ionic_force': [1.8552783280611038, -2.173237666487694, -12.846055001020432], 'ionic_force_magnitude': 13.160020847964342, 'motion_vector': [-2.82208251953125, 5.449005126953125, 2.03216552734375], 'cosine_ionic_motion': -0.5076259578248576, 'ionic_motion_component': -6.680368187942994, 'ionic_force_x': 1.8552783280611038, 'ionic_force_y': -2.173237666487694, 'ionic_force_z': -12.846055001020432, 'radial_force': 2.8574498472613796, 'axial_force': -12.846055001020432, 'before_closest_residue': 'SF', 'closest_residue': 1105, 'next_closest_residue': 98, 'contributions': [{'ion': 1355, 'force': [-0.9138748049736023, -0.6297469139099121, -4.202837944030762], 'magnitude': 4.346906661987305, 'distance': 8.73934555053711, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.33429224387299245, 'motion_component': -1.4531370892927156}, {'ion': 1380, 'force': [9.447088241577148, 4.048842430114746, -5.9594407081604], 'magnitude': 11.880888938903809, 'distance': 5.286211967468262, 'before_closest_residue': 1073, 'closest_residue': 1105, 'next_closest_residue': 1073, 'cosine_with_motion': -0.21756311411583418, 'motion_component': -2.584843313608019}, {'ion': 1443, 'force': [-0.18578504025936127, -0.21087370812892914, -1.5908935070037842], 'magnitude': 1.615526556968689, 'distance': 14.335472106933594, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.36940491676610593, 'motion_component': -0.5967834414567519}, {'ion': 2434, 'force': [-1.8904106616973877, -2.4841415882110596, -0.7933556437492371], 'magnitude': 3.2208733558654785, 'distance': 10.152715682983398, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.47134032227528494, 'motion_component': -1.51812747847017}, {'ion': 2443, 'force': [-4.601739406585693, -2.897317886352539, -0.29952719807624817], 'magnitude': 5.446115493774414, 'distance': 7.807744979858398, 'before_closest_residue': 130, 'closest_residue': 455, 'next_closest_residue': 780, 'cosine_with_motion': -0.09685378485089452, 'motion_component': -0.527476890051453}]}, 5898: {'frame': 5898, 'ionic_force': [-8.504436016082764, 11.964142084121704, -4.874931126832962], 'ionic_force_magnitude': 15.467096729899332, 'motion_vector': [1.28692626953125, 1.0255928039550781, -0.0074005126953125], 'cosine_ionic_motion': 0.053503810279040165, 'ionic_motion_component': 0.8275486090040964, 'ionic_force_x': -8.504436016082764, 'ionic_force_y': 11.964142084121704, 'ionic_force_z': -4.874931126832962, 'radial_force': 14.678764517516374, 'axial_force': -4.874931126832962, 'before_closest_residue': 1105, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1355, 'force': [-2.246494770050049, 1.9543259143829346, -3.1174850463867188], 'magnitude': 4.311013698577881, 'distance': 8.775650978088379, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.12173989718526873, 'motion_component': -0.5248223988331979}, {'ion': 1380, 'force': [1.3024711608886719, 6.837247848510742, -1.0843136310577393], 'magnitude': 7.044155597686768, 'distance': 6.865221977233887, 'before_closest_residue': 1105, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.7502090673975343, 'motion_component': 5.2845892541990045}, {'ion': 1443, 'force': [-0.6266984939575195, 0.5076103806495667, -1.6870962381362915], 'magnitude': 1.8699499368667603, 'distance': 13.32459545135498, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.08885512461797455, 'motion_component': -0.16615464063826718}, {'ion': 2434, 'force': [-3.711239814758301, -0.4314489960670471, -0.2661377489566803], 'magnitude': 3.745701313018799, 'distance': 9.414612770080566, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.8463017020136312, 'motion_component': -3.1699934160905885}, {'ion': 2443, 'force': [-3.2224740982055664, 3.096406936645508, 1.2801015377044678], 'magnitude': 4.6487345695495605, 'distance': 8.450874328613281, 'before_closest_residue': 455, 'closest_residue': 780, 'next_closest_residue': 748, 'cosine_with_motion': -0.12822213597355978, 'motion_component': -0.5960707047619811}]}, 5899: {'frame': 5899, 'ionic_force': [-6.799471914768219, 9.492137521505356, -5.600397616624832], 'ionic_force_magnitude': 12.949824188427762, 'motion_vector': [-1.2925643920898438, 0.4482421875, -0.7178955078125], 'cosine_ionic_motion': 0.8528839683401198, 'ionic_motion_component': 11.04469744313314, 'ionic_force_x': -6.799471914768219, 'ionic_force_y': 9.492137521505356, 'ionic_force_z': -5.600397616624832, 'radial_force': 11.676193431375298, 'axial_force': -5.600397616624832, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1355, 'force': [-1.5860280990600586, 2.484849214553833, -3.0621752738952637], 'magnitude': 4.250514984130859, 'distance': 8.837882995605469, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.816529670001961, 'motion_component': 3.4706716480274054}, {'ion': 1380, 'force': [1.502514123916626, 3.8119521141052246, -0.36482638120651245], 'magnitude': 4.113590717315674, 'distance': 8.98376750946045, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.00448254038297453, 'motion_component': 0.01843933504465589}, {'ion': 1443, 'force': [-0.44899803400039673, 0.7380704879760742, -1.5459970235824585], 'magnitude': 1.7710037231445312, 'distance': 13.691761016845703, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.7386375500883181, 'motion_component': 1.3081298281740104}, {'ion': 2434, 'force': [-5.232437610626221, -0.4004041254520416, -0.13199836015701294], 'magnitude': 5.249395370483398, 'distance': 7.952696323394775, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.8234643314790869, 'motion_component': 4.322689741515248}, {'ion': 2443, 'force': [-1.034522294998169, 2.8576698303222656, -0.4954005777835846], 'magnitude': 3.079274892807007, 'distance': 10.383524894714355, 'before_closest_residue': 780, 'closest_residue': 748, 'next_closest_residue': 780, 'cosine_with_motion': 0.6250715130958738, 'motion_component': 1.9247671286365629}]}, 5900: {'frame': 5900, 'ionic_force': [-6.1381120681762695, 8.840319886803627, -5.065477430820465], 'ionic_force_magnitude': 11.894819757552376, 'motion_vector': [1.6382980346679688, 0.11060333251953125, 0.5860443115234375], 'cosine_ionic_motion': -0.5808999323825219, 'ionic_motion_component': -6.909699992864462, 'ionic_force_x': -6.1381120681762695, 'ionic_force_y': 8.840319886803627, 'ionic_force_z': -5.065477430820465, 'radial_force': 10.762326675143571, 'axial_force': -5.065477430820465, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1355, 'force': [-1.8010727167129517, 2.0751216411590576, -2.528494358062744], 'magnitude': 3.734069585800171, 'distance': 9.429265022277832, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6455951833243415, 'motion_component': -2.4106974082634594}, {'ion': 1380, 'force': [0.7935147881507874, 3.8666439056396484, -0.5172351598739624], 'magnitude': 3.980971336364746, 'distance': 9.132181167602539, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1105, 'cosine_with_motion': 0.20524595466575268, 'motion_component': 0.8170782686594613}, {'ion': 1443, 'force': [-0.539768397808075, 0.6087048649787903, -1.3261784315109253], 'magnitude': 1.555834412574768, 'distance': 14.607885360717773, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5877023443381678, 'motion_component': -0.9143675408841645}, {'ion': 2434, 'force': [-3.400973320007324, 0.1036798506975174, -0.37451714277267456], 'magnitude': 3.423102617263794, 'distance': 9.848250389099121, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.9684545174849846, 'motion_component': -3.315119277919867}, {'ion': 2443, 'force': [-1.189812421798706, 2.1861696243286133, -0.3190523386001587], 'magnitude': 2.5093395709991455, 'distance': 11.502422332763672, 'before_closest_residue': 748, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.4330199266346829, 'motion_component': -1.0865940833195076}]}, 5901: {'frame': 5901, 'ionic_force': [-7.439622104167938, 9.131087750196457, -4.992527484893799], 'ionic_force_magnitude': 12.792578756530364, 'motion_vector': [-0.2744865417480469, -0.7472152709960938, 0.6619415283203125], 'cosine_ionic_motion': -0.6105029271010953, 'ionic_motion_component': -7.809906776033078, 'ionic_force_x': -7.439622104167938, 'ionic_force_y': 9.131087750196457, 'ionic_force_z': -4.992527484893799, 'radial_force': 11.77814673684328, 'axial_force': -4.992527484893799, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1355, 'force': [-1.4037278890609741, 2.735112428665161, -2.956904888153076], 'magnitude': 4.265510082244873, 'distance': 8.822335243225098, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8187622495734076, 'motion_component': -3.4924388454826705}, {'ion': 1380, 'force': [1.2992652654647827, 3.4894778728485107, -0.26489782333374023], 'magnitude': 3.7329232692718506, 'distance': 9.430712699890137, 'before_closest_residue': 1073, 'closest_residue': 1105, 'next_closest_residue': 1073, 'cosine_with_motion': -0.8123221702917955, 'motion_component': -3.032336416243023}, {'ion': 1443, 'force': [-0.41779905557632446, 0.741924524307251, -1.4480189085006714], 'magnitude': 1.6798115968704224, 'distance': 14.058492660522461, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8039778328249968, 'motion_component': -1.3505312414997288}, {'ion': 2434, 'force': [-5.164675235748291, 0.30420610308647156, -0.35055652260780334], 'magnitude': 5.185489654541016, 'distance': 8.001550674438477, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.17849948460629902, 'motion_component': 0.9256072060184977}, {'ion': 2443, 'force': [-1.7526851892471313, 1.8603668212890625, 0.02785065770149231], 'magnitude': 2.5560996532440186, 'distance': 11.396726608276367, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 748, 'cosine_with_motion': -0.3365313831905415, 'motion_component': -0.8602077719029388}]}, 5902: {'frame': 5902, 'ionic_force': [-7.47670590877533, 10.180595852434635, -5.091444402933121], 'ionic_force_magnitude': 13.618680892989754, 'motion_vector': [-0.6989402770996094, 0.07197189331054688, -0.5127105712890625], 'cosine_ionic_motion': 0.7233805888715068, 'ionic_motion_component': 9.851489404024067, 'ionic_force_x': -7.47670590877533, 'ionic_force_y': 10.180595852434635, 'ionic_force_z': -5.091444402933121, 'radial_force': 12.631138632638201, 'axial_force': -5.091444402933121, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1355, 'force': [-2.3436784744262695, 3.635133743286133, -3.490668773651123], 'magnitude': 5.558038711547852, 'distance': 7.728732109069824, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.7631541126482841, 'motion_component': 4.241640120977877}, {'ion': 1380, 'force': [1.7799241542816162, 3.8899707794189453, -0.24371981620788574], 'magnitude': 4.284787178039551, 'distance': 8.802467346191406, 'before_closest_residue': 1105, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.2251530332435537, 'motion_component': -0.9647328522041647}, {'ion': 1443, 'force': [-0.6318591833114624, 0.8132873177528381, -1.8050473928451538], 'magnitude': 2.078191041946411, 'distance': 12.639395713806152, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.7886742332344485, 'motion_component': 1.6390157971740118}, {'ion': 2434, 'force': [-4.041162490844727, 0.0778370276093483, 0.15670618414878845], 'magnitude': 4.044948577880859, 'distance': 9.059673309326172, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.7815590684252294, 'motion_component': 3.161366311019386}, {'ion': 2443, 'force': [-2.2399299144744873, 1.7643669843673706, 0.2912853956222534], 'magnitude': 2.866203784942627, 'distance': 10.762557983398438, 'before_closest_residue': 780, 'closest_residue': 748, 'next_closest_residue': 780, 'cosine_with_motion': 0.6190068769033602, 'motion_component': 1.7741998450811902}]}, 5903: {'frame': 5903, 'ionic_force': [-7.226976692676544, 9.150095321238041, -4.231179058551788], 'ionic_force_magnitude': 12.403882969850992, 'motion_vector': [-2.064189910888672, -0.9773674011230469, 0.5256500244140625], 'cosine_ionic_motion': 0.12902546839686596, 'ionic_motion_component': 1.600416810124933, 'ionic_force_x': -7.226976692676544, 'ionic_force_y': 9.150095321238041, 'ionic_force_z': -4.231179058551788, 'radial_force': 11.65990722536986, 'axial_force': -4.231179058551788, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1355, 'force': [-1.8546229600906372, 2.477461338043213, -2.9006059169769287], 'magnitude': 4.241574764251709, 'distance': 8.847192764282227, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.011850426762347991, 'motion_component': -0.05026446999784895}, {'ion': 1380, 'force': [1.4170900583267212, 4.401101589202881, -0.24274271726608276], 'magnitude': 4.629985332489014, 'distance': 8.467968940734863, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.6777590970009262, 'motion_component': -3.1380146253485997}, {'ion': 1443, 'force': [-0.5996553301811218, 0.7718545794487, -1.4985142946243286], 'magnitude': 1.7891035079956055, 'distance': 13.62232780456543, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.07256903406377582, 'motion_component': -0.12983350805516558}, {'ion': 2434, 'force': [-4.2714080810546875, 0.0717788115143776, 0.005224108695983887], 'magnitude': 4.272014141082764, 'distance': 8.815616607666016, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.8739216207863854, 'motion_component': 3.733405692233334}, {'ion': 2443, 'force': [-1.9183803796768188, 1.4278990030288696, 0.40545976161956787], 'magnitude': 2.4255878925323486, 'distance': 11.69931697845459, 'before_closest_residue': 748, 'closest_residue': 780, 'next_closest_residue': 455, 'cosine_with_motion': 0.4885923536268643, 'motion_component': 1.1851236810123673}]}, 5904: {'frame': 5904, 'ionic_force': [-9.568521454930305, 7.556034505367279, -3.6204235684126616], 'ionic_force_magnitude': 12.718401121779435, 'motion_vector': [0.26805877685546875, -0.65460205078125, 0.54949951171875], 'cosine_ionic_motion': -0.8339597165242312, 'ionic_motion_component': -10.606634194160641, 'ionic_force_x': -9.568521454930305, 'ionic_force_y': 7.556034505367279, 'ionic_force_z': -3.6204235684126616, 'radial_force': 12.192221302115644, 'axial_force': -3.6204235684126616, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1355, 'force': [-2.7520177364349365, 2.0397398471832275, -2.4019126892089844], 'magnitude': 4.183697700500488, 'distance': 8.908178329467773, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.9053642438427174, 'motion_component': -3.787770130145411}, {'ion': 1380, 'force': [-0.21680445969104767, 5.097675800323486, -0.02414863370358944], 'magnitude': 5.102341175079346, 'distance': 8.066484451293945, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.7457649127659219, 'motion_component': -3.8051470526533926}, {'ion': 1443, 'force': [-0.8819059133529663, 0.5921956896781921, -1.4838796854019165], 'magnitude': 1.8249253034591675, 'distance': 13.487966537475586, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8806016873471738, 'motion_component': -1.6070323817126706}, {'ion': 2434, 'force': [-3.755582809448242, -0.6733697652816772, -0.06396784633398056], 'magnitude': 3.8160085678100586, 'distance': 9.327481269836426, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.17585336726810966, 'motion_component': -0.671057946384932}, {'ion': 2443, 'force': [-1.9622105360031128, 0.4997929334640503, 0.3534852862358093], 'magnitude': 2.0554840564727783, 'distance': 12.709017753601074, 'before_closest_residue': 780, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': -0.3578848286087576, 'motion_component': -0.7356265858207962}]}, 5905: {'frame': 5905, 'ionic_force': [-9.992130100727081, 6.58165055513382, -3.931290879845619], 'ionic_force_magnitude': 12.594277905529433, 'motion_vector': [0.7903480529785156, -0.9876708984375, -0.41739654541015625], 'cosine_ionic_motion': -0.7604122752570438, 'ionic_motion_component': -9.576843517363152, 'ionic_force_x': -9.992130100727081, 'ionic_force_y': 6.58165055513382, 'ionic_force_z': -3.931290879845619, 'radial_force': 11.964981737543502, 'axial_force': -3.931290879845619, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1355, 'force': [-3.319589138031006, 2.096099615097046, -2.7997121810913086], 'magnitude': 4.822000980377197, 'distance': 8.29765510559082, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5488417217053617, 'motion_component': -2.6465153476760293}, {'ion': 1380, 'force': [-1.1027723550796509, 4.649133205413818, -0.03528514876961708], 'magnitude': 4.778262138366699, 'distance': 8.335545539855957, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.8560484604784877, 'motion_component': -4.090424162976559}, {'ion': 1443, 'force': [-0.942359983921051, 0.5759227275848389, -1.6433050632476807], 'magnitude': 1.9799445867538452, 'distance': 12.949187278747559, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.23800220727946045, 'motion_component': -0.47123119947199754}, {'ion': 2434, 'force': [-2.8171496391296387, -1.0690206289291382, 0.05009468272328377], 'magnitude': 3.0135769844055176, 'distance': 10.496098518371582, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.29684243476094296, 'motion_component': -0.8945575505990111}, {'ion': 2443, 'force': [-1.8102589845657349, 0.32951563596725464, 0.49691683053970337], 'magnitude': 1.9059234857559204, 'distance': 13.198248863220215, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': -0.7734389045849858, 'motion_component': -1.4741154031700958}]}, 5906: {'frame': 5906, 'ionic_force': [-10.922582864761353, 10.523097217082977, -6.046317458152771], 'ionic_force_magnitude': 16.327778363345114, 'motion_vector': [1.9758110046386719, 3.4515724182128906, -0.8893280029296875], 'cosine_ionic_motion': 0.3023330582001712, 'ionic_motion_component': 4.936427166204714, 'ionic_force_x': -10.922582864761353, 'ionic_force_y': 10.523097217082977, 'ionic_force_z': -6.046317458152771, 'radial_force': 15.1670165648277, 'axial_force': -6.046317458152771, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1355, 'force': [-4.033276081085205, 1.9656189680099487, -3.9555554389953613], 'magnitude': 5.981420516967773, 'distance': 7.450181484222412, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.09571965613329209, 'motion_component': 0.5725395255051566}, {'ion': 1380, 'force': [0.23750650882720947, 8.032539367675781, -0.7383502721786499], 'magnitude': 8.06989860534668, 'distance': 6.414089202880859, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.8772632129877416, 'motion_component': 7.079424943052482}, {'ion': 1443, 'force': [-1.2005337476730347, 0.7920025587081909, -2.096895217895508], 'magnitude': 2.542738437652588, 'distance': 11.426630973815918, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.2148583606219969, 'motion_component': 0.5463286174781139}, {'ion': 2434, 'force': [-3.1640639305114746, -0.9320102334022522, 0.2620435059070587], 'magnitude': 3.308868408203125, 'distance': 10.016806602478027, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.7194509242662153, 'motion_component': -2.3805684658359643}, {'ion': 2443, 'force': [-2.7622156143188477, 0.6649465560913086, 0.48243996500968933], 'magnitude': 2.881793975830078, 'distance': 10.733406066894531, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': -0.30581543469071415, 'motion_component': -0.8812971210839531}]}, 5907: {'frame': 5907, 'ionic_force': [-9.553559362888336, 8.830352172255516, -5.354349387693219], 'ionic_force_magnitude': 14.068215002329891, 'motion_vector': [-1.1595115661621094, -0.7659034729003906, 0.1236724853515625], 'cosine_ionic_motion': 0.18607521899512322, 'ionic_motion_component': 2.6177461874290127, 'ionic_force_x': -9.553559362888336, 'ionic_force_y': 8.830352172255516, 'ionic_force_z': -5.354349387693219, 'radial_force': 13.009443338832337, 'axial_force': -5.354349387693219, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'contributions': [{'ion': 1355, 'force': [-1.5680482387542725, 3.1532657146453857, -3.071322202682495], 'magnitude': 4.672780513763428, 'distance': 8.429102897644043, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.14983111096125093, 'motion_component': -0.7001279323548903}, {'ion': 1380, 'force': [0.9171464443206787, 3.123924732208252, -0.38423049449920654], 'magnitude': 3.278367757797241, 'distance': 10.063294410705566, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.7660238977833006, 'motion_component': -2.5113081942758813}, {'ion': 1443, 'force': [-0.6362531781196594, 1.28103506565094, -1.8257994651794434], 'magnitude': 2.3193562030792236, 'distance': 11.964245796203613, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.14500558336337774, 'motion_component': -0.3363195816363458}, {'ion': 2434, 'force': [-5.875592231750488, -0.22285892069339752, -0.07418480515480042], 'magnitude': 5.880284786224365, 'distance': 7.51397705078125, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.8501420158589348, 'motion_component': 4.99907747936747}, {'ion': 2443, 'force': [-2.3908121585845947, 1.494985580444336, 0.0011875798227265477], 'magnitude': 2.8197457790374756, 'distance': 10.850857734680176, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': 0.4136630808352814, 'motion_component': 1.1664247125823328}]}, 5908: {'frame': 5908, 'ionic_force': [-11.456575185060501, 10.54627639055252, -7.669879510998726], 'ionic_force_magnitude': 17.35811373364363, 'motion_vector': [0.8431854248046875, 0.49897003173828125, 0.0274658203125], 'cosine_ionic_motion': -0.2708674020063873, 'ionic_motion_component': -4.701747170763442, 'ionic_force_x': -11.456575185060501, 'ionic_force_y': 10.54627639055252, 'ionic_force_z': -7.669879510998726, 'radial_force': 15.571674947701341, 'axial_f</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>5997</v>
+      </c>
+      <c r="B21" t="n">
+        <v>6562</v>
+      </c>
+      <c r="C21" t="n">
+        <v>1355</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>{5997: {'frame': 5997, 'ionic_force': [9.381639122962952, 3.428868383169174, -11.025252528488636], 'ionic_force_magnitude': 14.877112768933067, 'motion_vector': [0.7771873474121094, 0.3831329345703125, 0.82928466796875], 'cosine_ionic_motion': -0.03015511111987929, 'ionic_motion_component': -0.44862098869015166, 'ionic_force_x': 9.381639122962952, 'ionic_force_y': 3.428868383169174, 'ionic_force_z': -11.025252528488636, 'radial_force': 9.988608062318105, 'axial_force': -11.025252528488636, 'before_closest_residue': None, 'closest_residue': 780, 'next_closest_residue': 455, 'contributions': [{'ion': 1327, 'force': [0.5210571885108948, -0.15596595406532288, -1.7473162412643433], 'magnitude': 1.8300108909606934, 'distance': 13.469212532043457, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5029046882528586, 'motion_component': -0.9203210783935373}, {'ion': 1380, 'force': [3.0363898277282715, 0.8332290053367615, -0.6519385576248169], 'magnitude': 3.2154250144958496, 'distance': 10.161314010620117, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.554497784335778, 'motion_component': 1.782946013499606}, {'ion': 1443, 'force': [2.586791753768921, -0.8877150416374207, -4.0297532081604], 'magnitude': 4.8701581954956055, 'distance': 8.256528854370117, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.28615785628677687, 'motion_component': -1.3936340184841656}, {'ion': 1476, 'force': [1.3487483263015747, -1.712496280670166, -0.039044089615345], 'magnitude': 2.180204153060913, 'distance': 12.340150833129883, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.13757207651808118, 'motion_component': 0.2999352078664286}, {'ion': 2434, 'force': [-0.48151785135269165, -7.0847249031066895, -1.291944980621338], 'magnitude': 7.217638969421387, 'distance': 6.7822136878967285, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.48055241989325803, 'motion_component': -3.4684537373107496}, {'ion': 2443, 'force': [2.3701698780059814, 12.436541557312012, -3.2652554512023926], 'magnitude': 13.074676513671875, 'distance': 5.039106845855713, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.24864144878760677, 'motion_component': 3.250906495401992}]}, 5998: {'frame': 5998, 'ionic_force': [10.780787527561188, 0.28440017998218536, -7.232492357492447], 'ionic_force_magnitude': 12.985191907629991, 'motion_vector': [-0.7672195434570312, 2.2775001525878906, -1.0481185913085938], 'cosine_ionic_motion': -0.001263009889529832, 'ionic_motion_component': -0.016400425796779423, 'ionic_force_x': 10.780787527561188, 'ionic_force_y': 0.28440017998218536, 'ionic_force_z': -7.232492357492447, 'radial_force': 10.784538153152075, 'axial_force': -7.232492357492447, 'before_closest_residue': 780, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1327, 'force': [0.6711025238037109, -0.13265840709209442, -1.804991602897644], 'magnitude': 1.9302775859832764, 'distance': 13.114724159240723, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.21237849268114292, 'motion_component': 0.40994944295757296}, {'ion': 1380, 'force': [2.8374791145324707, 0.6517823338508606, -0.4846545159816742], 'magnitude': 2.95143985748291, 'distance': 10.606010437011719, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.02385020767435757, 'motion_component': -0.07039245638239944}, {'ion': 1443, 'force': [3.076692581176758, -0.8291545510292053, -3.541635036468506], 'magnitude': 4.764106750488281, 'distance': 8.347920417785645, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.04297902665725936, 'motion_component': -0.20475667152368615}, {'ion': 1476, 'force': [1.263065218925476, -1.5566960573196411, 0.03140932321548462], 'magnitude': 2.004899740219116, 'distance': 12.868345260620117, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.8650766728807576, 'motion_component': -1.7343919836517667}, {'ion': 2434, 'force': [-0.50923091173172, -8.268269538879395, -0.3708587884902954], 'magnitude': 8.29223346710205, 'distance': 6.327516555786133, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.8302967302675558, 'motion_component': -6.88501421705325}, {'ion': 2443, 'force': [3.441679000854492, 10.41939640045166, -1.061761736869812], 'magnitude': 11.024351119995117, 'distance': 5.487727642059326, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.7681364258085014, 'motion_component': 8.46820552903441}]}, 5999: {'frame': 5999, 'ionic_force': [6.903971970081329, -9.943094223737717, -11.683605313301086], 'ionic_force_magnitude': 16.8236911771107, 'motion_vector': [-1.3753700256347656, -4.601753234863281, -0.27584075927734375], 'cosine_ionic_motion': 0.48783230159410307, 'ionic_motion_component': 8.207139988238318, 'ionic_force_x': 6.903971970081329, 'ionic_force_y': -9.943094223737717, 'ionic_force_z': -11.683605313301086, 'radial_force': 12.104955667237903, 'axial_force': -11.683605313301086, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 780, 'contributions': [{'ion': 1327, 'force': [0.45604217052459717, 0.1768944263458252, -1.7557339668273926], 'magnitude': 1.822599172592163, 'distance': 13.49657154083252, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.10913884575298162, 'motion_component': -0.19891637349124203}, {'ion': 1380, 'force': [2.0143558979034424, 1.382273554801941, -0.6717885732650757], 'magnitude': 2.5336947441101074, 'distance': 11.447005271911621, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.7339383307098968, 'motion_component': -1.8595757916178342}, {'ion': 1443, 'force': [2.022075653076172, 0.4375012218952179, -3.6579012870788574], 'magnitude': 4.202432632446289, 'distance': 8.888298988342285, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.18723646755622428, 'motion_component': -0.7868486203393044}, {'ion': 1476, 'force': [2.0586459636688232, -1.9142779111862183, -0.18536603450775146], 'magnitude': 2.8172404766082764, 'distance': 10.855681419372559, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.44482233949506284, 'motion_component': 1.2531714830432583}, {'ion': 2434, 'force': [0.3335014283657074, -16.288362503051758, -3.843754291534424], 'magnitude': 16.73906898498535, 'distance': 4.453519821166992, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.9382599892586932, 'motion_component': 15.705598484353184}, {'ion': 2443, 'force': [0.01935085654258728, 6.262876987457275, -1.5690611600875854], 'magnitude': 6.456466197967529, 'distance': 7.170866012573242, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.9147867132530993, 'motion_component': -5.90628947647706}]}, 6000: {'frame': 6000, 'ionic_force': [5.517950534820557, 7.6139421463012695, -19.801055759191513], 'ionic_force_magnitude': 21.920349045819517, 'motion_vector': [-4.781524658203125, 2.4392776489257812, 0.5065383911132812], 'cosine_ionic_motion': -0.1509624024908215, 'ionic_motion_component': -3.3091485553943008, 'ionic_force_x': 5.517950534820557, 'ionic_force_y': 7.6139421463012695, 'ionic_force_z': -19.801055759191513, 'radial_force': 9.403185264151146, 'axial_force': -19.801055759191513, 'before_closest_residue': 455, 'closest_residue': 780, 'next_closest_residue': 1105, 'contributions': [{'ion': 1327, 'force': [0.27228718996047974, -0.34001588821411133, -1.6231095790863037], 'magnitude': 1.6805462837219238, 'distance': 14.055419921875, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.3259627221595233, 'motion_component': -0.5477954425251834}, {'ion': 1380, 'force': [3.8357651233673096, 0.6248253583908081, -1.3770771026611328], 'magnitude': 4.123086452484131, 'distance': 8.973416328430176, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.7878593598961018, 'motion_component': -3.2484122782963705}, {'ion': 1443, 'force': [1.5023193359375, -1.549290657043457, -3.5091614723205566], 'magnitude': 4.119645595550537, 'distance': 8.977163314819336, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5735767810263909, 'motion_component': -2.362933013233306}, {'ion': 1476, 'force': [1.1409306526184082, -1.8393505811691284, -0.37553462386131287], 'magnitude': 2.1968066692352295, 'distance': 12.293431282043457, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 130, 'cosine_with_motion': -0.8554532966122542, 'motion_component': -1.8792655123287687}, {'ion': 2434, 'force': [-0.8899776935577393, -4.16619348526001, -0.9849853515625], 'magnitude': 4.3725762367248535, 'distance': 8.713654518127441, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.27172446280525053, 'motion_component': -1.1881359802195564}, {'ion': 2443, 'force': [-0.3433740735054016, 14.883967399597168, -11.931187629699707], 'magnitude': 19.07887840270996, 'distance': 4.17150354385376, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.31015416168122784, 'motion_component': 5.917393768109569}]}, 6001: {'frame': 6001, 'ionic_force': [-5.739471256732941, 1.5717533826828003, -13.330579981207848], 'ionic_force_magnitude': 14.598503404055426, 'motion_vector': [1.7098503112792969, -0.131500244140625, 0.37758636474609375], 'cosine_ionic_motion': -0.5872436292990687, 'ionic_motion_component': -8.572878121332318, 'ionic_force_x': -5.739471256732941, 'ionic_force_y': 1.5717533826828003, 'ionic_force_z': -13.330579981207848, 'radial_force': 5.9507931406526335, 'axial_force': -13.330579981207848, 'before_closest_residue': 780, 'closest_residue': 1105, 'next_closest_residue': 'SF', 'contributions': [{'ion': 1327, 'force': [-0.37006884813308716, -0.10675269365310669, -1.939383625984192], 'magnitude': 1.9772597551345825, 'distance': 12.957976341247559, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.3891132324604061, 'motion_component': -0.7693779149979432}, {'ion': 1380, 'force': [4.8833489418029785, 6.641224384307861, -3.6172406673431396], 'magnitude': 9.002077102661133, 'distance': 6.0729217529296875, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.38656834232561726, 'motion_component': 3.479917939183366}, {'ion': 1443, 'force': [-1.8360635042190552, -0.6234139800071716, -6.40214204788208], 'magnitude': 6.689334392547607, 'distance': 7.044944763183594, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.4660847366346669, 'motion_component': -3.1177967411055856}, {'ion': 1476, 'force': [-1.7837971448898315, -6.105370998382568, 0.018659725785255432], 'magnitude': 6.360647678375244, 'distance': 7.224676132202148, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 130, 'cosine_with_motion': -0.20056350312584506, 'motion_component': -1.2757137265881193}, {'ion': 2434, 'force': [-2.968780040740967, -1.7256089448928833, -0.42890286445617676], 'magnitude': 3.460540294647217, 'distance': 9.79483413696289, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.8246681142989506, 'motion_component': -2.853797203169603}, {'ion': 2443, 'force': [-3.6641106605529785, 3.491675615310669, -0.9615705013275146], 'magnitude': 5.151905059814453, 'distance': 8.027588844299316, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.7834209858121003, 'motion_component': -4.036110359738709}]}, 6004: {'frame': 6004, 'ionic_force': [-13.262407958507538, 11.088155046105385, -8.382136479020119], 'ionic_force_magnitude': 19.2119457405354, 'motion_vector': [-0.223419189453125, 2.570514678955078, -0.7060775756835938], 'cosine_ionic_motion': 0.7274053216976897, 'ionic_motion_component': 13.974871571832711, 'ionic_force_x': -13.262407958507538, 'ionic_force_y': 11.088155046105385, 'ionic_force_z': -8.382136479020119, 'radial_force': 17.28695019904773, 'axial_force': -8.382136479020119, 'before_closest_residue': 'SF', 'closest_residue': 1105, 'next_closest_residue': 1105, 'contributions': [{'ion': 1327, 'force': [-0.7501986622810364, -0.13029859960079193, -1.3091551065444946], 'magnitude': 1.5144842863082886, 'distance': 14.805962562561035, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.186860844372352, 'motion_component': 0.28299782470996293}, {'ion': 1380, 'force': [-4.599451065063477, 13.990073204040527, -4.257678985595703], 'magnitude': 15.329870223999023, 'distance': 4.653715133666992, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.9752989250966534, 'motion_component': 14.95120619354374}, {'ion': 1443, 'force': [-2.4518744945526123, -0.6125720739364624, -2.5525479316711426], 'magnitude': 3.59199595451355, 'distance': 9.613933563232422, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.08070347547918504, 'motion_component': 0.28988654720289553}, {'ion': 1476, 'force': [-1.4830362796783447, -2.197493553161621, 0.07560582458972931], 'magnitude': 2.652186155319214, 'distance': 11.188375473022461, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 130, 'cosine_with_motion': -0.7569972136268932, 'motion_component': -2.0076974384426522}, {'ion': 2434, 'force': [-1.6397267580032349, -0.897940993309021, -0.09315349161624908], 'magnitude': 1.8718117475509644, 'distance': 13.317967414855957, 'before_closest_residue': 455, 'closest_residue': 423, 'next_closest_residue': 455, 'cosine_with_motion': -0.3746682915369973, 'motion_component': -0.7013085318627432}, {'ion': 2443, 'force': [-2.338120698928833, 0.9363870620727539, -0.2452067881822586], 'magnitude': 2.530564308166504, 'distance': 11.454083442687988, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.4583115526478856, 'motion_component': 1.15978683758948}]}, 6005: {'frame': 6005, 'ionic_force': [-11.751091122627258, 3.513936460018158, -5.2574396431446075], 'ionic_force_magnitude': 13.344533098562968, 'motion_vector': [-0.2879486083984375, 0.21361923217773438, 0.6275177001953125], 'cosine_ionic_motion': 0.08660157332649941, 'ionic_motion_component': 1.1556575616430993, 'ionic_force_x': -11.751091122627258, 'ionic_force_y': 3.513936460018158, 'ionic_force_z': -5.2574396431446075, 'radial_force': 12.265231021767756, 'axial_force': -5.2574396431446075, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 1105, 'contributions': [{'ion': 1380, 'force': [-1.5290939807891846, 5.18525505065918, -2.7910616397857666], 'magnitude': 6.0839972496032715, 'distance': 7.387109279632568, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.046274344769027524, 'motion_component': -0.2815329896728045}, {'ion': 1443, 'force': [-2.1018567085266113, 0.29880401492118835, -2.3693599700927734], 'magnitude': 3.181344509124756, 'distance': 10.215596199035645, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.35566691171394543, 'motion_component': -1.1314989344353963}, {'ion': 1476, 'force': [-1.9276835918426514, -2.4968819618225098, -0.44340747594833374], 'magnitude': 3.185434579849243, 'distance': 10.20903491973877, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 130, 'cosine_with_motion': -0.1114396492132857, 'motion_component': -0.3549837172213053}, {'ion': 2434, 'force': [-4.488006591796875, -0.4852888882160187, 0.6003507971763611], 'magnitude': 4.553913593292236, 'distance': 8.538402557373047, 'before_closest_residue': 423, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': 0.475624094121237, 'motion_component': 2.165951055586958}, {'ion': 2443, 'force': [-1.704450249671936, 1.0120482444763184, -0.25396135449409485], 'magnitude': 1.9984716176986694, 'distance': 12.88902473449707, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.37915073484901873, 'motion_component': 0.7577219696746003}]}, 6006: {'frame': 6006, 'ionic_force': [-11.669181168079376, 5.09692008793354, -6.636843234300613], 'ionic_force_magnitude': 14.35952894885207, 'motion_vector': [3.3086013793945312, -2.3047142028808594, -0.0504608154296875], 'cosine_ionic_motion': -0.8638428873633073, 'ionic_motion_component': -12.404376948353368, 'ionic_force_x': -11.669181168079376, 'ionic_force_y': 5.09692008793354, 'ionic_force_z': -6.636843234300613, 'radial_force': 12.733749782221999, 'axial_force': -6.636843234300613, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 1105, 'contributions': [{'ion': 1327, 'force': [-0.7694267630577087, 0.20096524059772491, -1.2440012693405151], 'magnitude': 1.4764631986618042, 'distance': 14.995388984680176, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.49482651686876605, 'motion_component': -0.7305931674763221}, {'ion': 1380, 'force': [-1.6209291219711304, 5.998019695281982, -2.354433298110962], 'magnitude': 6.644321918487549, 'distance': 7.06876802444458, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.7116686340399404, 'motion_component': -4.7285551762152656}, {'ion': 1443, 'force': [-2.171865224838257, 0.4668664336204529, -2.2036139965057373], 'magnitude': 3.129037857055664, 'distance': 10.300626754760742, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6459600570181461, 'motion_component': -2.0212334267683243}, {'ion': 1476, 'force': [-3.098361015319824, -2.754167318344116, -0.36075103282928467], 'magnitude': 4.161180019378662, 'distance': 8.93224811553955, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 98, 'cosine_with_motion': -0.23155389581540803, 'motion_component': -0.9635374656188068}, {'ion': 2434, 'force': [-2.578646183013916, 0.22548645734786987, -0.3415878117084503], 'magnitude': 2.6109275817871094, 'distance': 11.276430130004883, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 'SF', 'cosine_with_motion': -0.858060532463983, 'motion_component': -2.240333857713003}, {'ion': 2443, 'force': [-1.42995285987854, 0.9597495794296265, -0.13245582580566406], 'magnitude': 1.7272605895996094, 'distance': 13.864049911499023, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.9958682908568361, 'motion_component': -1.7201240045553075}]}, 6007: {'frame': 6007, 'ionic_force': [-8.5225989818573, 11.005497053265572, -12.623888924717903], 'ionic_force_magnitude': 18.7914403486962, 'motion_vector': [2.3887977600097656, 0.3354644775390625, 2.6361465454101562], 'cosine_ionic_motion': -0.7438233596257194, 'ionic_motion_component': -13.977512292373508, 'ionic_force_x': -8.5225989818573, 'ionic_force_y': 11.005497053265572, 'ionic_force_z': -12.623888924717903, 'radial_force': 13.919614175507604, 'axial_force': -12.623888924717903, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 'SF', 'contributions': [{'ion': 1327, 'force': [-0.6066397428512573, -0.07653407752513885, -1.803540825843811], 'magnitude': 1.904370903968811, 'distance': 13.203627586364746, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.915413701296586, 'motion_component': -1.7432872690928678}, {'ion': 1380, 'force': [3.8302056789398193, 13.930157661437988, -4.655093669891357], 'magnitude': 15.178592681884766, 'distance': 4.676848411560059, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.02859949875737043, 'motion_component': 0.434100132452798}, {'ion': 1443, 'force': [-2.181785821914673, -0.8094444274902344, -4.307274341583252], 'magnitude': 4.895712852478027, 'distance': 8.234951972961426, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.9625209946089894, 'motion_component': -4.712226165570627}, {'ion': 1476, 'force': [-1.5309606790542603, -3.3161826133728027, -0.14249469339847565], 'magnitude': 3.655299186706543, 'distance': 9.530322074890137, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 130, 'cosine_with_motion': -0.39393060059103735, 'motion_component': -1.43993422116767}, {'ion': 2434, 'force': [-4.577861785888672, -0.5349699258804321, -0.9441246390342712], 'magnitude': 4.704719066619873, 'distance': 8.400443077087402, 'before_closest_residue': 455, 'closest_residue': 'SF', 'next_closest_residue': 455, 'cosine_with_motion': -0.8092180961137404, 'motion_component': -3.8071439082249348}, {'ion': 2443, 'force': [-3.455556631088257, 1.8124704360961914, -0.7713607549667358], 'magnitude': 3.9775516986846924, 'distance': 9.13610553741455, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.6810775388365401, 'motion_component': -2.7090211738439223}]}, 6009: {'frame': 6009, 'ionic_force': [-7.961302757263184, 8.177349001169205, -15.085426807403564], 'ionic_force_magnitude': 18.916169808956028, 'motion_vector': [3.8805274963378906, 4.743255615234375, -1.0284576416015625], 'cosine_ionic_motion': 0.1991376659376658, 'ionic_motion_component': 3.7669219042360447, 'ionic_force_x': -7.961302757263184, 'ionic_force_y': 8.177349001169205, 'ionic_force_z': -15.085426807403564, 'radial_force': 11.41277259388486, 'axial_force': -15.085426807403564, 'before_closest_residue': 'SF', 'closest_residue': 1105, 'next_closest_residue': 130, 'contributions': [{'ion': 1327, 'force': [-0.591535210609436, -0.1539454162120819, -1.536857008934021], 'magnitude': 1.6539475917816162, 'distance': 14.167987823486328, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.1406026487890743, 'motion_component': -0.23254940922222112}, {'ion': 1380, 'force': [0.541907787322998, 12.025218963623047, -9.050501823425293], 'magnitude': 15.060250282287598, 'distance': 4.695187568664551, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.7314129639106994, 'motion_component': 11.015262292895684}, {'ion': 1443, 'force': [-2.206110715866089, -0.993217945098877, -3.5082154273986816], 'magnitude': 4.261570453643799, 'distance': 8.826412200927734, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.3649277443025154, 'motion_component': -1.555165255618455}, {'ion': 1476, 'force': [-0.4248296022415161, -2.8931193351745605, -0.22868134081363678], 'magnitude': 2.933072566986084, 'distance': 10.639166831970215, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.8304569898762885, 'motion_component': -2.4357906364350237}, {'ion': 2434, 'force': [-2.3827462196350098, -0.7271773219108582, -0.04096989333629608], 'magnitude': 2.491574764251709, 'distance': 11.543355941772461, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': -0.8172516378812329, 'motion_component': -2.0362435784710797}, {'ion': 2443, 'force': [-2.897988796234131, 0.9195900559425354, -0.720201313495636], 'magnitude': 3.124527931213379, 'distance': 10.30805778503418, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.3163970260731719, 'motion_component': -0.9885913490203828}]}, 6010: {'frame': 6010, 'ionic_force': [-3.6213796138763428, 1.774631679058075, -10.690930426120758], 'ionic_force_magnitude': 11.426272414058323, 'motion_vector': [1.1203804016113281, -1.3056755065917969, -0.7982025146484375], 'cosine_ionic_motion': 0.09963000981851038, 'ionic_motion_component': 1.138399632801605, 'ionic_force_x': -3.6213796138763428, 'ionic_force_y': 1.774631679058075, 'ionic_force_z': -10.690930426120758, 'radial_force': 4.032828771980736, 'axial_force': -10.690930426120758, 'before_closest_residue': 1105, 'closest_residue': 130, 'next_closest_residue': 130, 'contributions': [{'ion': 1327, 'force': [-0.1575925350189209, 0.3570076823234558, -1.512939453125], 'magnitude': 1.5624581575393677, 'distance': 14.576889038085938, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.19063718239012178, 'motion_component': 0.2978626321694442}, {'ion': 1380, 'force': [1.4782865047454834, 3.0387051105499268, -1.537086009979248], 'magnitude': 3.7123701572418213, 'distance': 9.456782341003418, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.15401513443536977, 'motion_component': -0.5717612086865387}, {'ion': 1443, 'force': [-0.25140249729156494, 0.9879297614097595, -3.684279203414917], 'magnitude': 3.822711229324341, 'distance': 9.319299697875977, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.1888517298913497, 'motion_component': 0.7219256417490847}, {'ion': 1476, 'force': [2.1201860904693604, -6.282724380493164, -2.145188093185425], 'magnitude': 6.969192981719971, 'distance': 6.902045249938965, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.92986771215663, 'motion_component': 6.4804272558418035}, {'ion': 2434, 'force': [-5.255415439605713, 0.688380777835846, -0.6865726113319397], 'magnitude': 5.344590187072754, 'distance': 7.881553649902344, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': -0.6154733611346858, 'motion_component': -3.289452726313776}, {'ion': 2443, 'force': [-1.5554417371749878, 2.985332727432251, -1.1248650550842285], 'magnitude': 3.54921555519104, 'distance': 9.671700477600098, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.7045506025710427, 'motion_component': -2.5006020400647486}]}, 6011: {'frame': 6011, 'ionic_force': [-4.111999347805977, 4.2266088128089905, -12.676829218864441], 'ionic_force_magnitude': 13.981228835017564, 'motion_vector': [-0.2661705017089844, -1.283233642578125, 3.399566650390625], 'cosine_ionic_motion': -0.9310030034089785, 'ionic_motion_component': -13.016566036749564, 'ionic_force_x': -4.111999347805977, 'ionic_force_y': 4.2266088128089905, 'ionic_force_z': -12.676829218864441, 'radial_force': 5.89684328203416, 'axial_force': -12.676829218864441, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 'SF', 'contributions': [{'ion': 1380, 'force': [2.3445777893066406, 1.8577836751937866, -1.650367259979248], 'magnitude': 3.4164481163024902, 'distance': 9.857836723327637, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.6923878073754544, 'motion_component': -2.3655069752017326}, {'ion': 1443, 'force': [0.19824711978435516, 0.7226526141166687, -3.8288686275482178], 'magnitude': 3.901508092880249, 'distance': 9.224711418151855, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.984644180768522, 'motion_component': -3.841597024019926}, {'ion': 1476, 'force': [1.8675719499588013, -4.334394454956055, -1.7466002702713013], 'magnitude': 5.032435894012451, 'distance': 8.122316360473633, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.04759856881063422, 'motion_component': -0.2395367544916089}, {'ion': 2434, 'force': [-6.596822261810303, 2.5684547424316406, -3.428205728530884], 'magnitude': 7.865597248077393, 'distance': 6.49685525894165, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 130, 'cosine_with_motion': -0.46041497050577473, 'motion_component': -3.6214386713071427}, {'ion': 2443, 'force': [-1.9255739450454712, 3.412112236022949, -2.02278733253479], 'magnitude': 4.4093098640441895, 'distance': 8.677282333374023, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.6686956584488439, 'motion_component': -2.948486366220995}]}, 6013: {'frame': 6013, 'ionic_force': [13.507776856422424, 12.524327024817467, -10.32847486436367], 'ionic_force_magnitude': 21.118622020654342, 'motion_vector': [-0.33412933349609375, -3.45306396484375, 0.26458740234375], 'cosine_ionic_motion': -0.6871974397232127, 'ionic_motion_component': -14.512662983075925, 'ionic_force_x': 13.507776856422424, 'ionic_force_y': 12.524327024817467, 'ionic_force_z': -10.32847486436367, 'radial_force': 18.420608106886004, 'axial_force': -10.32847486436367, 'before_closest_residue': 'SF', 'closest_residue': 455, 'next_closest_residue': 748, 'contributions': [{'ion': 1327, 'force': [0.4487518072128296, 0.17691664397716522, -2.0343520641326904], 'magnitude': 2.090757369995117, 'distance': 12.601354598999023, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.17858886796218035, 'motion_component': -0.37338597583429944}, {'ion': 1380, 'force': [2.8208999633789062, 1.3959943056106567, -0.5538100600242615], 'magnitude': 3.1957757472991943, 'distance': 10.192503929138184, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.5314827701352313, 'motion_component': -1.6984997186537467}, {'ion': 1443, 'force': [2.2907891273498535, 0.40284377336502075, -4.769194602966309], 'magnitude': 5.306148529052734, 'distance': 7.9100518226623535, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.18516005038430078, 'motion_component': -0.9824867792408724}, {'ion': 1476, 'force': [2.0120725631713867, -2.631169557571411, 0.06651456654071808], 'magnitude': 3.3129916191101074, 'distance': 10.010571479797363, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.7314185945024936, 'motion_component': 2.4231836691692252}, {'ion': 2434, 'force': [7.2099080085754395, 4.52037239074707, -1.7856876850128174], 'magnitude': 8.695125579833984, 'distance': 6.179183483123779, 'before_closest_residue': 130, 'closest_residue': 'SF', 'next_closest_residue': 'SF', 'cosine_with_motion': -0.6112071813001704, 'motion_component': -5.314523608002732}, {'ion': 2443, 'force': [-1.2746446132659912, 8.659369468688965, -1.2519450187683105], 'magnitude': 8.84176254272461, 'distance': 6.127729892730713, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.9689188712793316, 'motion_component': -8.566950580467749}]}, 6014: {'frame': 6014, 'ionic_force': [17.058067679405212, 13.762900233268738, -12.238668072968721], 'ionic_force_magnitude': 25.10338805791723, 'motion_vector': [-3.6916656494140625, 0.4512596130371094, -6.285575866699219], 'cosine_ionic_motion': 0.10998618155531045, 'ionic_motion_component': 2.761025796591497, 'ionic_force_x': 17.058067679405212, 'ionic_force_y': 13.762900233268738, 'ionic_force_z': -12.238668072968721, 'radial_force': 21.91791723193783, 'axial_force': -12.238668072968721, 'before_closest_residue': 455, 'closest_residue': 748, 'next_closest_residue': 130, 'contributions': [{'ion': 1327, 'force': [0.44926393032073975, -0.363325715065</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>6160</v>
+      </c>
+      <c r="B22" t="n">
+        <v>6359</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1443</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>{6160: {'frame': 6160, 'ionic_force': [3.740715362073388, 2.176445934921503, -12.598692059516907], 'ionic_force_magnitude': 13.321295355115527, 'motion_vector': [2.4038047790527344, -0.042205810546875, -2.1078033447265625], 'cosine_ionic_motion': 0.8324384974001108, 'ionic_motion_component': 11.089159088835444, 'ionic_force_x': 3.740715362073388, 'ionic_force_y': 2.176445934921503, 'ionic_force_z': -12.598692059516907, 'radial_force': 4.327801789325404, 'axial_force': -12.598692059516907, 'before_closest_residue': None, 'closest_residue': 130, 'next_closest_residue': 455, 'contributions': [{'ion': 1327, 'force': [-0.22856654226779938, 0.7065204977989197, -8.549403190612793], 'magnitude': 8.581591606140137, 'distance': 6.219924449920654, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.6356556463125634, 'motion_component': 5.454936947654412}, {'ion': 1341, 'force': [-0.0005797222838737071, 0.04265621677041054, -2.332738161087036], 'magnitude': 2.3331282138824463, 'distance': 11.928881645202637, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.6587010552503938, 'motion_component': 1.5368340101219817}, {'ion': 1355, 'force': [-1.527624487876892, -3.6898083686828613, -0.8481869697570801], 'magnitude': 4.082614898681641, 'distance': 9.017784118652344, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.13242233380003088, 'motion_component': -0.5406293782664431}, {'ion': 1380, 'force': [5.1329145431518555, 4.496638774871826, -0.7909724116325378], 'magnitude': 6.869658946990967, 'distance': 6.95186710357666, 'before_closest_residue': 1073, 'closest_residue': 1105, 'next_closest_residue': 1073, 'cosine_with_motion': 0.6290118362515426, 'motion_component': 4.321096572897298}, {'ion': 1476, 'force': [-4.47384786605835, 4.564768314361572, -0.8368766903877258], 'magnitude': 6.446145057678223, 'distance': 7.176604270935059, 'before_closest_residue': 748, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.4455485038776503, 'motion_component': -2.872070320188927}, {'ion': 2443, 'force': [4.838419437408447, -3.9443295001983643, 0.7594853639602661], 'magnitude': 6.288470268249512, 'distance': 7.266019344329834, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.507117132671062, 'motion_component': 3.1889909130123653}]}, 6161: {'frame': 6161, 'ionic_force': [2.045816570520401, 2.513314615935087, -12.963244438171387], 'ionic_force_magnitude': 13.362178795491031, 'motion_vector': [4.460853576660156, 2.02520751953125, 0.9477462768554688], 'cosine_ionic_motion': 0.02894916806440939, 'ionic_motion_component': 0.3868239596573573, 'ionic_force_x': 2.045816570520401, 'ionic_force_y': 2.513314615935087, 'ionic_force_z': -12.963244438171387, 'radial_force': 3.2406968076154223, 'axial_force': -12.963244438171387, 'before_closest_residue': 130, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1327, 'force': [0.9507448077201843, 0.019289210438728333, -3.7588417530059814], 'magnitude': 3.8772642612457275, 'distance': 9.253506660461426, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.03709964672148767, 'motion_component': 0.14384513881447392}, {'ion': 1341, 'force': [0.26577094197273254, -0.029373470693826675, -1.5081979036331177], 'magnitude': 1.531717300415039, 'distance': 14.722437858581543, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.03968436262683752, 'motion_component': -0.06078522508307371}, {'ion': 1355, 'force': [-0.5799313187599182, -3.2436165809631348, -1.537106990814209], 'magnitude': 3.6359410285949707, 'distance': 9.555658340454102, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.5849542921591248, 'motion_component': -2.1268592782617333}, {'ion': 1380, 'force': [2.139223337173462, 1.9624422788619995, -1.0930858850479126], 'magnitude': 3.1019821166992188, 'distance': 10.345450401306152, 'before_closest_residue': 1105, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.8063528161229908, 'motion_component': 2.5012920002790526}, {'ion': 1476, 'force': [-4.092360019683838, 5.589524745941162, -4.061839580535889], 'magnitude': 8.030488014221191, 'distance': 6.429809093475342, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 748, 'cosine_with_motion': -0.2691477355049505, 'motion_component': -2.161387671528992}, {'ion': 2443, 'force': [3.3623688220977783, -1.7849515676498413, -1.0041723251342773], 'magnitude': 3.9369959831237793, 'distance': 9.1830415725708, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 130, 'cosine_with_motion': 0.5310442425551404, 'motion_component': 2.0907191092921558}]}, 6162: {'frame': 6162, 'ionic_force': [7.763323903083801, 2.8181435465812683, -6.318853139877319], 'ionic_force_magnitude': 10.398992070228124, 'motion_vector': [-1.7015113830566406, -2.5169944763183594, 0.5141983032226562], 'cosine_ionic_motion': -0.7350036857169278, 'ionic_motion_component': -7.643297499358775, 'ionic_force_x': 7.763323903083801, 'ionic_force_y': 2.8181435465812683, 'ionic_force_z': -6.318853139877319, 'radial_force': 8.259003031439688, 'axial_force': -6.318853139877319, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 780, 'contributions': [{'ion': 1327, 'force': [1.9486887454986572, 0.7575831413269043, -2.100437641143799], 'magnitude': 2.963639259338379, 'distance': 10.584158897399902, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.690161551578687, 'motion_component': -2.045389947290012}, {'ion': 1355, 'force': [1.829471230506897, -3.8013644218444824, -1.9934921264648438], 'magnitude': 4.665977478027344, 'distance': 8.435245513916016, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.3776782357281483, 'motion_component': 1.7622382018976808}, {'ion': 1380, 'force': [1.3906784057617188, 0.7438085079193115, -0.29142385721206665], 'magnitude': 1.603797197341919, 'distance': 14.387797355651855, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.8879747581624139, 'motion_component': -1.424131411579718}, {'ion': 1476, 'force': [0.6493955850601196, 5.551018238067627, -1.8384053707122803], 'magnitude': 5.883472919464111, 'distance': 7.511940956115723, 'before_closest_residue': 780, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.8837793439367987, 'motion_component': -5.199691748076372}, {'ion': 2443, 'force': [1.9450899362564087, -0.43290191888809204, -0.09509414434432983], 'magnitude': 1.9949489831924438, 'distance': 12.900399208068848, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 98, 'cosine_with_motion': -0.369093526402772, 'motion_component': -0.7363227905610161}]}, 6163: {'frame': 6163, 'ionic_force': [5.693150162696838, 11.41169948130846, -10.106098487973213], 'ionic_force_magnitude': 16.271818290385536, 'motion_vector': [-5.470054626464844, -0.9522628784179688, -5.482391357421875], 'cosine_ionic_motion': 0.10551406260941289, 'ionic_motion_component': 1.7169056538607292, 'ionic_force_x': 5.693150162696838, 'ionic_force_y': 11.41169948130846, 'ionic_force_z': -10.106098487973213, 'radial_force': 12.752993524138198, 'axial_force': -10.106098487973213, 'before_closest_residue': 455, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1327, 'force': [2.395063638687134, 0.08514890819787979, -3.508793830871582], 'magnitude': 4.249142646789551, 'distance': 8.839310646057129, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.18260500011970154, 'motion_component': 0.7759147168334264}, {'ion': 1341, 'force': [0.5789742469787598, -0.06532517075538635, -1.6003326177597046], 'magnitude': 1.7030980587005615, 'distance': 13.962050437927246, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.4265788997687441, 'motion_component': 0.7265057019041103}, {'ion': 1355, 'force': [0.5200189352035522, -3.328923225402832, -0.7997344136238098], 'magnitude': 3.462907075881958, 'distance': 9.791486740112305, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.1743087750944642, 'motion_component': 0.603615071780343}, {'ion': 1380, 'force': [2.3475747108459473, 0.65799880027771, -0.3588736653327942], 'magnitude': 2.4643173217773438, 'distance': 11.607020378112793, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.5980863138118124, 'motion_component': -1.4738744496265603}, {'ion': 1476, 'force': [-2.214129686355591, 15.15945053100586, -3.8823859691619873], 'magnitude': 15.804563522338867, 'distance': 4.583294868469238, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': 0.15374813144196073, 'motion_component': 2.429922126119237}, {'ion': 2443, 'force': [2.065648317337036, -1.0966503620147705, 0.044022008776664734], 'magnitude': 2.3391201496124268, 'distance': 11.913593292236328, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.5750783357621444, 'motion_component': -1.345177304391929}]}, 6164: {'frame': 6164, 'ionic_force': [0.7338058315217495, -0.6169207841157913, -9.97306752204895], 'ionic_force_magnitude': 10.019038778824891, 'motion_vector': [0.8026161193847656, -1.9557952880859375, 2.9555435180664062], 'cosine_ionic_motion': -0.7602959620299808, 'ionic_motion_component': -7.617434726962355, 'ionic_force_x': 0.7338058315217495, 'ionic_force_y': -0.6169207841157913, 'ionic_force_z': -9.97306752204895, 'radial_force': 0.9586773452258945, 'axial_force': -9.97306752204895, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1327, 'force': [-0.05467653647065163, -0.15348537266254425, -1.8620142936706543], 'magnitude': 1.8691293001174927, 'distance': 13.327520370483398, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.772514375988365, 'motion_component': -1.4439292905769412}, {'ion': 1355, 'force': [-0.5475013852119446, -1.3620316982269287, -1.0494215488433838], 'magnitude': 1.8044871091842651, 'distance': 13.564136505126953, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.13377577768711005, 'motion_component': -0.24139666538441507}, {'ion': 1380, 'force': [1.875036597251892, 1.458633303642273, -2.697950601577759], 'magnitude': 3.594761610031128, 'distance': 9.610234260559082, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.7136182945906884, 'motion_component': -2.565287626893147}, {'ion': 1476, 'force': [-2.0720303058624268, 1.2611353397369385, -2.7867367267608643], 'magnitude': 3.6945464611053467, 'distance': 9.47956657409668, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 780, 'cosine_with_motion': -0.9210902306061706, 'motion_component': -3.403010647426644}, {'ion': 2443, 'force': [1.5329774618148804, -1.8211723566055298, -1.576944351196289], 'magnitude': 2.8554232120513916, 'distance': 10.782855987548828, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.01267389165193761, 'motion_component': 0.036189325337053546}]}, 6165: {'frame': 6165, 'ionic_force': [0.8527390398085117, -2.051217794418335, -13.607491910457611], 'ionic_force_magnitude': 13.78762105670595, 'motion_vector': [-0.4117393493652344, 4.247417449951172, -2.2331161499023438], 'cosine_ionic_motion': 0.3211122018333723, 'ionic_motion_component': 4.427373355563015, 'ionic_force_x': 0.8527390398085117, 'ionic_force_y': -2.051217794418335, 'ionic_force_z': -13.607491910457611, 'radial_force': 2.221409082126019, 'axial_force': -13.607491910457611, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 455, 'contributions': [{'ion': 1327, 'force': [0.062102917581796646, -0.7361721992492676, -2.4836835861206055], 'magnitude': 2.591233491897583, 'distance': 11.319201469421387, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.191820151327965, 'motion_component': 0.49705077928710883}, {'ion': 1355, 'force': [-0.45634692907333374, -1.6045798063278198, -0.6252397894859314], 'magnitude': 1.7815312147140503, 'distance': 13.651247024536133, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.6096663689107369, 'motion_component': -1.0861397009811737}, {'ion': 1380, 'force': [4.697567462921143, 1.9251720905303955, -4.4325270652771], 'magnitude': 6.739490032196045, 'distance': 7.018681526184082, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.4972713830043761, 'motion_component': 3.351355452952653}, {'ion': 1476, 'force': [-5.758725166320801, 1.1061946153640747, -4.493953704833984], 'magnitude': 7.38797664642334, 'distance': 6.703571796417236, 'before_closest_residue': 748, 'closest_residue': 780, 'next_closest_residue': 748, 'cosine_with_motion': 0.4807118246685845, 'motion_component': 3.5514878332571698}, {'ion': 2443, 'force': [2.308140754699707, -2.7418324947357178, -1.5720877647399902], 'magnitude': 3.9136452674865723, 'distance': 9.210395812988281, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.48200098437439737, 'motion_component': -1.88638086113815}]}, 6166: {'frame': 6166, 'ionic_force': [1.4523009806871414, 1.297539383172989, -11.587992548942566], 'ionic_force_magnitude': 11.750504580814315, 'motion_vector': [2.0425567626953125, -2.522167205810547, 0.7178115844726562], 'cosine_ionic_motion': -0.22080468377105897, 'ionic_motion_component': -2.5945664481170847, 'ionic_force_x': 1.4523009806871414, 'ionic_force_y': 1.297539383172989, 'ionic_force_z': -11.587992548942566, 'radial_force': 1.9475077893014379, 'axial_force': -11.587992548942566, 'before_closest_residue': 780, 'closest_residue': 455, 'next_closest_residue': 780, 'contributions': [{'ion': 1327, 'force': [0.08723576366901398, 0.26207712292671204, -2.5743675231933594], 'magnitude': 2.5891432762145996, 'distance': 11.323769569396973, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.2708206249400485, 'motion_component': -0.7011933863444675}, {'ion': 1355, 'force': [-0.8347313404083252, -2.0121395587921143, -1.8562531471252441], 'magnitude': 2.8620200157165527, 'distance': 10.770421981811523, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.21417882627641824, 'motion_component': 0.6129840574588599}, {'ion': 1380, 'force': [1.436957836151123, 2.019728899002075, -1.8128858804702759], 'magnitude': 3.0709457397460938, 'distance': 10.39759635925293, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.33899412500374865, 'motion_component': -1.041032571015542}, {'ion': 1476, 'force': [-1.8430176973342896, 1.9066798686981201, -2.2257046699523926], 'magnitude': 3.462066411972046, 'distance': 9.792675018310547, 'before_closest_residue': 780, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.8838473596501303, 'motion_component': -3.0599382305185827}, {'ion': 2443, 'force': [2.605856418609619, -0.8788069486618042, -3.118781328201294], 'magnitude': 4.158074855804443, 'distance': 8.935583114624023, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.3834980879752371, 'motion_component': 1.5946137473633613}]}, 6167: {'frame': 6167, 'ionic_force': [1.0688188672065735, 1.0091578364372253, -11.419165134429932], 'ionic_force_magnitude': 11.513388105901736, 'motion_vector': [-0.13602447509765625, -1.4195594787597656, 3.152008056640625], 'cosine_ionic_motion': -0.9432504973964883, 'ionic_motion_component': -10.860009057610624, 'ionic_force_x': 1.0688188672065735, 'ionic_force_y': 1.0091578364372253, 'ionic_force_z': -11.419165134429932, 'radial_force': 1.4699569074430054, 'axial_force': -11.419165134429932, 'before_closest_residue': 455, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1327, 'force': [0.37463992834091187, -0.28571516275405884, -2.148576259613037], 'magnitude': 2.199629068374634, 'distance': 12.285541534423828, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8433436197672336, 'motion_component': -1.8550431665611884}, {'ion': 1355, 'force': [-0.322290301322937, -1.734464168548584, -1.1195731163024902], 'magnitude': 2.089421033859253, 'distance': 12.605382919311523, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.14150674080026152, 'motion_component': -0.2956671842401728}, {'ion': 1380, 'force': [2.3296315670013428, 1.3743340969085693, -2.2760865688323975], 'magnitude': 3.535045623779297, 'distance': 9.691065788269043, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.7720531629281498, 'motion_component': -2.729243149966913}, {'ion': 1476, 'force': [-3.17857027053833, 2.7836079597473145, -4.389988899230957], 'magnitude': 6.092929363250732, 'distance': 7.381692886352539, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 748, 'cosine_with_motion': -0.8233954713653064, 'motion_component': -5.016890211807125}, {'ion': 2443, 'force': [1.865407943725586, -1.1286048889160156, -1.4849402904510498], 'magnitude': 2.6379051208496094, 'distance': 11.218620300292969, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.36512508896735857, 'motion_component': -0.9631653441107701}]}, 6168: {'frame': 6168, 'ionic_force': [-7.520926967263222, 6.472836136817932, -23.5761159658432], 'ionic_force_magnitude': 25.579194556042808, 'motion_vector': [-0.9997520446777344, 3.4777908325195312, -1.7257232666015625], 'cosine_ionic_motion': 0.6895845985397099, 'ionic_motion_component': 17.639018608897914, 'ionic_force_x': -7.520926967263222, 'ionic_force_y': 6.472836136817932, 'ionic_force_z': -23.5761159658432, 'radial_force': 9.922799509261651, 'axial_force': -23.5761159658432, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 455, 'contributions': [{'ion': 1327, 'force': [1.1435531377792358, -1.7503900527954102, -4.134721279144287], 'magnitude': 4.633303165435791, 'distance': 8.464936256408691, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.005134544083482439, 'motion_component': -0.023789899881023757}, {'ion': 1341, 'force': [0.19866521656513214, -0.4084584712982178, -1.6042498350143433], 'magnitude': 1.667310357093811, 'distance': 14.111098289489746, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.1719448265095522, 'motion_component': 0.2866853847935005}, {'ion': 1355, 'force': [-0.2531542479991913, -2.0059866905212402, -0.5837475061416626], 'magnitude': 2.104478597640991, 'distance': 12.560206413269043, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.6774825447554669, 'motion_component': -1.4257476217592426}, {'ion': 1380, 'force': [4.757066249847412, 1.4454026222229004, -1.5462619066238403], 'magnitude': 5.206706523895264, 'distance': 7.985230922698975, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.14081311710588393, 'motion_component': 0.7331725904093531}, {'ion': 1476, 'force': [-15.625587463378906, 11.02933120727539, -14.86202335357666], 'magnitude': 24.22157859802246, 'distance': 3.702267646789551, 'before_closest_residue': 748, 'closest_residue': 748, 'next_closest_residue': 780, 'cosine_with_motion': 0.820002155604511, 'motion_component': 19.861746642845787}, {'ion': 2443, 'force': [2.2585301399230957, -1.8370624780654907, -0.8451120853424072], 'magnitude': 3.031496524810791, 'distance': 10.465030670166016, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.591473065178646, 'motion_component': -1.7930485609347073}]}, 6169: {'frame': 6169, 'ionic_force': [3.391502261161804, 2.702711671590805, -11.971076011657715], 'ionic_force_magnitude': 12.732383863366104, 'motion_vector': [0.38364410400390625, 1.7301025390625, 2.6249771118164062], 'cosine_ionic_motion': -0.631031291326958, 'ionic_motion_component': -8.034532630970435, 'ionic_force_x': 3.391502261161804, 'ionic_force_y': 2.702711671590805, 'ionic_force_z': -11.971076011657715, 'radial_force': 4.336696665345501, 'axial_force': -11.971076011657715, 'before_closest_residue': 780, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1327, 'force': [0.43922919034957886, 0.3048649728298187, -4.18452787399292], 'magnitude': 4.2185468673706055, 'distance': 8.871306419372559, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7700364697131815, 'motion_component': -3.2484350091106715}, {'ion': 1355, 'force': [-1.1267592906951904, -3.0149948596954346, -1.965143084526062], 'magnitude': 3.7711493968963623, 'distance': 9.382793426513672, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.904814890937976, 'motion_component': -3.4121921389138965}, {'ion': 1380, 'force': [1.8862299919128418, 2.4746272563934326, -1.5418955087661743], 'magnitude': 3.4726195335388184, 'distance': 9.77778434753418, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.08706382729268759, 'motion_component': 0.302339534481046}, {'ion': 1476, 'force': [-0.951141893863678, 4.275298595428467, -2.218920946121216], 'magnitude': 4.909832954406738, 'distance': 8.223102569580078, 'before_closest_residue': 748, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.0776314130857838, 'motion_component': 0.3811572663705402}, {'ion': 2443, 'force': [3.143944263458252, -1.3370842933654785, -2.0605885982513428], 'magnitude': 3.989762544631958, 'distance': 9.122114181518555, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.5156703286833915, 'motion_component': -2.057402172322913}]}, 6170: {'frame': 6170, 'ionic_force': [5.667690142989159, 1.7710587978363037, -13.184255957603455], 'ionic_force_magnitude': 14.459736027256238, 'motion_vector': [3.7403221130371094, -1.5651435852050781, 1.4440078735351562], 'cosine_ionic_motion': -0.009819873621377127, 'ionic_motion_component': -0.14199278038613003, 'ionic_force_x': 5.667690142989159, 'ionic_force_y': 1.7710587978363037, 'ionic_force_z': -13.184255957603455, 'radial_force': 5.9379593146408345, 'axial_force': -13.184255957603455, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1327, 'force': [1.4770755767822266, 2.068378448486328, -6.052678108215332], 'magnitude': 6.564666748046875, 'distance': 7.1115241050720215, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.22837603245973107, 'motion_component': -1.499212623473511}, {'ion': 1341, 'force': [0.2155987173318863, 0.3436358571052551, -2.0001230239868164], 'magnitude': 2.0408480167388916, 'distance': 12.754508018493652, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.2982298195332479, 'motion_component': -0.6086417278985303}, {'ion': 1355, 'force': [-2.284257650375366, -6.364039421081543, -2.5249183177948], 'magnitude': 7.217620372772217, 'distance': 6.782222270965576, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.0717600629576406, 'motion_component': -0.5179368895331322}, {'ion': 1380, 'force': [1.8270621299743652, 2.4519355297088623, -0.6305731534957886], 'magnitude': 3.1221413612365723, 'distance': 10.311996459960938, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.1552046801965146, 'motion_component': 0.4845709438187029}, {'ion': 1476, 'force': [-0.3435497581958771, 4.183430194854736, -0.503319263458252], 'magnitude': 4.22758150100708, 'distance': 8.861822128295898, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 748, 'cosine_with_motion': -0.47041022787114467, 'motion_component': -1.9886975530248403}, {'ion': 2443, 'force': [4.775761127471924, -0.9122818112373352, -1.4726440906524658], 'magnitude': 5.080239295959473, 'distance': 8.084012031555176, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.7849876604316632, 'motion_component': 3.9879252955995987}]}, 6171: {'frame': 6171, 'ionic_force': [10.627623319625854, -0.529610387980938, -5.966325297951698], 'ionic_force_magnitude': 12.19934023412295, 'motion_vector': [-1.0708656311035156, 1.0283088684082031, -2.1849288940429688], 'cosine_ionic_motion': 0.0344641513177246, 'ionic_motion_component': 0.4204399078052192, 'ionic_force_x': 10.627623319625854, 'ionic_force_y': -0.529610387980938, 'ionic_force_z': -5.966325297951698, 'radial_force': 10.640811274847072, 'axial_force': -5.966325297951698, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1327, 'force': [3.3019585609436035, 0.4475037753582001, -3.7688305377960205], 'magnitude': 5.030633449554443, 'distance': 8.123771667480469, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.38820542392481705, 'motion_component': 1.9529192173632346}, {'ion': 1341, 'force': [0.8308365941047668, 0.05887822061777115, -1.8445522785186768], 'magnitude': 2.0238895416259766, 'distance': 12.807832717895508, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5987381498916219, 'motion_component': 1.2117799274345193}, {'ion': 1355, 'force': [0.8886405825614929, -4.7136969566345215, -0.3486242890357971], 'magnitude': 4.809382438659668, 'distance': 8.308533668518066, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.39647626158736854, 'motion_component': -1.9068059919821962}, {'ion': 1380, 'force': [2.0485944747924805, 1.2774423360824585, -0.12629811465740204], 'magnitude': 2.4175503253936768, 'distance': 11.71875, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.09461183391256422, 'motion_component': -0.22872886755479094}, {'ion': 1476, 'force': [0.9028506278991699, 3.0675549507141113, 0.21530672907829285], 'magnitude': 3.2049007415771484, 'distance': 10.177983283996582, 'before_closest_residue': 780, 'closest_residue': 748, 'next_closest_residue': 780, 'cosine_with_motion': 0.2028247685813136, 'motion_component': 0.6500332783282765}, {'ion': 2443, 'force': [2.654742479324341, -0.6672927141189575, -0.09332680702209473], 'magnitude': 2.7389135360717773, 'distance': 11.009811401367188, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.45958287714503704, 'motion_component': -1.2587577407312978}]}, 6172: {'frame': 6172, 'ionic_force': [7.3180464617908, 0.31938037276268005, -8.137867994606495], 'ionic_force_magnitude': 10.94900467335162, 'motion_vector': [0.2743377685546875, -2.2898902893066406, -0.9024124145507812], 'cosine_ionic_motion': 0.31789813815261664, 'ionic_motion_component': 3.4806682002827785, 'ionic_force_x': 7.3180464617908, 'ionic_force_y': 0.31938037276268005, 'ionic_force_z': -8.137867994606495, 'radial_force': 7.325012480496868, 'axial_force': -8.137867994606495, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 780, 'contributions': [{'ion': 1327, 'force': [1.9322783946990967, 0.7810750007629395, -3.4608781337738037], 'magnitude': 4.039981842041016, 'distance': 9.065240859985352, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.18637019902355048, 'motion_component': 0.7529322689500795}, {'ion': 1341, 'force': [0.4868040978908539, 0.19157400727272034, -1.5694613456726074], 'magnitude': 1.654354214668274, 'distance': 14.16624641418457, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.27121075699936276, 'motion_component': 0.4486786489014434}, {'ion': 1355, 'force': [0.41514936089515686, -4.178457260131836, -1.8555198907852173], 'magnitude': 4.590730667114258, 'distance': 8.504095077514648, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.998896651421923, 'motion_component': 4.585665498980331}, {'ion': 1380, 'force': [1.7028212547302246, 1.3459678888320923, -0.46063730120658875], 'magnitude': 2.2188773155212402, 'distance': 12.232138633728027, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.4002253193375465, 'motion_component': -0.8880508790419137}, {'ion': 1476, 'force': [0.054844509810209274, 2.683497667312622, -0.06307730823755264], 'magnitude': 2.6847991943359375, 'distance': 11.120214462280273, 'before_closest_residue': 748, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.9133640530735111, 'motion_component': -2.4521990200139596}, {'ion': 2443, 'force': [2.726148843765259, -0.5042769312858582, -0.7282940149307251], 'magnitude': 2.8664603233337402, 'distance': 10.762076377868652, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.3605986416231447, 'motion_component': 1.033641706957674}]}, 6173: {'frame': 6173, 'ionic_force': [6.784936279058456, 2.012464940547943, -7.050760209560394], 'ionic_force_magnitude': 9.989924673416631, 'motion_vector': [-1.894927978515625, 0.30248260498046875, -0.6227035522460938], 'cosine_ionic_motion': -0.3898840075180566, 'ionic_motion_component': -3.8949118664751885, 'ionic_force_x': 6.784936279058456, 'ionic_force_y': 2.012464940547943, 'ionic_force_z': -7.050760209560394, 'radial_force': 7.077102192834173, 'axial_force': -7.050760209560394, 'before_closest_residue': 455, 'closest_residue': 780, 'next_closest_residue': 455, 'contributions': [{'ion': 1327, 'force': [1.4346952438354492, -0.13320499658584595, -2.9370408058166504], 'magnitude': 3.271437406539917, 'distance': 10.073948860168457, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.1409162394794962, 'motion_component': -0.46099865710665183}, {'ion': 1355, 'force': [0.2875460088253021, -2.611074686050415, -1.1207534074783325], 'magnitude': 2.8559556007385254, 'distance': 10.781850814819336, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.11052100472464929, 'motion_component': -0.31564307335446173}, {'ion': 1380, 'force': [2.0091943740844727, 1.0707746744155884, -0.7834347486495972], 'magnitude': 2.407735586166382, 'distance': 11.742610931396484, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.616692648196802, 'motion_component': -1.484832807733362}, {'ion': 1476, 'force': [0.7840487957000732, 4.45212459564209, -1.336418628692627], 'magnitude': 4.714038848876953, 'distance': 8.392135620117188, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.07288648656682731, 'motion_component': 0.34358971695424145}, {'ion': 2443, 'force': [2.269451856613159, -0.7661546468734741, -0.8731126189231873], 'magnitude': 2.549456834793091, 'distance': 11.411564826965</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>6449</v>
+      </c>
+      <c r="B23" t="n">
+        <v>6727</v>
+      </c>
+      <c r="C23" t="n">
+        <v>1341</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>{6449: {'frame': 6449, 'ionic_force': [11.088144078850746, 3.661605954170227, -9.956974852830172], 'ionic_force_magnitude': 15.345867375188023, 'motion_vector': [4.9669189453125, 1.6391181945800781, 0.8033828735351562], 'cosine_ionic_motion': 0.6536010129993487, 'ionic_motion_component': 10.030074461776548, 'ionic_force_x': 11.088144078850746, 'ionic_force_y': 3.661605954170227, 'ionic_force_z': -9.956974852830172, 'radial_force': 11.67708427977497, 'axial_force': -9.956974852830172, 'before_closest_residue': None, 'closest_residue': 130, 'next_closest_residue': 423, 'contributions': [{'ion': 1327, 'force': [3.5316085815429688, 2.2948412895202637, -0.9144463539123535], 'magnitude': 4.309845447540283, 'distance': 8.776840209960938, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.9018499490514568, 'motion_component': 3.886833904588357}, {'ion': 1330, 'force': [0.982691764831543, 1.5302084684371948, -6.489742279052734], 'magnitude': 6.739731311798096, 'distance': 7.018555641174316, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.060995501340076516, 'motion_component': 0.41109328010102075}, {'ion': 1355, 'force': [4.765550136566162, -4.245543003082275, 0.05606735870242119], 'magnitude': 6.3826518058776855, 'distance': 7.212211608886719, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.49610838474725943, 'motion_component': 3.1664871931964558}, {'ion': 1465, 'force': [0.14122642576694489, 0.30911684036254883, -1.894454836845398], 'magnitude': 1.924696683883667, 'distance': 13.133724212646484, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.030813358422604537, 'motion_component': -0.0593063682007644}, {'ion': 1476, 'force': [1.6670671701431274, 3.772982358932495, -0.7143987417221069], 'magnitude': 4.186272144317627, 'distance': 8.905438423156738, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 'SF', 'cosine_with_motion': 0.6270415061553786, 'motion_component': 2.6249663850423235}]}, 6450: {'frame': 6450, 'ionic_force': [11.005028426647186, 3.282705068588257, -4.414879508316517], 'ionic_force_magnitude': 12.303575265409675, 'motion_vector': [1.8098068237304688, -1.3127899169921875, -0.8244171142578125], 'cosine_ionic_motion': 0.6564770741103358, 'ionic_motion_component': 8.077015091332441, 'ionic_force_x': 11.005028426647186, 'ionic_force_y': 3.282705068588257, 'ionic_force_z': -4.414879508316517, 'radial_force': 11.484197979774107, 'axial_force': -4.414879508316517, 'before_closest_residue': 130, 'closest_residue': 423, 'next_closest_residue': 455, 'contributions': [{'ion': 1327, 'force': [1.6276063919067383, 0.8470562100410461, -0.08977655321359634], 'magnitude': 1.8370264768600464, 'distance': 13.44346809387207, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1105, 'cosine_with_motion': 0.4357820526866752, 'motion_component': 0.8005432095816627}, {'ion': 1330, 'force': [3.048281192779541, 1.3634477853775024, -2.819413661956787], 'magnitude': 4.370366096496582, 'distance': 8.71585750579834, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5810470822417294, 'motion_component': 2.5393885799464826}, {'ion': 1355, 'force': [2.8688948154449463, -1.2304490804672241, 0.45329388976097107], 'magnitude': 3.1543681621551514, 'distance': 10.259184837341309, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.855926739227634, 'motion_component': 2.699907953572965}, {'ion': 1465, 'force': [0.7390469908714294, 0.3952198624610901, -1.5287773609161377], 'magnitude': 1.7434303760528564, 'distance': 13.79960823059082, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5004290581086671, 'motion_component': 0.8724632119970935}, {'ion': 1476, 'force': [2.7211990356445312, 1.9074302911758423, -0.4302058219909668], 'magnitude': 3.3508644104003906, 'distance': 9.953839302062988, 'before_closest_residue': 1105, 'closest_residue': 'SF', 'next_closest_residue': 1105, 'cosine_with_motion': 0.34758559608259115, 'motion_component': 1.164712165083948}]}, 6451: {'frame': 6451, 'ionic_force': [8.739684104919434, 0.469412237405777, -2.0718104019761086], 'ionic_force_magnitude': 8.994155015572286, 'motion_vector': [-1.5418739318847656, -2.056304931640625, -0.31626129150390625], 'cosine_ionic_motion': -0.5918854713098048, 'ionic_motion_component': -5.323509680425447, 'ionic_force_x': 8.739684104919434, 'ionic_force_y': 0.469412237405777, 'ionic_force_z': -2.0718104019761086, 'radial_force': 8.75228119420347, 'axial_force': -2.0718104019761086, 'before_closest_residue': 423, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1327, 'force': [1.4240713119506836, 0.4835692346096039, -0.21571895480155945], 'magnitude': 1.5193264484405518, 'distance': 14.782349586486816, 'before_closest_residue': 1073, 'closest_residue': 1105, 'next_closest_residue': 1073, 'cosine_with_motion': -0.7934879036563897, 'motion_component': -1.2055671890198612}, {'ion': 1330, 'force': [2.4229938983917236, 0.5128621459007263, -2.0453357696533203], 'magnitude': 3.212059259414673, 'distance': 10.166635513305664, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.49817160709433006, 'motion_component': -1.6001567804949488}, {'ion': 1355, 'force': [2.7083451747894287, -1.8824938535690308, -0.10277257114648819], 'magnitude': 3.2999210357666016, 'distance': 10.030377388000488, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.03188205537431328, 'motion_component': -0.10520826545217403}, {'ion': 1476, 'force': [2.1842737197875977, 1.3554747104644775, 0.2920168936252594], 'magnitude': 2.5872063636779785, 'distance': 11.328006744384766, 'before_closest_residue': 'SF', 'closest_residue': 1105, 'next_closest_residue': 780, 'cosine_with_motion': -0.932502786587697, 'motion_component': -2.4125772285907994}]}, 6452: {'frame': 6452, 'ionic_force': [10.327910542488098, 1.1043216735124588, -5.13695291057229], 'ionic_force_magnitude': 11.58764634158565, 'motion_vector': [-0.060070037841796875, 3.2151107788085938, 1.4912796020507812], 'cosine_ionic_motion': -0.11517049748322489, 'ionic_motion_component': -1.3345549938200902, 'ionic_force_x': 10.327910542488098, 'ionic_force_y': 1.1043216735124588, 'ionic_force_z': -5.13695291057229, 'radial_force': 10.386783069469882, 'axial_force': -5.13695291057229, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 423, 'contributions': [{'ion': 1327, 'force': [1.7840296030044556, 0.277847021818161, -0.3307577669620514], 'magnitude': 1.8355820178985596, 'distance': 13.44875717163086, 'before_closest_residue': 1105, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.045015155333941806, 'motion_component': 0.08262900902508541}, {'ion': 1330, 'force': [2.474438190460205, -0.39485305547714233, -2.829497814178467], 'magnitude': 3.7795252799987793, 'distance': 9.372391700744629, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.4208171612386723, 'motion_component': -1.590489089812813}, {'ion': 1355, 'force': [2.0291547775268555, -1.468042254447937, -0.032318416982889175], 'magnitude': 2.504727840423584, 'distance': 11.513007164001465, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.5507784216766087, 'motion_component': -1.379550057396542}, {'ion': 1465, 'force': [0.6779139041900635, -0.06925506889820099, -1.4678304195404053], 'magnitude': 1.6182984113693237, 'distance': 14.323189735412598, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.4275121960333371, 'motion_component': -0.6918422968968603}, {'ion': 1476, 'force': [3.3623740673065186, 2.758625030517578, -0.4765484929084778], 'magnitude': 4.3752336502075195, 'distance': 8.711008071899414, 'before_closest_residue': 1105, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.5130463007121352, 'motion_component': 2.2446974624236695}]}, 6453: {'frame': 6453, 'ionic_force': [9.139528214931488, 2.8800260424613953, -3.7206843197345734], 'ionic_force_magnitude': 10.279543657376202, 'motion_vector': [-0.720062255859375, 0.6362991333007812, 0.15360260009765625], 'cosine_ionic_motion': -0.5318267452065297, 'ionic_motion_component': -5.466936245510812, 'ionic_force_x': 9.139528214931488, 'ionic_force_y': 2.8800260424613953, 'ionic_force_z': -3.7206843197345734, 'radial_force': 9.582563644285624, 'axial_force': -3.7206843197345734, 'before_closest_residue': 455, 'closest_residue': 423, 'next_closest_residue': 455, 'contributions': [{'ion': 1327, 'force': [1.5509934425354004, 0.7286680340766907, -0.15393760800361633], 'magnitude': 1.7205332517623901, 'distance': 13.891127586364746, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.40423643446915525, 'motion_component': -0.695502212911935}, {'ion': 1330, 'force': [2.758227825164795, 1.1968661546707153, -2.8668406009674072], 'magnitude': 4.15440559387207, 'distance': 8.939528465270996, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.41182200202131236, 'motion_component': -1.7108755555546544}, {'ion': 1355, 'force': [3.0123891830444336, -1.6359062194824219, 0.6324722766876221], 'magnitude': 3.4857852458953857, 'distance': 9.75930118560791, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.9176910640590641, 'motion_component': -3.1988739910453567}, {'ion': 1465, 'force': [0.8180946707725525, 0.47484707832336426, -1.7255505323410034], 'magnitude': 1.9678118228912354, 'distance': 12.989046096801758, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.2882548305003571, 'motion_component': -0.5672312566884852}, {'ion': 1476, 'force': [0.9998230934143066, 2.115550994873047, 0.39317214488983154], 'magnitude': 2.3727171421051025, 'distance': 11.828947067260742, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 1105, 'cosine_with_motion': 0.29735811219878866, 'motion_component': 0.7055466857160209}]}, 6454: {'frame': 6454, 'ionic_force': [11.519911527633667, 2.6967788338661194, -4.047921255230904], 'ionic_force_magnitude': 12.504664896423474, 'motion_vector': [1.3884010314941406, -1.9174156188964844, -1.4060287475585938], 'cosine_ionic_motion': 0.4796662185340068, 'ionic_motion_component': 5.998065324902385, 'ionic_force_x': 11.519911527633667, 'ionic_force_y': 2.6967788338661194, 'ionic_force_z': -4.047921255230904, 'radial_force': 11.831355699297328, 'axial_force': -4.047921255230904, 'before_closest_residue': 423, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1327, 'force': [1.6504477262496948, 0.7416374683380127, -0.09881125390529633], 'magnitude': 1.8121168613433838, 'distance': 13.535551071166992, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.20210468545852037, 'motion_component': 0.36623730695197043}, {'ion': 1330, 'force': [3.0074729919433594, 1.765475869178772, -3.316441059112549], 'magnitude': 4.812543869018555, 'distance': 8.305804252624512, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.41155781151904886, 'motion_component': 1.980640093093207}, {'ion': 1355, 'force': [3.105611801147461, -2.121004343032837, 0.69764643907547], 'magnitude': 3.824943780899048, 'distance': 9.316579818725586, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 130, 'cosine_with_motion': 0.7024427580038051, 'motion_component': 2.686804031990011}, {'ion': 1465, 'force': [0.7477613687515259, 0.573081910610199, -1.774617314338684], 'magnitude': 2.009187936782837, 'distance': 12.854605674743652, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.44007607183732467, 'motion_component': 0.884195577283851}, {'ion': 1476, 'force': [3.008617639541626, 1.7375879287719727, 0.44430193305015564], 'magnitude': 3.502626895904541, 'distance': 9.735810279846191, 'before_closest_residue': 780, 'closest_residue': 1105, 'next_closest_residue': 748, 'cosine_with_motion': 0.022893770199989852, 'motion_component': 0.08018833834593231}]}, 6455: {'frame': 6455, 'ionic_force': [12.358292996883392, 6.324190944433212, -5.279603046365082], 'ionic_force_magnitude': 14.852508381605297, 'motion_vector': [-0.5884780883789062, -1.5783882141113281, 0.5686721801757812], 'cosine_ionic_motion': -0.7671182394454574, 'ionic_motion_component': -11.393630081045956, 'ionic_force_x': 12.358292996883392, 'ionic_force_y': 6.324190944433212, 'ionic_force_z': -5.279603046365082, 'radial_force': 13.882463646574701, 'axial_force': -5.279603046365082, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1327, 'force': [1.4005006551742554, 0.43182238936424255, -0.22161030769348145], 'magnitude': 1.482222557067871, 'distance': 14.966226577758789, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.6192032869882479, 'motion_component': -0.9177970962816141}, {'ion': 1330, 'force': [2.4547295570373535, 0.45704543590545654, -2.393592596054077], 'magnitude': 3.458883285522461, 'distance': 9.79718017578125, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5735505794656885, 'motion_component': -1.9838444846666337}, {'ion': 1355, 'force': [2.053807497024536, -1.2260771989822388, 0.0074832020327448845], 'magnitude': 2.3919544219970703, 'distance': 11.781282424926758, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 98, 'cosine_with_motion': 0.17185773231780294, 'motion_component': 0.4110758833959836}, {'ion': 1465, 'force': [0.7318766713142395, 0.13336181640625, -1.374646544456482], 'magnitude': 1.5630360841751099, 'distance': 14.574193954467773, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5120317863135961, 'motion_component': -0.800324184106337}, {'ion': 1476, 'force': [5.717378616333008, 6.528038501739502, -1.2972368001937866], 'magnitude': 8.77419662475586, 'distance': 6.151278018951416, 'before_closest_residue': 1105, 'closest_residue': 748, 'next_closest_residue': 780, 'cosine_with_motion': -0.923473711829239, 'motion_component': -8.102740021611602}]}, 6456: {'frame': 6456, 'ionic_force': [9.233830749988556, 1.1224905923008919, -4.864724556449801], 'ionic_force_magnitude': 10.497102479225585, 'motion_vector': [0.4046783447265625, 0.90826416015625, -0.1713714599609375], 'cosine_ionic_motion': 0.5277719062348334, 'ionic_motion_component': 5.540075785403283, 'ionic_force_x': 9.233830749988556, 'ionic_force_y': 1.1224905923008919, 'ionic_force_z': -4.864724556449801, 'radial_force': 9.301807106645365, 'axial_force': -4.864724556449801, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1327, 'force': [1.8978043794631958, 0.4435109794139862, -0.23132824897766113], 'magnitude': 1.9626197814941406, 'distance': 13.006216049194336, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.6112616198270099, 'motion_component': 1.1996741161612672}, {'ion': 1330, 'force': [2.841651201248169, -0.0774279534816742, -3.014273166656494], 'magnitude': 4.143286228179932, 'distance': 8.951516151428223, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.3818119092933767, 'motion_component': 1.5819559606615972}, {'ion': 1355, 'force': [1.5171762704849243, -1.7436965703964233, -0.024102753028273582], 'magnitude': 2.3114676475524902, 'distance': 11.984643936157227, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.41403437645778535, 'motion_component': -0.9570270502468217}, {'ion': 1465, 'force': [0.7945194840431213, 0.04755014926195145, -1.6000595092773438], 'magnitude': 1.7870961427688599, 'distance': 13.629975318908691, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.3543289360404364, 'motion_component': 0.6332198785321617}, {'ion': 1476, 'force': [2.1826794147491455, 2.4525539875030518, 0.005039121489971876], 'magnitude': 3.2831594944000244, 'distance': 10.055949211120605, 'before_closest_residue': 748, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.9388069691631643, 'motion_component': 3.082252959352908}]}, 6457: {'frame': 6457, 'ionic_force': [9.096073269844055, 2.163865104317665, -4.737605880945921], 'ionic_force_magnitude': 10.481687392935767, 'motion_vector': [-0.11692047119140625, 0.4889183044433594, -0.9179763793945312], 'cosine_ionic_motion': 0.39593006496444544, 'ionic_motion_component': 4.1500151704220665, 'ionic_force_x': 9.096073269844055, 'ionic_force_y': 2.163865104317665, 'ionic_force_z': -4.737605880945921, 'radial_force': 9.349912358950496, 'axial_force': -4.737605880945921, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1327, 'force': [1.7632050514221191, 0.5160462856292725, -0.29753151535987854], 'magnitude': 1.8611074686050415, 'distance': 13.356212615966797, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1105, 'cosine_with_motion': 0.16391204728999575, 'motion_component': 0.3050579272681855}, {'ion': 1330, 'force': [2.496544122695923, 0.2790150046348572, -2.758460760116577], 'magnitude': 3.730909824371338, 'distance': 9.433257102966309, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.6086652807854851, 'motion_component': 2.270875241323065}, {'ion': 1355, 'force': [1.7096211910247803, -1.5737277269363403, -0.002807583659887314], 'magnitude': 2.3236677646636963, 'distance': 11.953140258789062, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.39751123302335817, 'motion_component': -0.9236840021138677}, {'ion': 1465, 'force': [0.7106510400772095, 0.08507032692432404, -1.5122408866882324], 'magnitude': 1.6730613708496094, 'distance': 14.086824417114258, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.7690871425186415, 'motion_component': 1.2867299912699872}, {'ion': 1476, 'force': [2.4160518646240234, 2.8574612140655518, -0.16656513512134552], 'magnitude': 3.7456822395324707, 'distance': 9.414636611938477, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.32331517770345275, 'motion_component': 1.211035906255364}]}, 6458: {'frame': 6458, 'ionic_force': [7.916607975959778, 2.0578590631484985, -4.374101959168911], 'ionic_force_magnitude': 9.27578749853713, 'motion_vector': [1.0696640014648438, -0.24401092529296875, -0.6402435302734375], 'cosine_ionic_motion': 0.9137336519254561, 'ionic_motion_component': 8.475599185522823, 'ionic_force_x': 7.916607975959778, 'ionic_force_y': 2.0578590631484985, 'ionic_force_z': -4.374101959168911, 'radial_force': 8.179698391066285, 'axial_force': -4.374101959168911, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1327, 'force': [1.6573450565338135, 0.6732655763626099, -0.3442486822605133], 'magnitude': 1.821698784828186, 'distance': 13.499906539916992, 'before_closest_residue': 1073, 'closest_residue': 1105, 'next_closest_residue': 1073, 'cosine_with_motion': 0.7903435021550261, 'motion_component': 1.4397677682584291}, {'ion': 1330, 'force': [2.1297972202301025, 0.3772757053375244, -2.3562591075897217], 'magnitude': 3.198488712310791, 'distance': 10.188179969787598, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.909348525788148, 'motion_component': 2.9085410090015955}, {'ion': 1355, 'force': [1.8750309944152832, -1.692273497581482, -0.19635580480098724], 'magnitude': 2.5333943367004395, 'distance': 11.447684288024902, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.7906118493156139, 'motion_component': 2.002931512535695}, {'ion': 1465, 'force': [0.6408071517944336, 0.15025389194488525, -1.3914772272109985], 'magnitude': 1.5392916202545166, 'distance': 14.686171531677246, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.7874154182272478, 'motion_component': 1.212062011077471}, {'ion': 1476, 'force': [1.613627552986145, 2.549337387084961, -0.08576113730669022], 'magnitude': 3.018322229385376, 'distance': 10.487844467163086, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 130, 'cosine_with_motion': 0.30225307836269955, 'motion_component': 0.9122972296447824}]}, 6459: {'frame': 6459, 'ionic_force': [10.070922791957855, -0.5866779759526253, -2.2287999242544174], 'ionic_force_magnitude': 10.33127417269528, 'motion_vector': [-1.1145095825195312, -2.0631027221679688, 1.3752975463867188], 'cosine_ionic_motion': -0.46569356277561985, 'ionic_motion_component': -4.81120787749421, 'ionic_force_x': 10.070922791957855, 'ionic_force_y': -0.5866779759526253, 'ionic_force_z': -2.2287999242544174, 'radial_force': 10.087996675705444, 'axial_force': -2.2287999242544174, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1327, 'force': [1.3782541751861572, 0.488964319229126, -0.2811233103275299], 'magnitude': 1.4891947507858276, 'distance': 14.931151390075684, 'before_closest_residue': 1105, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.7241283073273487, 'motion_component': -1.0783680709431334}, {'ion': 1330, 'force': [1.798455834388733, 0.22501133382320404, -1.8021730184555054], 'magnitude': 2.5559539794921875, 'distance': 11.397051811218262, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7120000779386864, 'motion_component': -1.8198394788149406}, {'ion': 1355, 'force': [1.6811152696609497, -1.412225365638733, -0.18546278774738312], 'magnitude': 2.2033896446228027, 'distance': 12.275053977966309, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.131036077420042, 'motion_component': 0.2887235227632176}, {'ion': 1465, 'force': [0.7065557837486267, 0.13394781947135925, -1.2894666194915771], 'magnitude': 1.476444125175476, 'distance': 14.995485305786133, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7068925848535891, 'motion_component': -1.0436874044938556}, {'ion': 1476, 'force': [4.506541728973389, -0.022376082837581635, 1.3294258117675781], 'magnitude': 4.698594570159912, 'distance': 8.405916213989258, 'before_closest_residue': 780, 'closest_residue': 130, 'next_closest_residue': 1105, 'cosine_with_motion': -0.24646441555121948, 'motion_component': -1.1580363934527225}]}, 6460: {'frame': 6460, 'ionic_force': [10.501655519008636, -0.10368964076042175, -3.4797102883458138], 'ionic_force_magnitude': 11.063629778347849, 'motion_vector': [-4.040958404541016, 4.321376800537109, 0.48625946044921875], 'cosine_ionic_motion': -0.6787244499052771, 'ionic_motion_component': -7.5091560352647875, 'ionic_force_x': 10.501655519008636, 'ionic_force_y': -0.10368964076042175, 'ionic_force_z': -3.4797102883458138, 'radial_force': 10.502167403994548, 'axial_force': -3.4797102883458138, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1327, 'force': [1.7326629161834717, 0.26751768589019775, -0.18968352675437927], 'magnitude': 1.7634246349334717, 'distance': 13.721152305603027, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.5672191023917383, 'motion_component': -1.000248120969888}, {'ion': 1330, 'force': [2.9949021339416504, -0.2766885459423065, -2.8809821605682373], 'magnitude': 4.164859294891357, 'distance': 8.928301811218262, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5945175260413068, 'motion_component': -2.476081887604808}, {'ion': 1355, 'force': [1.500700831413269, -1.4485684633255005, -0.06197259575128555], 'magnitude': 2.0866944789886475, 'distance': 12.613615989685059, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.9973273968062647, 'motion_component': -2.0811176520772103}, {'ion': 1465, 'force': [0.7845519185066223, -0.08523333072662354, -1.5313416719436646], 'magnitude': 1.7227286100387573, 'distance': 13.88227367401123, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.4188348006950093, 'motion_component': -0.7215386801651054}, {'ion': 1476, 'force': [3.488837718963623, 1.439283013343811, 1.184269666671753], 'magnitude': 3.955504894256592, 'distance': 9.161531448364258, 'before_closest_residue': 130, 'closest_residue': 1105, 'next_closest_residue': 1105, 'cosine_with_motion': -0.3110019460566897, 'motion_component': -1.2301697156885645}]}, 6461: {'frame': 6461, 'ionic_force': [9.932420074939728, 2.0168667435646057, -6.994688577950001], 'ionic_force_magnitude': 12.314478807845129, 'motion_vector': [1.1206817626953125, -1.6179962158203125, -0.19561004638671875], 'cosine_ionic_motion': 0.3791964013859275, 'ionic_motion_component': 4.669606048878139, 'ionic_force_x': 9.932420074939728, 'ionic_force_y': 2.0168667435646057, 'ionic_force_z': -6.994688577950001, 'radial_force': 10.135123087874296, 'axial_force': -6.994688577950001, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1327, 'force': [2.1432230472564697, 1.4571622610092163, -0.19045372307300568], 'magnitude': 2.598653554916382, 'distance': 11.30302906036377, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.01584520331532757, 'motion_component': 0.041176191507181326}, {'ion': 1330, 'force': [2.3041412830352783, 2.8984789848327637, -5.283723831176758], 'magnitude': 6.451975345611572, 'distance': 7.173360824584961, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.08415776090292298, 'motion_component': -0.5429837928883217}, {'ion': 1355, 'force': [4.2389912605285645, -5.536309242248535, 0.24877865612506866], 'magnitude': 6.977224349975586, 'distance': 6.898071765899658, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 130, 'cosine_with_motion': 0.9898079870830155, 'motion_component': 6.906112256101975}, {'ion': 1465, 'force': [0.33492982387542725, 0.5356461405754089, -1.8747485876083374], 'magnitude': 1.9783267974853516, 'distance': 12.95448112487793, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.031844101211086266, 'motion_component': -0.06299803976510887}, {'ion': 1476, 'force': [0.911134660243988, 2.661888599395752, 0.10545890778303146], 'magnitude': 2.8154821395874023, 'distance': 10.859070777893066, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 780, 'cosine_with_motion': -0.5937529033887871, 'motion_component': -1.6717006091549076}]}, 6462: {'frame': 6462, 'ionic_force': [17.567132353782654, 1.7452539205551147, -1.5626121181994677], 'ionic_force_magnitude': 17.72263544212525, 'motion_vector': [4.015556335449219, -1.5489654541015625, -0.00579833984375], 'cosine_ionic_motion': 0.8894839537147118, 'ionic_motion_component': 15.763999843306046, 'ionic_force_x': 17.567132353782654, 'ionic_force_y': 1.7452539205551147, 'ionic_force_z': -1.5626121181994677, 'radial_force': 17.653612955498097, 'axial_force': -1.5626121181994677, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1327, 'force': [2.2711713314056396, 1.3109850883483887, -0.3511980175971985], 'magnitude': 2.64579701423645, 'distance': 11.201876640319824, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.6227399651913887, 'motion_component': 1.6476434611698196}, {'ion': 1330, 'force': [3.1668646335601807, 2.0477538108825684, -5.296675682067871], 'magnitude': 6.502084255218506, 'distance': 7.145666599273682, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.34217069584171755, 'motion_component': 2.224822717614096}, {'ion': 1355, 'force': [5.7192840576171875, -7.260217189788818, 0.016965268179774284], 'magnitude': 9.242362022399902, 'distance': 5.993459224700928, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 98, 'cosine_with_motion': 0.860054081373168, 'motion_component': 7.948930985423409}, {'ion': 1465, 'force': [0.5201071500778198, 0.3467801809310913, -1.9481827020645142], 'magnitude': 2.0460166931152344, 'distance': 12.738388061523438, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.1774553755351891, 'motion_component': 0.36307663779865335}, {'ion': 1476, 'force': [5.889705181121826, 5.299952030181885, 6.016479015350342], 'magnitude': 9.948675155639648, 'distance': 5.776787757873535, 'before_closest_residue': 1105, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.3597992195773787, 'motion_component': 3.5795255754979527}]}, 6463: {'frame': 6463, 'ionic_force': [15.515380442142487, 2.0406659450381994, -1.9564794301986694], 'ionic_force_magnitude': 15.770832556477377, 'motion_vector': [-1.9192962646484375, 4.6290435791015625, 0.8290939331054688], 'cosine_ionic_motion': -0.2740715950300907, 'ionic_motion_component': -4.322337233706238, 'ionic_force_x': 15.515380442142487, 'ionic_force_y': 2.0406659450381994, 'ionic_force_z': -1.9564794301986694, 'radial_force': 15.649004689233633, 'axial_force': -1.9564794301986694, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 423, 'contributions': [{'ion': 1327, 'force': [1.7279499769210815, 0.4192473888397217, -0.20830027759075165], 'magnitude': 1.7902426719665527, 'distance': 13.617992401123047, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1105, 'cosine_with_motion': -0.17028570485659653, 'motion_component': -0.3048527198939759}, {'ion': 1330, 'force': [2.942939281463623, -0.07083207368850708, -2.4105186462402344], 'magnitude': 3.8048007488250732, 'distance': 9.341208457946777, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.4126534114558553, 'motion_component': -1.570064019902123}, {'ion': 1355, 'force': [1.4266270399093628, -1.3901089429855347, 0.13944165408611298], 'magnitude': 1.9967752695083618, 'distance': 12.894497871398926, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.893040155913853, 'motion_component': -1.783200516420262}, {'ion': 1465, 'force': [0.8499615788459778, -0.021102407947182655, -1.4299547672271729], 'magnitude': 1.6636258363723755, 'distance': 14.126716613769531, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.34491933978937955, 'motion_component': -0.5738166950758564}, {'ion': 1476, 'force': [8.567902565002441, 3.103461980819702, 1.9528526067733765], 'magnitude': 9.319552421569824, 'distance': 5.968586444854736, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 455, 'cosine_with_motion': -0.009700397960359285, 'motion_component': -0.09040337073399485}]}, 6464: {'frame': 6464, 'ionic_force': [11.33767420053482, 4.5525089502334595, -1.6449899077415466], 'ionic_force_magnitude'</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>6569</v>
+      </c>
+      <c r="B24" t="n">
+        <v>6670</v>
+      </c>
+      <c r="C24" t="n">
+        <v>1465</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>{6569: {'frame': 6569, 'ionic_force': [8.93659296631813, 4.198592029511929, -11.964962244033813], 'ionic_force_magnitude': 15.51293622681027, 'motion_vector': [0.9375572204589844, 4.542621612548828, 3.9090347290039062], 'cosine_ionic_motion': -0.20531702194883455, 'ionic_motion_component': -3.185069867770875, 'ionic_force_x': 8.93659296631813, 'ionic_force_y': 4.198592029511929, 'ionic_force_z': -11.964962244033813, 'radial_force': 9.87374644579897, 'axial_force': -11.964962244033813, 'before_closest_residue': None, 'closest_residue': 455, 'next_closest_residue': 423, 'contributions': [{'ion': 1327, 'force': [2.5776994228363037, 1.23420250415802, -1.3029985427856445], 'magnitude': 3.1409544944763184, 'distance': 10.281067848205566, 'before_closest_residue': 1105, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.15377313307214993, 'motion_component': 0.4829944183947106}, {'ion': 1330, 'force': [3.5478971004486084, -3.1198573112487793, -2.1965181827545166], 'magnitude': 5.210160732269287, 'distance': 7.982583522796631, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.6148617942807654, 'motion_component': -3.20352882053065}, {'ion': 1341, 'force': [1.5748634338378906, 5.740958213806152, -3.378621816635132], 'magnitude': 6.844989776611328, 'distance': 6.964383125305176, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.3455697276985564, 'motion_component': 2.365421161972364}, {'ion': 1359, 'force': [1.0105098485946655, 0.24263377487659454, -3.6123909950256348], 'magnitude': 3.7589054107666016, 'distance': 9.398062705993652, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5294201717457786, 'motion_component': -1.990040356360307}, {'ion': 1374, 'force': [0.22562316060066223, 0.10065484791994095, -1.4744327068328857], 'magnitude': 1.494987964630127, 'distance': 14.902193069458008, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5618215292436758, 'motion_component': -0.8399164247898128}]}, 6570: {'frame': 6570, 'ionic_force': [12.369088254868984, 9.554802000522614, -1.3525469191372395], 'ionic_force_magnitude': 15.688147395227915, 'motion_vector': [0.08165740966796875, 0.8572654724121094, 0.46636962890625], 'cosine_ionic_motion': 0.5578220875076787, 'ionic_motion_component': 8.751195129134187, 'ionic_force_x': 12.369088254868984, 'ionic_force_y': 9.554802000522614, 'ionic_force_z': -1.3525469191372395, 'radial_force': 15.629734019679567, 'axial_force': -1.3525469191372395, 'before_closest_residue': 455, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1327, 'force': [1.5750917196273804, 1.453436017036438, -0.059865642338991165], 'magnitude': 2.1440553665161133, 'distance': 12.443742752075195, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.6413605893494628, 'motion_component': 1.3751127123759574}, {'ion': 1330, 'force': [8.851373672485352, -0.5448993444442749, 0.612082302570343], 'magnitude': 8.889227867126465, 'distance': 6.1113481521606445, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.06215821404243742, 'motion_component': 0.5525385419218214}, {'ion': 1341, 'force': [-0.1118030920624733, 4.923777103424072, 3.27870774269104], 'magnitude': 5.9165873527526855, 'distance': 7.490889549255371, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.9908006826356204, 'motion_component': 5.862158742332892}, {'ion': 1359, 'force': [1.5930393934249878, 2.9040167331695557, -3.243910789489746], 'magnitude': 4.636167049407959, 'distance': 8.462321281433105, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.24375800960093685, 'motion_component': 1.130102852027684}, {'ion': 1374, 'force': [0.4613865613937378, 0.8184714913368225, -1.9395605325698853], 'magnitude': 2.155149221420288, 'distance': 12.411674499511719, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.07828591522281605, 'motion_component': -0.1687178298596086}]}, 6571: {'frame': 6571, 'ionic_force': [10.874882519245148, 11.021745204925537, -1.5739329904317856], 'ionic_force_magnitude': 15.563393017849684, 'motion_vector': [-0.7143974304199219, 2.6378211975097656, 0.46242523193359375], 'cosine_ionic_motion': 0.4770052911616335, 'ionic_motion_component': 7.423820817942322, 'ionic_force_x': 10.874882519245148, 'ionic_force_y': 11.021745204925537, 'ionic_force_z': -1.5739329904317856, 'radial_force': 15.483602202642729, 'axial_force': -1.5739329904317856, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1327, 'force': [0.9435466527938843, 1.3866626024246216, -0.0861724466085434], 'magnitude': 1.6794461011886597, 'distance': 14.060022354125977, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.6324180897014997, 'motion_component': 1.0621120842852612}, {'ion': 1330, 'force': [7.051734924316406, 1.6229393482208252, 0.9881018400192261], 'magnitude': 7.3032355308532715, 'distance': 6.742351531982422, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.014810253427721524, 'motion_component': -0.10816276256291779}, {'ion': 1341, 'force': [0.5937607288360596, 3.663236141204834, 2.101393938064575], 'magnitude': 4.264704704284668, 'distance': 8.82316780090332, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.8637998705639303, 'motion_component': 3.683851482704153}, {'ion': 1359, 'force': [1.727158784866333, 3.3323826789855957, -2.602457046508789], 'magnitude': 4.5673441886901855, 'distance': 8.525839805603027, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.501837686085301, 'motion_component': 2.29206552316883}, {'ion': 1374, 'force': [0.5586814284324646, 1.0165244340896606, -1.9747992753982544], 'magnitude': 2.290257453918457, 'distance': 12.040011405944824, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.21567643245512247, 'motion_component': 0.49395454936455074}]}, 6572: {'frame': 6572, 'ionic_force': [4.297864839434624, 8.788159370422363, -1.320813924074173], 'ionic_force_magnitude': 9.871572150372959, 'motion_vector': [0.8923988342285156, -0.882781982421875, -0.6154251098632812], 'cosine_ionic_motion': -0.2253358781914698, 'ionic_motion_component': -2.224419379634747, 'ionic_force_x': 4.297864839434624, 'ionic_force_y': 8.788159370422363, 'ionic_force_z': -1.320813924074173, 'radial_force': 9.782810807635544, 'axial_force': -1.320813924074173, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1330, 'force': [3.4389588832855225, 2.7700512409210205, 0.2946772277355194], 'magnitude': 4.425658702850342, 'distance': 8.661239624023438, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.07147438925554626, 'motion_component': 0.31632126731567206}, {'ion': 1341, 'force': [-0.10774736106395721, 2.0299341678619385, 1.3322513103485107], 'magnitude': 2.430459976196289, 'distance': 11.687585830688477, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.7969983098200872, 'motion_component': -1.9370725058540001}, {'ion': 1359, 'force': [0.6919946074485779, 2.870731830596924, -1.4831961393356323], 'magnitude': 3.304516315460205, 'distance': 10.02340030670166, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.21730627483870296, 'motion_component': -0.718092146719588}, {'ion': 1374, 'force': [0.2746587097644806, 1.1174421310424805, -1.4645463228225708], 'magnitude': 1.8625279664993286, 'distance': 13.351118087768555, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.061434877066536324, 'motion_component': 0.11442417383104164}]}, 6573: {'frame': 6573, 'ionic_force': [6.707516588270664, 9.176944971084595, -0.1950500402599573], 'ionic_force_magnitude': 11.368603357600545, 'motion_vector': [-0.3231239318847656, -0.48430633544921875, 0.06146240234375], 'cosine_ionic_motion': -0.995217753560235, 'ionic_motion_component': -11.31423589466856, 'ionic_force_x': 6.707516588270664, 'ionic_force_y': 9.176944971084595, 'ionic_force_z': -0.1950500402599573, 'radial_force': 11.366930007008971, 'axial_force': -0.1950500402599573, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1327, 'force': [0.9881269335746765, 1.1771571636199951, 0.006705602630972862], 'magnitude': 1.5369250774383545, 'distance': 14.697473526000977, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.9880008358344904, 'motion_component': -1.5184832920336617}, {'ion': 1330, 'force': [4.258534908294678, 1.36393404006958, 1.1857856512069702], 'magnitude': 4.62617826461792, 'distance': 8.471452713012695, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.7250604061209903, 'motion_component': -3.354258527189531}, {'ion': 1341, 'force': [-0.05445399135351181, 2.8371944427490234, 1.6453436613082886], 'magnitude': 3.28021240234375, 'distance': 10.060464859008789, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 'SF', 'cosine_with_motion': -0.6537031557818106, 'motion_component': -2.144285189327313}, {'ion': 1359, 'force': [1.1280900239944458, 2.8237078189849854, -1.7318087816238403], 'magnitude': 3.499296188354492, 'distance': 9.740442276000977, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8974276319060125, 'motion_component': -3.14036519314781}, {'ion': 1374, 'force': [0.387218713760376, 0.9749515056610107, -1.3010761737823486], 'magnitude': 1.6713072061538696, 'distance': 14.094215393066406, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6921791265166704, 'motion_component': -1.1568440041993604}]}, 6574: {'frame': 6574, 'ionic_force': [9.922765612602234, 10.655503034591675, -1.8789064027369022], 'ionic_force_magnitude': 14.680984694259426, 'motion_vector': [0.2715606689453125, -0.07678985595703125, -0.05289459228515625], 'cosine_ionic_motion': 0.4687223494525201, 'ionic_motion_component': 6.881305638169765, 'ionic_force_x': 9.922765612602234, 'ionic_force_y': 10.655503034591675, 'ionic_force_z': -1.8789064027369022, 'radial_force': 14.560254885228959, 'axial_force': -1.8789064027369022, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1327, 'force': [0.8655595183372498, 1.3287378549575806, -0.03194442763924599], 'magnitude': 1.5861141681671143, 'distance': 14.467777252197266, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': 0.295794977559575, 'motion_component': 0.4691645916303158}, {'ion': 1330, 'force': [6.645339488983154, 1.9468575716018677, 1.6377795934677124], 'magnitude': 7.115694999694824, 'distance': 6.830624103546143, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.7677054146793523, 'motion_component': 5.462757472369846}, {'ion': 1341, 'force': [0.7769212126731873, 3.7414112091064453, 0.19452917575836182], 'magnitude': 3.826173782348633, 'distance': 9.315082550048828, 'before_closest_residue': 780, 'closest_residue': 'SF', 'next_closest_residue': 780, 'cosine_with_motion': -0.07883855880427347, 'motion_component': -0.3016500287318795}, {'ion': 1359, 'force': [1.2521162033081055, 2.632829427719116, -2.2195000648498535], 'magnitude': 3.664118766784668, 'distance': 9.518845558166504, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.24262122220108004, 'motion_component': 0.8889929729182668}, {'ion': 1374, 'force': [0.3828291893005371, 1.005666971206665, -1.459770679473877], 'magnitude': 1.8135199546813965, 'distance': 13.530313491821289, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.19963431493602773, 'motion_component': 0.3620408168458269}]}, 6575: {'frame': 6575, 'ionic_force': [6.102406769990921, 8.403478920459747, -1.6997588761150837], 'ionic_force_magnitude': 10.52364036776126, 'motion_vector': [-0.7413291931152344, 0.8488311767578125, 0.4405517578125], 'cosine_ionic_motion': 0.14609900437198084, 'ionic_motion_component': 1.5374933800987063, 'ionic_force_x': 6.102406769990921, 'ionic_force_y': 8.403478920459747, 'ionic_force_z': -1.6997588761150837, 'radial_force': 10.385462259959464, 'axial_force': -1.6997588761150837, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1330, 'force': [3.698859691619873, 1.877339243888855, -0.03207122161984444], 'magnitude': 4.148131370544434, 'distance': 8.94628620147705, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.2316347697950632, 'motion_component': -0.96085146489291}, {'ion': 1341, 'force': [0.6937668323516846, 2.8005433082580566, 1.644039273262024], 'magnitude': 3.320725917816162, 'distance': 9.998907089233398, 'before_closest_residue': 'SF', 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.6438655630588777, 'motion_component': 2.1381010385898946}, {'ion': 1359, 'force': [1.2716120481491089, 2.7411482334136963, -1.8873075246810913], 'magnitude': 3.5626986026763916, 'distance': 9.653382301330566, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.12819220190672265, 'motion_component': 0.45671016417391286}, {'ion': 1374, 'force': [0.4381681978702545, 0.9844481348991394, -1.4244194030761719], 'magnitude': 1.7860851287841797, 'distance': 13.633832931518555, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.05400995022278874, 'motion_component': -0.09646636963300992}]}, 6576: {'frame': 6576, 'ionic_force': [5.697530130855739, 9.966541528701782, -1.1423418633639812], 'ionic_force_magnitude': 11.536842920320106, 'motion_vector': [0.1239013671875, -0.14241409301757812, -0.3520050048828125], 'cosine_ionic_motion': -0.06756220567549721, 'ionic_motion_component': -0.7794545542285709, 'ionic_force_x': 5.697530130855739, 'ionic_force_y': 9.966541528701782, 'ionic_force_z': -1.1423418633639812, 'radial_force': 11.480148066786693, 'axial_force': -1.1423418633639812, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1327, 'force': [0.8476411700248718, 1.4078731536865234, 0.05625929310917854], 'magnitude': 1.6443136930465698, 'distance': 14.209431648254395, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.17552367847627473, 'motion_component': -0.28861598567276614}, {'ion': 1330, 'force': [3.670255661010742, 1.709186315536499, 0.31133517622947693], 'magnitude': 4.060667991638184, 'distance': 9.042120933532715, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.06273120196461206, 'motion_component': 0.25473058028006434}, {'ion': 1341, 'force': [0.002328316681087017, 2.6095755100250244, 1.5804171562194824], 'magnitude': 3.050837278366089, 'distance': 10.431806564331055, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.7612668469814414, 'motion_component': -2.322501282066058}, {'ion': 1359, 'force': [0.9095866680145264, 3.105701446533203, -1.6332862377166748], 'magnitude': 3.624962568283081, 'distance': 9.570117950439453, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.16943698437349575, 'motion_component': 0.6142027188966424}, {'ion': 1374, 'force': [0.2677183151245117, 1.1342051029205322, -1.4570672512054443], 'magnitude': 1.8657810688018799, 'distance': 13.339473724365234, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5159927105714089, 'motion_component': 0.9627294710664245}]}, 6577: {'frame': 6577, 'ionic_force': [10.770041853189468, 11.033284544944763, -1.4359604306519032], 'ionic_force_magnitude': 15.48512679081343, 'motion_vector': [2.2769126892089844, -2.477092742919922, -0.91888427734375], 'cosine_ionic_motion': -0.027561089715659084, 'ionic_motion_component': -0.42678696873996497, 'ionic_force_x': 10.770041853189468, 'ionic_force_y': 11.033284544944763, 'ionic_force_z': -1.4359604306519032, 'radial_force': 15.41840359340648, 'axial_force': -1.4359604306519032, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1327, 'force': [1.0223180055618286, 1.2306550741195679, 0.052624136209487915], 'magnitude': 1.6007546186447144, 'distance': 14.401464462280273, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1105, 'cosine_with_motion': -0.13775037653817027, 'motion_component': -0.22050455002434874}, {'ion': 1330, 'force': [7.852027416229248, 3.727412223815918, 1.5429376363754272], 'magnitude': 8.827717781066895, 'distance': 6.132602691650391, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.23473986102912722, 'motion_component': 2.0722171355634664}, {'ion': 1341, 'force': [0.4523809254169464, 1.9864200353622437, 0.05863363668322563], 'magnitude': 2.0381243228912354, 'distance': 12.76302719116211, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 'SF', 'cosine_with_motion': -0.5548802485993717, 'motion_component': -1.1309149590530434}, {'ion': 1359, 'force': [1.0853403806686401, 2.987722158432007, -1.669343113899231], 'magnitude': 3.5904252529144287, 'distance': 9.616036415100098, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.27116527483362757, 'motion_component': -0.9735986645634576}, {'ion': 1374, 'force': [0.3579751253128052, 1.1010750532150269, -1.420812726020813], 'magnitude': 1.832817792892456, 'distance': 13.458894729614258, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.09492783318420045, 'motion_component': -0.17398542697419472}]}, 6578: {'frame': 6578, 'ionic_force': [11.297083020210266, 8.097006931900978, -3.776877298951149], 'ionic_force_magnitude': 14.403138829856085, 'motion_vector': [-1.2792587280273438, 0.96728515625, 1.4186248779296875], 'cosine_ionic_motion': -0.38838770659146066, 'ionic_motion_component': -5.594002057846219, 'ionic_force_x': 11.297083020210266, 'ionic_force_y': 8.097006931900978, 'ionic_force_z': -3.776877298951149, 'radial_force': 13.899122491034303, 'axial_force': -3.776877298951149, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'contributions': [{'ion': 1327, 'force': [1.3949049711227417, 1.2103792428970337, -0.1234259232878685], 'magnitude': 1.8509489297866821, 'distance': 13.392813682556152, 'before_closest_residue': 1073, 'closest_residue': 1105, 'next_closest_residue': 1073, 'cosine_with_motion': -0.19901989675176637, 'motion_component': -0.36837565457455934}, {'ion': 1330, 'force': [4.5826263427734375, 0.2037651091814041, 0.11392490565776825], 'magnitude': 4.588568687438965, 'distance': 8.506098747253418, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.5601713361052677, 'motion_component': -2.57038469530253}, {'ion': 1341, 'force': [2.695676326751709, 3.7334976196289062, 0.10549106448888779], 'magnitude': 4.606170177459717, 'distance': 8.48983097076416, 'before_closest_residue': 780, 'closest_residue': 'SF', 'next_closest_residue': 780, 'cosine_with_motion': 0.031689497765525536, 'motion_component': 0.1459672195302515}, {'ion': 1359, 'force': [2.0399694442749023, 2.267669677734375, -2.4146974086761475], 'magnitude': 3.8903167247772217, 'distance': 9.237970352172852, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.46119819915256116, 'motion_component': -1.7942070947055129}, {'ion': 1374, 'force': [0.5839059352874756, 0.681695282459259, -1.458169937133789], 'magnitude': 1.7122832536697388, 'distance': 13.924551963806152, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5881046354072257, 'motion_component': -1.0070017571075702}]}, 6579: {'frame': 6579, 'ionic_force': [9.608516097068787, 8.373697221279144, -1.9300379157066345], 'ionic_force_magnitude': 12.89059475343761, 'motion_vector': [2.924358367919922, -6.608238220214844, -2.4186172485351562], 'cosine_ionic_motion': -0.22974953235812362, 'ionic_motion_component': -2.9616081164203725, 'ionic_force_x': 9.608516097068787, 'ionic_force_y': 8.373697221279144, 'ionic_force_z': -1.9300379157066345, 'radial_force': 12.745288805723, 'axial_force': -1.9300379157066345, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 455, 'contributions': [{'ion': 1327, 'force': [1.3253157138824463, 1.562822699546814, 0.09811156988143921], 'magnitude': 2.0514633655548096, 'distance': 12.721465110778809, 'before_closest_residue': 1105, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.4278845029472088, 'motion_component': -0.8777894316682975}, {'ion': 1330, 'force': [5.451991558074951, 0.6885251402854919, 1.5081236362457275], 'magnitude': 5.698483943939209, 'distance': 7.632896900177002, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.17837929729573904, 'motion_component': 1.0164915061803086}, {'ion': 1341, 'force': [0.3505029082298279, 1.43211030960083, 0.5435124635696411], 'magnitude': 1.5713682174682617, 'distance': 14.535503387451172, 'before_closest_residue': 'SF', 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.8145078473890567, 'motion_component': -1.2798917314959368}, {'ion': 1359, 'force': [1.873288631439209, 3.515359878540039, -2.291175127029419], 'magnitude': 4.595263957977295, 'distance': 8.499899864196777, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.3487003992758554, 'motion_component': -1.6023703007219012}, {'ion': 1374, 'force': [0.6074172854423523, 1.1748791933059692, -1.7886104583740234], 'magnitude': 2.2245054244995117, 'distance': 12.216654777526855, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.09802088427497478, 'motion_component': -0.21804798582489582}]}, 6580: {'frame': 6580, 'ionic_force': [9.401102185249329, 2.19012341927737, -3.330233727581799], 'ionic_force_magnitude': 10.211161519116729, 'motion_vector': [0.0558624267578125, 1.9655532836914062, -0.0980682373046875], 'cosine_ionic_motion': 0.2564989404926745, 'ionic_motion_component': 2.6191521108530096, 'ionic_force_x': 9.401102185249329, 'ionic_force_y': 2.19012341927737, 'ionic_force_z': -3.330233727581799, 'radial_force': 9.652842218184595, 'axial_force': -3.330233727581799, 'before_closest_residue': 423, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1327, 'force': [1.994491696357727, 0.5432167649269104, -0.318158358335495], 'magnitude': 2.091484308242798, 'distance': 12.599164009094238, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1105, 'cosine_with_motion': 0.2939362459607358, 'motion_component': 0.6147630256647435}, {'ion': 1330, 'force': [1.841148018836975, -1.1111570596694946, 0.003038342110812664], 'magnitude': 2.1504664421081543, 'distance': 12.425180435180664, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.491633106325562, 'motion_component': -1.0572404228431884}, {'ion': 1341, 'force': [3.1475207805633545, 2.842928171157837, 0.6421310901641846], 'magnitude': 4.289692401885986, 'distance': 8.797432899475098, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.6750076766192781, 'motion_component': 2.89557522958656}, {'ion': 1359, 'force': [1.743165135383606, -0.0841091051697731, -2.3038322925567627], 'magnitude': 2.8902149200439453, 'distance': 10.717759132385254, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.0277650151279751, 'motion_component': 0.08024686087711674}, {'ion': 1374, 'force': [0.674776554107666, -0.0007553519681096077, -1.3534125089645386], 'magnitude': 1.5122994184494019, 'distance': 14.816655158996582, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.05673966670334128, 'motion_component': 0.08580736227417984}]}, 6581: {'frame': 6581, 'ionic_force': [8.237632095813751, 2.8010704964399338, -3.125244453549385], 'ionic_force_magnitude': 9.245092285447901, 'motion_vector': [-1.0904083251953125, 0.6786651611328125, -0.0248260498046875], 'cosine_ionic_motion': -0.5897330513000432, 'ionic_motion_component': -5.45213648304768, 'ionic_force_x': 8.237632095813751, 'ionic_force_y': 2.8010704964399338, 'ionic_force_z': -3.125244453549385, 'radial_force': 8.700837802878933, 'axial_force': -3.125244453549385, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'contributions': [{'ion': 1327, 'force': [1.5015419721603394, 0.9385555386543274, -0.21082422137260437], 'magnitude': 1.7832446098327637, 'distance': 13.644686698913574, 'before_closest_residue': 1073, 'closest_residue': 1105, 'next_closest_residue': 1105, 'cosine_with_motion': -0.434396371589925, 'motion_component': -0.7746350255753975}, {'ion': 1330, 'force': [2.607945680618286, -0.777786374092102, -0.1844618171453476], 'magnitude': 2.7277021408081055, 'distance': 11.032414436340332, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 780, 'cosine_with_motion': -0.9609020723946794, 'motion_component': -2.621054553634242}, {'ion': 1341, 'force': [1.963555932044983, 2.088361978530884, 0.7296456098556519], 'magnitude': 2.9579031467437744, 'distance': 10.594417572021484, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 'SF', 'cosine_with_motion': -0.1952496148674068, 'motion_component': -0.5775294285032408}, {'ion': 1359, 'force': [1.4981328248977661, 0.38405388593673706, -2.148705005645752], 'magnitude': 2.6474199295043945, 'distance': 11.198442459106445, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.38801482743793303, 'motion_component': -1.0272382066311811}, {'ion': 1374, 'force': [0.6664556860923767, 0.16788546741008759, -1.310899019241333], 'magnitude': 1.480136752128601, 'distance': 14.976768493652344, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.3051604131494634, 'motion_component': -0.45167915777951295}]}, 6582: {'frame': 6582, 'ionic_force': [13.439601302146912, 8.873756095767021, -5.538107238709927], 'ionic_force_magnitude': 17.030474514683455, 'motion_vector': [-3.5965843200683594, -4.00225830078125, 1.7977447509765625], 'cosine_ionic_motion': -0.9709190363327294, 'ionic_motion_component': -16.535211904085568, 'ionic_force_x': 13.439601302146912, 'ionic_force_y': 8.873756095767021, 'ionic_force_z': -5.538107238709927, 'radial_force': 16.104857354470152, 'axial_force': -5.538107238709927, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 'SF', 'contributions': [{'ion': 1327, 'force': [1.7381343841552734, 1.2546632289886475, -0.4241744577884674], 'magnitude': 2.1852266788482666, 'distance': 12.32596206665039, 'before_closest_residue': 1105, 'closest_residue': 1105, 'next_closest_residue': 1105, 'cosine_with_motion': -0.9708103909504258, 'motion_component': -2.1214406083064645}, {'ion': 1330, 'force': [7.226673126220703, 3.71441388130188, -0.0353500172495842], 'magnitude': 8.125449180603027, 'distance': 6.392126560211182, 'before_closest_residue': 98, 'closest_residue': 780, 'next_closest_residue': 130, 'cosine_with_motion': -0.8877053495316299, 'motion_component': -7.21300471545702}, {'ion': 1341, 'force': [2.3823862075805664, 2.991396427154541, -1.2005852460861206], 'magnitude': 4.008194446563721, 'distance': 9.101116180419922, 'before_closest_residue': 780, 'closest_residue': 'SF', 'next_closest_residue': 780, 'cosine_with_motion': -0.9982316294542771, 'motion_component': -4.0011063288809225}, {'ion': 1359, 'force': [1.5048085451126099, 0.7228309512138367, -2.4776906967163086], 'magnitude': 2.987621784210205, 'distance': 10.541592597961426, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7527915131617094, 'motion_component': -2.249056399859022}, {'ion': 1374, 'force': [0.5875990390777588, 0.19045160710811615, -1.4003068208694458], 'magnitude': 1.5304913520812988, 'distance': 14.728333473205566, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.621110192406535, 'motion_component': -0.9506037495882076}]}, 6617: {'frame': 6617, 'ionic_force': [25.495893580839038, -9.819616988301277, -19.05839467048645], 'ionic_force_magnitude': 33.31197794635483, 'motion_vector': [-0.17819976806640625, -0.8794822692871094, 1.2368545532226562], 'cosine_ionic_motion': -0.3826768616619429, 'ionic_motion_component': -12.747723176262921, 'ionic_force_x': 25.495893580839038, 'ionic_force_y': -9.819616988301277, 'ionic_force_z': -19.05839467048645, 'radial_force': 27.321520222754888, 'axial_force': -19.05839467048645, 'before_closest_residue': 'SF', 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1327, 'force': [4.0314860343933105, 3.0800936222076416, -2.2007877826690674], 'magnitude': 5.530219078063965, 'distance': 7.748147487640381, 'before_closest_residue': 1073, 'closest_residue': 1073, 'next_closest_residue': 1073, 'cosine_with_motion': -0.7276769114328192, 'motion_component': -4.024212750117133}, {'ion': 1330, 'force': [-0.8541614413261414, -2.234247922897339, -0.8133053779602051], 'magnitude': 2.526444435119629, 'distance': 11.463418960571289, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.2878422361281663, 'motion_component': 0.7272173987333486}, {'ion': 1341, 'force': [22.168386459350586, -9.734976768493652, -8.426047325134277], 'magnitude': 25.636016845703125, 'distance': 3.598684310913086, 'before_closest_residue': 455, 'closest_residue': 130, 'next_closest_residue': 98, 'cosine_with_motion': -0.14832395750175315, 'motion_component': -3.8024356024668147}, {'ion': 1359, 'force': [0.1290685534477234, -0.7988556623458862, -5.832190990447998], 'magnitude': 5.888062477111816, 'distance': 7.509012222290039, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.726202608861233, 'motion_component': -4.2759263983362}, {'ion': 1374, 'force': [0.02111397497355938, -0.13163025677204132, -1.7860631942749023], 'magnitude': 1.7910315990447998, 'distance': 13.61499309539795, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.7662433952410148, 'motion_component': -1.372366105542772}]}, 6618: {'frame': 6618, 'ionic_force': [7.006479242816567, -3.3669902831315994, -11.937614440917969], 'ionic_force_magnitude': 14.245490987913868, 'motion_vector': [0.8625411987304688, 1.1436653137207031, -2.8303680419921875], 'cosine_ionic_motion': 0.7962100082199257, 'ionic_motion_component': 11.342402496583778, 'ionic_force_x': 7.006479242816567, 'ionic_force_y': -3.3669902831315994, 'ionic_force_z': -11.937614440917969, 'radial_force': 7.773504675931058, 'axial_force': -11.937614440917969, 'before_closest_re</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
         <v>6716</v>
       </c>
-      <c r="B5" t="n">
+      <c r="B25" t="n">
         <v>6748</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C25" t="n">
         <v>1374</v>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>{6716: {'frame': 6716, 'ionic_force': [3.5372003372758627, 2.6352185904979706, -13.3009512424469], 'ionic_force_magnitude': 14.013260405761406, 'motion_vector': [2.1366920471191406, 6.534908294677734, 0.9935302734375], 'cosine_ionic_motion': 0.11879090077260183, 'ionic_motion_component': 1.6646478263614333, 'ionic_force_x': 3.5372003372758627, 'ionic_force_y': 2.6352185904979706, 'ionic_force_z': -13.3009512424469, 'radial_force': 4.410914105458254, 'axial_force': -13.3009512424469, 'before_closest_residue': None, 'closest_residue': 780, 'next_closest_residue': 455, 'contributions': [{'ion': 1327, 'force': [1.9013433456420898, -1.8896634578704834, -1.5707390308380127], 'magnitude': 3.106952667236328, 'distance': 10.33717155456543, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.4562221165872038, 'motion_component': np.float64(-1.4174605754747915)}, {'ion': 1330, 'force': [1.3640469312667847, -2.8642194271087646, -0.5391140580177307], 'magnitude': 3.217921733856201, 'distance': 10.157370567321777, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.7308927258320043, 'motion_component': np.float64(-2.3519556602151077)}, {'ion': 1341, 'force': [3.074054718017578, 10.045456886291504, -7.949360370635986], 'magnitude': 13.173964500427246, 'distance': 5.020081996917725, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.702786246731144, 'motion_component': np.float64(9.258481228729863)}, {'ion': 1359, 'force': [-2.778268337249756, -2.3256843090057373, -0.9613978266716003], 'magnitude': 3.748582124710083, 'distance': 9.410994529724121, 'before_closest_residue': 423, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': -0.8482782703144434, 'motion_component': np.float64(-3.179840794185729)}, {'ion': 1400, 'force': [-0.023976320400834084, -0.330671101808548, -2.2803399562835693], 'magnitude': 2.3043150901794434, 'distance': 12.003229141235352, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.2797257697648916, 'motion_component': np.float64(-0.6445763441196359)}]}, 6717: {'frame': 6717, 'ionic_force': [0.5450510084629059, 4.748510509729385, -11.099060416221619], 'ionic_force_magnitude': 12.084476603716624, 'motion_vector': [-2.882415771484375, -8.947956085205078, 1.36480712890625], 'cosine_ionic_motion': -0.5157803651546883, 'ionic_motion_component': -6.232935755368247, 'ionic_force_x': 0.5450510084629059, 'ionic_force_y': 4.748510509729385, 'ionic_force_z': -11.099060416221619, 'radial_force': 4.779689599005029, 'axial_force': -11.099060416221619, 'before_closest_residue': 780, 'closest_residue': 455, 'next_closest_residue': 780, 'contributions': [{'ion': 1327, 'force': [3.7785017490386963, 0.381460577249527, -2.1780126094818115], 'magnitude': 4.377936363220215, 'distance': 8.708318710327148, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.41544024505267596, 'motion_component': np.float64(-1.8187709444652604)}, {'ion': 1330, 'force': [8.046460151672363, -2.481989860534668, -1.290306568145752], 'magnitude': 8.518842697143555, 'distance': 6.242790222167969, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 130, 'cosine_with_motion': -0.03392759388441384, 'motion_component': np.float64(-0.28902384491516386)}, {'ion': 1341, 'force': [0.29557427763938904, 3.0619518756866455, -0.5244418382644653], 'magnitude': 3.1205694675445557, 'distance': 10.314593315124512, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 748, 'cosine_with_motion': -0.9771509240004413, 'motion_component': np.float64(-3.049267163667653)}, {'ion': 1359, 'force': [-12.195097923278809, 2.7431704998016357, -4.48800802230835], 'magnitude': 13.281100273132324, 'distance': 4.99979305267334, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': 0.035512542081213586, 'motion_component': np.float64(0.47164561801915283)}, {'ion': 1400, 'force': [0.6196127533912659, 1.0439174175262451, -2.6182913780212402], 'magnitude': 2.886023759841919, 'distance': 10.72553825378418, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5362116516285387, 'motion_component': np.float64(-1.5475195795965124)}]}, 6718: {'frame': 6718, 'ionic_force': [-15.745279282331467, -6.038105010986328, -8.724656969308853], 'ionic_force_magnitude': 18.98663137669303, 'motion_vector': [-0.8591651916503906, -0.15292739868164062, -0.16278839111328125], 'cosine_ionic_motion': 0.941654600054518, 'ionic_motion_component': 17.878848775402435, 'ionic_force_x': -15.745279282331467, 'ionic_force_y': -6.038105010986328, 'ionic_force_z': -8.724656969308853, 'radial_force': 16.863348771887352, 'axial_force': -8.724656969308853, 'before_closest_residue': 455, 'closest_residue': 780, 'next_closest_residue': 1105, 'contributions': [{'ion': 1327, 'force': [1.6139215230941772, -3.2655606269836426, -0.8199718594551086], 'magnitude': 3.733762502670288, 'distance': 9.429652214050293, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.22740658575106223, 'motion_component': np.float64(-0.8490821923351985)}, {'ion': 1330, 'force': [0.4008204936981201, -2.449448347091675, 0.07108324766159058], 'magnitude': 2.483043909072876, 'distance': 11.5631685256958, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 98, 'cosine_with_motion': 0.008458746980975155, 'motion_component': np.float64(0.021003440249473652)}, {'ion': 1340, 'force': [-0.1447393000125885, -0.5571725368499756, -1.7205244302749634], 'magnitude': 1.8142753839492798, 'distance': 13.527496337890625, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.3040179972274526, 'motion_component': np.float64(0.551572355841353)}, {'ion': 1341, 'force': [-15.274748802185059, 4.401199817657471, -2.545541286468506], 'magnitude': 16.098703384399414, 'distance': 4.54123067855835, 'before_closest_residue': 780, 'closest_residue': 748, 'next_closest_residue': 780, 'cosine_with_motion': 0.900194890649546, 'motion_component': np.float64(14.491971667476406)}, {'ion': 1359, 'force': [-1.6921180486679077, -1.7458655834197998, -0.0793391764163971], 'magnitude': 2.432612895965576, 'distance': 11.682413101196289, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 423, 'cosine_with_motion': 0.8028370445889909, 'motion_component': np.float64(1.9529916373492413)}, {'ion': 1400, 'force': [-0.6484151482582092, -2.421257734298706, -3.6303634643554688], 'magnitude': 4.4116291999816895, 'distance': 8.67500114440918, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.3877006632017084, 'motion_component': np.float64(1.7103914746028686)}]}, 6719: {'frame': 6719, 'ionic_force': [-13.247648186981678, -7.324256241321564, -7.235395602881908], 'ionic_force_magnitude': 16.777838403822457, 'motion_vector': [3.021942138671875, 1.1164970397949219, -1.1178054809570312], 'cosine_ionic_motion': -0.7013024980662967, 'ionic_motion_component': -11.766339984753339, 'ionic_force_x': -13.247648186981678, 'ionic_force_y': -7.324256241321564, 'ionic_force_z': -7.235395602881908, 'radial_force': 15.13753321960275, 'axial_force': -7.235395602881908, 'before_closest_residue': 780, 'closest_residue': 1105, 'next_closest_residue': 780, 'contributions': [{'ion': 1327, 'force': [1.420046091079712, -3.122454881668091, -0.8165378570556641], 'magnitude': 3.5260443687438965, 'distance': 9.7034273147583, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.14286728851306163, 'motion_component': np.float64(0.5037564096968339)}, {'ion': 1330, 'force': [0.10633199661970139, -2.712059497833252, -0.04335900396108627], 'magnitude': 2.714489459991455, 'distance': 11.059231758117676, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.28717403087952637, 'motion_component': np.float64(-0.7795308899562283)}, {'ion': 1340, 'force': [-0.22071534395217896, -0.5099888443946838, -1.6464329957962036], 'magnitude': 1.737683892250061, 'distance': 13.822405815124512, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.10193220999201093, 'motion_component': np.float64(0.1771259648225083)}, {'ion': 1341, 'force': [-12.584758758544922, 2.7286531925201416, -1.619233250617981], 'magnitude': 12.978583335876465, 'distance': 5.057727336883545, 'before_closest_residue': 748, 'closest_residue': 780, 'next_closest_residue': 748, 'cosine_with_motion': -0.7495715800440138, 'motion_component': np.float64(-9.728376991680793)}, {'ion': 1359, 'force': [-1.4268096685409546, -1.9060715436935425, -0.11701104044914246], 'magnitude': 2.383817672729492, 'distance': 11.801372528076172, 'before_closest_residue': 455, 'closest_residue': 423, 'next_closest_residue': 455, 'cosine_with_motion': -0.776132534249492, 'motion_component': np.float64(-1.8501583614498278)}, {'ion': 1400, 'force': [-0.5417425036430359, -1.8023346662521362, -2.992821455001831], 'magnitude': 3.535374879837036, 'distance': 9.690614700317383, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.025218295532721334, 'motion_component': np.float64(-0.0891561282175708)}]}, 6720: {'frame': 6720, 'ionic_force': [-13.87582477927208, -1.1168306767940521, -19.71669414639473], 'ionic_force_magnitude': 24.135738068850632, 'motion_vector': [-2.0362319946289062, -3.377918243408203, 1.4120712280273438], 'cosine_ionic_motion': 0.041395254739074926, 'ionic_motion_component': 0.9991050256756602, 'ionic_force_x': -13.87582477927208, 'ionic_force_y': -1.1168306767940521, 'ionic_force_z': -19.71669414639473, 'radial_force': 13.920697686024551, 'axial_force': -19.71669414639473, 'before_closest_residue': 1105, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1327, 'force': [1.9507142305374146, -2.5765552520751953, -0.8716263175010681], 'magnitude': 3.3471860885620117, 'distance': 9.959306716918945, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.24963399482009194, 'motion_component': np.float64(0.8355714608759257)}, {'ion': 1330, 'force': [0.7414261698722839, -2.502897262573242, -0.2262757122516632], 'magnitude': 2.620192527770996, 'distance': 11.256476402282715, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 130, 'cosine_with_motion': 0.6035741375210052, 'motion_component': np.float64(1.581480363051632)}, {'ion': 1340, 'force': [0.15693143010139465, -0.3897511661052704, -1.5432026386260986], 'magnitude': 1.5993773937225342, 'distance': 14.40766429901123, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.17642624695933348, 'motion_component': np.float64(-0.2821721389973071)}, {'ion': 1341, 'force': [-16.80057144165039, 8.428204536437988, -13.408795356750488], 'magnitude': 23.088733673095703, 'distance': 3.792005777359009, 'before_closest_residue': 780, 'closest_residue': 748, 'next_closest_residue': 780, 'cosine_with_motion': -0.13640637058778973, 'motion_component': np.float64(-3.1494503699860275)}, {'ion': 1359, 'force': [-0.39115285873413086, -2.5806212425231934, -0.5263550877571106], 'magnitude': 2.6626408100128174, 'distance': 11.166389465332031, 'before_closest_residue': 423, 'closest_residue': 455, 'next_closest_residue': 423, 'cosine_with_motion': 0.7862480782728855, 'motion_component': np.float64(2.0934962423746057)}, {'ion': 1400, 'force': [0.4668276906013489, -1.4952102899551392, -3.140439033508301], 'magnitude': 3.5094072818756104, 'distance': 9.726400375366211, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.02274474388170812, 'motion_component': np.float64(-0.07982056901541412)}]}, 6721: {'frame': 6721, 'ionic_force': [-14.872821755707264, -15.005798995494843, -8.689001321792603], 'ionic_force_magnitude': 22.844552401838538, 'motion_vector': [-1.2706642150878906, 0.12684249877929688, -0.00298309326171875], 'cosine_ionic_motion': 0.5834652896842984, 'ionic_motion_component': 13.329003384846859, 'ionic_force_x': -14.872821755707264, 'ionic_force_y': -15.005798995494843, 'ionic_force_z': -8.689001321792603, 'radial_force': 21.127584586748984, 'axial_force': -8.689001321792603, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 1105, 'contributions': [{'ion': 1327, 'force': [0.9067454934120178, -1.875288724899292, -0.39515984058380127], 'magnitude': 2.120152473449707, 'distance': 12.513692855834961, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.5129856540705134, 'motion_component': np.float64(-1.0876078009618537)}, {'ion': 1340, 'force': [-0.07977346330881119, -0.7151584029197693, -1.4344522953033447], 'magnitude': 1.6048266887664795, 'distance': 14.38318157196045, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.00728621658859265, 'motion_component': np.float64(0.011693114916961955)}, {'ion': 1341, 'force': [-14.652534484863281, -8.45791244506836, -4.700499057769775], 'magnitude': 17.559263229370117, 'distance': 4.348263740539551, 'before_closest_residue': 748, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.7831130895059822, 'motion_component': np.float64(13.750889233616203)}, {'ion': 1359, 'force': [-0.839736819267273, -1.8682215213775635, -0.06597363948822021], 'magnitude': 2.0493321418762207, 'distance': 12.728078842163086, 'before_closest_residue': 455, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.3172573445902172, 'motion_component': np.float64(0.6501656636034504)}, {'ion': 1400, 'force': [-0.20752248167991638, -2.0892179012298584, -2.092916488647461], 'magnitude': 2.964489221572876, 'distance': 10.5826416015625, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.0013031289237940694, 'motion_component': np.float64(0.0038631116715133196)}]}, 6722: {'frame': 6722, 'ionic_force': [-6.684693954885006, -13.338739812374115, -3.4362437799572945], 'ionic_force_magnitude': 15.310613454985583, 'motion_vector': [1.3387413024902344, 0.14303207397460938, 0.6805572509765625], 'cosine_ionic_motion': -0.5712972146225438, 'ionic_motion_component': -8.746910820995705, 'ionic_force_x': -6.684693954885006, 'ionic_force_y': -13.338739812374115, 'ionic_force_z': -3.4362437799572945, 'radial_force': 14.920023895848505, 'axial_force': -3.4362437799572945, 'before_closest_residue': 780, 'closest_residue': 1105, 'next_closest_residue': 780, 'contributions': [{'ion': 1327, 'force': [0.8192603588104248, -2.1865477561950684, -0.48868289589881897], 'magnitude': 2.3855795860290527, 'distance': 11.797014236450195, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.12544368299866207, 'motion_component': np.float64(0.2992558798166547)}, {'ion': 1330, 'force': [0.035064585506916046, -1.5158445835113525, 0.15978534519672394], 'magnitude': 1.5246460437774658, 'distance': 14.756539344787598, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 98, 'cosine_with_motion': -0.026577019886595728, 'motion_component': np.float64(-0.040520549308438625)}, {'ion': 1340, 'force': [-0.26287201046943665, -0.7818873524665833, -1.5102778673171997], 'magnitude': 1.7208685874938965, 'distance': 13.889774322509766, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5745508499662869, 'motion_component': np.float64(-0.9887265207963449)}, {'ion': 1341, 'force': [-5.845896244049072, -5.083929061889648, 0.5223320722579956], 'magnitude': 7.764899730682373, 'distance': 6.538846492767334, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.6998287725945069, 'motion_component': np.float64(-5.4341002734692445)}, {'ion': 1359, 'force': [-0.7654677033424377, -1.5446780920028687, -0.07922738045454025], 'magnitude': 1.7257601022720337, 'distance': 13.870075225830078, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.49918877829101976, 'motion_component': np.float64(-0.8614801146791009)}, {'ion': 1400, 'force': [-0.6647829413414001, -2.2258529663085938, -2.040173053741455], 'magnitude': 3.0917088985443115, 'distance': 10.362624168395996, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5567597574552943, 'motion_component': np.float64(-1.7213390931081953)}]}, 6723: {'frame': 6723, 'ionic_force': [-0.576256413012743, -13.915500223636627, 1.1806349493563175], 'ionic_force_magnitude': 13.977378753228765, 'motion_vector': [-0.162322998046875, 2.1346893310546875, 1.369384765625], 'cosine_ionic_motion': -0.7881157163108534, 'ionic_motion_component': -11.015791868248991, 'ionic_force_x': -0.576256413012743, 'ionic_force_y': -13.915500223636627, 'ionic_force_z': 1.1806349493563175, 'radial_force': 13.927426823630032, 'axial_force': 1.1806349493563175, 'before_closest_residue': 1105, 'closest_residue': 780, 'next_closest_residue': 748, 'contributions': [{'ion': 1327, 'force': [0.9342626333236694, -2.013418436050415, -0.30056488513946533], 'magnitude': 2.239874839782715, 'distance': 12.17466926574707, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.8540059906302656, 'motion_component': np.float64(-1.9128666113018717)}, {'ion': 1340, 'force': [-0.046403419226408005, -0.8943821787834167, -1.6315449476242065], 'magnitude': 1.8611855506896973, 'distance': 13.355932235717773, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8744132028960275, 'motion_component': np.float64(-1.627445223510299)}, {'ion': 1341, 'force': [-0.5979642868041992, -6.457273483276367, 5.619952201843262], 'magnitude': 8.581247329711914, 'distance': 6.2200493812561035, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.27473154144593465, 'motion_component': np.float64(-2.357539292708914)}, {'ion': 1359, 'force': [-0.7437008619308472, -1.861376404762268, 0.03603336587548256], 'magnitude': 2.004772186279297, 'distance': 12.868754386901855, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.746521141604162, 'motion_component': np.float64(-1.4966048168416326)}, {'ion': 1400, 'force': [-0.12245047837495804, -2.68904972076416, -2.543240785598755], 'magnitude': 3.703249454498291, 'distance': 9.46842098236084, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.9778807589389066, 'motion_component': np.float64(-3.6213363463983046)}]}, 6724: {'frame': 6724, 'ionic_force': [-4.113540604710579, -15.694007158279419, 7.197184890508652], 'ionic_force_magnitude': 17.748874537245857, 'motion_vector': [-0.3926811218261719, -2.1882896423339844, -1.7566070556640625], 'cosine_ionic_motion': 0.46361911761555036, 'ionic_motion_component': 8.228717551627033, 'ionic_force_x': -4.113540604710579, 'ionic_force_y': -15.694007158279419, 'ionic_force_z': 7.197184890508652, 'radial_force': 16.224151040677853, 'axial_force': 7.197184890508652, 'before_closest_residue': 780, 'closest_residue': 748, 'next_closest_residue': 780, 'contributions': [{'ion': 1327, 'force': [1.648600697517395, -2.8385839462280273, -0.17031431198120117], 'magnitude': 3.2870123386383057, 'distance': 10.050053596496582, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.6295567558755207, 'motion_component': np.float64(2.0693608177461815)}, {'ion': 1330, 'force': [0.29793599247932434, -1.9125957489013672, 0.4574536979198456], 'magnitude': 1.9889826774597168, 'distance': 12.919733047485352, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.5792989369094492, 'motion_component': np.float64(1.1522155722582466)}, {'ion': 1340, 'force': [-0.16771666705608368, -1.0057437419891357, -2.1990678310394287], 'magnitude': 2.423953056335449, 'distance': 11.703262329101562, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.892467519191024, 'motion_component': np.float64(2.163299418899779)}, {'ion': 1341, 'force': [-4.0101213455200195, -2.7143781185150146, 13.681194305419922], 'magnitude': 14.512890815734863, 'distance': 4.7829084396362305, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.40168469073769564, 'motion_component': np.float64(-5.829606053067735)}, {'ion': 1359, 'force': [-1.2397170066833496, -2.3678457736968994, 0.34243643283843994], 'magnitude': 2.6945972442626953, 'distance': 11.099977493286133, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 455, 'cosine_with_motion': 0.6636283760801129, 'motion_component': np.float64(1.7882112262072525)}, {'ion': 1400, 'force': [-0.6425222754478455, -4.854859828948975, -4.914517402648926], 'magnitude': 6.9379377365112305, 'distance': 6.917574405670166, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.9924039216805082, 'motion_component': np.float64(6.885236625128063)}]}, 6725: {'frame': 6725, 'ionic_force': [-2.6017091125249863, -10.550699651241302, -2.3864914998412132], 'ionic_force_magnitude': 11.125713240764084, 'motion_vector': [-0.458587646484375, 0.23482513427734375, -0.8922119140625], 'cosine_ionic_motion': 0.07370003850582965, 'ionic_motion_component': 0.8199654942491318, 'ionic_force_x': -2.6017091125249863, 'ionic_force_y': -10.550699651241302, 'ionic_force_z': -2.3864914998412132, 'radial_force': 10.866745301004293, 'axial_force': -2.3864914998412132, 'before_closest_residue': 748, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1327, 'force': [1.0887424945831299, -2.387108087539673, -0.3622821271419525], 'magnitude': 2.648564338684082, 'distance': 11.196022987365723, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.2699394138825094, 'motion_component': np.float64(-0.7149519319481872)}, {'ion': 1340, 'force': [-0.15459378063678741, -0.8115611672401428, -1.453180193901062], 'magnitude': 1.6716049909591675, 'distance': 14.0929594039917, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.6833375908502632, 'motion_component': np.float64(1.1422705673000157)}, {'ion': 1341, 'force': [-2.5049638748168945, -3.5627336502075195, 1.4722782373428345], 'magnitude': 4.5973381996154785, 'distance': 8.497982025146484, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.21143109657537829, 'motion_component': np.float64(-0.9720202514220446)}, {'ion': 1359, 'force': [-0.7145503759384155, -1.7946149110794067, 0.0394371822476387], 'magnitude': 1.9320404529571533, 'distance': 13.108739852905273, 'before_closest_residue': 423, 'closest_residue': 455, 'next_closest_residue': 423, 'cosine_with_motion': -0.06476746148457564, 'motion_component': np.float64(-0.1251333539189594)}, {'ion': 1400, 'force': [-0.3163435757160187, -1.9946818351745605, -2.082744598388672], 'magnitude': 2.9011471271514893, 'distance': 10.697546005249023, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5135211624013504, 'motion_component': np.float64(1.489800382213538)}]}, 6726: {'frame': 6726, 'ionic_force': [-10.677393078804016, -23.184772431850433, 0.8381237275898457], 'ionic_force_magnitude': 25.53904553930575, 'motion_vector': [1.3153266906738281, 2.5401535034179688, 0.22161865234375], 'cosine_ionic_motion': -0.992876176707314, 'ionic_motion_component': -25.357109891819874, 'ionic_force_x': -10.677393078804016, 'ionic_force_y': -23.184772431850433, 'ionic_force_z': 0.8381237275898457, 'radial_force': 25.525289335793705, 'axial_force': 0.8381237275898457, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1327, 'force': [0.9742769598960876, -2.260103225708008, -0.6310176849365234], 'magnitude': 2.5407607555389404, 'distance': 11.431077003479004, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.6309460379872143, 'motion_component': np.float64(-1.6030829678477687)}, {'ion': 1330, 'force': [0.2411656230688095, -1.9719338417053223, -0.08398731797933578], 'magnitude': 1.9884008169174194, 'distance': 12.921623229980469, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 98, 'cosine_with_motion': -0.8256838073146171, 'motion_component': np.float64(-1.6417903558745526)}, {'ion': 1340, 'force': [-0.16953469812870026, -0.6895309090614319, -1.4364378452301025], 'magnitude': 1.602357268333435, 'distance': 14.394261360168457, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.49874044444684573, 'motion_component': np.float64(-0.7991603382369856)}, {'ion': 1341, 'force': [-10.608416557312012, -15.084050178527832, 5.144473552703857], 'magnitude': 19.145042419433594, 'distance': 4.1642889976501465, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 130, 'cosine_with_motion': -0.9308319385126406, 'motion_component': np.float64(-17.82081769047824)}, {'ion': 1359, 'force': [-0.7096368670463562, -1.4897035360336304, -0.05674480274319649], 'magnitude': 1.6510666608810425, 'distance': 14.180342674255371, 'before_closest_residue': 455, 'closest_residue': 423, 'next_closest_residue': 455, 'cosine_with_motion': -0.9985275775958757, 'motion_component': np.float64(-1.6486355819412137)}, {'ion': 1400, 'force': [-0.4052475392818451, -1.689450740814209, -2.0981621742248535], 'magnitude': 2.7241060733795166, 'distance': 11.039693832397461, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6767809384082066, 'motion_component': np.float64(-1.8436230626847667)}]}, 6727: {'frame': 6727, 'ionic_force': [0.19401564449071884, -14.893806159496307, -1.191986322402954], 'ionic_force_magnitude': 14.942688358516785, 'motion_vector': [1.3554725646972656, -0.12535858154296875, 0.22263336181640625], 'cosine_ionic_motion': 0.09046943077024892, 'ionic_motion_component': 1.3518565099722388, 'ionic_force_x': 0.19401564449071884, 'ionic_force_y': -14.893806159496307, 'ionic_force_z': -1.191986322402954, 'radial_force': 14.895069787918326, 'axial_force': -1.191986322402954, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1327, 'force': [1.8957452774047852, -2.660691261291504, -0.9064188599586487], 'magnitude': 3.3903868198394775, 'distance': 9.895651817321777, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.5776476013357499, 'motion_component': np.float64(1.9584488572086751)}, {'ion': 1330, 'force': [0.34051114320755005, -2.0693624019622803, 0.12192656844854355], 'magnitude': 2.1007320880889893, 'distance': 12.571402549743652, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 130, 'cosine_with_motion': 0.25818029144636306, 'motion_component': np.float64(0.5423675841303569)}, {'ion': 1340, 'force': [-0.05866319686174393, -0.5451573729515076, -1.6288466453552246], 'magnitude': 1.718656301498413, 'distance': 13.898711204528809, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.15768551634272415, 'motion_component': np.float64(-0.27100719913138205)}, {'ion': 1341, 'force': [0.5644397735595703, -4.90380334854126, 4.14929723739624], 'magnitude': 6.448452949523926, 'distance': 7.175320148468018, 'before_closest_residue': 780, 'closest_residue': 130, 'next_closest_residue': None, 'cosine_with_motion': 0.25898652287047647, 'motion_component': np.float64(1.6700624406497229)}, {'ion': 1359, 'force': [-2.4074676036834717, -2.86397123336792, 0.0936751738190651], 'magnitude': 3.74259352684021, 'distance': 9.4185209274292, 'before_closest_residue': 423, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': -0.5585431036967348, 'motion_component': np.float64(-2.090399820727341)}, {'ion': 1400, 'force': [-0.14054974913597107, -1.850820541381836, -3.0216197967529297], 'magnitude': 3.546191930770874, 'distance': 9.675823211669922, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.12904417269620683, 'motion_component': np.float64(-0.4576154020114362)}]}, 6728: {'frame': 6728, 'ionic_force': [2.4772854894399643, -9.180881977081299, -5.546252265572548], 'ionic_force_magnitude': 11.008471804326641, 'motion_vector': [-2.3235855102539062, 0.4115257263183594, -0.305999755859375], 'cosine_ionic_motion': -0.2991903423675208, 'ionic_motion_component': -3.293628448079687, 'ionic_force_x': 2.4772854894399643, 'ionic_force_y': -9.180881977081299, 'ionic_force_z': -5.546252265572548, 'radial_force': 9.509234315826172, 'axial_force': -5.546252265572548, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1327, 'force': [1.678908109664917, -2.0583689212799072, -0.4516320526599884], 'magnitude': 2.694361925125122, 'distance': 11.100461959838867, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.7190427304193472, 'motion_component': np.float64(-1.9373614066475815)}, {'ion': 1330, 'force': [0.7343487739562988, -2.256716012954712, 0.1098492294549942], 'magnitude': 2.375731945037842, 'distance': 11.82143783569336, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 98, 'cosine_with_motion': -0.4720684228718054, 'motion_component': np.float64(-1.1215080188962099)}, {'ion': 1340, 'force': [0.15440182387828827, -0.5537362098693848, -1.7548797130584717], 'magnitude': 1.8466365337371826, 'distance': 13.408442497253418, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.011299252569514797, 'motion_component': np.float64(-0.020865612699471292)}, {'ion': 1359, 'force': [-0.4944912791252136, -2.2753615379333496, -0.14022064208984375], 'magnitude': 2.3326923847198486, 'distance': 11.929996490478516, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 423, 'cosine_with_motion': 0.046036121737723396, 'motion_component': np.float64(0.10738810882518735)}, {'ion': 1400, 'force': [0.40411806106567383, -2.0366992950439453, -3.3093690872192383], 'magnitude': 3.9068374633789062, 'distance': 9.218417167663574, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.08223573685554021, 'motion_component': np.float64(-0.3212816598479833)}]}, 6729: {'frame': 6729, 'ionic_force': [-0.138140469789505, -10.870651006698608, -5.780998468399048], 'ionic_force_magnitude': 12.313004482678599, 'motion_vector': [6.845603942871094, -0.24485015869140625, 2.0646591186523438], 'cosine_ionic_motion': -0.1160126310210488, 'ionic_motion_component': -1.4284640458095121, 'ionic_force_x': -0.138140469789505, 'ionic_force_y': -10.870651006698608, 'ionic_force_z': -5.780998468399048, 'radial_force': 10.871528691901206, 'axial_force': -5.780998468399048, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 748, 'contributions': [{'ion': 1327, 'force': [1.820922613143921, -3.5445034503936768, -0.7323452830314636], 'magnitude': 4.051616191864014, 'distance': 9.052215576171875, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.40781161798980436, 'motion_component': np.float64(1.652296140602055)}, {'ion': 1330, 'force': [0.3618646264076233, -3.04648756980896, -0.05099794268608093], 'magnitude': 3.0683274269104004, 'dista</t>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>{6716: {'frame': 6716, 'ionic_force': [3.5372003354132175, 2.635218560695648, -13.300951480865479], 'ionic_force_magnitude': 14.013260625986366, 'motion_vector': [2.1366920471191406, 6.534908294677734, 0.9935302734375], 'cosine_ionic_motion': 0.1187908944309096, 'ionic_motion_component': 1.6646477636543684, 'ionic_force_x': 3.5372003354132175, 'ionic_force_y': 2.635218560695648, 'ionic_force_z': -13.300951480865479, 'radial_force': 4.4109140861597185, 'axial_force': -13.300951480865479, 'before_closest_residue': None, 'closest_residue': 780, 'next_closest_residue': 455, 'contributions': [{'ion': 1327, 'force': [1.9013433456420898, -1.8896634578704834, -1.5707390308380127], 'magnitude': 3.106952667236328, 'distance': 10.33717155456543, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.4562221165872038, 'motion_component': -1.4174605754747915}, {'ion': 1330, 'force': [1.3640469312667847, -2.8642194271087646, -0.5391140580177307], 'magnitude': 3.217921733856201, 'distance': 10.157370567321777, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.7308927258320043, 'motion_component': -2.3519556602151077}, {'ion': 1341, 'force': [3.074054718017578, 10.045456886291504, -7.949360370635986], 'magnitude': 13.173964500427246, 'distance': 5.020081996917725, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.702786246731144, 'motion_component': 9.258481228729863}, {'ion': 1359, 'force': [-2.778268337249756, -2.3256843090057373, -0.9613978266716003], 'magnitude': 3.748582124710083, 'distance': 9.410994529724121, 'before_closest_residue': 423, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': -0.8482782703144434, 'motion_component': -3.179840794185729}, {'ion': 1400, 'force': [-0.023976322263479233, -0.33067113161087036, -2.2803401947021484], 'magnitude': 2.3043153285980225, 'distance': 12.003229141235352, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.2797257678152574, 'motion_component': -0.6445764068267018}]}, 6717: {'frame': 6717, 'ionic_force': [0.5450510084629059, 4.748510509729385, -11.099060416221619], 'ionic_force_magnitude': 12.084476603716624, 'motion_vector': [-2.882415771484375, -8.947956085205078, 1.36480712890625], 'cosine_ionic_motion': -0.5157803651546883, 'ionic_motion_component': -6.232935755368247, 'ionic_force_x': 0.5450510084629059, 'ionic_force_y': 4.748510509729385, 'ionic_force_z': -11.099060416221619, 'radial_force': 4.779689599005029, 'axial_force': -11.099060416221619, 'before_closest_residue': 780, 'closest_residue': 455, 'next_closest_residue': 780, 'contributions': [{'ion': 1327, 'force': [3.7785017490386963, 0.381460577249527, -2.1780126094818115], 'magnitude': 4.377936363220215, 'distance': 8.708318710327148, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.41544024505267596, 'motion_component': -1.8187709444652604}, {'ion': 1330, 'force': [8.046460151672363, -2.481989860534668, -1.290306568145752], 'magnitude': 8.518842697143555, 'distance': 6.242790222167969, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 130, 'cosine_with_motion': -0.03392759388441384, 'motion_component': -0.28902384491516386}, {'ion': 1341, 'force': [0.29557427763938904, 3.0619518756866455, -0.5244418382644653], 'magnitude': 3.1205694675445557, 'distance': 10.314593315124512, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 748, 'cosine_with_motion': -0.9771509240004413, 'motion_component': -3.049267163667653}, {'ion': 1359, 'force': [-12.195097923278809, 2.7431704998016357, -4.48800802230835], 'magnitude': 13.281100273132324, 'distance': 4.99979305267334, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': 0.035512542081213586, 'motion_component': 0.47164561801915283}, {'ion': 1400, 'force': [0.6196127533912659, 1.0439174175262451, -2.6182913780212402], 'magnitude': 2.886023759841919, 'distance': 10.72553825378418, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5362116516285387, 'motion_component': -1.5475195795965124}]}, 6718: {'frame': 6718, 'ionic_force': [-15.74527932703495, -6.038105010986328, -8.724657155573368], 'ionic_force_magnitude': 18.986631499356328, 'motion_vector': [-0.8591651916503906, -0.15292739868164062, -0.16278839111328125], 'cosine_ionic_motion': 0.9416545980486678, 'ionic_motion_component': 17.878848852824557, 'ionic_force_x': -15.74527932703495, 'ionic_force_y': -6.038105010986328, 'ionic_force_z': -8.724657155573368, 'radial_force': 16.863348813626917, 'axial_force': -8.724657155573368, 'before_closest_residue': 455, 'closest_residue': 780, 'next_closest_residue': 1105, 'contributions': [{'ion': 1327, 'force': [1.6139215230941772, -3.2655608654022217, -0.8199719190597534], 'magnitude': 3.733762741088867, 'distance': 9.429652214050293, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.22740655832611156, 'motion_component': -0.8490821403328379}, {'ion': 1330, 'force': [0.40082046389579773, -2.4494481086730957, 0.07108324021100998], 'magnitude': 2.483043670654297, 'distance': 11.5631685256958, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 98, 'cosine_with_motion': 0.008458743424691165, 'motion_component': 0.021003429387131622}, {'ion': 1340, 'force': [-0.1447393149137497, -0.5571725368499756, -1.720524549484253], 'magnitude': 1.8142755031585693, 'distance': 13.527496337890625, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.3040179980827136, 'motion_component': 0.5515723921234557}, {'ion': 1341, 'force': [-15.274748802185059, 4.401199817657471, -2.545541286468506], 'magnitude': 16.098703384399414, 'distance': 4.54123067855835, 'before_closest_residue': 780, 'closest_residue': 748, 'next_closest_residue': 780, 'cosine_with_motion': 0.900194890649546, 'motion_component': 14.491971667476406}, {'ion': 1359, 'force': [-1.6921180486679077, -1.7458655834197998, -0.0793391764163971], 'magnitude': 2.432612895965576, 'distance': 11.682413101196289, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 423, 'cosine_with_motion': 0.8028370445889909, 'motion_component': 1.9529916373492413}, {'ion': 1400, 'force': [-0.6484151482582092, -2.421257734298706, -3.6303634643554688], 'magnitude': 4.4116291999816895, 'distance': 8.67500114440918, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.3877006632017084, 'motion_component': 1.7103914746028686}]}, 6719: {'frame': 6719, 'ionic_force': [-13.247648186981678, -7.324256241321564, -7.235395602881908], 'ionic_force_magnitude': 16.777838403822457, 'motion_vector': [3.021942138671875, 1.1164970397949219, -1.1178054809570312], 'cosine_ionic_motion': -0.7013024980662967, 'ionic_motion_component': -11.766339984753339, 'ionic_force_x': -13.247648186981678, 'ionic_force_y': -7.324256241321564, 'ionic_force_z': -7.235395602881908, 'radial_force': 15.13753321960275, 'axial_force': -7.235395602881908, 'before_closest_residue': 780, 'closest_residue': 1105, 'next_closest_residue': 780, 'contributions': [{'ion': 1327, 'force': [1.420046091079712, -3.122454881668091, -0.8165378570556641], 'magnitude': 3.5260443687438965, 'distance': 9.7034273147583, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.14286728851306163, 'motion_component': 0.5037564096968339}, {'ion': 1330, 'force': [0.10633199661970139, -2.712059497833252, -0.04335900396108627], 'magnitude': 2.714489459991455, 'distance': 11.059231758117676, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.28717403087952637, 'motion_component': -0.7795308899562283}, {'ion': 1340, 'force': [-0.22071534395217896, -0.5099888443946838, -1.6464329957962036], 'magnitude': 1.737683892250061, 'distance': 13.822405815124512, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.10193220999201093, 'motion_component': 0.1771259648225083}, {'ion': 1341, 'force': [-12.584758758544922, 2.7286531925201416, -1.619233250617981], 'magnitude': 12.978583335876465, 'distance': 5.057727336883545, 'before_closest_residue': 748, 'closest_residue': 780, 'next_closest_residue': 748, 'cosine_with_motion': -0.7495715800440138, 'motion_component': -9.728376991680793}, {'ion': 1359, 'force': [-1.4268096685409546, -1.9060715436935425, -0.11701104044914246], 'magnitude': 2.383817672729492, 'distance': 11.801372528076172, 'before_closest_residue': 455, 'closest_residue': 423, 'next_closest_residue': 455, 'cosine_with_motion': -0.776132534249492, 'motion_component': -1.8501583614498278}, {'ion': 1400, 'force': [-0.5417425036430359, -1.8023346662521362, -2.992821455001831], 'magnitude': 3.535374879837036, 'distance': 9.690614700317383, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.025218295532721334, 'motion_component': -0.0891561282175708}]}, 6720: {'frame': 6720, 'ionic_force': [-13.875824749469757, -1.1168307960033417, -19.71669438481331], 'ionic_force_magnitude': 24.135738251999413, 'motion_vector': [-2.0362319946289062, -3.377918243408203, 1.4120712280273438], 'cosine_ionic_motion': 0.04139525447767722, 'ionic_motion_component': 0.999105026948124, 'ionic_force_x': -13.875824749469757, 'ionic_force_y': -1.1168307960033417, 'ionic_force_z': -19.71669438481331, 'radial_force': 13.920697665882228, 'axial_force': -19.71669438481331, 'before_closest_residue': 1105, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1327, 'force': [1.9507142305374146, -2.5765552520751953, -0.8716263175010681], 'magnitude': 3.3471860885620117, 'distance': 9.959306716918945, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.24963399482009194, 'motion_component': 0.8355714608759257}, {'ion': 1330, 'force': [0.7414261698722839, -2.502897262573242, -0.2262757122516632], 'magnitude': 2.620192527770996, 'distance': 11.256476402282715, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 130, 'cosine_with_motion': 0.6035741375210052, 'motion_component': 1.581480363051632}, {'ion': 1340, 'force': [0.15693143010139465, -0.3897511661052704, -1.5432026386260986], 'magnitude': 1.5993773937225342, 'distance': 14.40766429901123, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.17642624695933348, 'motion_component': -0.2821721389973071}, {'ion': 1341, 'force': [-16.80057144165039, 8.428204536437988, -13.408795356750488], 'magnitude': 23.088733673095703, 'distance': 3.792005777359009, 'before_closest_residue': 780, 'closest_residue': 748, 'next_closest_residue': 780, 'cosine_with_motion': -0.13640637058778973, 'motion_component': -3.1494503699860275}, {'ion': 1359, 'force': [-0.39115285873413086, -2.5806212425231934, -0.5263550877571106], 'magnitude': 2.6626408100128174, 'distance': 11.166389465332031, 'before_closest_residue': 423, 'closest_residue': 455, 'next_closest_residue': 423, 'cosine_with_motion': 0.7862480782728855, 'motion_component': 2.0934962423746057}, {'ion': 1400, 'force': [0.46682772040367126, -1.4952104091644287, -3.14043927192688], 'magnitude': 3.5094075202941895, 'distance': 9.726400375366211, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.022744741781503392, 'motion_component': -0.0798205677429511}]}, 6721: {'frame': 6721, 'ionic_force': [-14.872823670506477, -15.005800008773804, -8.68900191783905], 'ionic_force_magnitude': 22.84455454075444, 'motion_vector': [-1.2706642150878906, 0.12684249877929688, -0.00298309326171875], 'cosine_ionic_motion': 0.5834653141139671, 'ionic_motion_component': 13.329005190914943, 'ionic_force_x': -14.872823670506477, 'ionic_force_y': -15.005800008773804, 'ionic_force_z': -8.68900191783905, 'radial_force': 21.127586654355333, 'axial_force': -8.68900191783905, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 1105, 'contributions': [{'ion': 1327, 'force': [0.9067454934120178, -1.875288724899292, -0.39515984058380127], 'magnitude': 2.120152473449707, 'distance': 12.513692855834961, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.5129856540705134, 'motion_component': -1.0876078009618537}, {'ion': 1340, 'force': [-0.07977347075939178, -0.7151584625244141, -1.4344524145126343], 'magnitude': 1.604826807975769, 'distance': 14.38318157196045, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.0072862170865083615, 'motion_component': 0.011693116688635014}, {'ion': 1341, 'force': [-14.652536392211914, -8.457913398742676, -4.700499534606934], 'magnitude': 17.55926513671875, 'distance': 4.348263740539551, 'before_closest_residue': 748, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': 0.7831130950979465, 'motion_component': 13.75089103791261}, {'ion': 1359, 'force': [-0.839736819267273, -1.8682215213775635, -0.06597363948822021], 'magnitude': 2.0493321418762207, 'distance': 12.728078842163086, 'before_closest_residue': 455, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': 0.3172573445902172, 'motion_component': 0.6501656636034504}, {'ion': 1400, 'force': [-0.20752248167991638, -2.0892179012298584, -2.092916488647461], 'magnitude': 2.964489221572876, 'distance': 10.5826416015625, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.0013031289237940694, 'motion_component': 0.0038631116715133196}]}, 6722: {'frame': 6722, 'ionic_force': [-6.684693541377783, -13.338738977909088, -3.4362437948584557], 'ionic_force_magnitude': 15.310612550797314, 'motion_vector': [1.3387413024902344, 0.14303207397460938, 0.6805572509765625], 'cosine_ionic_motion': -0.5712972196657156, 'ionic_motion_component': -8.746910381649515, 'ionic_force_x': -6.684693541377783, 'ionic_force_y': -13.338738977909088, 'ionic_force_z': -3.4362437948584557, 'radial_force': 14.920022964557695, 'axial_force': -3.4362437948584557, 'before_closest_residue': 780, 'closest_residue': 1105, 'next_closest_residue': 780, 'contributions': [{'ion': 1327, 'force': [0.81926029920578, -2.1865475177764893, -0.4886828362941742], 'magnitude': 2.3855793476104736, 'distance': 11.797014236450195, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.12544369478288375, 'motion_component': 0.2992558764165798}, {'ion': 1330, 'force': [0.03506458178162575, -1.515844464302063, 0.15978533029556274], 'magnitude': 1.5246459245681763, 'distance': 14.756539344787598, 'before_closest_residue': 130, 'closest_residue': 130, 'next_closest_residue': 98, 'cosine_with_motion': -0.026577021145496933, 'motion_component': -0.04052054803409777}, {'ion': 1340, 'force': [-0.26287201046943665, -0.7818873524665833, -1.5102778673171997], 'magnitude': 1.7208685874938965, 'distance': 13.889774322509766, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5745508499662869, 'motion_component': -0.9887265207963449}, {'ion': 1341, 'force': [-5.845895767211914, -5.08392858505249, 0.5223320126533508], 'magnitude': 7.764898777008057, 'distance': 6.538846492767334, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.699828776593821, 'motion_component': -5.434099831997331}, {'ion': 1359, 'force': [-0.7654677033424377, -1.5446780920028687, -0.07922738045454025], 'magnitude': 1.7257601022720337, 'distance': 13.870075225830078, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.49918877829101976, 'motion_component': -0.8614801146791009}, {'ion': 1400, 'force': [-0.6647829413414001, -2.2258529663085938, -2.040173053741455], 'magnitude': 3.0917088985443115, 'distance': 10.362624168395996, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.5567597574552943, 'motion_component': -1.7213390931081953}]}, 6723: {'frame': 6723, 'ionic_force': [-0.5762564726173878, -13.915500342845917, 1.1806349530816078], 'ionic_force_magnitude': 13.977378874682344, 'motion_vector': [-0.162322998046875, 2.1346893310546875, 1.369384765625], 'cosine_ionic_motion': -0.7881157162106749, 'ionic_motion_component': -11.015791962568233, 'ionic_force_x': -0.5762564726173878, 'ionic_force_y': -13.915500342845917, 'ionic_force_z': 1.1806349530816078, 'radial_force': 13.92742694520342, 'axial_force': 1.1806349530816078, 'before_closest_residue': 1105, 'closest_residue': 780, 'next_closest_residue': 748, 'contributions': [{'ion': 1327, 'force': [0.9342626333236694, -2.013418436050415, -0.30056488513946533], 'magnitude': 2.239874839782715, 'distance': 12.17466926574707, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.8540059906302656, 'motion_component': -1.9128666113018717}, {'ion': 1340, 'force': [-0.046403419226408005, -0.8943821787834167, -1.6315449476242065], 'magnitude': 1.8611855506896973, 'distance': 13.355932235717773, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.8744132028960275, 'motion_component': -1.627445223510299}, {'ion': 1341, 'force': [-0.5979642868041992, -6.457273483276367, 5.619952201843262], 'magnitude': 8.581247329711914, 'distance': 6.2200493812561035, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.27473154144593465, 'motion_component': -2.357539292708914}, {'ion': 1359, 'force': [-0.7437009215354919, -1.8613765239715576, 0.03603336960077286], 'magnitude': 2.004772424697876, 'distance': 12.868754386901855, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.7465211391778789, 'motion_component': -1.4966049111608775}, {'ion': 1400, 'force': [-0.12245047837495804, -2.68904972076416, -2.543240785598755], 'magnitude': 3.703249454498291, 'distance': 9.46842098236084, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.9778807589389066, 'motion_component': -3.6213363463983046}]}, 6724: {'frame': 6724, 'ionic_force': [-4.113540753722191, -15.694007277488708, 7.197184890508652], 'ionic_force_magnitude': 17.748874677189196, 'motion_vector': [-0.3926811218261719, -2.1882896423339844, -1.7566070556640625], 'cosine_ionic_motion': 0.4636191203107351, 'ionic_motion_component': 8.228717664343938, 'ionic_force_x': -4.113540753722191, 'ionic_force_y': -15.694007277488708, 'ionic_force_z': 7.197184890508652, 'radial_force': 16.224151193772876, 'axial_force': 7.197184890508652, 'before_closest_residue': 780, 'closest_residue': 748, 'next_closest_residue': 780, 'contributions': [{'ion': 1327, 'force': [1.648600697517395, -2.8385839462280273, -0.17031431198120117], 'magnitude': 3.2870123386383057, 'distance': 10.050053596496582, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.6295567558755207, 'motion_component': 2.0693608177461815}, {'ion': 1330, 'force': [0.29793596267700195, -1.9125956296920776, 0.4574536681175232], 'magnitude': 1.9889825582504272, 'distance': 12.919733047485352, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.579298938670601, 'motion_component': 1.1522155027986862}, {'ion': 1340, 'force': [-0.16771666705608368, -1.0057437419891357, -2.1990678310394287], 'magnitude': 2.423953056335449, 'distance': 11.703262329101562, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.892467519191024, 'motion_component': 2.163299418899779}, {'ion': 1341, 'force': [-4.0101213455200195, -2.7143781185150146, 13.681194305419922], 'magnitude': 14.512890815734863, 'distance': 4.7829084396362305, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.40168469073769564, 'motion_component': -5.829606053067735}, {'ion': 1359, 'force': [-1.2397171258926392, -2.3678460121154785, 0.34243646264076233], 'magnitude': 2.6945974826812744, 'distance': 11.099977493286133, 'before_closest_residue': 423, 'closest_residue': 423, 'next_closest_residue': 455, 'cosine_with_motion': 0.6636283776503213, 'motion_component': 1.7882114083837164}, {'ion': 1400, 'force': [-0.6425222754478455, -4.854859828948975, -4.914517402648926], 'magnitude': 6.9379377365112305, 'distance': 6.917574405670166, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.9924039216805082, 'motion_component': 6.885236625128063}]}, 6725: {'frame': 6725, 'ionic_force': [-2.6017091274261475, -10.550699710845947, -2.3864916190505028], 'ionic_force_magnitude': 11.125713326343421, 'motion_vector': [-0.458587646484375, 0.23482513427734375, -0.8922119140625], 'cosine_ionic_motion': 0.07370004659283276, 'ionic_motion_component': 0.8199655905300105, 'ionic_force_x': -2.6017091274261475, 'ionic_force_y': -10.550699710845947, 'ionic_force_z': -2.3864916190505028, 'radial_force': 10.866745362443039, 'axial_force': -2.3864916190505028, 'before_closest_residue': 748, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1327, 'force': [1.0887424945831299, -2.387108087539673, -0.3622821271419525], 'magnitude': 2.648564338684082, 'distance': 11.196022987365723, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.2699394138825094, 'motion_component': -0.7149519319481872}, {'ion': 1340, 'force': [-0.1545937955379486, -0.8115612268447876, -1.4531803131103516], 'magnitude': 1.671605110168457, 'distance': 14.0929594039917, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.683337593691137, 'motion_component': 1.1422706635808932}, {'ion': 1341, 'force': [-2.5049638748168945, -3.5627336502075195, 1.4722782373428345], 'magnitude': 4.5973381996154785, 'distance': 8.497982025146484, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'cosine_with_motion': -0.21143109657537829, 'motion_component': -0.9720202514220446}, {'ion': 1359, 'force': [-0.7145503759384155, -1.7946149110794067, 0.0394371822476387], 'magnitude': 1.9320404529571533, 'distance': 13.108739852905273, 'before_closest_residue': 423, 'closest_residue': 455, 'next_closest_residue': 423, 'cosine_with_motion': -0.06476746148457564, 'motion_component': -0.1251333539189594}, {'ion': 1400, 'force': [-0.3163435757160187, -1.9946818351745605, -2.082744598388672], 'magnitude': 2.9011471271514893, 'distance': 10.697546005249023, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': 0.5135211624013504, 'motion_component': 1.489800382213538}]}, 6726: {'frame': 6726, 'ionic_force': [-10.6773931235075, -23.184772670269012, 0.8381237238645554], 'ionic_force_magnitude': 25.539045774313546, 'motion_vector': [1.3153266906738281, 2.5401535034179688, 0.22161865234375], 'cosine_ionic_motion': -0.9928761766499101, 'ionic_motion_component': -25.357110123687477, 'ionic_force_x': -10.6773931235075, 'ionic_force_y': -23.184772670269012, 'ionic_force_z': 0.8381237238645554, 'radial_force': 25.525289571050475, 'axial_force': 0.8381237238645554, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1327, 'force': [0.9742769598960876, -2.260103225708008, -0.6310176849365234], 'magnitude': 2.5407607555389404, 'distance': 11.431077003479004, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.6309460379872143, 'motion_component': -1.6030829678477687}, {'ion': 1330, 'force': [0.2411656379699707, -1.9719339609146118, -0.08398731797933578], 'magnitude': 1.988400936126709, 'distance': 12.921623229980469, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 98, 'cosine_with_motion': -0.8256838071159796, 'motion_component': -1.6417904545858815}, {'ion': 1340, 'force': [-0.16953469812870026, -0.6895309090614319, -1.4364378452301025], 'magnitude': 1.602357268333435, 'distance': 14.394261360168457, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.49874044444684573, 'motion_component': -0.7991603382369856}, {'ion': 1341, 'force': [-10.608416557312012, -15.084050178527832, 5.144473552703857], 'magnitude': 19.145042419433594, 'distance': 4.1642889976501465, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 130, 'cosine_with_motion': -0.9308319385126406, 'motion_component': -17.82081769047824}, {'ion': 1359, 'force': [-0.709636926651001, -1.48970365524292, -0.056744806468486786], 'magnitude': 1.651066780090332, 'distance': 14.180342674255371, 'before_closest_residue': 455, 'closest_residue': 423, 'next_closest_residue': 455, 'cosine_with_motion': -0.9985275776246425, 'motion_component': -1.6486357150974915}, {'ion': 1400, 'force': [-0.4052475392818451, -1.689450740814209, -2.0981621742248535], 'magnitude': 2.7241060733795166, 'distance': 11.039693832397461, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.6767809384082066, 'motion_component': -1.8436230626847667}]}, 6727: {'frame': 6727, 'ionic_force': [0.19401593878865242, -14.893805980682373, -1.1919869855046272], 'ionic_force_magnitude': 14.942688237004964, 'motion_vector': [1.3554725646972656, -0.12535858154296875, 0.22263336181640625], 'cosine_ionic_motion': 0.09046944261007141, 'ionic_motion_component': 1.3518566758979096, 'ionic_force_x': 0.19401593878865242, 'ionic_force_y': -14.893805980682373, 'ionic_force_z': -1.1919869855046272, 'radial_force': 14.895069612952941, 'axial_force': -1.1919869855046272, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1327, 'force': [1.8957453966140747, -2.660691499710083, -0.9064189195632935], 'magnitude': 3.3903872966766357, 'distance': 9.895651817321777, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.5776475934913463, 'motion_component': 1.9584489864026418}, {'ion': 1330, 'force': [0.34051114320755005, -2.0693624019622803, 0.12192656844854355], 'magnitude': 2.1007320880889893, 'distance': 12.571402549743652, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 130, 'cosine_with_motion': 0.25818029144636306, 'motion_component': 0.5423675841303569}, {'ion': 1340, 'force': [-0.058663200587034225, -0.5451574325561523, -1.6288467645645142], 'magnitude': 1.7186564207077026, 'distance': 13.898711204528809, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.15768551440409598, 'motion_component': -0.2710072166161883}, {'ion': 1341, 'force': [0.5644397139549255, -4.903802871704102, 4.149296760559082], 'magnitude': 6.448452472686768, 'distance': 7.175320148468018, 'before_closest_residue': 780, 'closest_residue': 130, 'next_closest_residue': None, 'cosine_with_motion': 0.25898652222747937, 'motion_component': 1.670062261776156}, {'ion': 1359, 'force': [-2.4074673652648926, -2.86397123336792, 0.0936751663684845], 'magnitude': 3.74259352684021, 'distance': 9.4185209274292, 'before_closest_residue': 423, 'closest_residue': 455, 'next_closest_residue': 455, 'cosine_with_motion': -0.5585430643324164, 'motion_component': -2.0903995876372625}, {'ion': 1400, 'force': [-0.14054974913597107, -1.850820541381836, -3.0216197967529297], 'magnitude': 3.546191930770874, 'distance': 9.675823211669922, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.12904417269620683, 'motion_component': -0.4576154020114362}]}, 6728: {'frame': 6728, 'ionic_force': [2.4772856384515762, -9.180882215499878, -5.546252489089966], 'ionic_force_magnitude': 11.008472149308323, 'motion_vector': [-2.3235855102539062, 0.4115257263183594, -0.305999755859375], 'cosine_ionic_motion': -0.2991903473440756, 'ionic_motion_component': -3.2936286060791398, 'ionic_force_x': 2.4772856384515762, 'ionic_force_y': -9.180882215499878, 'ionic_force_z': -5.546252489089966, 'radial_force': 9.509234584831756, 'axial_force': -5.546252489089966, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 780, 'contributions': [{'ion': 1327, 'force': [1.678908109664917, -2.0583689212799072, -0.4516320526599884], 'magnitude': 2.694361925125122, 'distance': 11.100461959838867, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': -0.7190427304193472, 'motion_component': -1.9373614066475815}, {'ion': 1330, 'force': [0.7343488931655884, -2.256716251373291, 0.1098492443561554], 'magnitude': 2.375732183456421, 'distance': 11.82143783569336, 'before_closest_residue': 98, 'closest_residue': 130, 'next_closest_residue': 98, 'cosine_with_motion': -0.47206843757298744, 'motion_component': -1.121508178453884}, {'ion': 1340, 'force': [0.15440182387828827, -0.5537362098693848, -1.7548797130584717], 'magnitude': 1.8466365337371826, 'distance': 13.408442497253418, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.011299252569514797, 'motion_component': -0.020865612699471292}, {'ion': 1359, 'force': [-0.4944912791252136, -2.2753615379333496, -0.14022064208984375], 'magnitude': 2.3326923847198486, 'distance': 11.929996490478516, 'before_closest_residue': 455, 'closest_residue': 455, 'next_closest_residue': 423, 'cosine_with_motion': 0.046036121737723396, 'motion_component': 0.10738810882518735}, {'ion': 1400, 'force': [0.4041180908679962, -2.0366992950439453, -3.3093693256378174], 'magnitude': 3.9068377017974854, 'distance': 9.218417167663574, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.08223573214076878, 'motion_component': -0.3212816582897684}]}, 6729: {'frame': 6729, 'ionic_force': [-0.1381404548883438, -10.870651245117188, -5.780998591333628], 'ionic_force_magnitude': 12.313004750719704, 'motion_vector': [6.845603942871094, -0.24485015869140625, 2.0646591186523438], 'cosine_ionic_motion': -0.1160126295562164, 'ionic_motion_component': -1.4284640588691777, 'ionic_force_x': -0.1381404548883438, 'ionic_force_y': -10.870651245117188, 'ionic_force_z': -5.780998591333628, 'radial_force': 10.871528930111193, 'axial_force': -5.780998591333628, 'before_closest_residue': 780, 'closest_residue': 780, 'next_closest_residue': 748, 'contributions': [{'ion': 1327, 'force': [1.820922613143921, -3.5445034503936768, -0.7323452830314636], 'magnitude': 4.051616191864014, 'distance': 9.052215576171875, 'before_closest_residue': 98, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.40781161798980436, 'motion_component': 1.652296140602055}, {'ion': 1330, 'force': [0.3618646562099457, -3.046487808227539, -0.05099794641137123], 'magnitude': 3.0683276653289795, 'distance': 10.402031898498535, 'before_closest_residue': 130, 'closest_residue': 98, 'next_closest_residue': 98, 'cosine_with_motion': 0.14202929470439557, 'motion_component': 0.43579241709412253}, {'ion': 1340, 'force': [-0.1966351717710495, -0.5052287578582764, -1.6221227645874023], 'magnitude': 1.7103227376937866, 'distance': 13.932531356811523, 'before_closest_residue': None, 'closest_residue': None, 'next_closest_residue': None, 'cosine_with_motion': -0.37360282117611954, 'motion_component': -0.638981387348994}, {'ion': 1359, 'force': [-1.4620943069458008, -2.0969743728637695, -0.17865630984306335], 'magnitude': 2.5626041889190674, 'distance': 11.382254600524902, 'before_closest_residue': 455, 'closest_residue': 423, 'next_closest_residue': 423, 'cosine_with_motion': -0.5380403441470379, 'motion_component': -1.3787843484740705}, {'ion': 1400, 'force': [-0.66219824552</t>
         </is>
       </c>
     </row>

</xml_diff>